<commit_message>
Refresh: 2026-08-23 06:00 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -365,8 +365,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblWeather" displayName="tblWeather" ref="A4:J38" headerRowCount="1">
-  <autoFilter ref="A4:J38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblWeather" displayName="tblWeather" ref="A4:J37" headerRowCount="1">
+  <autoFilter ref="A4:J37"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Game id"/>
     <tableColumn id="2" name="Venue"/>
@@ -689,7 +689,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-23T04:20:20+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-23T06:00:13+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23T04:20:20+00:00</t>
+          <t>2026-08-23T06:00:13+00:00</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3628,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3638,23 +3638,23 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>DAL -2.5</t>
+          <t>PIT -3</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.5101</v>
+        <v>0.5097</v>
       </c>
       <c r="G31" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>-0.0134</v>
+        <v>-0.0138</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>-0.02613350288850708</v>
+        <v>-0.0250340463292979</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0.5</v>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -3679,23 +3679,23 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>PIT -3</t>
+          <t>DAL -2.5</t>
         </is>
       </c>
       <c r="E32" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5097</v>
+        <v>0.5094</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>-0.0138</v>
+        <v>-0.0141</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>-0.0250340463292979</v>
+        <v>-0.0275104067761156</v>
       </c>
       <c r="J32" s="14" t="n">
         <v>0.5</v>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -4212,23 +4212,23 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>ATL +3</t>
+          <t>NYG +2.5</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.4903</v>
+        <v>0.4906</v>
       </c>
       <c r="G45" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>-0.0299</v>
+        <v>-0.0297</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>-0.05931477362409254</v>
+        <v>-0.06339868413297528</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>0.5</v>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -4253,23 +4253,23 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>NYG +2.5</t>
+          <t>ATL +3</t>
         </is>
       </c>
       <c r="E46" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4899</v>
+        <v>0.4903</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H46" s="13" t="n">
-        <v>-0.0302</v>
+        <v>-0.0299</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>-0.06477558802058375</v>
+        <v>-0.05931477362409254</v>
       </c>
       <c r="J46" s="14" t="n">
         <v>0.5</v>
@@ -6036,7 +6036,7 @@
         </is>
       </c>
       <c r="D9" s="22" t="n">
-        <v>-2.43</v>
+        <v>-2.39</v>
       </c>
       <c r="E9" s="22" t="n">
         <v>2.5</v>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D22" s="18" t="n">
         <v>-0.07000000000000001</v>
@@ -7270,7 +7270,7 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D23" s="16" t="n">
         <v>-0.34</v>
@@ -7302,7 +7302,7 @@
         </is>
       </c>
       <c r="C24" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24" s="18" t="n">
         <v>-0.47</v>
@@ -7334,7 +7334,7 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25" s="16" t="n">
         <v>-0.65</v>
@@ -7366,7 +7366,7 @@
         </is>
       </c>
       <c r="C26" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D26" s="18" t="n">
         <v>-0.8100000000000001</v>
@@ -7398,7 +7398,7 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D27" s="16" t="n">
         <v>-1.39</v>
@@ -7430,7 +7430,7 @@
         </is>
       </c>
       <c r="C28" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="18" t="n">
         <v>-1.86</v>
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D29" s="16" t="n">
         <v>-2</v>
@@ -7494,7 +7494,7 @@
         </is>
       </c>
       <c r="C30" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D30" s="18" t="n">
         <v>-2.32</v>
@@ -7526,7 +7526,7 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D31" s="16" t="n">
         <v>-2.63</v>
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="C32" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D32" s="18" t="n">
         <v>-3.17</v>
@@ -7590,7 +7590,7 @@
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D33" s="16" t="n">
         <v>-3.24</v>
@@ -7622,7 +7622,7 @@
         </is>
       </c>
       <c r="C34" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D34" s="18" t="n">
         <v>-3.76</v>
@@ -7654,7 +7654,7 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D35" s="16" t="n">
         <v>-4.7</v>
@@ -7686,7 +7686,7 @@
         </is>
       </c>
       <c r="C36" s="12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D36" s="18" t="n">
         <v>-5.61</v>
@@ -9250,14 +9250,14 @@
       <c r="I36" s="12" t="n"/>
       <c r="J36" s="12" t="n"/>
       <c r="K36" s="17" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="L36" s="17" t="n">
         <v>13</v>
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>13:59 - 4th</t>
+          <t>Final</t>
         </is>
       </c>
     </row>
@@ -27924,12 +27924,12 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>Rome Odunze</t>
+          <t>Cairo Santos</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D130" s="5" t="inlineStr">
@@ -27944,7 +27944,7 @@
       </c>
       <c r="F130" s="5" t="inlineStr">
         <is>
-          <t>Odunze brought in one of two targets for 18 yards in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
+          <t>Santos connected on field-goal attempts of 45, 26 and 44 yards and missed wide right from 53 yards in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
         </is>
       </c>
     </row>
@@ -27956,7 +27956,7 @@
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Colston Loveland</t>
+          <t>Sam Roush</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
@@ -27976,7 +27976,7 @@
       </c>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>Loveland brought in one of three targets for 10 yards in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
+          <t>Roush brought in two of three targets for 30 yards in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
         </is>
       </c>
     </row>
@@ -27988,12 +27988,12 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>Caleb Williams</t>
+          <t>Rome Odunze</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D132" s="5" t="inlineStr">
@@ -28008,7 +28008,7 @@
       </c>
       <c r="F132" s="5" t="inlineStr">
         <is>
-          <t>Williams completed two of five passes for 28 yards with no touchdowns or interceptions in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
+          <t>Odunze brought in one of two targets for 18 yards in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
         </is>
       </c>
     </row>
@@ -28020,27 +28020,27 @@
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>Tyrique Stevenson</t>
+          <t>Colston Loveland</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>Stevenson (undisclosed) returned to practice Thursday following a week-long absence, Brad Biggs of the Chicago Tribune reports.</t>
+          <t>Loveland brought in one of three targets for 10 yards in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
         </is>
       </c>
     </row>
@@ -28052,7 +28052,7 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Tyson Bagent</t>
+          <t>Caleb Williams</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
@@ -28062,17 +28062,17 @@
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>Bagent is still dealing with a hamstring injury and did not join the team on its trip to Cincinnati for a preseason game this Saturday, Courtney Cronin of ESPN.com reports.</t>
+          <t>Williams completed two of five passes for 28 yards with no touchdowns or interceptions in the Bears' 27-9 preseason loss to the Bengals on Saturday.</t>
         </is>
       </c>
     </row>
@@ -28084,12 +28084,12 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>Xavier Woods</t>
+          <t>Tyrique Stevenson</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="F135" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Stevenson (undisclosed) returned to practice Thursday following a week-long absence, Brad Biggs of the Chicago Tribune reports.</t>
         </is>
       </c>
     </row>
@@ -28116,12 +28116,12 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>Nephi Sewell</t>
+          <t>Tyson Bagent</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
@@ -28131,12 +28131,12 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t>Concussion</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F136" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Bagent is still dealing with a hamstring injury and did not join the team on its trip to Cincinnati for a preseason game this Saturday, Courtney Cronin of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -28148,12 +28148,12 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Ruben Hyppolite II</t>
+          <t>Xavier Woods</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
@@ -28180,27 +28180,27 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>Nikola Kalinic</t>
+          <t>Nephi Sewell</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D138" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Concussion</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -28212,27 +28212,27 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>Coby Bryant</t>
+          <t>Ruben Hyppolite II</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F139" s="4" t="inlineStr">
         <is>
-          <t>out</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -28244,17 +28244,17 @@
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>Luther Burden III</t>
+          <t>Nikola Kalinic</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D140" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E140" s="5" t="inlineStr">
@@ -28264,7 +28264,7 @@
       </c>
       <c r="F140" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -28276,27 +28276,27 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>Dallis Flowers</t>
+          <t>Coby Bryant</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F141" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>out</t>
         </is>
       </c>
     </row>
@@ -28308,17 +28308,17 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>Jonathan Garvin</t>
+          <t>Luther Burden III</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
@@ -28328,7 +28328,7 @@
       </c>
       <c r="F142" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -28340,25 +28340,29 @@
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Ozzy Trapilo</t>
+          <t>Dallis Flowers</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F143" s="4" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F143" s="4" t="inlineStr">
+        <is>
+          <t>ir</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -28368,7 +28372,7 @@
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>Dayo Odeyingbo</t>
+          <t>Jonathan Garvin</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr">
@@ -28378,15 +28382,19 @@
       </c>
       <c r="D144" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F144" s="5" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>ir</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -28396,12 +28404,12 @@
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>Zavion Thomas</t>
+          <t>Ozzy Trapilo</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
@@ -28414,11 +28422,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F145" s="4" t="inlineStr">
-        <is>
-          <t>Thomas (knee) was a full participant in Tuesday's practice, Brad Biggs of the Chicago Tribune reports.</t>
-        </is>
-      </c>
+      <c r="F145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -28428,29 +28432,25 @@
       </c>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>Kyle Monangai</t>
+          <t>Dayo Odeyingbo</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D146" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="F146" s="5" t="inlineStr">
-        <is>
-          <t>Monangai (knee) is considered week-to-week, Adam Jahns of AllCHGO.com reports.</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -28460,12 +28460,12 @@
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Marcus Davenport</t>
+          <t>Zavion Thomas</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
@@ -28480,7 +28480,7 @@
       </c>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>The Bears signed Davenport to a contract Monday, NFL reporter Jordan Schultz reports.</t>
+          <t>Thomas (knee) was a full participant in Tuesday's practice, Brad Biggs of the Chicago Tribune reports.</t>
         </is>
       </c>
     </row>
@@ -28492,7 +28492,7 @@
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>Salvon Ahmed</t>
+          <t>Kyle Monangai</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
@@ -28502,17 +28502,17 @@
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
         <is>
-          <t>Ahmed was among the Bears' top performers in Saturday's 34-10 preseason win over the Browns, which was highlighted by his 49-yard touchdown catch, Courtney Cronin of ESPN.com reports.</t>
+          <t>Monangai (knee) is considered week-to-week, Adam Jahns of AllCHGO.com reports.</t>
         </is>
       </c>
     </row>
@@ -28524,12 +28524,12 @@
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Braxton Jones</t>
+          <t>Marcus Davenport</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -28544,7 +28544,7 @@
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>Jones (knee) returned to practice Sunday, Adam Hoge of AllCHGO.com reports.</t>
+          <t>The Bears signed Davenport to a contract Monday, NFL reporter Jordan Schultz reports.</t>
         </is>
       </c>
     </row>
@@ -28556,12 +28556,12 @@
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>Cam Lewis</t>
+          <t>Salvon Ahmed</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D150" s="5" t="inlineStr">
@@ -28576,7 +28576,7 @@
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
-          <t>Lewis made one tackle assist during Saturday's preseason opener against the Browns.</t>
+          <t>Ahmed was among the Bears' top performers in Saturday's 34-10 preseason win over the Browns, which was highlighted by his 49-yard touchdown catch, Courtney Cronin of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -28588,12 +28588,12 @@
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Montez Sweat</t>
+          <t>Braxton Jones</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
@@ -28608,7 +28608,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>Sweat (undisclosed) was a full participant in Sunday's practice, Adam Hoge of AllCHGO.com reports.</t>
+          <t>Jones (knee) returned to practice Sunday, Adam Hoge of AllCHGO.com reports.</t>
         </is>
       </c>
     </row>
@@ -28620,7 +28620,7 @@
       </c>
       <c r="B152" s="5" t="inlineStr">
         <is>
-          <t>Kyler Gordon</t>
+          <t>Cam Lewis</t>
         </is>
       </c>
       <c r="C152" s="5" t="inlineStr">
@@ -28630,17 +28630,17 @@
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F152" s="5" t="inlineStr">
         <is>
-          <t>Bears coach Ben Johnson said Saturday that Gordon's timeline to return to practice from his calf injury is "unknown," Courtney Cronin of ESPN.com reports.</t>
+          <t>Lewis made one tackle assist during Saturday's preseason opener against the Browns.</t>
         </is>
       </c>
     </row>
@@ -28652,12 +28652,12 @@
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>D'Andre Swift</t>
+          <t>Montez Sweat</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
@@ -28672,7 +28672,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>Swift has been one of the brightest stars of training camp for the Bears, Courtney Cronin of ESPN.com reports.</t>
+          <t>Sweat (undisclosed) was a full participant in Sunday's practice, Adam Hoge of AllCHGO.com reports.</t>
         </is>
       </c>
     </row>
@@ -28684,27 +28684,27 @@
       </c>
       <c r="B154" s="5" t="inlineStr">
         <is>
-          <t>Jahdae Walker</t>
+          <t>Kyler Gordon</t>
         </is>
       </c>
       <c r="C154" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D154" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F154" s="5" t="inlineStr">
         <is>
-          <t>Walker was listed as a second-string wide receiver on the Bears' first unofficial depth chart that was released Tuesday, Kevin Fishbain of The Athletic reports.</t>
+          <t>Bears coach Ben Johnson said Saturday that Gordon's timeline to return to practice from his calf injury is "unknown," Courtney Cronin of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -28716,12 +28716,12 @@
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Joe Burrow</t>
+          <t>Evan McPherson</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
@@ -28736,7 +28736,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>Bengals head coach Zac Taylor said that Burrow and other key starters are in line to be rested for Saturday's preseason game against the Bears, Jay Morrison of SI.com reports.</t>
+          <t>McPherson connected on field-goal attempts of 25 and 58 yards while also knocking home all three PATs in the Bengals' 27-9 preseason win over the Bears on Saturday.</t>
         </is>
       </c>
     </row>
@@ -28748,27 +28748,27 @@
       </c>
       <c r="B156" s="5" t="inlineStr">
         <is>
-          <t>Myles Murphy</t>
+          <t>Colbie Young</t>
         </is>
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E156" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F156" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Young brought in three of eight targets for 48 yards and a touchdown in the Bengals' 27-9 preseason win over the Bears on Saturday.</t>
         </is>
       </c>
     </row>
@@ -28780,27 +28780,27 @@
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Dax Hill</t>
+          <t>Joe Burrow</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>Soreness</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Bengals head coach Zac Taylor said that Burrow and other key starters are in line to be rested for Saturday's preseason game against the Bears, Jay Morrison of SI.com reports.</t>
         </is>
       </c>
     </row>
@@ -28812,12 +28812,12 @@
       </c>
       <c r="B158" s="5" t="inlineStr">
         <is>
-          <t>McKinnley Jackson</t>
+          <t>Myles Murphy</t>
         </is>
       </c>
       <c r="C158" s="5" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D158" s="5" t="inlineStr">
@@ -28844,25 +28844,29 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Josh Kattus</t>
+          <t>Dax Hill</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F159" s="4" t="inlineStr"/>
+          <t>Soreness</t>
+        </is>
+      </c>
+      <c r="F159" s="4" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="5" t="inlineStr">
@@ -28872,12 +28876,12 @@
       </c>
       <c r="B160" s="5" t="inlineStr">
         <is>
-          <t>Bryan Cook</t>
+          <t>McKinnley Jackson</t>
         </is>
       </c>
       <c r="C160" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D160" s="5" t="inlineStr">
@@ -28904,12 +28908,12 @@
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Kris Jenkins Jr.</t>
+          <t>Josh Kattus</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
@@ -28932,25 +28936,29 @@
       </c>
       <c r="B162" s="5" t="inlineStr">
         <is>
-          <t>Cam Grandy</t>
+          <t>Bryan Cook</t>
         </is>
       </c>
       <c r="C162" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D162" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F162" s="5" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -28960,12 +28968,12 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Jack Endries</t>
+          <t>Kris Jenkins Jr.</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
@@ -28978,11 +28986,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F163" s="4" t="inlineStr">
-        <is>
-          <t>Endries caught a 17-yard touchdown reception from Joe Flacco in Thursday's preseason opener against the Lions. He's competing with veteran Tanner Hudson for a roster spot, Geoff Hobson of Bengals.com reports.</t>
-        </is>
-      </c>
+      <c r="F163" s="4" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="inlineStr">
@@ -28992,12 +28996,12 @@
       </c>
       <c r="B164" s="5" t="inlineStr">
         <is>
-          <t>B.J. Hill</t>
+          <t>Cam Grandy</t>
         </is>
       </c>
       <c r="C164" s="5" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D164" s="5" t="inlineStr">
@@ -29010,11 +29014,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F164" s="5" t="inlineStr">
-        <is>
-          <t>The Bengals activated Hill (undisclosed) from the active/PUP list Saturday after he passed a physical.</t>
-        </is>
-      </c>
+      <c r="F164" s="5" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -29024,12 +29024,12 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Colbie Young</t>
+          <t>Jack Endries</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D165" s="4" t="inlineStr">
@@ -29044,7 +29044,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>Young caught two of four targets for 28 yards in Thursday's 16-14 preseason win over the Lions.</t>
+          <t>Endries caught a 17-yard touchdown reception from Joe Flacco in Thursday's preseason opener against the Lions. He's competing with veteran Tanner Hudson for a roster spot, Geoff Hobson of Bengals.com reports.</t>
         </is>
       </c>
     </row>
@@ -29056,12 +29056,12 @@
       </c>
       <c r="B166" s="5" t="inlineStr">
         <is>
-          <t>Mike Gesicki</t>
+          <t>B.J. Hill</t>
         </is>
       </c>
       <c r="C166" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D166" s="5" t="inlineStr">
@@ -29076,7 +29076,7 @@
       </c>
       <c r="F166" s="5" t="inlineStr">
         <is>
-          <t>Gesicki didn't catch his only target in Thursday's 16-14 preseason win over the Lions.</t>
+          <t>The Bengals activated Hill (undisclosed) from the active/PUP list Saturday after he passed a physical.</t>
         </is>
       </c>
     </row>
@@ -29088,12 +29088,12 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Tee Higgins</t>
+          <t>Mike Gesicki</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
@@ -29108,7 +29108,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>Higgins and quarterback Joe Burrow have had no trouble connecting at practice, Dan Hoard of the Bengals' official website reports.</t>
+          <t>Gesicki didn't catch his only target in Thursday's 16-14 preseason win over the Lions.</t>
         </is>
       </c>
     </row>
@@ -29120,12 +29120,12 @@
       </c>
       <c r="B168" s="5" t="inlineStr">
         <is>
-          <t>Chase Brown</t>
+          <t>Tee Higgins</t>
         </is>
       </c>
       <c r="C168" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D168" s="5" t="inlineStr">
@@ -29140,7 +29140,7 @@
       </c>
       <c r="F168" s="5" t="inlineStr">
         <is>
-          <t>Brown rushed five times for 16 yards in Thursday's preseason-opening 16-14 win over the Lions.</t>
+          <t>Higgins and quarterback Joe Burrow have had no trouble connecting at practice, Dan Hoard of the Bengals' official website reports.</t>
         </is>
       </c>
     </row>
@@ -29152,12 +29152,12 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Ja'Marr Chase</t>
+          <t>Chase Brown</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
@@ -29172,7 +29172,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>Chase caught his only target for 16 yards in Thursday's preseason-opening 16-14 win over the Lions.</t>
+          <t>Brown rushed five times for 16 yards in Thursday's preseason-opening 16-14 win over the Lions.</t>
         </is>
       </c>
     </row>
@@ -29184,12 +29184,12 @@
       </c>
       <c r="B170" s="5" t="inlineStr">
         <is>
-          <t>Cashius Howell</t>
+          <t>Ja'Marr Chase</t>
         </is>
       </c>
       <c r="C170" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D170" s="5" t="inlineStr">
@@ -29204,7 +29204,7 @@
       </c>
       <c r="F170" s="5" t="inlineStr">
         <is>
-          <t>Howell has "been a monster in camp," particularly surprising the Bengals' coaching staff with his strength, Sports Illustrated's Albert Breer reports.</t>
+          <t>Chase caught his only target for 16 yards in Thursday's preseason-opening 16-14 win over the Lions.</t>
         </is>
       </c>
     </row>
@@ -29216,12 +29216,12 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Erick All Jr.</t>
+          <t>Cashius Howell</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
@@ -29236,7 +29236,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>All (knee) passed his conditioning test and is all set to participate in training camp, Dan Hoard of the Bengals' official site reports.</t>
+          <t>Howell has "been a monster in camp," particularly surprising the Bengals' coaching staff with his strength, Sports Illustrated's Albert Breer reports.</t>
         </is>
       </c>
     </row>
@@ -29248,12 +29248,12 @@
       </c>
       <c r="B172" s="5" t="inlineStr">
         <is>
-          <t>Jonathan Allen</t>
+          <t>Erick All Jr.</t>
         </is>
       </c>
       <c r="C172" s="5" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D172" s="5" t="inlineStr">
@@ -29266,7 +29266,11 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F172" s="5" t="inlineStr"/>
+      <c r="F172" s="5" t="inlineStr">
+        <is>
+          <t>All (knee) passed his conditioning test and is all set to participate in training camp, Dan Hoard of the Bengals' official site reports.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -29276,29 +29280,25 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Shemar Stewart</t>
+          <t>Jonathan Allen</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="F173" s="4" t="inlineStr">
-        <is>
-          <t>Stewart will miss several weeks due to a hyperextended knee, head coach Zac Taylor revealed Thursday, Charlie Goldsmith of FOX19 Cincinnati reports.</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="inlineStr">
@@ -29308,27 +29308,27 @@
       </c>
       <c r="B174" s="5" t="inlineStr">
         <is>
-          <t>Josh Newton</t>
+          <t>Shemar Stewart</t>
         </is>
       </c>
       <c r="C174" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D174" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F174" s="5" t="inlineStr">
         <is>
-          <t>Newton (hamstring) is expected to compete for the Bengals' starting cornerback role, Chris Roling of USA Today reports.</t>
+          <t>Stewart will miss several weeks due to a hyperextended knee, head coach Zac Taylor revealed Thursday, Charlie Goldsmith of FOX19 Cincinnati reports.</t>
         </is>
       </c>
     </row>
@@ -29340,12 +29340,12 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Connor Lew</t>
+          <t>Josh Newton</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
@@ -29360,7 +29360,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>Lew (knee) participated in Cincinnati's training camp Wednesday, Dan Hoard of the team's official site reports.</t>
+          <t>Newton (hamstring) is expected to compete for the Bengals' starting cornerback role, Chris Roling of USA Today reports.</t>
         </is>
       </c>
     </row>
@@ -29372,12 +29372,12 @@
       </c>
       <c r="B176" s="5" t="inlineStr">
         <is>
-          <t>DJ Turner II</t>
+          <t>Connor Lew</t>
         </is>
       </c>
       <c r="C176" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D176" s="5" t="inlineStr">
@@ -29392,7 +29392,7 @@
       </c>
       <c r="F176" s="5" t="inlineStr">
         <is>
-          <t>Turner (calf) was active in Wednesday's training camp practice, mixing it up with Ja'Marr Chase during 7-on-7 and 11-on-11 drills, Geoff Hobson of the Bengals' official site reports.</t>
+          <t>Lew (knee) participated in Cincinnati's training camp Wednesday, Dan Hoard of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -29404,12 +29404,12 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Charlie Jones</t>
+          <t>DJ Turner II</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
@@ -29424,7 +29424,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>Jones (ankle) is participating at the Bengals' training camp, Sam Greene and Jacob Sebastian of The Cincinnati Enquirer report.</t>
+          <t>Turner (calf) was active in Wednesday's training camp practice, mixing it up with Ja'Marr Chase during 7-on-7 and 11-on-11 drills, Geoff Hobson of the Bengals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -29436,12 +29436,12 @@
       </c>
       <c r="B178" s="5" t="inlineStr">
         <is>
-          <t>Tahj Brooks</t>
+          <t>Charlie Jones</t>
         </is>
       </c>
       <c r="C178" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D178" s="5" t="inlineStr">
@@ -29456,7 +29456,7 @@
       </c>
       <c r="F178" s="5" t="inlineStr">
         <is>
-          <t>Brooks will compete against Samaje Perine in training camp for the No. 2 running back role behind Chase Brown, Michael Hull of the Bengals' official site reports.</t>
+          <t>Jones (ankle) is participating at the Bengals' training camp, Sam Greene and Jacob Sebastian of The Cincinnati Enquirer report.</t>
         </is>
       </c>
     </row>
@@ -29468,12 +29468,12 @@
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>Evan McPherson</t>
+          <t>Tahj Brooks</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
@@ -29488,7 +29488,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>McPherson will again work as Cincinnati's primary kicker during the upcoming season following a bounce-back performance last year, John Sheeran of A to Z Sports reports.</t>
+          <t>Brooks will compete against Samaje Perine in training camp for the No. 2 running back role behind Chase Brown, Michael Hull of the Bengals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -30288,12 +30288,12 @@
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>Jaydon Blue</t>
+          <t>Joe Milton III</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -30306,7 +30306,11 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F205" s="4" t="inlineStr"/>
+      <c r="F205" s="4" t="inlineStr">
+        <is>
+          <t>Milton completed nine of 13 passes for 179 yards with two touchdowns and no interceptions and rushed three times for two yards and another score in the Cowboys' 34-13 preseason win over the Cardinals on Saturday.</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="5" t="inlineStr">
@@ -30316,27 +30320,27 @@
       </c>
       <c r="B206" s="5" t="inlineStr">
         <is>
-          <t>Zion Childress</t>
+          <t>Jaydon Blue</t>
         </is>
       </c>
       <c r="C206" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D206" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E206" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F206" s="5" t="inlineStr">
         <is>
-          <t>Childress (hamstring) returned to practice as a limited participant Thursday, Calvin Watkins of The Dallas Morning News reports.</t>
+          <t>Blue (shoulder) rushed 15 times for 75 yards in the Cowboys' 34-13 preseason win over the Cardinals on Saturday. He also returned one kickoff for 26 yards.</t>
         </is>
       </c>
     </row>
@@ -30348,27 +30352,27 @@
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>Michael Trigg</t>
+          <t>Malik Davis</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>Toe</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>Trigg (toe) did not practice Thursday, Tommy Yarrish of the Cowboys' official site reports.</t>
+          <t>Davis rushed five times for 29 yards and brought in his only target for an eight-yard touchdown in the Cowboys' 34-13 preseason win over the Cardinals on Saturday. He also committed a fumble but recovered and ran back one kickoff for 31 yards.</t>
         </is>
       </c>
     </row>
@@ -30380,12 +30384,12 @@
       </c>
       <c r="B208" s="5" t="inlineStr">
         <is>
-          <t>Tyler Guyton</t>
+          <t>Julius Wood</t>
         </is>
       </c>
       <c r="C208" s="5" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D208" s="5" t="inlineStr">
@@ -30395,12 +30399,12 @@
       </c>
       <c r="E208" s="5" t="inlineStr">
         <is>
-          <t>Soreness</t>
+          <t>Concussion</t>
         </is>
       </c>
       <c r="F208" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Wood has entered the league's concussion protocol and has been ruled out for the rest of Saturday's preseason game against the Cardinals, Patrik Walker of the Cowboys' official site reports.</t>
         </is>
       </c>
     </row>
@@ -30412,12 +30416,12 @@
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>Phil Mafah</t>
+          <t>Zion Childress</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
@@ -30432,7 +30436,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Childress (hamstring) returned to practice as a limited participant Thursday, Calvin Watkins of The Dallas Morning News reports.</t>
         </is>
       </c>
     </row>
@@ -30444,25 +30448,29 @@
       </c>
       <c r="B210" s="5" t="inlineStr">
         <is>
-          <t>Jalen Thompson</t>
+          <t>Michael Trigg</t>
         </is>
       </c>
       <c r="C210" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D210" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E210" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F210" s="5" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F210" s="5" t="inlineStr">
+        <is>
+          <t>Trigg (toe) did not practice Thursday, Tommy Yarrish of the Cowboys' official site reports.</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
@@ -30472,12 +30480,12 @@
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>Jonathan Bullard</t>
+          <t>Tyler Guyton</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr">
@@ -30504,27 +30512,27 @@
       </c>
       <c r="B212" s="5" t="inlineStr">
         <is>
-          <t>Princeton Fant</t>
+          <t>Phil Mafah</t>
         </is>
       </c>
       <c r="C212" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D212" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E212" s="5" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F212" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -30536,12 +30544,12 @@
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>Ajani Cornelius</t>
+          <t>Jalen Thompson</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr">
@@ -30564,25 +30572,29 @@
       </c>
       <c r="B214" s="5" t="inlineStr">
         <is>
-          <t>P.J. Locke</t>
+          <t>Jonathan Bullard</t>
         </is>
       </c>
       <c r="C214" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D214" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E214" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F214" s="5" t="inlineStr"/>
+          <t>Soreness</t>
+        </is>
+      </c>
+      <c r="F214" s="5" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -30592,25 +30604,29 @@
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>James Houston</t>
+          <t>Princeton Fant</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F215" s="4" t="inlineStr"/>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="F215" s="4" t="inlineStr">
+        <is>
+          <t>ir</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="5" t="inlineStr">
@@ -30620,12 +30636,12 @@
       </c>
       <c r="B216" s="5" t="inlineStr">
         <is>
-          <t>DeMarvion Overshown</t>
+          <t>Ajani Cornelius</t>
         </is>
       </c>
       <c r="C216" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D216" s="5" t="inlineStr">
@@ -30638,11 +30654,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F216" s="5" t="inlineStr">
-        <is>
-          <t>Overshown (lower body) participated at the Cowboys' training camp practice Monday, Todd Archer of ESPN.com reports.</t>
-        </is>
-      </c>
+      <c r="F216" s="5" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
@@ -30652,12 +30664,12 @@
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>Jaishawn Barham</t>
+          <t>P.J. Locke</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
@@ -30670,11 +30682,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F217" s="4" t="inlineStr">
-        <is>
-          <t>Barham (groin) returned to practice Monday, Todd Archer of ESPN.com reports.</t>
-        </is>
-      </c>
+      <c r="F217" s="4" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="5" t="inlineStr">
@@ -30684,7 +30692,7 @@
       </c>
       <c r="B218" s="5" t="inlineStr">
         <is>
-          <t>Von Miller</t>
+          <t>James Houston</t>
         </is>
       </c>
       <c r="C218" s="5" t="inlineStr">
@@ -30702,11 +30710,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F218" s="5" t="inlineStr">
-        <is>
-          <t>Miller is not expected to practice with the Cowboys this week, Calvin Watkins of The Dallas Morning News reports.</t>
-        </is>
-      </c>
+      <c r="F218" s="5" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
@@ -30716,12 +30720,12 @@
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>Alijah Clark</t>
+          <t>DeMarvion Overshown</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
@@ -30736,7 +30740,7 @@
       </c>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>Clark (ankle) recorded one tackle in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
+          <t>Overshown (lower body) participated at the Cowboys' training camp practice Monday, Todd Archer of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -30748,12 +30752,12 @@
       </c>
       <c r="B220" s="5" t="inlineStr">
         <is>
-          <t>Camden Brown</t>
+          <t>Jaishawn Barham</t>
         </is>
       </c>
       <c r="C220" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D220" s="5" t="inlineStr">
@@ -30768,7 +30772,7 @@
       </c>
       <c r="F220" s="5" t="inlineStr">
         <is>
-          <t>Brown caught all three of his targets for 62 yards and two touchdowns during Saturday night's preseason game against the Seahawks.</t>
+          <t>Barham (groin) returned to practice Monday, Todd Archer of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -30780,12 +30784,12 @@
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>Anthony Smith</t>
+          <t>Von Miller</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
@@ -30800,7 +30804,7 @@
       </c>
       <c r="F221" s="4" t="inlineStr">
         <is>
-          <t>Smith brought in two of five targets for 28 yards and rushed once for nine yards in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
+          <t>Miller is not expected to practice with the Cowboys this week, Calvin Watkins of The Dallas Morning News reports.</t>
         </is>
       </c>
     </row>
@@ -30812,12 +30816,12 @@
       </c>
       <c r="B222" s="5" t="inlineStr">
         <is>
-          <t>Marquez Valdes-Scantling</t>
+          <t>Alijah Clark</t>
         </is>
       </c>
       <c r="C222" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D222" s="5" t="inlineStr">
@@ -30832,7 +30836,7 @@
       </c>
       <c r="F222" s="5" t="inlineStr">
         <is>
-          <t>Valdes-Scantling failed to bring in his only target in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
+          <t>Clark (ankle) recorded one tackle in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
         </is>
       </c>
     </row>
@@ -30844,12 +30848,12 @@
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>Brandon Aubrey</t>
+          <t>Camden Brown</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
@@ -30864,7 +30868,7 @@
       </c>
       <c r="F223" s="4" t="inlineStr">
         <is>
-          <t>Aubrey made his only field-goal attempt from 29 yards and knocked home both extra-point tries in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
+          <t>Brown caught all three of his targets for 62 yards and two touchdowns during Saturday night's preseason game against the Seahawks.</t>
         </is>
       </c>
     </row>
@@ -30876,7 +30880,7 @@
       </c>
       <c r="B224" s="5" t="inlineStr">
         <is>
-          <t>Ryan Flournoy</t>
+          <t>Anthony Smith</t>
         </is>
       </c>
       <c r="C224" s="5" t="inlineStr">
@@ -30896,7 +30900,7 @@
       </c>
       <c r="F224" s="5" t="inlineStr">
         <is>
-          <t>Flournoy isn't suited up ahead of Saturday's preseason opener versus Seattle, Nick Harris of the Fort Worth Star-Telegram reports.</t>
+          <t>Smith brought in two of five targets for 28 yards and rushed once for nine yards in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
         </is>
       </c>
     </row>
@@ -30908,12 +30912,12 @@
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>Jake Ferguson</t>
+          <t>Marquez Valdes-Scantling</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
@@ -30928,7 +30932,7 @@
       </c>
       <c r="F225" s="4" t="inlineStr">
         <is>
-          <t>Ferguson isn't suited up for Saturday's preseason contest against the Seahawks, Nick Harris of the Fort Worth Star-Telegram reports.</t>
+          <t>Valdes-Scantling failed to bring in his only target in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
         </is>
       </c>
     </row>
@@ -30940,12 +30944,12 @@
       </c>
       <c r="B226" s="5" t="inlineStr">
         <is>
-          <t>Dak Prescott</t>
+          <t>Brandon Aubrey</t>
         </is>
       </c>
       <c r="C226" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D226" s="5" t="inlineStr">
@@ -30960,7 +30964,7 @@
       </c>
       <c r="F226" s="5" t="inlineStr">
         <is>
-          <t>Prescott isn't slated to play in Saturday's preseason matchup versus Seattle, Nick Harris of the Fort Worth Star-Telegram reports.</t>
+          <t>Aubrey made his only field-goal attempt from 29 yards and knocked home both extra-point tries in the Cowboys' 17-7 preseason win over the Seahawks on Saturday.</t>
         </is>
       </c>
     </row>
@@ -30972,12 +30976,12 @@
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>Devin Moore</t>
+          <t>Ryan Flournoy</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
@@ -30992,7 +30996,7 @@
       </c>
       <c r="F227" s="4" t="inlineStr">
         <is>
-          <t>Moore (groin) was an active participant at the Cowboys' training camp practice Thursday, Tommy Yarrish of the team's official site reports.</t>
+          <t>Flournoy isn't suited up ahead of Saturday's preseason opener versus Seattle, Nick Harris of the Fort Worth Star-Telegram reports.</t>
         </is>
       </c>
     </row>
@@ -31004,12 +31008,12 @@
       </c>
       <c r="B228" s="5" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>Jake Ferguson</t>
         </is>
       </c>
       <c r="C228" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D228" s="5" t="inlineStr">
@@ -31024,7 +31028,7 @@
       </c>
       <c r="F228" s="5" t="inlineStr">
         <is>
-          <t>Pickens has impressed throughout the Cowboys' training camp, Dan Rogers of SB Nation reports.</t>
+          <t>Ferguson isn't suited up for Saturday's preseason contest against the Seahawks, Nick Harris of the Fort Worth Star-Telegram reports.</t>
         </is>
       </c>
     </row>
@@ -31036,12 +31040,12 @@
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>CeeDee Lamb</t>
+          <t>Dak Prescott</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
@@ -31056,7 +31060,7 @@
       </c>
       <c r="F229" s="4" t="inlineStr">
         <is>
-          <t>Lamb recently told reporters that he and QB Dak Prescott are "hitting on all cylinders" at training camp, Tommy Yarish of DallasCowboys.com reports.</t>
+          <t>Prescott isn't slated to play in Saturday's preseason matchup versus Seattle, Nick Harris of the Fort Worth Star-Telegram reports.</t>
         </is>
       </c>
     </row>
@@ -35964,7 +35968,7 @@
       </c>
       <c r="F384" s="5" t="inlineStr">
         <is>
-          <t>Walker rushed twice for four yards in the Chiefs' 16-15 preseason loss to the Bengals on Saturday.</t>
+          <t>Walker rushed twice for four yards in the Chiefs' 16-15 preseason loss to the Buccaneers on Saturday.</t>
         </is>
       </c>
     </row>
@@ -38340,7 +38344,7 @@
       </c>
       <c r="F459" s="4" t="inlineStr">
         <is>
-          <t>Rickert (knee) won't return to the Ram's preseason matchup versus the Saints on Saturday.</t>
+          <t>Rickert (knee) won't return to the Rams' preseason matchup versus the Saints on Saturday.</t>
         </is>
       </c>
     </row>
@@ -46940,27 +46944,27 @@
       </c>
       <c r="B730" s="5" t="inlineStr">
         <is>
-          <t>Chris Braswell</t>
+          <t>Ted Hurst III</t>
         </is>
       </c>
       <c r="C730" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D730" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E730" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F730" s="5" t="inlineStr">
         <is>
-          <t>Braswell (undisclosed) did not play in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday, Greg Auman of Fox Sports reports.</t>
+          <t>Hurst failed to bring in his only target in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
         </is>
       </c>
     </row>
@@ -46972,27 +46976,27 @@
       </c>
       <c r="B731" s="4" t="inlineStr">
         <is>
-          <t>Baker Mayfield</t>
+          <t>Chris Braswell</t>
         </is>
       </c>
       <c r="C731" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D731" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E731" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F731" s="4" t="inlineStr">
         <is>
-          <t>Mayfield completed two of four passes for 10 yards with no touchdowns or interceptions in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
+          <t>Braswell (undisclosed) did not play in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday, Greg Auman of Fox Sports reports.</t>
         </is>
       </c>
     </row>
@@ -47004,12 +47008,12 @@
       </c>
       <c r="B732" s="5" t="inlineStr">
         <is>
-          <t>Kenny Gainwell</t>
+          <t>Baker Mayfield</t>
         </is>
       </c>
       <c r="C732" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D732" s="5" t="inlineStr">
@@ -47024,7 +47028,7 @@
       </c>
       <c r="F732" s="5" t="inlineStr">
         <is>
-          <t>Gainwell rushed once for no gain in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
+          <t>Mayfield completed two of four passes for 10 yards with no touchdowns or interceptions in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
         </is>
       </c>
     </row>
@@ -47036,7 +47040,7 @@
       </c>
       <c r="B733" s="4" t="inlineStr">
         <is>
-          <t>Bucky Irving</t>
+          <t>Kenny Gainwell</t>
         </is>
       </c>
       <c r="C733" s="4" t="inlineStr">
@@ -47056,7 +47060,7 @@
       </c>
       <c r="F733" s="4" t="inlineStr">
         <is>
-          <t>Irving rushed three times for 14 yards in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
+          <t>Gainwell rushed once for no gain in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
         </is>
       </c>
     </row>
@@ -47068,27 +47072,27 @@
       </c>
       <c r="B734" s="5" t="inlineStr">
         <is>
-          <t>Dennis Houston</t>
+          <t>Bucky Irving</t>
         </is>
       </c>
       <c r="C734" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D734" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E734" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F734" s="5" t="inlineStr">
         <is>
-          <t>Houston has been ruled out for the rest of Saturday's preseason game against the Chiefs due to a groin injury.</t>
+          <t>Irving rushed three times for 14 yards in the Buccaneers' 16-15 preseason win over the Chiefs on Saturday.</t>
         </is>
       </c>
     </row>
@@ -47100,27 +47104,27 @@
       </c>
       <c r="B735" s="4" t="inlineStr">
         <is>
-          <t>Zyon McCollum</t>
+          <t>Dennis Houston</t>
         </is>
       </c>
       <c r="C735" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D735" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E735" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F735" s="4" t="inlineStr">
         <is>
-          <t>McCollum (groin) practiced Thursday and might even see some snaps in Saturday's preseason game against the Chiefs, Scott Smith of the Buccaneers' official site reports.</t>
+          <t>Houston has been ruled out for the rest of Saturday's preseason game against the Chiefs due to a groin injury.</t>
         </is>
       </c>
     </row>
@@ -47132,12 +47136,12 @@
       </c>
       <c r="B736" s="5" t="inlineStr">
         <is>
-          <t>Vita Vea</t>
+          <t>Zyon McCollum</t>
         </is>
       </c>
       <c r="C736" s="5" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D736" s="5" t="inlineStr">
@@ -47152,7 +47156,7 @@
       </c>
       <c r="F736" s="5" t="inlineStr">
         <is>
-          <t>Vea (back) and the Buccaneers reached an agreement on a one-year, $30 million extension Wednesday, Adam Schefter of ESPN reports.</t>
+          <t>McCollum (groin) practiced Thursday and might even see some snaps in Saturday's preseason game against the Chiefs, Scott Smith of the Buccaneers' official site reports.</t>
         </is>
       </c>
     </row>
@@ -47164,27 +47168,27 @@
       </c>
       <c r="B737" s="4" t="inlineStr">
         <is>
-          <t>Cade Otton</t>
+          <t>Vita Vea</t>
         </is>
       </c>
       <c r="C737" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D737" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E737" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F737" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Vea (back) and the Buccaneers reached an agreement on a one-year, $30 million extension Wednesday, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -47196,12 +47200,12 @@
       </c>
       <c r="B738" s="5" t="inlineStr">
         <is>
-          <t>Tez Johnson</t>
+          <t>Cade Otton</t>
         </is>
       </c>
       <c r="C738" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D738" s="5" t="inlineStr">
@@ -47211,7 +47215,7 @@
       </c>
       <c r="E738" s="5" t="inlineStr">
         <is>
-          <t>Strain</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F738" s="5" t="inlineStr">
@@ -47228,7 +47232,7 @@
       </c>
       <c r="B739" s="4" t="inlineStr">
         <is>
-          <t>Jalen McMillan</t>
+          <t>Tez Johnson</t>
         </is>
       </c>
       <c r="C739" s="4" t="inlineStr">
@@ -47243,7 +47247,7 @@
       </c>
       <c r="E739" s="4" t="inlineStr">
         <is>
-          <t>Soreness</t>
+          <t>Strain</t>
         </is>
       </c>
       <c r="F739" s="4" t="inlineStr">
@@ -47260,27 +47264,27 @@
       </c>
       <c r="B740" s="5" t="inlineStr">
         <is>
-          <t>Kadarius Calloway</t>
+          <t>Jalen McMillan</t>
         </is>
       </c>
       <c r="C740" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D740" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E740" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Soreness</t>
         </is>
       </c>
       <c r="F740" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -47292,27 +47296,27 @@
       </c>
       <c r="B741" s="4" t="inlineStr">
         <is>
-          <t>Emeka Egbuka</t>
+          <t>Kadarius Calloway</t>
         </is>
       </c>
       <c r="C741" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D741" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E741" s="4" t="inlineStr">
         <is>
-          <t>Sprain</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F741" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -47324,25 +47328,29 @@
       </c>
       <c r="B742" s="5" t="inlineStr">
         <is>
-          <t>JJ Roberts</t>
+          <t>Emeka Egbuka</t>
         </is>
       </c>
       <c r="C742" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D742" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E742" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F742" s="5" t="inlineStr"/>
+          <t>Sprain</t>
+        </is>
+      </c>
+      <c r="F742" s="5" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="743">
       <c r="A743" s="4" t="inlineStr">
@@ -47352,12 +47360,12 @@
       </c>
       <c r="B743" s="4" t="inlineStr">
         <is>
-          <t>Tristan Wirfs</t>
+          <t>JJ Roberts</t>
         </is>
       </c>
       <c r="C743" s="4" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D743" s="4" t="inlineStr">
@@ -47380,29 +47388,25 @@
       </c>
       <c r="B744" s="5" t="inlineStr">
         <is>
-          <t>Billy Schrauth</t>
+          <t>Tristan Wirfs</t>
         </is>
       </c>
       <c r="C744" s="5" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D744" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E744" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="F744" s="5" t="inlineStr">
-        <is>
-          <t>Schrauth (knee) did not participate in Tuesday's practice, Greg Auman of Fox Sports reports.</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F744" s="5" t="inlineStr"/>
     </row>
     <row r="745">
       <c r="A745" s="4" t="inlineStr">
@@ -47412,27 +47416,27 @@
       </c>
       <c r="B745" s="4" t="inlineStr">
         <is>
-          <t>Jake Browning</t>
+          <t>Billy Schrauth</t>
         </is>
       </c>
       <c r="C745" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D745" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E745" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F745" s="4" t="inlineStr">
         <is>
-          <t>Browning (back) practiced Monday after missing Friday's preseason game against the Jets, Rick Stroud of the Tampa Bay Times reports.</t>
+          <t>Schrauth (knee) did not participate in Tuesday's practice, Greg Auman of Fox Sports reports.</t>
         </is>
       </c>
     </row>
@@ -47444,12 +47448,12 @@
       </c>
       <c r="B746" s="5" t="inlineStr">
         <is>
-          <t>Chris Godwin Jr.</t>
+          <t>Jake Browning</t>
         </is>
       </c>
       <c r="C746" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D746" s="5" t="inlineStr">
@@ -47464,7 +47468,7 @@
       </c>
       <c r="F746" s="5" t="inlineStr">
         <is>
-          <t>Godwin didn't play in Friday's 24-16 preseason victory over the Jets.</t>
+          <t>Browning (back) practiced Monday after missing Friday's preseason game against the Jets, Rick Stroud of the Tampa Bay Times reports.</t>
         </is>
       </c>
     </row>
@@ -47476,7 +47480,7 @@
       </c>
       <c r="B747" s="4" t="inlineStr">
         <is>
-          <t>Ted Hurst III</t>
+          <t>Chris Godwin Jr.</t>
         </is>
       </c>
       <c r="C747" s="4" t="inlineStr">
@@ -47496,7 +47500,7 @@
       </c>
       <c r="F747" s="4" t="inlineStr">
         <is>
-          <t>Hurst brought in two of six targets for 19 yards in the Buccaneers' 24-16 preseason win over the Jets on Friday.</t>
+          <t>Godwin didn't play in Friday's 24-16 preseason victory over the Jets.</t>
         </is>
       </c>
     </row>
@@ -49322,7 +49326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49406,54 +49410,50 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>401874101</t>
+          <t>401873297</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>State Farm Stadium</t>
+          <t>Nissan Stadium</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>retractable</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>108.1</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>7.6</v>
+        <v>5.6</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>11</v>
+        <v>12.3</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>108°F · retractable roof — effect halved</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>401873297</t>
+          <t>401873298</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Nissan Stadium</t>
+          <t>Highmark Stadium</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -49462,20 +49462,20 @@
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>82.90000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>5.6</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>12.3</v>
+        <v>12.1</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I6" s="22" t="n">
@@ -49486,12 +49486,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>401873298</t>
+          <t>401873299</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Highmark Stadium</t>
+          <t>Huntington Bank Field</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -49500,142 +49500,142 @@
         </is>
       </c>
       <c r="D7" s="15" t="n">
-        <v>74.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>6.7</v>
+        <v>5.1</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>12.1</v>
+        <v>21.7</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Wind 5 mph (gusts 22)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>401873299</t>
+          <t>401873641</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Huntington Bank Field</t>
+          <t>Allegiant Stadium</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>dome</t>
         </is>
       </c>
       <c r="D8" s="17" t="n">
-        <v>72.3</v>
+        <v>108.5</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>9.800000000000001</v>
+        <v>18.8</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>21.7</v>
+        <v>16.1</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I8" s="22" t="n">
-        <v>-0.8</v>
+        <v>0</v>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Wind 10 mph (gusts 22)</t>
+          <t>Indoors — weather ignored</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>401873641</t>
+          <t>401873300</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Allegiant Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>dome</t>
+          <t>canopy</t>
         </is>
       </c>
       <c r="D9" s="15" t="n">
-        <v>108.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>18</v>
+        <v>8.1</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>16.1</v>
+        <v>6.9</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>Indoors — weather ignored</t>
-        </is>
-      </c>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>401873300</t>
+          <t>401873302</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>M&amp;T Bank Stadium</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>canopy</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>78.40000000000001</v>
+        <v>83.7</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>8.300000000000001</v>
+        <v>2.7</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>6.9</v>
+        <v>8.1</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I10" s="22" t="n">
@@ -49646,34 +49646,34 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>401873302</t>
+          <t>401873304</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>M&amp;T Bank Stadium</t>
+          <t>Hard Rock Stadium</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>canopy</t>
         </is>
       </c>
       <c r="D11" s="15" t="n">
-        <v>86.2</v>
+        <v>89.5</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>2</v>
+        <v>10.5</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>8.1</v>
+        <v>11.6</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
@@ -49684,30 +49684,30 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>401873304</t>
+          <t>401873307</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Hard Rock Stadium</t>
+          <t>Bank of America Stadium</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>canopy</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D12" s="17" t="n">
-        <v>89.09999999999999</v>
+        <v>82</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>12.1</v>
+        <v>4</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>11.6</v>
+        <v>4.7</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -49715,23 +49715,19 @@
         </is>
       </c>
       <c r="I12" s="22" t="n">
-        <v>-0.68</v>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>Wind 12 mph (gusts 12) · canopy — wind damped</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>401873307</t>
+          <t>401873303</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Bank of America Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -49740,20 +49736,20 @@
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>85.90000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>4.7</v>
+        <v>10.1</v>
       </c>
       <c r="G13" s="15" t="n">
         <v>25</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Drizzle</t>
         </is>
       </c>
       <c r="I13" s="9" t="n">
@@ -49764,12 +49760,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>401873303</t>
+          <t>401873306</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>EverBank Stadium</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -49778,36 +49774,40 @@
         </is>
       </c>
       <c r="D14" s="17" t="n">
-        <v>79.2</v>
+        <v>91.5</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>7.6</v>
+        <v>11.2</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>10.1</v>
+        <v>11.2</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I14" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="5" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>67% chance of rain</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>401873306</t>
+          <t>401873301</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>EverBank Stadium</t>
+          <t>Lincoln Financial Field</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -49816,16 +49816,16 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>94.8</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>8.4</v>
+        <v>7.4</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>11.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -49833,23 +49833,19 @@
         </is>
       </c>
       <c r="I15" s="9" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>67% chance of rain · 95°F</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>401873301</t>
+          <t>401873305</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Lincoln Financial Field</t>
+          <t>Arrowhead Stadium</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -49858,20 +49854,20 @@
         </is>
       </c>
       <c r="D16" s="17" t="n">
-        <v>79.59999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>4.1</v>
+        <v>10.6</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>9.199999999999999</v>
+        <v>14.5</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I16" s="22" t="n">
@@ -49882,92 +49878,96 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>401873305</t>
+          <t>401874048</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Arrowhead Stadium</t>
+          <t>AT&amp;T Stadium</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>retractable</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>84.40000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>8.800000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>14.5</v>
+        <v>6</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="4" t="inlineStr"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>93°F · retractable roof — effect halved</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>401874048</t>
+          <t>401874102</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>AT&amp;T Stadium</t>
+          <t>Lambeau Field</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>retractable</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D18" s="17" t="n">
-        <v>98.3</v>
+        <v>63.7</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>8.4</v>
+        <v>12.6</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="G18" s="17" t="n">
         <v>2</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I18" s="22" t="n">
-        <v>-0.25</v>
+        <v>-0.8</v>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>98°F · retractable roof — effect halved</t>
+          <t>Wind 13 mph (gusts 19)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>401874102</t>
+          <t>401873614</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Lambeau Field</t>
+          <t>Empower Field at Mile High</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -49976,62 +49976,58 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>63.5</v>
+        <v>82.2</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>13.8</v>
+        <v>7.7</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>19</v>
+        <v>7.4</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>Wind 14 mph (gusts 19)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>401873614</t>
+          <t>401873308</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Empower Field at Mile High</t>
+          <t>Lucas Oil Stadium</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>retractable</t>
         </is>
       </c>
       <c r="D20" s="17" t="n">
-        <v>74.59999999999999</v>
+        <v>78.7</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>9.699999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="F20" s="17" t="n">
-        <v>7.4</v>
+        <v>2.2</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I20" s="22" t="n">
@@ -50042,34 +50038,34 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>401873308</t>
+          <t>401874394</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Lucas Oil Stadium</t>
+          <t>Nissan Stadium</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>retractable</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>79.59999999999999</v>
+        <v>88.8</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>2.2</v>
+        <v>5.6</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I21" s="9" t="n">
@@ -50080,36 +50076,24 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>401874394</t>
+          <t>401872656</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Nissan Stadium</t>
+          <t>Lumen Field</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="D22" s="17" t="n">
-        <v>91.2</v>
-      </c>
-      <c r="E22" s="17" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G22" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Partly cloudy</t>
-        </is>
-      </c>
+          <t>canopy</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="5" t="n"/>
       <c r="I22" s="22" t="n">
         <v>0</v>
       </c>
@@ -50118,17 +50102,17 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>401872656</t>
+          <t>401872657</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Lumen Field</t>
+          <t>Melbourne Cricket Ground</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>canopy</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D23" s="15" t="n"/>
@@ -50144,12 +50128,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>401872657</t>
+          <t>401872658</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Melbourne Cricket Ground</t>
+          <t>Acrisure Stadium</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -50170,17 +50154,17 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>401872658</t>
+          <t>401872659</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Acrisure Stadium</t>
+          <t>Lucas Oil Stadium</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>retractable</t>
         </is>
       </c>
       <c r="D25" s="15" t="n"/>
@@ -50196,12 +50180,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>401872659</t>
+          <t>401872660</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Lucas Oil Stadium</t>
+          <t>Reliant Stadium</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -50222,17 +50206,17 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>401872660</t>
+          <t>401872661</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Reliant Stadium</t>
+          <t>Bank of America Stadium</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>retractable</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D27" s="15" t="n"/>
@@ -50248,12 +50232,12 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>401872661</t>
+          <t>401872922</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Bank of America Stadium</t>
+          <t>EverBank Stadium</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -50274,17 +50258,17 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>401872922</t>
+          <t>401872923</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>EverBank Stadium</t>
+          <t>Ford Field</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>dome</t>
         </is>
       </c>
       <c r="D29" s="15" t="n"/>
@@ -50300,17 +50284,17 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>401872923</t>
+          <t>401872924</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Ford Field</t>
+          <t>Nissan Stadium</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>dome</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D30" s="17" t="n"/>
@@ -50326,12 +50310,12 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>401872924</t>
+          <t>401872925</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Nissan Stadium</t>
+          <t>Paycor Stadium</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -50352,17 +50336,17 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>401872925</t>
+          <t>401872926</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Paycor Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>canopy</t>
         </is>
       </c>
       <c r="D32" s="17" t="n"/>
@@ -50378,17 +50362,17 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>401872926</t>
+          <t>401872927</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>U.S. Bank Stadium</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>canopy</t>
+          <t>dome</t>
         </is>
       </c>
       <c r="D33" s="15" t="n"/>
@@ -50404,12 +50388,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>401872927</t>
+          <t>401872928</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>U.S. Bank Stadium</t>
+          <t>Allegiant Stadium</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -50430,17 +50414,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>401872928</t>
+          <t>401872929</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Allegiant Stadium</t>
+          <t>Lincoln Financial Field</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>dome</t>
+          <t>open</t>
         </is>
       </c>
       <c r="D35" s="15" t="n"/>
@@ -50456,12 +50440,12 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>401872929</t>
+          <t>401872930</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Lincoln Financial Field</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -50482,12 +50466,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>401872930</t>
+          <t>401872931</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Arrowhead Stadium</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -50504,32 +50488,6 @@
         <v>0</v>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>401872931</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Arrowhead Stadium</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="D38" s="17" t="n"/>
-      <c r="E38" s="17" t="n"/>
-      <c r="F38" s="17" t="n"/>
-      <c r="G38" s="17" t="n"/>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh: 2026-08-23 13:45 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -689,7 +689,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-23T06:00:13+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-23T13:45:14+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23T06:00:13+00:00</t>
+          <t>2026-08-23T13:45:14+00:00</t>
         </is>
       </c>
     </row>
@@ -23972,27 +23972,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Dadrion Taylor-Demerson</t>
+          <t>Chad Ryland</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Taylor-Demerson is questionable to return to Saturday's preseason game against the Cowboys due to a rib injury.</t>
+          <t>Ryland made field goals of 38 and 31 yards, missed a 62-yarder wide right and knocked through his only extra-point try in the Cardinals' 34-13 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -24004,12 +24004,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Blake Gillikin</t>
+          <t>Dadrion Taylor-Demerson</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Gillikin sustained a groin injury during pregame warmups and is questionable to play in Saturday's preseason game against the Cowboys, Darren Urban of the Cardinals' official site reports.</t>
+          <t>Taylor-Demerson is questionable to return to Saturday's preseason game against the Cowboys due to a rib injury.</t>
         </is>
       </c>
     </row>
@@ -24036,12 +24036,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Trey Benson</t>
+          <t>Blake Gillikin</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -24056,7 +24056,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Benson (knee) has not been present for any portion of the Cardinals' previous two full-squad practices this week, Theo Mackie of The Arizona Republic reports.</t>
+          <t>Gillikin sustained a groin injury during pregame warmups and is questionable to play in Saturday's preseason game against the Cowboys, Darren Urban of the Cardinals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -24068,17 +24068,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Tip Reiman</t>
+          <t>Trey Benson</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -24088,7 +24088,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Reiman (ankle) will not be back for the start of the regular season, Darren Urban of the Cardinals' official site reports.</t>
+          <t>Benson (knee) has not been present for any portion of the Cardinals' previous two full-squad practices this week, Theo Mackie of The Arizona Republic reports.</t>
         </is>
       </c>
     </row>
@@ -24100,12 +24100,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Josh Sweat</t>
+          <t>Tip Reiman</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -24120,7 +24120,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Sweat (knee) is almost ready to be activated off the PUP list, Darren Urban of the Cardinals' official site reports.</t>
+          <t>Reiman (ankle) will not be back for the start of the regular season, Darren Urban of the Cardinals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -24132,27 +24132,27 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Garrett Williams</t>
+          <t>Josh Sweat</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Williams (Achilles) was activated from the PUP list by the Cardinals on Thursday, Darren Urban of the Cardinals' official site reports.</t>
+          <t>Sweat (knee) is almost ready to be activated off the PUP list, Darren Urban of the Cardinals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -24164,27 +24164,27 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Carson Beck</t>
+          <t>Garrett Williams</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Coach Mike LaFleur said Beck (ribs) "most likely" won't suit up for Saturday's preseason contest against the Cowboys, Josh Weinfuss of ESPN.com reports.</t>
+          <t>Williams (Achilles) was activated from the PUP list by the Cardinals on Thursday, Darren Urban of the Cardinals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -24196,7 +24196,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Jacoby Brissett</t>
+          <t>Carson Beck</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -24206,17 +24206,17 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Coach Mike LaFleur said Thursday that Brissett won't suit up for Saturday's preseason game against the Cowboys, Josh Weinfuss of ESPN.com reports.</t>
+          <t>Coach Mike LaFleur said Beck (ribs) "most likely" won't suit up for Saturday's preseason contest against the Cowboys, Josh Weinfuss of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -24228,27 +24228,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Xavier Weaver</t>
+          <t>Jacoby Brissett</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Concussion</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Coach Mike LaFleur said Thursday that Brissett won't suit up for Saturday's preseason game against the Cowboys, Josh Weinfuss of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -24260,12 +24260,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Elijah Higgins</t>
+          <t>Xavier Weaver</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -24292,27 +24292,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Austin Keys</t>
+          <t>Elijah Higgins</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Concussion</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -24324,25 +24324,29 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Valentin Senn</t>
+          <t>Austin Keys</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>ir</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -24352,29 +24356,25 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Chase Bisontis</t>
+          <t>Valentin Senn</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>ir</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -24384,12 +24384,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Joey Blount</t>
+          <t>Chase Bisontis</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -24399,7 +24399,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Stinger</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -24416,27 +24416,27 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Zachary Carter</t>
+          <t>Joey Blount</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Stinger</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -24448,17 +24448,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Jameson Geers</t>
+          <t>Zachary Carter</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -24468,7 +24468,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -24480,27 +24480,27 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Jameson Geers</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Sprain</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Coach Mike LaFleur confirmed Tuesday that Love does not need surgery to address his ankle injury, Tyler Drake of ArizonaSports.com reports.</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -24512,7 +24512,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Tyler Allgeier</t>
+          <t>Jeremiyah Love</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -24522,17 +24522,17 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Sprain</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Allgeier could open the regular season as the Cardinals' primary running back, as Adam Schefter of ESPN reports that Jeremiyah Love sustained a high-ankle sprain in Thursday's preseason win over the Raiders.</t>
+          <t>Coach Mike LaFleur confirmed Tuesday that Love does not need surgery to address his ankle injury, Tyler Drake of ArizonaSports.com reports.</t>
         </is>
       </c>
     </row>
@@ -24544,7 +24544,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Tre Stewart</t>
+          <t>Tyler Allgeier</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -24564,7 +24564,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>The Cardinals signed Stewart to a contract Saturday.</t>
+          <t>Allgeier could open the regular season as the Cardinals' primary running back, as Adam Schefter of ESPN reports that Jeremiyah Love sustained a high-ankle sprain in Thursday's preseason win over the Raiders.</t>
         </is>
       </c>
     </row>
@@ -24576,12 +24576,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Baylor Cupp</t>
+          <t>Tre Stewart</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -24596,7 +24596,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>The Cardinals signed Cupp to a contract Saturday.</t>
+          <t>The Cardinals signed Stewart to a contract Saturday.</t>
         </is>
       </c>
     </row>
@@ -24608,27 +24608,27 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>James Conner</t>
+          <t>Baylor Cupp</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Head coach Mike LaFleur said Saturday that there is no timeline for Conner (foot) to participate in 11-on-11 drills in training camp practice, Darren Urban of the Cardinals' official site reports.</t>
+          <t>The Cardinals signed Cupp to a contract Saturday.</t>
         </is>
       </c>
     </row>
@@ -24640,27 +24640,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Trey McBride</t>
+          <t>James Conner</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>McBride played one snap in Thursday's 27-14 preseason win over the Raiders.</t>
+          <t>Head coach Mike LaFleur said Saturday that there is no timeline for Conner (foot) to participate in 11-on-11 drills in training camp practice, Darren Urban of the Cardinals' official site reports.</t>
         </is>
       </c>
     </row>
@@ -24672,12 +24672,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr.</t>
+          <t>Trey McBride</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -24692,7 +24692,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Harrison brought in his only target for seven yards and a touchdown and also drew a 20-yard pass interference penalty in the Cardinals' 27-14 preseason win over the Raiders on Thursday.</t>
+          <t>McBride played one snap in Thursday's 27-14 preseason win over the Raiders.</t>
         </is>
       </c>
     </row>
@@ -24704,7 +24704,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Michael Wilson</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -24724,7 +24724,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Wilson brought in both targets for 23 yards in the Cardinals' 27-14 preseason win over the Raiders on Thursday.</t>
+          <t>Harrison brought in his only target for seven yards and a touchdown and also drew a 20-yard pass interference penalty in the Cardinals' 27-14 preseason win over the Raiders on Thursday.</t>
         </is>
       </c>
     </row>
@@ -24736,12 +24736,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Shawn Bowman</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -24756,7 +24756,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>The Cardinals signed Bowman to a contract Sunday, Zach Gershman of the team's official site reports.</t>
+          <t>Wilson brought in both targets for 23 yards in the Cardinals' 27-14 preseason win over the Raiders on Thursday.</t>
         </is>
       </c>
     </row>
@@ -35024,27 +35024,27 @@
       </c>
       <c r="B355" s="4" t="inlineStr">
         <is>
-          <t>Tanner Koziol</t>
+          <t>Parker Washington</t>
         </is>
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F355" s="4" t="inlineStr">
         <is>
-          <t>Koziol played 18 snaps (13 on offense, five on special teams) but didn't show up in the box score otherwise during the Jaguars' 34-17 preseason loss to the Panthers on Friday.</t>
+          <t>Washington (undisclosed) was spotted at Sunday's walkthrough, Ryan O'Halloran of The Florida Times-Union reports.</t>
         </is>
       </c>
     </row>
@@ -35056,7 +35056,7 @@
       </c>
       <c r="B356" s="5" t="inlineStr">
         <is>
-          <t>Nate Boerkircher</t>
+          <t>Tanner Koziol</t>
         </is>
       </c>
       <c r="C356" s="5" t="inlineStr">
@@ -35076,7 +35076,7 @@
       </c>
       <c r="F356" s="5" t="inlineStr">
         <is>
-          <t>Boerkircher did not participate in Friday's 34-17 preseason loss to Carolina.</t>
+          <t>Koziol played 18 snaps (13 on offense, five on special teams) but didn't show up in the box score otherwise during the Jaguars' 34-17 preseason loss to the Panthers on Friday.</t>
         </is>
       </c>
     </row>
@@ -35088,7 +35088,7 @@
       </c>
       <c r="B357" s="4" t="inlineStr">
         <is>
-          <t>Brenton Strange</t>
+          <t>Nate Boerkircher</t>
         </is>
       </c>
       <c r="C357" s="4" t="inlineStr">
@@ -35108,7 +35108,7 @@
       </c>
       <c r="F357" s="4" t="inlineStr">
         <is>
-          <t>Strange did not play in the Jaguars' 34-17 preseason loss to the Panthers on Friday.</t>
+          <t>Boerkircher did not participate in Friday's 34-17 preseason loss to Carolina.</t>
         </is>
       </c>
     </row>
@@ -35120,12 +35120,12 @@
       </c>
       <c r="B358" s="5" t="inlineStr">
         <is>
-          <t>Travis Hunter</t>
+          <t>Brenton Strange</t>
         </is>
       </c>
       <c r="C358" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D358" s="5" t="inlineStr">
@@ -35140,7 +35140,7 @@
       </c>
       <c r="F358" s="5" t="inlineStr">
         <is>
-          <t>Hunter did not play in the Jaguars' 34-17 preseason loss to the Panthers on Friday.</t>
+          <t>Strange did not play in the Jaguars' 34-17 preseason loss to the Panthers on Friday.</t>
         </is>
       </c>
     </row>
@@ -35152,12 +35152,12 @@
       </c>
       <c r="B359" s="4" t="inlineStr">
         <is>
-          <t>Ameer Abdullah</t>
+          <t>Travis Hunter</t>
         </is>
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D359" s="4" t="inlineStr">
@@ -35172,7 +35172,7 @@
       </c>
       <c r="F359" s="4" t="inlineStr">
         <is>
-          <t>Abdullah carried the ball six times for 45 yards and caught three of four targets for 37 yards in Friday's 34-17 preseason loss to the Panthers.</t>
+          <t>Hunter did not play in the Jaguars' 34-17 preseason loss to the Panthers on Friday.</t>
         </is>
       </c>
     </row>
@@ -35184,12 +35184,12 @@
       </c>
       <c r="B360" s="5" t="inlineStr">
         <is>
-          <t>CJ Williams</t>
+          <t>Ameer Abdullah</t>
         </is>
       </c>
       <c r="C360" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D360" s="5" t="inlineStr">
@@ -35204,7 +35204,7 @@
       </c>
       <c r="F360" s="5" t="inlineStr">
         <is>
-          <t>Williams caught all four of his targets for 22 yards and gained two rushing yards on his lone carry during Friday's 34-17 preseason loss to the Panthers.</t>
+          <t>Abdullah carried the ball six times for 45 yards and caught three of four targets for 37 yards in Friday's 34-17 preseason loss to the Panthers.</t>
         </is>
       </c>
     </row>
@@ -35216,7 +35216,7 @@
       </c>
       <c r="B361" s="4" t="inlineStr">
         <is>
-          <t>Josh Cameron</t>
+          <t>CJ Williams</t>
         </is>
       </c>
       <c r="C361" s="4" t="inlineStr">
@@ -35236,7 +35236,7 @@
       </c>
       <c r="F361" s="4" t="inlineStr">
         <is>
-          <t>Cameron caught both his targets for 41 yards in Friday's 34-17 preseason loss to the Panthers.</t>
+          <t>Williams caught all four of his targets for 22 yards and gained two rushing yards on his lone carry during Friday's 34-17 preseason loss to the Panthers.</t>
         </is>
       </c>
     </row>
@@ -35248,12 +35248,12 @@
       </c>
       <c r="B362" s="5" t="inlineStr">
         <is>
-          <t>Nick Mullens</t>
+          <t>Josh Cameron</t>
         </is>
       </c>
       <c r="C362" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D362" s="5" t="inlineStr">
@@ -35268,7 +35268,7 @@
       </c>
       <c r="F362" s="5" t="inlineStr">
         <is>
-          <t>Mullens completed six of seven passes for 65 yards in Friday's 34-17 preseason loss to the Panthers.</t>
+          <t>Cameron caught both his targets for 41 yards in Friday's 34-17 preseason loss to the Panthers.</t>
         </is>
       </c>
     </row>
@@ -35280,27 +35280,27 @@
       </c>
       <c r="B363" s="4" t="inlineStr">
         <is>
-          <t>Jakobi Meyers</t>
+          <t>Nick Mullens</t>
         </is>
       </c>
       <c r="C363" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D363" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E363" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F363" s="4" t="inlineStr">
         <is>
-          <t>Head coach Liam Coen said after Friday's 34-17 preseason loss to the Panthers that Meyers jammed his right hand during Wednesday's joint practice with Carolina, Juston Lewis of The Florida Times-Union reports.</t>
+          <t>Mullens completed six of seven passes for 65 yards in Friday's 34-17 preseason loss to the Panthers.</t>
         </is>
       </c>
     </row>
@@ -35312,27 +35312,27 @@
       </c>
       <c r="B364" s="5" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Jakobi Meyers</t>
         </is>
       </c>
       <c r="C364" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D364" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E364" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F364" s="5" t="inlineStr">
         <is>
-          <t>Lawrence won't play in Friday's preseason game against the Panthers, John Shipley of SI.com reports.</t>
+          <t>Head coach Liam Coen said after Friday's 34-17 preseason loss to the Panthers that Meyers jammed his right hand during Wednesday's joint practice with Carolina, Juston Lewis of The Florida Times-Union reports.</t>
         </is>
       </c>
     </row>
@@ -35344,27 +35344,27 @@
       </c>
       <c r="B365" s="4" t="inlineStr">
         <is>
-          <t>Parker Washington</t>
+          <t>Trevor Lawrence</t>
         </is>
       </c>
       <c r="C365" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D365" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E365" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F365" s="4" t="inlineStr">
         <is>
-          <t>Washington (undisclosed) is expected to return to practice next week, ESPN's Adam Schefter reports.</t>
+          <t>Lawrence won't play in Friday's preseason game against the Panthers, John Shipley of SI.com reports.</t>
         </is>
       </c>
     </row>
@@ -49424,20 +49424,20 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>82.90000000000001</v>
+        <v>82.7</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>5.6</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>12.3</v>
+        <v>12.1</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I5" s="9" t="n">
@@ -49465,13 +49465,13 @@
         <v>70.5</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>5.6</v>
+        <v>7.4</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>12.1</v>
+        <v>20.6</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -49479,9 +49479,13 @@
         </is>
       </c>
       <c r="I6" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="5" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Wind 7 mph (gusts 21)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -49500,16 +49504,16 @@
         </is>
       </c>
       <c r="D7" s="15" t="n">
-        <v>73</v>
+        <v>73.3</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>5.1</v>
+        <v>6.2</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>21.7</v>
+        <v>9.4</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -49517,13 +49521,9 @@
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>Wind 5 mph (gusts 22)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -49542,16 +49542,16 @@
         </is>
       </c>
       <c r="D8" s="17" t="n">
-        <v>108.5</v>
+        <v>107.4</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>18.8</v>
+        <v>20</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>16.1</v>
+        <v>20.4</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -49584,10 +49584,10 @@
         </is>
       </c>
       <c r="D9" s="15" t="n">
-        <v>78.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>6.9</v>
@@ -49597,7 +49597,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
@@ -49622,20 +49622,20 @@
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>83.7</v>
+        <v>86.7</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>8.1</v>
+        <v>6.9</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I10" s="22" t="n">
@@ -49660,26 +49660,30 @@
         </is>
       </c>
       <c r="D11" s="15" t="n">
-        <v>89.5</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>10.5</v>
+        <v>13.9</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>11.6</v>
+        <v>14.3</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4" t="inlineStr"/>
+        <v>-0.68</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Wind 14 mph (gusts 14) · canopy — wind damped</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -49698,16 +49702,16 @@
         </is>
       </c>
       <c r="D12" s="17" t="n">
-        <v>82</v>
+        <v>85.3</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>4</v>
+        <v>5.6</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>4.7</v>
+        <v>13.2</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -49736,20 +49740,20 @@
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>80.5</v>
+        <v>84.7</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>4.4</v>
+        <v>6.8</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>10.1</v>
+        <v>12.3</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Drizzle</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I13" s="9" t="n">
@@ -49774,16 +49778,16 @@
         </is>
       </c>
       <c r="D14" s="17" t="n">
-        <v>91.5</v>
+        <v>93.2</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>11.2</v>
+        <v>8.9</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>11.2</v>
+        <v>12.8</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -49791,11 +49795,11 @@
         </is>
       </c>
       <c r="I14" s="22" t="n">
-        <v>-1</v>
+        <v>-1.5</v>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>67% chance of rain</t>
+          <t>61% chance of rain · 93°F</t>
         </is>
       </c>
     </row>
@@ -49816,16 +49820,16 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>81.59999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>7.4</v>
+        <v>4.7</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -49854,26 +49858,30 @@
         </is>
       </c>
       <c r="D16" s="17" t="n">
-        <v>89.3</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>10.6</v>
+        <v>11.4</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>14.5</v>
+        <v>19</v>
       </c>
       <c r="G16" s="17" t="n">
         <v>7</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I16" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="5" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Wind 11 mph (gusts 19)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -49892,20 +49900,20 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>93.3</v>
+        <v>101.9</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>10.7</v>
+        <v>8</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>6</v>
+        <v>10.5</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I17" s="9" t="n">
@@ -49913,7 +49921,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>93°F · retractable roof — effect halved</t>
+          <t>102°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -49934,30 +49942,26 @@
         </is>
       </c>
       <c r="D18" s="17" t="n">
-        <v>63.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>12.6</v>
+        <v>7.8</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G18" s="17" t="n">
         <v>2</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I18" s="22" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Wind 13 mph (gusts 19)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -49976,26 +49980,30 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>82.2</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>7.7</v>
+        <v>13.2</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>7.4</v>
+        <v>21</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="4" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Wind 13 mph (gusts 21)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -50014,20 +50022,20 @@
         </is>
       </c>
       <c r="D20" s="17" t="n">
-        <v>78.7</v>
+        <v>76.2</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>0.7</v>
+        <v>6.1</v>
       </c>
       <c r="F20" s="17" t="n">
-        <v>2.2</v>
+        <v>7.2</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I20" s="22" t="n">
@@ -50052,16 +50060,16 @@
         </is>
       </c>
       <c r="D21" s="15" t="n">
-        <v>88.8</v>
+        <v>88.3</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>4</v>
+        <v>5.4</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh: 2026-08-23 16:56 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -689,7 +689,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-23T13:45:14+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-23T16:56:41+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23T13:45:14+00:00</t>
+          <t>2026-08-23T16:56:41+00:00</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -3023,23 +3023,23 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>CLE +7.5</t>
+          <t>NE +3.5</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5356</v>
+        <v>0.5327</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0.0117</v>
+        <v>0.0089</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0.02260161108580988</v>
+        <v>0.01706011721804213</v>
       </c>
       <c r="J16" s="14" t="n">
         <v>0.5</v>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -3064,23 +3064,23 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>NE +3.5</t>
+          <t>NO +7</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.5327</v>
+        <v>0.5323</v>
       </c>
       <c r="G17" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.01706011721804213</v>
+        <v>0.01531241952910156</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>0.5</v>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3105,23 +3105,23 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>NO +7</t>
+          <t>CLE +7.5</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5323</v>
+        <v>0.5313</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0074</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.01531241952910156</v>
+        <v>0.01421344402886232</v>
       </c>
       <c r="J18" s="14" t="n">
         <v>0.5</v>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -3720,23 +3720,23 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>MIA +3.5</t>
+          <t>MIN -1.5</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>0.5048</v>
+        <v>0.5044999999999999</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>-0.0183</v>
+        <v>-0.0185</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>-0.03638401763136451</v>
+        <v>-0.03680188589386885</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.5</v>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -3761,23 +3761,23 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>MIN -1.5</t>
+          <t>MIA +3.5</t>
         </is>
       </c>
       <c r="E34" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5044999999999999</v>
+        <v>0.5034999999999999</v>
       </c>
       <c r="G34" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H34" s="13" t="n">
-        <v>-0.0185</v>
+        <v>-0.0194</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.03680188589386885</v>
+        <v>-0.03879346990146776</v>
       </c>
       <c r="J34" s="14" t="n">
         <v>0.5</v>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -4130,23 +4130,23 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>GB +1.5</t>
+          <t>LV -3.5</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>0.4955</v>
+        <v>0.4965</v>
       </c>
       <c r="G43" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>-0.0261</v>
+        <v>-0.0253</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>-0.05410720501522198</v>
+        <v>-0.05211562100762307</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>0.5</v>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -4171,23 +4171,23 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>LV -3.5</t>
+          <t>GB +1.5</t>
         </is>
       </c>
       <c r="E44" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4952</v>
+        <v>0.4955</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H44" s="13" t="n">
-        <v>-0.0262</v>
+        <v>-0.0261</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>-0.05452507327772632</v>
+        <v>-0.05410720501522198</v>
       </c>
       <c r="J44" s="14" t="n">
         <v>0.5</v>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -4786,23 +4786,23 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>DET -7</t>
+          <t>JAX -7.5</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>0.4677</v>
+        <v>0.4687</v>
       </c>
       <c r="G59" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H59" s="8" t="n">
-        <v>-0.0423</v>
+        <v>-0.0419</v>
       </c>
       <c r="I59" s="8" t="n">
-        <v>-0.101227913867188</v>
+        <v>-0.1051225349379531</v>
       </c>
       <c r="J59" s="10" t="n">
         <v>0.5</v>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -4827,23 +4827,23 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>SEA -3.5</t>
+          <t>DET -7</t>
         </is>
       </c>
       <c r="E60" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4673</v>
+        <v>0.4677</v>
       </c>
       <c r="G60" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H60" s="13" t="n">
-        <v>-0.0425</v>
+        <v>-0.0423</v>
       </c>
       <c r="I60" s="13" t="n">
-        <v>-0.1079692081271329</v>
+        <v>-0.101227913867188</v>
       </c>
       <c r="J60" s="14" t="n">
         <v>0.5</v>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -4868,23 +4868,23 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>JAX -7.5</t>
+          <t>SEA -3.5</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>0.4644</v>
+        <v>0.4673</v>
       </c>
       <c r="G61" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H61" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0425</v>
       </c>
       <c r="I61" s="8" t="n">
-        <v>-0.1135107019949007</v>
+        <v>-0.1079692081271329</v>
       </c>
       <c r="J61" s="10" t="n">
         <v>0.5</v>
@@ -6138,7 +6138,7 @@
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>4.21</v>
+        <v>4.28</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>-3.5</v>
@@ -6342,7 +6342,7 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>7.73</v>
+        <v>7.97</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>-7.5</v>
@@ -24768,7 +24768,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Michael Penix Jr.</t>
+          <t>Tua Tagovailoa</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -24778,17 +24778,17 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Penix (knee) has been cleared to participate in 11-on-11 drills, Marc Raimondi of ESPN.com reports.</t>
+          <t>Tagovailoa's teammate, Michael Penix (knee), is in line to return to 11-on-11 drills in Monday's practice, Will McFadden of the Falcons' official site reports.</t>
         </is>
       </c>
     </row>
@@ -24800,27 +24800,27 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Nick Folk</t>
+          <t>Michael Penix Jr.</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Folk made both of his field-goal attempts and all four PAT tries in Saturday's 34-6 preseason win over the Colts.</t>
+          <t>Penix (knee) has been cleared to participate in 11-on-11 drills, Marc Raimondi of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -24832,12 +24832,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Zachariah Branch</t>
+          <t>Nick Folk</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -24852,7 +24852,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Branch caught two of three targets for 15 yards and added a five-yard punt return in Saturday's 34-6 preseason win over the Colts.</t>
+          <t>Folk made both of his field-goal attempts and all four PAT tries in Saturday's 34-6 preseason win over the Colts.</t>
         </is>
       </c>
     </row>
@@ -24864,12 +24864,12 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Tua Tagovailoa</t>
+          <t>Zachariah Branch</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -24884,7 +24884,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Tagovailoa didn't play in Saturday's 34-6 preseason win over the Colts.</t>
+          <t>Branch caught two of three targets for 15 yards and added a five-yard punt return in Saturday's 34-6 preseason win over the Colts.</t>
         </is>
       </c>
     </row>
@@ -29500,27 +29500,27 @@
       </c>
       <c r="B180" s="5" t="inlineStr">
         <is>
-          <t>Dillon Gabriel</t>
+          <t>Alex Wright</t>
         </is>
       </c>
       <c r="C180" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D180" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F180" s="5" t="inlineStr">
         <is>
-          <t>Gabriel didn't complete his only pass attempt in Saturday's 31-7 preseason loss to the Bills.</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -29532,7 +29532,7 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Deshaun Watson</t>
+          <t>Dillon Gabriel</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -29552,7 +29552,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>Watson completed five of 12 passes for 36 yards, no touchdowns and one interception in Saturday's 31-7 preseason loss to the Bills. He also rushed twice for 13 yards.</t>
+          <t>Gabriel didn't complete his only pass attempt in Saturday's 31-7 preseason loss to the Bills.</t>
         </is>
       </c>
     </row>
@@ -29564,7 +29564,7 @@
       </c>
       <c r="B182" s="5" t="inlineStr">
         <is>
-          <t>Shedeur Sanders</t>
+          <t>Deshaun Watson</t>
         </is>
       </c>
       <c r="C182" s="5" t="inlineStr">
@@ -29584,7 +29584,7 @@
       </c>
       <c r="F182" s="5" t="inlineStr">
         <is>
-          <t>Sanders completed nine of 11 passes for 74 yards, one touchdown and one interception in Saturday's 31-7 preseason loss to the Bills. He also rushed once for two yards.</t>
+          <t>Watson completed five of 12 passes for 36 yards, no touchdowns and one interception in Saturday's 31-7 preseason loss to the Bills. He also rushed twice for 13 yards.</t>
         </is>
       </c>
     </row>
@@ -29596,12 +29596,12 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Isaiah Bond</t>
+          <t>Shedeur Sanders</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
@@ -29616,7 +29616,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>Bond cleared concussion protocol during Saturday's preseason game against the Bills.</t>
+          <t>Sanders completed nine of 11 passes for 74 yards, one touchdown and one interception in Saturday's 31-7 preseason loss to the Bills. He also rushed once for two yards.</t>
         </is>
       </c>
     </row>
@@ -29628,7 +29628,7 @@
       </c>
       <c r="B184" s="5" t="inlineStr">
         <is>
-          <t>Jerry Jeudy</t>
+          <t>Isaiah Bond</t>
         </is>
       </c>
       <c r="C184" s="5" t="inlineStr">
@@ -29648,7 +29648,7 @@
       </c>
       <c r="F184" s="5" t="inlineStr">
         <is>
-          <t>Jeudy will not play in the Browns' preseason game against the Bills on Saturday, Daniel Oyefusi of ESPN.com reports.</t>
+          <t>Bond cleared concussion protocol during Saturday's preseason game against the Bills.</t>
         </is>
       </c>
     </row>
@@ -29660,27 +29660,27 @@
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Alex Wright</t>
+          <t>Jerry Jeudy</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>Wright (lower leg) is not expected to play in Saturday's preseason game against the Bills, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
+          <t>Jeudy will not play in the Browns' preseason game against the Bills on Saturday, Daniel Oyefusi of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -33455,7 +33455,7 @@
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Fracture</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F305" s="4" t="inlineStr">
@@ -34155,7 +34155,7 @@
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F327" s="4" t="inlineStr">
@@ -38996,12 +38996,12 @@
       </c>
       <c r="B480" s="5" t="inlineStr">
         <is>
-          <t>Chris Bell</t>
+          <t>Ronnie Harrison Jr.</t>
         </is>
       </c>
       <c r="C480" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D480" s="5" t="inlineStr">
@@ -39011,12 +39011,12 @@
       </c>
       <c r="E480" s="5" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Hamstring</t>
         </is>
       </c>
       <c r="F480" s="5" t="inlineStr">
         <is>
-          <t>Head coach Jeff Hafley told reporters Saturday that Bell (knee) is "close" to being cleared to fully participate in practice, C. Isaiah Smalls II of the Miami Herald reports.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -39028,27 +39028,27 @@
       </c>
       <c r="B481" s="4" t="inlineStr">
         <is>
-          <t>Kevin Coleman Jr.</t>
+          <t>Trey Moore</t>
         </is>
       </c>
       <c r="C481" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D481" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E481" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Ankle</t>
         </is>
       </c>
       <c r="F481" s="4" t="inlineStr">
         <is>
-          <t>Coleman (undisclosed) caught two of five targets for 32 yards in Saturday's 26-3 preseason loss to the Giants.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -39060,27 +39060,27 @@
       </c>
       <c r="B482" s="5" t="inlineStr">
         <is>
-          <t>James Ester</t>
+          <t>Chris Bell</t>
         </is>
       </c>
       <c r="C482" s="5" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D482" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E482" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F482" s="5" t="inlineStr">
         <is>
-          <t>Ester (undisclosed) reverted to Miami's injured reserve Saturday, Aaron Wilson of KPRC 2 Houston reports.</t>
+          <t>Head coach Jeff Hafley told reporters Saturday that Bell (knee) is "close" to being cleared to fully participate in practice, C. Isaiah Smalls II of the Miami Herald reports.</t>
         </is>
       </c>
     </row>
@@ -39092,27 +39092,27 @@
       </c>
       <c r="B483" s="4" t="inlineStr">
         <is>
-          <t>Ollie Gordon II</t>
+          <t>Kevin Coleman Jr.</t>
         </is>
       </c>
       <c r="C483" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D483" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E483" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F483" s="4" t="inlineStr">
         <is>
-          <t>Gordon exited Miami's preseason game versus the Giants on Sunday with an undisclosed injury, Chris Perkins of the South Florida Sun Sentinel reports.</t>
+          <t>Coleman (undisclosed) caught two of five targets for 32 yards in Saturday's 26-3 preseason loss to the Giants.</t>
         </is>
       </c>
     </row>
@@ -39124,27 +39124,27 @@
       </c>
       <c r="B484" s="5" t="inlineStr">
         <is>
-          <t>Malik Washington</t>
+          <t>James Ester</t>
         </is>
       </c>
       <c r="C484" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D484" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E484" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F484" s="5" t="inlineStr">
         <is>
-          <t>Washington is not playing in Saturday's preseason game against the Giants, C. Isaiah Smalls II of the Miami Herald reports.</t>
+          <t>Ester (undisclosed) reverted to Miami's injured reserve Saturday, Aaron Wilson of KPRC 2 Houston reports.</t>
         </is>
       </c>
     </row>
@@ -39156,27 +39156,27 @@
       </c>
       <c r="B485" s="4" t="inlineStr">
         <is>
-          <t>Malik Willis</t>
+          <t>Ollie Gordon II</t>
         </is>
       </c>
       <c r="C485" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D485" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E485" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F485" s="4" t="inlineStr">
         <is>
-          <t>Willis is not in uniform for Saturday's preseason game against the Giants, David Furones of the South Florida Sun Sentinel reports.</t>
+          <t>Gordon exited Miami's preseason game versus the Giants on Sunday with an undisclosed injury, Chris Perkins of the South Florida Sun Sentinel reports.</t>
         </is>
       </c>
     </row>
@@ -39188,12 +39188,12 @@
       </c>
       <c r="B486" s="5" t="inlineStr">
         <is>
-          <t>De'Von Achane</t>
+          <t>Malik Washington</t>
         </is>
       </c>
       <c r="C486" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D486" s="5" t="inlineStr">
@@ -39208,7 +39208,7 @@
       </c>
       <c r="F486" s="5" t="inlineStr">
         <is>
-          <t>Achane is not in uniform for Saturday's preseason game against the Giants, David Furones of the South Florida Sun Sentinel reports.</t>
+          <t>Washington is not playing in Saturday's preseason game against the Giants, C. Isaiah Smalls II of the Miami Herald reports.</t>
         </is>
       </c>
     </row>
@@ -39220,27 +39220,27 @@
       </c>
       <c r="B487" s="4" t="inlineStr">
         <is>
-          <t>JuJu Brents</t>
+          <t>Malik Willis</t>
         </is>
       </c>
       <c r="C487" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D487" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E487" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F487" s="4" t="inlineStr">
         <is>
-          <t>Brents (undisclosed) is trending in the right direction but did not participate in full-team drills against the Giants on Thursday, Alain Poupart of SI.com reports.</t>
+          <t>Willis is not in uniform for Saturday's preseason game against the Giants, David Furones of the South Florida Sun Sentinel reports.</t>
         </is>
       </c>
     </row>
@@ -39252,27 +39252,27 @@
       </c>
       <c r="B488" s="5" t="inlineStr">
         <is>
-          <t>Ethan Robinson</t>
+          <t>De'Von Achane</t>
         </is>
       </c>
       <c r="C488" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D488" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E488" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F488" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>Achane is not in uniform for Saturday's preseason game against the Giants, David Furones of the South Florida Sun Sentinel reports.</t>
         </is>
       </c>
     </row>
@@ -39284,17 +39284,17 @@
       </c>
       <c r="B489" s="4" t="inlineStr">
         <is>
-          <t>Jamaree Salyer</t>
+          <t>JuJu Brents</t>
         </is>
       </c>
       <c r="C489" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D489" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E489" s="4" t="inlineStr">
@@ -39304,7 +39304,7 @@
       </c>
       <c r="F489" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>Brents (undisclosed) is trending in the right direction but did not participate in full-team drills against the Giants on Thursday, Alain Poupart of SI.com reports.</t>
         </is>
       </c>
     </row>
@@ -39316,17 +39316,17 @@
       </c>
       <c r="B490" s="5" t="inlineStr">
         <is>
-          <t>Zach Sieler</t>
+          <t>Ethan Robinson</t>
         </is>
       </c>
       <c r="C490" s="5" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D490" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E490" s="5" t="inlineStr">
@@ -39336,7 +39336,7 @@
       </c>
       <c r="F490" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -39348,17 +39348,17 @@
       </c>
       <c r="B491" s="4" t="inlineStr">
         <is>
-          <t>Ben Sims</t>
+          <t>Jamaree Salyer</t>
         </is>
       </c>
       <c r="C491" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D491" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E491" s="4" t="inlineStr">
@@ -39368,7 +39368,7 @@
       </c>
       <c r="F491" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -39380,7 +39380,7 @@
       </c>
       <c r="B492" s="5" t="inlineStr">
         <is>
-          <t>Kenneth Grant</t>
+          <t>Zach Sieler</t>
         </is>
       </c>
       <c r="C492" s="5" t="inlineStr">
@@ -39412,12 +39412,12 @@
       </c>
       <c r="B493" s="4" t="inlineStr">
         <is>
-          <t>Lonnie Johnson Jr.</t>
+          <t>Ben Sims</t>
         </is>
       </c>
       <c r="C493" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D493" s="4" t="inlineStr">
@@ -39444,7 +39444,7 @@
       </c>
       <c r="B494" s="5" t="inlineStr">
         <is>
-          <t>Rene Konga</t>
+          <t>Kenneth Grant</t>
         </is>
       </c>
       <c r="C494" s="5" t="inlineStr">
@@ -39454,7 +39454,7 @@
       </c>
       <c r="D494" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E494" s="5" t="inlineStr">
@@ -39464,7 +39464,7 @@
       </c>
       <c r="F494" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -39476,12 +39476,12 @@
       </c>
       <c r="B495" s="4" t="inlineStr">
         <is>
-          <t>Jordyn Brooks</t>
+          <t>Lonnie Johnson Jr.</t>
         </is>
       </c>
       <c r="C495" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D495" s="4" t="inlineStr">
@@ -39508,17 +39508,17 @@
       </c>
       <c r="B496" s="5" t="inlineStr">
         <is>
-          <t>Quinn Ewers</t>
+          <t>Rene Konga</t>
         </is>
       </c>
       <c r="C496" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D496" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E496" s="5" t="inlineStr">
@@ -39528,7 +39528,7 @@
       </c>
       <c r="F496" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -39540,12 +39540,12 @@
       </c>
       <c r="B497" s="4" t="inlineStr">
         <is>
-          <t>Clelin Ferrell</t>
+          <t>Jordyn Brooks</t>
         </is>
       </c>
       <c r="C497" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D497" s="4" t="inlineStr">
@@ -39572,27 +39572,27 @@
       </c>
       <c r="B498" s="5" t="inlineStr">
         <is>
-          <t>Caleb Douglas</t>
+          <t>Quinn Ewers</t>
         </is>
       </c>
       <c r="C498" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D498" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E498" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F498" s="5" t="inlineStr">
         <is>
-          <t>Douglas (lower body) returned to practice Tuesday, David Furones of the South Florida Sun Sentinel reports.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -39604,27 +39604,27 @@
       </c>
       <c r="B499" s="4" t="inlineStr">
         <is>
-          <t>Mark Gronowski</t>
+          <t>Clelin Ferrell</t>
         </is>
       </c>
       <c r="C499" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D499" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E499" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F499" s="4" t="inlineStr">
         <is>
-          <t>The Dolphins signed Gronowski to a contract Sunday.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -39636,12 +39636,12 @@
       </c>
       <c r="B500" s="5" t="inlineStr">
         <is>
-          <t>Greg Dulcich</t>
+          <t>Caleb Douglas</t>
         </is>
       </c>
       <c r="C500" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D500" s="5" t="inlineStr">
@@ -39656,7 +39656,7 @@
       </c>
       <c r="F500" s="5" t="inlineStr">
         <is>
-          <t>Dulcich played 13 snaps on offense but didn't show up in the box score otherwise during the Dolphins' 20-7 preseason loss to the Commanders on Friday.</t>
+          <t>Douglas (lower body) returned to practice Tuesday, David Furones of the South Florida Sun Sentinel reports.</t>
         </is>
       </c>
     </row>
@@ -39668,12 +39668,12 @@
       </c>
       <c r="B501" s="4" t="inlineStr">
         <is>
-          <t>Jaylen Wright</t>
+          <t>Mark Gronowski</t>
         </is>
       </c>
       <c r="C501" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D501" s="4" t="inlineStr">
@@ -39688,7 +39688,7 @@
       </c>
       <c r="F501" s="4" t="inlineStr">
         <is>
-          <t>Wright rushed six times for 22 yards and failed to bring in his only target in the Dolphins' 20-7 preseason loss to the Commanders on Friday. He also returned one kickoff for no gain.</t>
+          <t>The Dolphins signed Gronowski to a contract Sunday.</t>
         </is>
       </c>
     </row>
@@ -39700,12 +39700,12 @@
       </c>
       <c r="B502" s="5" t="inlineStr">
         <is>
-          <t>Jalen Tolbert</t>
+          <t>Greg Dulcich</t>
         </is>
       </c>
       <c r="C502" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D502" s="5" t="inlineStr">
@@ -39720,7 +39720,7 @@
       </c>
       <c r="F502" s="5" t="inlineStr">
         <is>
-          <t>Tolbert secured one of three targets for 27 yards in the Dolphins' 20-7 preseason loss to the Commanders on Friday.</t>
+          <t>Dulcich played 13 snaps on offense but didn't show up in the box score otherwise during the Dolphins' 20-7 preseason loss to the Commanders on Friday.</t>
         </is>
       </c>
     </row>
@@ -39732,12 +39732,12 @@
       </c>
       <c r="B503" s="4" t="inlineStr">
         <is>
-          <t>Tutu Atwell</t>
+          <t>Jaylen Wright</t>
         </is>
       </c>
       <c r="C503" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D503" s="4" t="inlineStr">
@@ -39752,7 +39752,7 @@
       </c>
       <c r="F503" s="4" t="inlineStr">
         <is>
-          <t>Atwell is listed with the second-team offense on the Dolphins' first unofficial depth chart of training camp, David Furones of the South Florida Sun Sentinel reports.</t>
+          <t>Wright rushed six times for 22 yards and failed to bring in his only target in the Dolphins' 20-7 preseason loss to the Commanders on Friday. He also returned one kickoff for no gain.</t>
         </is>
       </c>
     </row>
@@ -39764,12 +39764,12 @@
       </c>
       <c r="B504" s="5" t="inlineStr">
         <is>
-          <t>Caedan Wallace</t>
+          <t>Jalen Tolbert</t>
         </is>
       </c>
       <c r="C504" s="5" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D504" s="5" t="inlineStr">
@@ -39784,7 +39784,7 @@
       </c>
       <c r="F504" s="5" t="inlineStr">
         <is>
-          <t>The Dolphins acquired Wallace from the Patriots on Monday.</t>
+          <t>Tolbert secured one of three targets for 27 yards in the Dolphins' 20-7 preseason loss to the Commanders on Friday.</t>
         </is>
       </c>
     </row>
@@ -40600,7 +40600,7 @@
       </c>
       <c r="F530" s="5" t="inlineStr">
         <is>
-          <t>Morton completed 13 of 17 passes for 129 yards with one touchdown and no interceptions while rushing once for minus-1 yard in the Patriot's 24-21 preseason win over the Eagles on Saturday.</t>
+          <t>Morton completed 13 of 17 passes for 129 yards with one touchdown and no interceptions while rushing once for minus-1 yard in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
         </is>
       </c>
     </row>
@@ -46148,12 +46148,12 @@
       </c>
       <c r="B705" s="4" t="inlineStr">
         <is>
-          <t>Julian Hicks</t>
+          <t>Jadarian Price</t>
         </is>
       </c>
       <c r="C705" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D705" s="4" t="inlineStr">
@@ -46168,7 +46168,7 @@
       </c>
       <c r="F705" s="4" t="inlineStr">
         <is>
-          <t>The Seahawks signed Hicks to a contract Saturday, John Boyle of the team's official site reports.</t>
+          <t>Price will not play in Sunday's preseason game against the Titans, Gregg Bell of The Tacoma News Tribune reports.</t>
         </is>
       </c>
     </row>
@@ -46180,7 +46180,7 @@
       </c>
       <c r="B706" s="5" t="inlineStr">
         <is>
-          <t>Jake Bobo</t>
+          <t>Julian Hicks</t>
         </is>
       </c>
       <c r="C706" s="5" t="inlineStr">
@@ -46190,17 +46190,17 @@
       </c>
       <c r="D706" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E706" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F706" s="5" t="inlineStr">
         <is>
-          <t>The Seahawks placed Bobo (knee) on injured reserve Saturday, John Boyle of the team's official site reports.</t>
+          <t>The Seahawks signed Hicks to a contract Saturday, John Boyle of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -46212,27 +46212,27 @@
       </c>
       <c r="B707" s="4" t="inlineStr">
         <is>
-          <t>Trevon Diggs</t>
+          <t>Jake Bobo</t>
         </is>
       </c>
       <c r="C707" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D707" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E707" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F707" s="4" t="inlineStr">
         <is>
-          <t>The Seahawks are slated to sign Diggs to a one-year deal, Adam Schefter of ESPN reports.</t>
+          <t>The Seahawks placed Bobo (knee) on injured reserve Saturday, John Boyle of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -46244,27 +46244,27 @@
       </c>
       <c r="B708" s="5" t="inlineStr">
         <is>
-          <t>Joseph Vaughn</t>
+          <t>Trevon Diggs</t>
         </is>
       </c>
       <c r="C708" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D708" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E708" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F708" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>The Seahawks are slated to sign Diggs to a one-year deal, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -46276,17 +46276,17 @@
       </c>
       <c r="B709" s="4" t="inlineStr">
         <is>
-          <t>Emanuel Wilson</t>
+          <t>Joseph Vaughn</t>
         </is>
       </c>
       <c r="C709" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D709" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E709" s="4" t="inlineStr">
@@ -46296,7 +46296,7 @@
       </c>
       <c r="F709" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -46308,17 +46308,17 @@
       </c>
       <c r="B710" s="5" t="inlineStr">
         <is>
-          <t>Robbie Ouzts</t>
+          <t>Emanuel Wilson</t>
         </is>
       </c>
       <c r="C710" s="5" t="inlineStr">
         <is>
-          <t>FB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D710" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E710" s="5" t="inlineStr">
@@ -46328,7 +46328,7 @@
       </c>
       <c r="F710" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -46340,27 +46340,27 @@
       </c>
       <c r="B711" s="4" t="inlineStr">
         <is>
-          <t>Tory Horton</t>
+          <t>Robbie Ouzts</t>
         </is>
       </c>
       <c r="C711" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>FB</t>
         </is>
       </c>
       <c r="D711" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E711" s="4" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F711" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -46372,27 +46372,27 @@
       </c>
       <c r="B712" s="5" t="inlineStr">
         <is>
-          <t>Shemar Jean-Charles</t>
+          <t>Tory Horton</t>
         </is>
       </c>
       <c r="C712" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D712" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E712" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Undisclosed</t>
         </is>
       </c>
       <c r="F712" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -46404,27 +46404,27 @@
       </c>
       <c r="B713" s="4" t="inlineStr">
         <is>
-          <t>Nick Emmanwori</t>
+          <t>Shemar Jean-Charles</t>
         </is>
       </c>
       <c r="C713" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D713" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E713" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F713" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -46436,27 +46436,27 @@
       </c>
       <c r="B714" s="5" t="inlineStr">
         <is>
-          <t>Anthony Hankerson</t>
+          <t>Nick Emmanwori</t>
         </is>
       </c>
       <c r="C714" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D714" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E714" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F714" s="5" t="inlineStr">
         <is>
-          <t>Hankerson and the Seahawks agreed on a contract Monday, John Boyle of the team's official website reports.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -46468,7 +46468,7 @@
       </c>
       <c r="B715" s="4" t="inlineStr">
         <is>
-          <t>Jadarian Price</t>
+          <t>Anthony Hankerson</t>
         </is>
       </c>
       <c r="C715" s="4" t="inlineStr">
@@ -46488,7 +46488,7 @@
       </c>
       <c r="F715" s="4" t="inlineStr">
         <is>
-          <t>Price (lower body) participated fully in Monday's practice, Bob Condotta of The Seattle Times reports.</t>
+          <t>Hankerson and the Seahawks agreed on a contract Monday, John Boyle of the team's official website reports.</t>
         </is>
       </c>
     </row>
@@ -49424,13 +49424,13 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>82.7</v>
+        <v>83.2</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>5.6</v>
+        <v>6.7</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>12.1</v>
+        <v>13.2</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>0</v>
@@ -49471,7 +49471,7 @@
         <v>20.6</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -49513,7 +49513,7 @@
         <v>9.4</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -49631,7 +49631,7 @@
         <v>6.9</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -49669,7 +49669,7 @@
         <v>14.3</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -49711,7 +49711,7 @@
         <v>13.2</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -49749,7 +49749,7 @@
         <v>12.3</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
         <v>12.8</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -49795,11 +49795,11 @@
         </is>
       </c>
       <c r="I14" s="22" t="n">
-        <v>-1.5</v>
+        <v>-0.5</v>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>61% chance of rain · 93°F</t>
+          <t>93°F</t>
         </is>
       </c>
     </row>
@@ -49829,7 +49829,7 @@
         <v>9.4</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -49867,7 +49867,7 @@
         <v>19</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
@@ -49909,7 +49909,7 @@
         <v>10.5</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -49989,7 +49989,7 @@
         <v>21</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
@@ -50031,7 +50031,7 @@
         <v>7.2</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh: 2026-08-23 19:57 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -689,7 +689,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-23T19:56:25+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-23T19:57:37+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23T19:56:25+00:00</t>
+          <t>2026-08-23T19:57:37+00:00</t>
         </is>
       </c>
     </row>
@@ -2609,19 +2609,19 @@
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>-112</v>
+        <v>-108</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5888</v>
+        <v>0.5858</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.5283</v>
+        <v>0.5192</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>0.044</v>
+        <v>0.046</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>0.1145574022904216</v>
+        <v>0.1281919050894967</v>
       </c>
       <c r="J6" s="14" t="n">
         <v>0.15</v>
@@ -2727,28 +2727,28 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>SEA ML</t>
+          <t>SEA +3.5</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>164</v>
+        <v>-105</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.4136</v>
+        <v>0.5502</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.3788</v>
+        <v>0.5122</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>0.0308</v>
+        <v>0.0329</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.09120300354675681</v>
+        <v>0.07419026293050812</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>0.15</v>
@@ -2772,28 +2772,28 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>SEA +4.5</t>
+          <t>SEA ML</t>
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>-115</v>
+        <v>154</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5668</v>
+        <v>0.4307</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.3937</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>0.0288</v>
+        <v>0.0323</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>0.05970271346067979</v>
+        <v>0.0930713376416743</v>
       </c>
       <c r="J10" s="14" t="n">
         <v>0.15</v>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3109,23 +3109,23 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>CAR ML</t>
+          <t>NE ML</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4611</v>
+        <v>0.4102</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.4464</v>
+        <v>0.3937</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.0143</v>
+        <v>0.016</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.0325138851490685</v>
+        <v>0.04157344040829225</v>
       </c>
       <c r="J18" s="14" t="n">
         <v>0.5</v>
@@ -3140,33 +3140,33 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>CAR ML</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>-105</v>
+        <v>124</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.5266999999999999</v>
+        <v>0.4611</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.4464</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.0141</v>
+        <v>0.0143</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.02824070440763249</v>
+        <v>0.0325138851490685</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>0.5</v>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -3191,23 +3191,23 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Over 40.5</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E20" s="12" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.538</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>0.0139</v>
+        <v>0.0141</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>0.02712503029680507</v>
+        <v>0.02824070440763249</v>
       </c>
       <c r="J20" s="14" t="n">
         <v>0.5</v>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -3232,23 +3232,23 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>Over 40.5</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>0.5241</v>
+        <v>0.538</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>0.0118</v>
+        <v>0.0139</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>0.02330043912717339</v>
+        <v>0.02712503029680507</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>0.5</v>
@@ -3263,33 +3263,33 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>CLE +7.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="E22" s="12" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5353</v>
+        <v>0.5241</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>0.0113</v>
+        <v>0.0118</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>0.02190365162224267</v>
+        <v>0.02330043912717339</v>
       </c>
       <c r="J22" s="14" t="n">
         <v>0.5</v>
@@ -3304,33 +3304,33 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>NO ML</t>
+          <t>CLE +7.5</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>250</v>
+        <v>-110</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0.2972</v>
+        <v>0.5353</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>0.2857</v>
+        <v>0.5238</v>
       </c>
       <c r="H23" s="8" t="n">
         <v>0.0113</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>0.03991163697142053</v>
+        <v>0.02190365162224267</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>0.5</v>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -3355,23 +3355,23 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>NE ML</t>
+          <t>NO ML</t>
         </is>
       </c>
       <c r="E24" s="12" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4111</v>
+        <v>0.2972</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.4</v>
+        <v>0.2857</v>
       </c>
       <c r="H24" s="13" t="n">
-        <v>0.0109</v>
+        <v>0.0113</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>0.02741697578924818</v>
+        <v>0.03991163697142053</v>
       </c>
       <c r="J24" s="14" t="n">
         <v>0.5</v>
@@ -3386,33 +3386,33 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>CAR +2.5</t>
+          <t>SF ML</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>-102</v>
+        <v>160</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>0.5141</v>
+        <v>0.3952</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>0.505</v>
+        <v>0.3846</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0105</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.0180591736369381</v>
+        <v>0.02738011685610797</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>0.5</v>
@@ -3444,16 +3444,16 @@
         <v>-110</v>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5327</v>
+        <v>0.534</v>
       </c>
       <c r="G26" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>0.0089</v>
+        <v>0.0101</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>0.01706011721804213</v>
+        <v>0.01944210719035699</v>
       </c>
       <c r="J26" s="14" t="n">
         <v>0.5</v>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -3478,23 +3478,23 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>NO +7</t>
+          <t>CAR +2.5</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.5323</v>
+        <v>0.5141</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.505</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.01531241952910156</v>
+        <v>0.0180591736369381</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>0.5</v>
@@ -3509,33 +3509,33 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>BAL @ IND</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>IND ML</t>
+          <t>NO +7</t>
         </is>
       </c>
       <c r="E28" s="12" t="n">
-        <v>150</v>
+        <v>-110</v>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4077</v>
+        <v>0.5323</v>
       </c>
       <c r="G28" s="13" t="n">
-        <v>0.4</v>
+        <v>0.5238</v>
       </c>
       <c r="H28" s="13" t="n">
-        <v>0.0076</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>0.0189591996912486</v>
+        <v>0.01531241952910156</v>
       </c>
       <c r="J28" s="14" t="n">
         <v>0.5</v>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>BAL @ IND</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -3560,23 +3560,23 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>SF ML</t>
+          <t>IND ML</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>0.3966</v>
+        <v>0.4077</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.3937</v>
+        <v>0.4</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.0029</v>
+        <v>0.0076</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.007300801423401726</v>
+        <v>0.0189591996912486</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>0.5</v>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -3765,23 +3765,23 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>WSH +4.5</t>
+          <t>SF +3.5</t>
         </is>
       </c>
       <c r="E34" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5209</v>
+        <v>0.522</v>
       </c>
       <c r="G34" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H34" s="13" t="n">
-        <v>-0.0029</v>
+        <v>-0.0018</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.00557688940705281</v>
+        <v>-0.003423344769942216</v>
       </c>
       <c r="J34" s="14" t="n">
         <v>0.5</v>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3806,23 +3806,23 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>SF +3.5</t>
+          <t>WSH +4.5</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.5204</v>
+        <v>0.5209</v>
       </c>
       <c r="G35" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>-0.0034</v>
+        <v>-0.0029</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>-0.006504965748980907</v>
+        <v>-0.00557688940705281</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>0.5</v>
@@ -4387,16 +4387,16 @@
         <v>130</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>0.4165</v>
+        <v>0.4163</v>
       </c>
       <c r="G49" s="8" t="n">
         <v>0.4348</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>-0.0176</v>
+        <v>-0.0178</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>-0.04170524916936713</v>
+        <v>-0.04211347125206366</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>0.5</v>
@@ -4428,16 +4428,16 @@
         <v>-105</v>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4929</v>
+        <v>0.4931</v>
       </c>
       <c r="G50" s="13" t="n">
         <v>0.5122</v>
       </c>
       <c r="H50" s="13" t="n">
-        <v>-0.0185</v>
+        <v>-0.0184</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>-0.03491941307422497</v>
+        <v>-0.03456897245401863</v>
       </c>
       <c r="J50" s="14" t="n">
         <v>0.5</v>
@@ -4674,16 +4674,16 @@
         <v>-155</v>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5835</v>
+        <v>0.5837</v>
       </c>
       <c r="G56" s="13" t="n">
         <v>0.6078</v>
       </c>
       <c r="H56" s="13" t="n">
-        <v>-0.0229</v>
+        <v>-0.0227</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>-0.03967882301045061</v>
+        <v>-0.0393869186590014</v>
       </c>
       <c r="J56" s="14" t="n">
         <v>0.5</v>
@@ -5002,16 +5002,16 @@
         <v>-115</v>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.5071</v>
+        <v>0.5069</v>
       </c>
       <c r="G64" s="13" t="n">
         <v>0.5349</v>
       </c>
       <c r="H64" s="13" t="n">
-        <v>-0.0257</v>
+        <v>-0.0258</v>
       </c>
       <c r="I64" s="13" t="n">
-        <v>-0.04823004570995831</v>
+        <v>-0.04856547434225605</v>
       </c>
       <c r="J64" s="14" t="n">
         <v>0.5</v>
@@ -5518,33 +5518,33 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>LAR -3.5</t>
+          <t>LV ML</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
-        <v>-110</v>
+        <v>-205</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>0.4796</v>
+        <v>0.6278</v>
       </c>
       <c r="G77" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6721</v>
       </c>
       <c r="H77" s="8" t="n">
-        <v>-0.0366</v>
+        <v>-0.0367</v>
       </c>
       <c r="I77" s="8" t="n">
-        <v>-0.08440412516010987</v>
+        <v>-0.06538038662822776</v>
       </c>
       <c r="J77" s="10" t="n">
         <v>0.5</v>
@@ -5559,33 +5559,33 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>LV ML</t>
+          <t>PHI -4.5</t>
         </is>
       </c>
       <c r="E78" s="12" t="n">
-        <v>-205</v>
+        <v>-110</v>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.6278</v>
+        <v>0.4791</v>
       </c>
       <c r="G78" s="13" t="n">
-        <v>0.6721</v>
+        <v>0.5238</v>
       </c>
       <c r="H78" s="13" t="n">
-        <v>-0.0367</v>
+        <v>-0.0369</v>
       </c>
       <c r="I78" s="13" t="n">
-        <v>-0.06538038662822776</v>
+        <v>-0.08533220150203796</v>
       </c>
       <c r="J78" s="14" t="n">
         <v>0.5</v>
@@ -5600,7 +5600,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -5610,23 +5610,23 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>PHI -4.5</t>
+          <t>LAR -3.5</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>0.4791</v>
+        <v>0.478</v>
       </c>
       <c r="G79" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H79" s="8" t="n">
-        <v>-0.0369</v>
+        <v>-0.0375</v>
       </c>
       <c r="I79" s="8" t="n">
-        <v>-0.08533220150203796</v>
+        <v>-0.08748574613914867</v>
       </c>
       <c r="J79" s="10" t="n">
         <v>0.5</v>
@@ -5641,33 +5641,33 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>LAR ML</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E80" s="12" t="n">
-        <v>-185</v>
+        <v>-110</v>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.6034</v>
+        <v>0.4771</v>
       </c>
       <c r="G80" s="13" t="n">
-        <v>0.6491</v>
+        <v>0.5238</v>
       </c>
       <c r="H80" s="13" t="n">
-        <v>-0.0375</v>
+        <v>-0.038</v>
       </c>
       <c r="I80" s="13" t="n">
-        <v>-0.06982294310384429</v>
+        <v>-0.08908584867374703</v>
       </c>
       <c r="J80" s="14" t="n">
         <v>0.5</v>
@@ -5682,33 +5682,33 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>BAL @ IND</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>BAL -3.5</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>0.4771</v>
+        <v>0.4691</v>
       </c>
       <c r="G81" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5192</v>
       </c>
       <c r="H81" s="8" t="n">
-        <v>-0.038</v>
+        <v>-0.0397</v>
       </c>
       <c r="I81" s="8" t="n">
-        <v>-0.08908584867374703</v>
+        <v>-0.09649040432769079</v>
       </c>
       <c r="J81" s="10" t="n">
         <v>0.5</v>
@@ -5728,28 +5728,28 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>BAL -3.5</t>
+          <t>BAL ML</t>
         </is>
       </c>
       <c r="E82" s="12" t="n">
-        <v>-108</v>
+        <v>-180</v>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.4691</v>
+        <v>0.5923</v>
       </c>
       <c r="G82" s="13" t="n">
-        <v>0.5192</v>
+        <v>0.6429</v>
       </c>
       <c r="H82" s="13" t="n">
-        <v>-0.0397</v>
+        <v>-0.0399</v>
       </c>
       <c r="I82" s="13" t="n">
-        <v>-0.09649040432769079</v>
+        <v>-0.07787638073675418</v>
       </c>
       <c r="J82" s="14" t="n">
         <v>0.5</v>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>BAL @ IND</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -5774,23 +5774,23 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>BAL ML</t>
+          <t>LAR ML</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
-        <v>-180</v>
+        <v>-192</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>0.5923</v>
+        <v>0.6048</v>
       </c>
       <c r="G83" s="8" t="n">
-        <v>0.6429</v>
+        <v>0.6575</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>-0.0399</v>
+        <v>-0.0409</v>
       </c>
       <c r="I83" s="8" t="n">
-        <v>-0.07787638073675418</v>
+        <v>-0.07955712205271259</v>
       </c>
       <c r="J83" s="10" t="n">
         <v>0.5</v>
@@ -5846,33 +5846,33 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>SEA ML</t>
+          <t>CHI -2.5</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
-        <v>-180</v>
+        <v>-118</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>0.5889</v>
+        <v>0.4859</v>
       </c>
       <c r="G85" s="8" t="n">
-        <v>0.6429</v>
+        <v>0.5413</v>
       </c>
       <c r="H85" s="8" t="n">
-        <v>-0.0414</v>
+        <v>-0.042</v>
       </c>
       <c r="I85" s="8" t="n">
-        <v>-0.08313747713867009</v>
+        <v>-0.1022639614444939</v>
       </c>
       <c r="J85" s="10" t="n">
         <v>0.5</v>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -5897,23 +5897,23 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>CHI -2.5</t>
+          <t>DET -7</t>
         </is>
       </c>
       <c r="E86" s="12" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.4859</v>
+        <v>0.4677</v>
       </c>
       <c r="G86" s="13" t="n">
-        <v>0.5413</v>
+        <v>0.5238</v>
       </c>
       <c r="H86" s="13" t="n">
-        <v>-0.042</v>
+        <v>-0.0423</v>
       </c>
       <c r="I86" s="13" t="n">
-        <v>-0.1022639614444939</v>
+        <v>-0.101227913867188</v>
       </c>
       <c r="J86" s="14" t="n">
         <v>0.5</v>
@@ -5928,7 +5928,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -5938,23 +5938,23 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>DET -7</t>
+          <t>SEA -3.5</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>0.4677</v>
+        <v>0.466</v>
       </c>
       <c r="G87" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H87" s="8" t="n">
-        <v>-0.0423</v>
+        <v>-0.043</v>
       </c>
       <c r="I87" s="8" t="n">
-        <v>-0.101227913867188</v>
+        <v>-0.1103511980994479</v>
       </c>
       <c r="J87" s="10" t="n">
         <v>0.5</v>
@@ -5969,33 +5969,33 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>SEA -3.5</t>
+          <t>CHI ML</t>
         </is>
       </c>
       <c r="E88" s="12" t="n">
-        <v>-110</v>
+        <v>-148</v>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.4673</v>
+        <v>0.5389</v>
       </c>
       <c r="G88" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5968</v>
       </c>
       <c r="H88" s="13" t="n">
-        <v>-0.0425</v>
+        <v>-0.043</v>
       </c>
       <c r="I88" s="13" t="n">
-        <v>-0.1079692081271329</v>
+        <v>-0.09606695185565578</v>
       </c>
       <c r="J88" s="14" t="n">
         <v>0.5</v>
@@ -6015,28 +6015,28 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>CHI ML</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
-        <v>-148</v>
+        <v>-115</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>0.5389</v>
+        <v>0.4759</v>
       </c>
       <c r="G89" s="8" t="n">
-        <v>0.5968</v>
+        <v>0.5349</v>
       </c>
       <c r="H89" s="8" t="n">
-        <v>-0.043</v>
+        <v>-0.0435</v>
       </c>
       <c r="I89" s="8" t="n">
-        <v>-0.09606695185565578</v>
+        <v>-0.1103290525258087</v>
       </c>
       <c r="J89" s="10" t="n">
         <v>0.5</v>
@@ -6051,33 +6051,33 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>JAX -7.5</t>
         </is>
       </c>
       <c r="E90" s="12" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.4759</v>
+        <v>0.4647</v>
       </c>
       <c r="G90" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H90" s="13" t="n">
         <v>-0.0435</v>
       </c>
       <c r="I90" s="13" t="n">
-        <v>-0.1103290525258087</v>
+        <v>-0.1128127425313334</v>
       </c>
       <c r="J90" s="14" t="n">
         <v>0.5</v>
@@ -6092,33 +6092,33 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>JAX -7.5</t>
+          <t>SEA ML</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>-110</v>
+        <v>-185</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>0.4647</v>
+        <v>0.5898</v>
       </c>
       <c r="G91" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6491</v>
       </c>
       <c r="H91" s="8" t="n">
-        <v>-0.0435</v>
+        <v>-0.0436</v>
       </c>
       <c r="I91" s="8" t="n">
-        <v>-0.1128127425313334</v>
+        <v>-0.09060324316118262</v>
       </c>
       <c r="J91" s="10" t="n">
         <v>0.5</v>
@@ -6469,42 +6469,38 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>SEA @ TEN</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>TEN ML</t>
+          <t>Over 51.5</t>
         </is>
       </c>
       <c r="E100" s="12" t="n">
-        <v>-198</v>
+        <v>-110</v>
       </c>
       <c r="F100" s="13" t="n">
-        <v>0.5864</v>
+        <v>0.4445</v>
       </c>
       <c r="G100" s="13" t="n">
-        <v>0.6644</v>
+        <v>0.5238</v>
       </c>
       <c r="H100" s="13" t="n">
-        <v>-0.0489</v>
+        <v>-0.0492</v>
       </c>
       <c r="I100" s="13" t="n">
-        <v>-0.1164607636337045</v>
+        <v>-0.1514496874157239</v>
       </c>
       <c r="J100" s="14" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K100" s="5" t="inlineStr">
-        <is>
-          <t>Preseason — priced for reference only. Preseason results are decided by how long the starters played, which no rating model sees.</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="K100" s="5" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -6519,28 +6515,28 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>TEN -4.5</t>
+          <t>TEN ML</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
-        <v>-105</v>
+        <v>-185</v>
       </c>
       <c r="F101" s="8" t="n">
-        <v>0.4332</v>
+        <v>0.5693</v>
       </c>
       <c r="G101" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.6491</v>
       </c>
       <c r="H101" s="8" t="n">
-        <v>-0.0491</v>
+        <v>-0.0493</v>
       </c>
       <c r="I101" s="8" t="n">
-        <v>-0.1542631880325815</v>
+        <v>-0.1218307247308589</v>
       </c>
       <c r="J101" s="10" t="n">
         <v>0.15</v>
@@ -6559,38 +6555,42 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>SEA @ TEN</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Over 51.5</t>
+          <t>TEN -3.5</t>
         </is>
       </c>
       <c r="E102" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F102" s="13" t="n">
-        <v>0.4445</v>
+        <v>0.4498</v>
       </c>
       <c r="G102" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H102" s="13" t="n">
-        <v>-0.0492</v>
+        <v>-0.0502</v>
       </c>
       <c r="I102" s="13" t="n">
-        <v>-0.1514496874157239</v>
+        <v>-0.1590602411731166</v>
       </c>
       <c r="J102" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K102" s="5" t="inlineStr"/>
+        <v>0.15</v>
+      </c>
+      <c r="K102" s="5" t="inlineStr">
+        <is>
+          <t>Preseason — priced for reference only. Preseason results are decided by how long the starters played, which no rating model sees.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>SEA @ TEN</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -6692,32 +6692,28 @@
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Under 37.5</t>
+          <t>Under 38.5</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="F105" s="8" t="n">
-        <v>0.4112</v>
+        <v>0.4041</v>
       </c>
       <c r="G105" s="8" t="n">
-        <v>0.5192</v>
+        <v>0.5122</v>
       </c>
       <c r="H105" s="8" t="n">
         <v>-0.0529</v>
       </c>
       <c r="I105" s="8" t="n">
-        <v>-0.2081031290949362</v>
+        <v>-0.2109934210059127</v>
       </c>
       <c r="J105" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K105" s="4" t="inlineStr">
-        <is>
-          <t>Preseason — priced for reference only. Preseason results are decided by how long the starters played, which no rating model sees.</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="K105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -6727,7 +6723,7 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>SEA @ TEN</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
@@ -6737,28 +6733,32 @@
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>Under 38.5</t>
+          <t>Under 37.5</t>
         </is>
       </c>
       <c r="E106" s="12" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="F106" s="13" t="n">
-        <v>0.4041</v>
+        <v>0.4142</v>
       </c>
       <c r="G106" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5283</v>
       </c>
       <c r="H106" s="13" t="n">
-        <v>-0.0529</v>
+        <v>-0.0533</v>
       </c>
       <c r="I106" s="13" t="n">
-        <v>-0.2109934210059127</v>
+        <v>-0.2159633352905699</v>
       </c>
       <c r="J106" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K106" s="5" t="inlineStr"/>
+        <v>0.15</v>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>Preseason — priced for reference only. Preseason results are decided by how long the starters played, which no rating model sees.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>3</v>
+        <v>3.01</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>-3</v>
@@ -7913,7 +7913,7 @@
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>3.34</v>
+        <v>3.25</v>
       </c>
       <c r="E22" s="9" t="n">
         <v>-3.5</v>
@@ -7947,7 +7947,7 @@
         </is>
       </c>
       <c r="D23" s="22" t="n">
-        <v>2.65</v>
+        <v>2.58</v>
       </c>
       <c r="E23" s="22" t="n">
         <v>-3.5</v>
@@ -7981,10 +7981,10 @@
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>2.11</v>
+        <v>1.45</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>-4.5</v>
+        <v>-3.5</v>
       </c>
       <c r="F24" s="11" t="n">
         <v>41</v>
@@ -8132,7 +8132,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>3.76</v>
+        <v>3.75</v>
       </c>
       <c r="E5" s="16" t="n">
         <v>2.9</v>
@@ -8164,7 +8164,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>3.07</v>
+        <v>2.93</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>2.35</v>
@@ -8260,7 +8260,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>2.12</v>
+        <v>2.13</v>
       </c>
       <c r="E9" s="16" t="n">
         <v>-1.33</v>
@@ -8445,20 +8445,20 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>1.79</v>
+        <v>1.81</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>-1.14</v>
+        <v>-0.01</v>
       </c>
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="11" t="n"/>
@@ -8477,20 +8477,20 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="C16" s="12" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>1.67</v>
+        <v>1.79</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>0.64</v>
+        <v>0.61</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>-0.01</v>
+        <v>-1.14</v>
       </c>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="23" t="n"/>
@@ -8548,7 +8548,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="18" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="E18" s="18" t="n">
         <v>-0.24</v>
@@ -8644,7 +8644,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="E21" s="16" t="n">
         <v>1.87</v>
@@ -8868,7 +8868,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="18" t="n">
-        <v>-1.86</v>
+        <v>-1.87</v>
       </c>
       <c r="E28" s="18" t="n">
         <v>-1.28</v>
@@ -8932,7 +8932,7 @@
         <v>0</v>
       </c>
       <c r="D30" s="18" t="n">
-        <v>-2.32</v>
+        <v>-2.31</v>
       </c>
       <c r="E30" s="18" t="n">
         <v>-0.52</v>
@@ -9028,7 +9028,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>-3.24</v>
+        <v>-3.23</v>
       </c>
       <c r="E33" s="16" t="n">
         <v>-2.1</v>
@@ -9092,7 +9092,7 @@
         <v>0</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>-4.7</v>
+        <v>-4.69</v>
       </c>
       <c r="E35" s="16" t="n">
         <v>-1.02</v>
@@ -10726,16 +10726,16 @@
         </is>
       </c>
       <c r="G37" s="9" t="n">
-        <v>-4.5</v>
+        <v>-3.5</v>
       </c>
       <c r="H37" s="11" t="n">
         <v>37.5</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>-198</v>
+        <v>-185</v>
       </c>
       <c r="K37" s="15" t="n">
         <v>0</v>
@@ -11505,10 +11505,10 @@
         <v>44.5</v>
       </c>
       <c r="I54" s="12" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="J54" s="12" t="n">
-        <v>-180</v>
+        <v>-185</v>
       </c>
       <c r="K54" s="17" t="n">
         <v>0</v>
@@ -11558,10 +11558,10 @@
         <v>48.5</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>-185</v>
+        <v>-192</v>
       </c>
       <c r="K55" s="15" t="n">
         <v>0</v>
@@ -12936,10 +12936,10 @@
         <v>46.5</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="J81" s="7" t="n">
-        <v>-700</v>
+        <v>-675</v>
       </c>
       <c r="K81" s="15" t="n">
         <v>0</v>
@@ -18446,10 +18446,10 @@
         <v>46.5</v>
       </c>
       <c r="I185" s="7" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="J185" s="7" t="n">
-        <v>-440</v>
+        <v>-425</v>
       </c>
       <c r="K185" s="15" t="n">
         <v>0</v>
@@ -20772,7 +20772,7 @@
         </is>
       </c>
       <c r="G229" s="9" t="n">
-        <v>1.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H229" s="11" t="n">
         <v>46.5</v>
@@ -21043,10 +21043,10 @@
         <v>47.5</v>
       </c>
       <c r="I234" s="12" t="n">
-        <v>-166</v>
+        <v>-162</v>
       </c>
       <c r="J234" s="12" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="K234" s="17" t="n">
         <v>0</v>
@@ -25707,10 +25707,10 @@
         <v>44.5</v>
       </c>
       <c r="I322" s="12" t="n">
-        <v>-425</v>
+        <v>-410</v>
       </c>
       <c r="J322" s="12" t="n">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="K322" s="17" t="n">
         <v>0</v>
@@ -51958,10 +51958,10 @@
         <v>83</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>13.2</v>
+        <v>11.6</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Refresh: 2026-08-23 20:52 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -689,7 +689,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-23T19:57:37+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-23T20:52:05+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23T19:57:37+00:00</t>
+          <t>2026-08-23T20:52:05+00:00</t>
         </is>
       </c>
     </row>
@@ -8449,7 +8449,7 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>1.81</v>
@@ -8481,7 +8481,7 @@
         </is>
       </c>
       <c r="C16" s="12" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D16" s="18" t="n">
         <v>1.79</v>
@@ -32027,27 +32027,27 @@
       </c>
       <c r="B180" s="5" t="inlineStr">
         <is>
-          <t>Alex Wright</t>
+          <t>Shedeur Sanders</t>
         </is>
       </c>
       <c r="C180" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D180" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F180" s="5" t="inlineStr">
         <is>
-          <t>The Browns placed Wright on injured reserve Sunday due to a ruptured Achilles, Adam Schefter of ESPN reports.</t>
+          <t>Sanders will learn Monday if he or Deshaun Watson will start at quarterback for the Browns, Jeremy Fowler of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -32059,12 +32059,12 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Derek Barnett</t>
+          <t>Deshaun Watson</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
@@ -32079,7 +32079,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>Barnett and the Browns agreed to a one-year contract worth up to $5.5 million Sunday, Jeremy Fowler of ESPN.com reports.</t>
+          <t>Watson will learn Monday if he or Shedeur Sanders will be named starting quarterback for the Browns, Jeremy Fowler of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -32091,27 +32091,27 @@
       </c>
       <c r="B182" s="5" t="inlineStr">
         <is>
-          <t>Dillon Gabriel</t>
+          <t>Alex Wright</t>
         </is>
       </c>
       <c r="C182" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D182" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E182" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F182" s="5" t="inlineStr">
         <is>
-          <t>Gabriel didn't complete his only pass attempt in Saturday's 31-7 preseason loss to the Bills.</t>
+          <t>The Browns placed Wright on injured reserve Sunday due to a ruptured Achilles, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -32123,12 +32123,12 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Deshaun Watson</t>
+          <t>Derek Barnett</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
@@ -32143,7 +32143,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>Watson completed five of 12 passes for 36 yards, no touchdowns and one interception in Saturday's 31-7 preseason loss to the Bills. He also rushed twice for 13 yards.</t>
+          <t>Barnett and the Browns agreed to a one-year contract worth up to $5.5 million Sunday, Jeremy Fowler of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -32155,7 +32155,7 @@
       </c>
       <c r="B184" s="5" t="inlineStr">
         <is>
-          <t>Shedeur Sanders</t>
+          <t>Dillon Gabriel</t>
         </is>
       </c>
       <c r="C184" s="5" t="inlineStr">
@@ -32175,7 +32175,7 @@
       </c>
       <c r="F184" s="5" t="inlineStr">
         <is>
-          <t>Sanders completed nine of 11 passes for 74 yards, one touchdown and one interception in Saturday's 31-7 preseason loss to the Bills. He also rushed once for two yards.</t>
+          <t>Gabriel didn't complete his only pass attempt in Saturday's 31-7 preseason loss to the Bills.</t>
         </is>
       </c>
     </row>
@@ -44703,12 +44703,12 @@
       </c>
       <c r="B580" s="5" t="inlineStr">
         <is>
-          <t>Joshua Ezeudu</t>
+          <t>Malik Nabers</t>
         </is>
       </c>
       <c r="C580" s="5" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D580" s="5" t="inlineStr">
@@ -44718,12 +44718,12 @@
       </c>
       <c r="E580" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F580" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Giants coach John Harbaugh said Sunday that Nabers (knee) could be out of his red non-contact jersey at some point this week, Evan Barnes of Newsday reports.</t>
         </is>
       </c>
     </row>
@@ -44735,12 +44735,12 @@
       </c>
       <c r="B581" s="4" t="inlineStr">
         <is>
-          <t>Braxton Berrios</t>
+          <t>Joshua Ezeudu</t>
         </is>
       </c>
       <c r="C581" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D581" s="4" t="inlineStr">
@@ -44755,7 +44755,7 @@
       </c>
       <c r="F581" s="4" t="inlineStr">
         <is>
-          <t>Head coach John Harbaugh told reporters that Berrios did not play in Saturday's 26-3 preseason win over the Dolphins due to a soft-tissue issue, Paul Schwartz of the New York Post reports.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -44767,27 +44767,27 @@
       </c>
       <c r="B582" s="5" t="inlineStr">
         <is>
-          <t>Theo Johnson</t>
+          <t>Braxton Berrios</t>
         </is>
       </c>
       <c r="C582" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D582" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E582" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F582" s="5" t="inlineStr">
         <is>
-          <t>Johnson caught his only target for 12 yards in Saturday's 26-3 preseason win over the Dolphins.</t>
+          <t>Head coach John Harbaugh told reporters that Berrios did not play in Saturday's 26-3 preseason win over the Dolphins due to a soft-tissue issue, Paul Schwartz of the New York Post reports.</t>
         </is>
       </c>
     </row>
@@ -44799,12 +44799,12 @@
       </c>
       <c r="B583" s="4" t="inlineStr">
         <is>
-          <t>Darius Slayton</t>
+          <t>Theo Johnson</t>
         </is>
       </c>
       <c r="C583" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D583" s="4" t="inlineStr">
@@ -44819,7 +44819,7 @@
       </c>
       <c r="F583" s="4" t="inlineStr">
         <is>
-          <t>Slayton caught four of six targets for 58 yards in Saturday's 26-3 preseason win over the Dolphins.</t>
+          <t>Johnson caught his only target for 12 yards in Saturday's 26-3 preseason win over the Dolphins.</t>
         </is>
       </c>
     </row>
@@ -44831,12 +44831,12 @@
       </c>
       <c r="B584" s="5" t="inlineStr">
         <is>
-          <t>Tyrone Tracy Jr.</t>
+          <t>Darius Slayton</t>
         </is>
       </c>
       <c r="C584" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D584" s="5" t="inlineStr">
@@ -44851,7 +44851,7 @@
       </c>
       <c r="F584" s="5" t="inlineStr">
         <is>
-          <t>Tracy rushed six times for 26 yards, caught all three of his targets for 22 yards and lost a fumble in Saturday's 26-3 preseason win over the Dolphins.</t>
+          <t>Slayton caught four of six targets for 58 yards in Saturday's 26-3 preseason win over the Dolphins.</t>
         </is>
       </c>
     </row>
@@ -44863,7 +44863,7 @@
       </c>
       <c r="B585" s="4" t="inlineStr">
         <is>
-          <t>Devin Singletary</t>
+          <t>Tyrone Tracy Jr.</t>
         </is>
       </c>
       <c r="C585" s="4" t="inlineStr">
@@ -44883,7 +44883,7 @@
       </c>
       <c r="F585" s="4" t="inlineStr">
         <is>
-          <t>Singletary rushed eight times for 40 yards and a touchdown while catching his only target for four yards in Saturday's 26-3 preseason win over the Dolphins.</t>
+          <t>Tracy rushed six times for 26 yards, caught all three of his targets for 22 yards and lost a fumble in Saturday's 26-3 preseason win over the Dolphins.</t>
         </is>
       </c>
     </row>
@@ -44895,12 +44895,12 @@
       </c>
       <c r="B586" s="5" t="inlineStr">
         <is>
-          <t>Jaxson Dart</t>
+          <t>Devin Singletary</t>
         </is>
       </c>
       <c r="C586" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D586" s="5" t="inlineStr">
@@ -44915,7 +44915,7 @@
       </c>
       <c r="F586" s="5" t="inlineStr">
         <is>
-          <t>Dart didn't suit up for Saturday's 26-3 preseason win over the Dolphins.</t>
+          <t>Singletary rushed eight times for 40 yards and a touchdown while catching his only target for four yards in Saturday's 26-3 preseason win over the Dolphins.</t>
         </is>
       </c>
     </row>
@@ -44927,27 +44927,27 @@
       </c>
       <c r="B587" s="4" t="inlineStr">
         <is>
-          <t>Francis Mauigoa</t>
+          <t>Jaxson Dart</t>
         </is>
       </c>
       <c r="C587" s="4" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D587" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E587" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F587" s="4" t="inlineStr">
         <is>
-          <t>Mauigoa (upper body) had to leave Thursday's joint practice with the Dolphins due to a stinger, Dan Benton of USA Today reports.</t>
+          <t>Dart didn't suit up for Saturday's 26-3 preseason win over the Dolphins.</t>
         </is>
       </c>
     </row>
@@ -44959,27 +44959,27 @@
       </c>
       <c r="B588" s="5" t="inlineStr">
         <is>
-          <t>Najee Harris</t>
+          <t>Francis Mauigoa</t>
         </is>
       </c>
       <c r="C588" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D588" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E588" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F588" s="5" t="inlineStr">
         <is>
-          <t>Harris (Achilles) is participating in live drills Thursday, Jordan Raanan of ESPN.com reports.</t>
+          <t>Mauigoa (upper body) had to leave Thursday's joint practice with the Dolphins due to a stinger, Dan Benton of USA Today reports.</t>
         </is>
       </c>
     </row>
@@ -44991,27 +44991,27 @@
       </c>
       <c r="B589" s="4" t="inlineStr">
         <is>
-          <t>Malik Nabers</t>
+          <t>Najee Harris</t>
         </is>
       </c>
       <c r="C589" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D589" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E589" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F589" s="4" t="inlineStr">
         <is>
-          <t>Head coach John Harbaugh said that Nabers (knee) won't participate in the Giants' joint practices with the Dolphins this week, Jordan Raanan of ESPN.com reports.</t>
+          <t>Harris (Achilles) is participating in live drills Thursday, Jordan Raanan of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -51955,20 +51955,20 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>83</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>11.6</v>
+        <v>12.3</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I5" s="9" t="n">
@@ -52002,7 +52002,7 @@
         <v>22.4</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -52044,7 +52044,7 @@
         <v>13</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -52082,7 +52082,7 @@
         <v>19.5</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -52162,7 +52162,7 @@
         <v>7.4</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -52200,7 +52200,7 @@
         <v>13.4</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -52242,7 +52242,7 @@
         <v>2.9</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -52280,7 +52280,7 @@
         <v>6.5</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -52318,7 +52318,7 @@
         <v>10.1</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -52326,9 +52326,13 @@
         </is>
       </c>
       <c r="I14" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="5" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>56% chance of rain</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -52356,7 +52360,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -52394,7 +52398,7 @@
         <v>13.6</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
@@ -52432,7 +52436,7 @@
         <v>7.8</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -52474,7 +52478,7 @@
         <v>16.3</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -52512,7 +52516,7 @@
         <v>10.5</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
@@ -52588,7 +52592,7 @@
         <v>7.2</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh: 2026-08-24 08:03 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -692,7 +692,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-24T03:34:11+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-24T08:03:54+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-24T03:34:11+00:00</t>
+          <t>2026-08-24T08:03:54+00:00</t>
         </is>
       </c>
     </row>
@@ -3951,33 +3951,33 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>TEN -3</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.4897</v>
+        <v>0.5127</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>0.5</v>
+        <v>0.5238</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>-0.0102</v>
+        <v>-0.0109</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>-0.01914606343509778</v>
+        <v>-0.02118472397290833</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>0.5</v>
@@ -3992,33 +3992,33 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>TEN -3</t>
         </is>
       </c>
       <c r="E40" s="12" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5127</v>
+        <v>0.4887</v>
       </c>
       <c r="G40" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5</v>
       </c>
       <c r="H40" s="13" t="n">
-        <v>-0.0109</v>
+        <v>-0.0111</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.02118472397290833</v>
+        <v>-0.0209408624219064</v>
       </c>
       <c r="J40" s="14" t="n">
         <v>0.5</v>
@@ -4156,33 +4156,33 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>TEN ML</t>
+          <t>ATL +3</t>
         </is>
       </c>
       <c r="E44" s="12" t="n">
-        <v>-148</v>
+        <v>100</v>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.5802</v>
+        <v>0.4827</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.5968</v>
+        <v>0.5</v>
       </c>
       <c r="H44" s="13" t="n">
-        <v>-0.0161</v>
+        <v>-0.0167</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>-0.0274936344486636</v>
+        <v>-0.03207583043232859</v>
       </c>
       <c r="J44" s="14" t="n">
         <v>0.5</v>
@@ -4197,33 +4197,33 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>ATL +3</t>
+          <t>TEN ML</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>100</v>
+        <v>-148</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.4827</v>
+        <v>0.5793</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>0.5</v>
+        <v>0.5968</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>-0.0167</v>
+        <v>-0.0169</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>-0.03207583043232859</v>
+        <v>-0.02898030615415753</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>0.5</v>
@@ -4607,33 +4607,33 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>BUF -1.5</t>
+          <t>NYJ ML</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
-        <v>-105</v>
+        <v>124</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.4861</v>
+        <v>0.4207</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.4464</v>
       </c>
       <c r="H55" s="8" t="n">
-        <v>-0.0243</v>
+        <v>-0.024</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>-0.05094536914808651</v>
+        <v>-0.05718351511097874</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>0.5</v>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -4658,23 +4658,23 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>NYG +2.5</t>
+          <t>BUF -1.5</t>
         </is>
       </c>
       <c r="E56" s="12" t="n">
         <v>-105</v>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4859</v>
+        <v>0.4861</v>
       </c>
       <c r="G56" s="13" t="n">
         <v>0.5122</v>
       </c>
       <c r="H56" s="13" t="n">
-        <v>-0.0245</v>
+        <v>-0.0243</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>-0.0513240982517143</v>
+        <v>-0.05094536914808651</v>
       </c>
       <c r="J56" s="14" t="n">
         <v>0.5</v>
@@ -4694,28 +4694,28 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>NYG +2.5</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>0.4975</v>
+        <v>0.4859</v>
       </c>
       <c r="G57" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H57" s="8" t="n">
         <v>-0.0245</v>
       </c>
       <c r="I57" s="8" t="n">
-        <v>-0.05031031389922158</v>
+        <v>-0.0513240982517143</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>0.5</v>
@@ -4730,33 +4730,33 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>NYJ ML</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E58" s="12" t="n">
-        <v>124</v>
+        <v>-110</v>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.4198</v>
+        <v>0.4975</v>
       </c>
       <c r="G58" s="13" t="n">
-        <v>0.4464</v>
+        <v>0.5238</v>
       </c>
       <c r="H58" s="13" t="n">
-        <v>-0.0247</v>
+        <v>-0.0245</v>
       </c>
       <c r="I58" s="13" t="n">
-        <v>-0.05917149296025048</v>
+        <v>-0.05031031389922158</v>
       </c>
       <c r="J58" s="14" t="n">
         <v>0.5</v>
@@ -5034,16 +5034,16 @@
         <v>-120</v>
       </c>
       <c r="F65" s="8" t="n">
-        <v>0.5103</v>
+        <v>0.5113</v>
       </c>
       <c r="G65" s="8" t="n">
         <v>0.5455</v>
       </c>
       <c r="H65" s="8" t="n">
-        <v>-0.031</v>
+        <v>-0.0304</v>
       </c>
       <c r="I65" s="8" t="n">
-        <v>-0.0597714860381045</v>
+        <v>-0.05812694981548389</v>
       </c>
       <c r="J65" s="10" t="n">
         <v>0.5</v>
@@ -7702,7 +7702,7 @@
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>3.03</v>
+        <v>2.98</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>-3</v>
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="C12" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="18" t="n">
         <v>1.9</v>
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>1.88</v>
@@ -8326,7 +8326,7 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>1.79</v>
@@ -8358,7 +8358,7 @@
         </is>
       </c>
       <c r="C16" s="12" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D16" s="18" t="n">
         <v>1.76</v>
@@ -32020,7 +32020,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>Watson will learn Monday if he or Shedeur Sanders will be named starting quarterback for the Browns, Jeremy Fowler of ESPN reports.</t>
+          <t>Watson will learn Monday if he or Shedeur Sanders will be named the starting quarterback for the Browns, Jeremy Fowler of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -39880,27 +39880,27 @@
       </c>
       <c r="B432" s="5" t="inlineStr">
         <is>
-          <t>Tyler Biadasz</t>
+          <t>Gary Jennings</t>
         </is>
       </c>
       <c r="C432" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D432" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E432" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F432" s="5" t="inlineStr">
         <is>
-          <t>The Chargers placed Biadasz (knee) on injured reserve Sunday.</t>
+          <t>The Chargers signed Jennings to a contract Sunday.</t>
         </is>
       </c>
     </row>
@@ -39912,27 +39912,27 @@
       </c>
       <c r="B433" s="4" t="inlineStr">
         <is>
-          <t>Tre' Harris</t>
+          <t>Tyler Biadasz</t>
         </is>
       </c>
       <c r="C433" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D433" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E433" s="4" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F433" s="4" t="inlineStr">
         <is>
-          <t>Harris (undisclosed) will participate in Saturday's training camp practice, Alex Insdorf of BoltBeat.com reports.</t>
+          <t>The Chargers placed Biadasz (knee) on injured reserve Sunday.</t>
         </is>
       </c>
     </row>
@@ -39944,12 +39944,12 @@
       </c>
       <c r="B434" s="5" t="inlineStr">
         <is>
-          <t>Rashawn Slater</t>
+          <t>Tre' Harris</t>
         </is>
       </c>
       <c r="C434" s="5" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D434" s="5" t="inlineStr">
@@ -39959,12 +39959,12 @@
       </c>
       <c r="E434" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Undisclosed</t>
         </is>
       </c>
       <c r="F434" s="5" t="inlineStr">
         <is>
-          <t>Slater (undisclosed) was a limited participant in Saturday's practice, Alex Insdorf of BoltBeat.com reports.</t>
+          <t>Harris (undisclosed) will participate in Saturday's training camp practice, Alex Insdorf of BoltBeat.com reports.</t>
         </is>
       </c>
     </row>
@@ -39976,12 +39976,12 @@
       </c>
       <c r="B435" s="4" t="inlineStr">
         <is>
-          <t>Quentin Johnston</t>
+          <t>Rashawn Slater</t>
         </is>
       </c>
       <c r="C435" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D435" s="4" t="inlineStr">
@@ -39996,7 +39996,7 @@
       </c>
       <c r="F435" s="4" t="inlineStr">
         <is>
-          <t>Johnston (lower body) will not participate in Saturday's training camp practice, Alex Insdorf of BoltBeat.com reports.</t>
+          <t>Slater (undisclosed) was a limited participant in Saturday's practice, Alex Insdorf of BoltBeat.com reports.</t>
         </is>
       </c>
     </row>
@@ -40008,27 +40008,27 @@
       </c>
       <c r="B436" s="5" t="inlineStr">
         <is>
-          <t>Kimani Vidal</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="C436" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D436" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E436" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F436" s="5" t="inlineStr">
         <is>
-          <t>Vidal turned four carries into six yards while catching both targets for 10 yards during the Chargers' 41-17 preseason loss to the 49ers on Thursday. He also returned one kickoff for 27 yards.</t>
+          <t>Johnston (lower body) will not participate in Saturday's training camp practice, Alex Insdorf of BoltBeat.com reports.</t>
         </is>
       </c>
     </row>
@@ -40040,12 +40040,12 @@
       </c>
       <c r="B437" s="4" t="inlineStr">
         <is>
-          <t>KeAndre Lambert-Smith</t>
+          <t>Kimani Vidal</t>
         </is>
       </c>
       <c r="C437" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D437" s="4" t="inlineStr">
@@ -40060,7 +40060,7 @@
       </c>
       <c r="F437" s="4" t="inlineStr">
         <is>
-          <t>Lambert-Smith caught two of four targets for 14 yards in Thursday night's 41-17 preseason loss to the 49ers.</t>
+          <t>Vidal turned four carries into six yards while catching both targets for 10 yards during the Chargers' 41-17 preseason loss to the 49ers on Thursday. He also returned one kickoff for 27 yards.</t>
         </is>
       </c>
     </row>
@@ -40072,12 +40072,12 @@
       </c>
       <c r="B438" s="5" t="inlineStr">
         <is>
-          <t>Trey Lance</t>
+          <t>KeAndre Lambert-Smith</t>
         </is>
       </c>
       <c r="C438" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D438" s="5" t="inlineStr">
@@ -40092,7 +40092,7 @@
       </c>
       <c r="F438" s="5" t="inlineStr">
         <is>
-          <t>Lance completed 10 of 16 passes for 73 yards while rushing twice for 42 yards in Thursday's 41-17 preseason loss to the 49ers.</t>
+          <t>Lambert-Smith caught two of four targets for 14 yards in Thursday night's 41-17 preseason loss to the 49ers.</t>
         </is>
       </c>
     </row>
@@ -40104,12 +40104,12 @@
       </c>
       <c r="B439" s="4" t="inlineStr">
         <is>
-          <t>Cameron Dicker</t>
+          <t>Trey Lance</t>
         </is>
       </c>
       <c r="C439" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D439" s="4" t="inlineStr">
@@ -40124,7 +40124,7 @@
       </c>
       <c r="F439" s="4" t="inlineStr">
         <is>
-          <t>Dicker made his sole field-goal attempt but missed a PAT try in Thursday night's 41-17 preseason loss to the 49ers.</t>
+          <t>Lance completed 10 of 16 passes for 73 yards while rushing twice for 42 yards in Thursday's 41-17 preseason loss to the 49ers.</t>
         </is>
       </c>
     </row>
@@ -40136,12 +40136,12 @@
       </c>
       <c r="B440" s="5" t="inlineStr">
         <is>
-          <t>Charlie Kolar</t>
+          <t>Cameron Dicker</t>
         </is>
       </c>
       <c r="C440" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D440" s="5" t="inlineStr">
@@ -40156,7 +40156,7 @@
       </c>
       <c r="F440" s="5" t="inlineStr">
         <is>
-          <t>Kolar and David Njoku both started Thursday's preseason game against San Francisco. Kolar finished with one catch for nine yards on eight snaps.</t>
+          <t>Dicker made his sole field-goal attempt but missed a PAT try in Thursday night's 41-17 preseason loss to the 49ers.</t>
         </is>
       </c>
     </row>
@@ -40168,7 +40168,7 @@
       </c>
       <c r="B441" s="4" t="inlineStr">
         <is>
-          <t>David Njoku</t>
+          <t>Charlie Kolar</t>
         </is>
       </c>
       <c r="C441" s="4" t="inlineStr">
@@ -40188,7 +40188,7 @@
       </c>
       <c r="F441" s="4" t="inlineStr">
         <is>
-          <t>Njoku and Charlie Kolar both started Thursday's preseason game against San Francisco. Njoku finished with no targets on five snaps.</t>
+          <t>Kolar and David Njoku both started Thursday's preseason game against San Francisco. Kolar finished with one catch for nine yards on eight snaps.</t>
         </is>
       </c>
     </row>
@@ -40200,12 +40200,12 @@
       </c>
       <c r="B442" s="5" t="inlineStr">
         <is>
-          <t>Keaton Mitchell</t>
+          <t>David Njoku</t>
         </is>
       </c>
       <c r="C442" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D442" s="5" t="inlineStr">
@@ -40220,7 +40220,7 @@
       </c>
       <c r="F442" s="5" t="inlineStr">
         <is>
-          <t>Mitchell rushed three times for minus-1 yard and brought in his only target for 11 yards in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
+          <t>Njoku and Charlie Kolar both started Thursday's preseason game against San Francisco. Njoku finished with no targets on five snaps.</t>
         </is>
       </c>
     </row>
@@ -40232,12 +40232,12 @@
       </c>
       <c r="B443" s="4" t="inlineStr">
         <is>
-          <t>Ladd McConkey</t>
+          <t>Keaton Mitchell</t>
         </is>
       </c>
       <c r="C443" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D443" s="4" t="inlineStr">
@@ -40252,7 +40252,7 @@
       </c>
       <c r="F443" s="4" t="inlineStr">
         <is>
-          <t>McConkey failed to bring in his only target in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
+          <t>Mitchell rushed three times for minus-1 yard and brought in his only target for 11 yards in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
         </is>
       </c>
     </row>
@@ -40264,12 +40264,12 @@
       </c>
       <c r="B444" s="5" t="inlineStr">
         <is>
-          <t>Justin Herbert</t>
+          <t>Ladd McConkey</t>
         </is>
       </c>
       <c r="C444" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D444" s="5" t="inlineStr">
@@ -40284,7 +40284,7 @@
       </c>
       <c r="F444" s="5" t="inlineStr">
         <is>
-          <t>Herbert completed one of two passes for nine yards with no touchdowns or interceptions in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
+          <t>McConkey failed to bring in his only target in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
         </is>
       </c>
     </row>
@@ -40296,12 +40296,12 @@
       </c>
       <c r="B445" s="4" t="inlineStr">
         <is>
-          <t>Omarion Hampton</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
       <c r="C445" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D445" s="4" t="inlineStr">
@@ -40316,7 +40316,7 @@
       </c>
       <c r="F445" s="4" t="inlineStr">
         <is>
-          <t>Hampton rushed once for minus-1 yard and wasn't targeted in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
+          <t>Herbert completed one of two passes for nine yards with no touchdowns or interceptions in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
         </is>
       </c>
     </row>
@@ -40328,27 +40328,27 @@
       </c>
       <c r="B446" s="5" t="inlineStr">
         <is>
-          <t>Luke Grimm</t>
+          <t>Omarion Hampton</t>
         </is>
       </c>
       <c r="C446" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D446" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E446" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F446" s="5" t="inlineStr">
         <is>
-          <t>Grimm (undisclosed) reverted to the Chargers' injured-reserve list Thursday, per the NFL's transaction log.</t>
+          <t>Hampton rushed once for minus-1 yard and wasn't targeted in the Chargers' 41-17 preseason loss to the 49ers on Thursday night.</t>
         </is>
       </c>
     </row>
@@ -40360,7 +40360,7 @@
       </c>
       <c r="B447" s="4" t="inlineStr">
         <is>
-          <t>Liam Clifford</t>
+          <t>Luke Grimm</t>
         </is>
       </c>
       <c r="C447" s="4" t="inlineStr">
@@ -40370,17 +40370,17 @@
       </c>
       <c r="D447" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E447" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F447" s="4" t="inlineStr">
         <is>
-          <t>The Chargers signed Clifford on Wednesday.</t>
+          <t>Grimm (undisclosed) reverted to the Chargers' injured-reserve list Thursday, per the NFL's transaction log.</t>
         </is>
       </c>
     </row>
@@ -40392,12 +40392,12 @@
       </c>
       <c r="B448" s="5" t="inlineStr">
         <is>
-          <t>Junior Colson</t>
+          <t>Liam Clifford</t>
         </is>
       </c>
       <c r="C448" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D448" s="5" t="inlineStr">
@@ -40410,7 +40410,11 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F448" s="5" t="inlineStr"/>
+      <c r="F448" s="5" t="inlineStr">
+        <is>
+          <t>The Chargers signed Clifford on Wednesday.</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="4" t="inlineStr">
@@ -40420,12 +40424,12 @@
       </c>
       <c r="B449" s="4" t="inlineStr">
         <is>
-          <t>Nikko Reed</t>
+          <t>Junior Colson</t>
         </is>
       </c>
       <c r="C449" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D449" s="4" t="inlineStr">
@@ -40448,7 +40452,7 @@
       </c>
       <c r="B450" s="5" t="inlineStr">
         <is>
-          <t>Eric Rogers</t>
+          <t>Nikko Reed</t>
         </is>
       </c>
       <c r="C450" s="5" t="inlineStr">
@@ -40476,12 +40480,12 @@
       </c>
       <c r="B451" s="4" t="inlineStr">
         <is>
-          <t>Oronde Gadsden</t>
+          <t>Eric Rogers</t>
         </is>
       </c>
       <c r="C451" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D451" s="4" t="inlineStr">
@@ -40494,11 +40498,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F451" s="4" t="inlineStr">
-        <is>
-          <t>Gadsden caught two of three targets for 21 yards in Thursday's 21-7 preseason win over the Texans.</t>
-        </is>
-      </c>
+      <c r="F451" s="4" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" s="5" t="inlineStr">
@@ -40508,12 +40508,12 @@
       </c>
       <c r="B452" s="5" t="inlineStr">
         <is>
-          <t>Andre Carter II</t>
+          <t>Oronde Gadsden</t>
         </is>
       </c>
       <c r="C452" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D452" s="5" t="inlineStr">
@@ -40528,7 +40528,7 @@
       </c>
       <c r="F452" s="5" t="inlineStr">
         <is>
-          <t>The Chargers signed Carter on Monday, Aaron Wilson of KPRC 2 Houston reports.</t>
+          <t>Gadsden caught two of three targets for 21 yards in Thursday's 21-7 preseason win over the Texans.</t>
         </is>
       </c>
     </row>
@@ -40540,12 +40540,12 @@
       </c>
       <c r="B453" s="4" t="inlineStr">
         <is>
-          <t>Kendall Williamson</t>
+          <t>Andre Carter II</t>
         </is>
       </c>
       <c r="C453" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D453" s="4" t="inlineStr">
@@ -40560,7 +40560,7 @@
       </c>
       <c r="F453" s="4" t="inlineStr">
         <is>
-          <t>Williamson (ankle) participated in the Chargers' training camp Wednesday, Eric Smith of the team's official site reports.</t>
+          <t>The Chargers signed Carter on Monday, Aaron Wilson of KPRC 2 Houston reports.</t>
         </is>
       </c>
     </row>
@@ -40572,12 +40572,12 @@
       </c>
       <c r="B454" s="5" t="inlineStr">
         <is>
-          <t>Tuli Tuipulotu</t>
+          <t>Kendall Williamson</t>
         </is>
       </c>
       <c r="C454" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D454" s="5" t="inlineStr">
@@ -40592,7 +40592,7 @@
       </c>
       <c r="F454" s="5" t="inlineStr">
         <is>
-          <t>Tuipulotu did not participate in team drills Monday due his ongoing negotiations on an extension, Kris Rhim of ESPN.com reports.</t>
+          <t>Williamson (ankle) participated in the Chargers' training camp Wednesday, Eric Smith of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -45376,12 +45376,12 @@
       </c>
       <c r="B605" s="4" t="inlineStr">
         <is>
-          <t>Cade York</t>
+          <t>Dominic Richardson</t>
         </is>
       </c>
       <c r="C605" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D605" s="4" t="inlineStr">
@@ -45396,7 +45396,7 @@
       </c>
       <c r="F605" s="4" t="inlineStr">
         <is>
-          <t>York missed his sole field-goal attempt, but converted a PAT in Friday night's preseason game against the Steelers.</t>
+          <t>The Jets signed Richardson to a contract Sunday.</t>
         </is>
       </c>
     </row>
@@ -45408,12 +45408,12 @@
       </c>
       <c r="B606" s="5" t="inlineStr">
         <is>
-          <t>Cade Klubnik</t>
+          <t>Cade York</t>
         </is>
       </c>
       <c r="C606" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D606" s="5" t="inlineStr">
@@ -45428,7 +45428,7 @@
       </c>
       <c r="F606" s="5" t="inlineStr">
         <is>
-          <t>Klubnik completed 10 of 14 passes for 75 yards and recorded a 16-yard carry during the Jets' 17-0 preseason win over the Steelers on Friday.</t>
+          <t>York missed his sole field-goal attempt, but converted a PAT in Friday night's preseason game against the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45440,12 +45440,12 @@
       </c>
       <c r="B607" s="4" t="inlineStr">
         <is>
-          <t>Jason Sanders</t>
+          <t>Cade Klubnik</t>
         </is>
       </c>
       <c r="C607" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D607" s="4" t="inlineStr">
@@ -45460,7 +45460,7 @@
       </c>
       <c r="F607" s="4" t="inlineStr">
         <is>
-          <t>Sanders converted his sole field-goal attempt and only PAT in Friday night's preseason game against the Steelers.</t>
+          <t>Klubnik completed 10 of 14 passes for 75 yards and recorded a 16-yard carry during the Jets' 17-0 preseason win over the Steelers on Friday.</t>
         </is>
       </c>
     </row>
@@ -45472,27 +45472,27 @@
       </c>
       <c r="B608" s="5" t="inlineStr">
         <is>
-          <t>Isaiah Davis</t>
+          <t>Jason Sanders</t>
         </is>
       </c>
       <c r="C608" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D608" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E608" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F608" s="5" t="inlineStr">
         <is>
-          <t>Davis (knee) did not play in the Jets' 17-0 preseason win over the Steelers on Friday.</t>
+          <t>Sanders converted his sole field-goal attempt and only PAT in Friday night's preseason game against the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45504,27 +45504,27 @@
       </c>
       <c r="B609" s="4" t="inlineStr">
         <is>
-          <t>Mason Taylor</t>
+          <t>Isaiah Davis</t>
         </is>
       </c>
       <c r="C609" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D609" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E609" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F609" s="4" t="inlineStr">
         <is>
-          <t>Taylor caught his only target for 10 yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>Davis (knee) did not play in the Jets' 17-0 preseason win over the Steelers on Friday.</t>
         </is>
       </c>
     </row>
@@ -45536,12 +45536,12 @@
       </c>
       <c r="B610" s="5" t="inlineStr">
         <is>
-          <t>Adonai Mitchell</t>
+          <t>Mason Taylor</t>
         </is>
       </c>
       <c r="C610" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D610" s="5" t="inlineStr">
@@ -45556,7 +45556,7 @@
       </c>
       <c r="F610" s="5" t="inlineStr">
         <is>
-          <t>Mitchell caught both of his targets for 29 yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>Taylor caught his only target for 10 yards in Friday's 17-0 preseason win over the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45568,12 +45568,12 @@
       </c>
       <c r="B611" s="4" t="inlineStr">
         <is>
-          <t>Braelon Allen</t>
+          <t>Adonai Mitchell</t>
         </is>
       </c>
       <c r="C611" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D611" s="4" t="inlineStr">
@@ -45588,7 +45588,7 @@
       </c>
       <c r="F611" s="4" t="inlineStr">
         <is>
-          <t>Allen rushed three times for four yards and caught his lone target for five yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>Mitchell caught both of his targets for 29 yards in Friday's 17-0 preseason win over the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45600,12 +45600,12 @@
       </c>
       <c r="B612" s="5" t="inlineStr">
         <is>
-          <t>Omar Cooper Jr.</t>
+          <t>Braelon Allen</t>
         </is>
       </c>
       <c r="C612" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D612" s="5" t="inlineStr">
@@ -45620,7 +45620,7 @@
       </c>
       <c r="F612" s="5" t="inlineStr">
         <is>
-          <t>Cooper caught his only target for nine yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>Allen rushed three times for four yards and caught his lone target for five yards in Friday's 17-0 preseason win over the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45632,12 +45632,12 @@
       </c>
       <c r="B613" s="4" t="inlineStr">
         <is>
-          <t>Geno Smith</t>
+          <t>Omar Cooper Jr.</t>
         </is>
       </c>
       <c r="C613" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D613" s="4" t="inlineStr">
@@ -45652,7 +45652,7 @@
       </c>
       <c r="F613" s="4" t="inlineStr">
         <is>
-          <t>Smith completed all seven of his pass attempts for 65 yards and a touchdown in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>Cooper caught his only target for nine yards in Friday's 17-0 preseason win over the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45664,12 +45664,12 @@
       </c>
       <c r="B614" s="5" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Geno Smith</t>
         </is>
       </c>
       <c r="C614" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D614" s="5" t="inlineStr">
@@ -45684,7 +45684,7 @@
       </c>
       <c r="F614" s="5" t="inlineStr">
         <is>
-          <t>Wilson caught his only target for 10 yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>Smith completed all seven of his pass attempts for 65 yards and a touchdown in Friday's 17-0 preseason win over the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45696,27 +45696,27 @@
       </c>
       <c r="B615" s="4" t="inlineStr">
         <is>
-          <t>Chase Curtis</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="C615" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D615" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E615" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F615" s="4" t="inlineStr">
         <is>
-          <t>Curtis (knee) is out for the remainder of Friday's preseason contest at Pittsburgh.</t>
+          <t>Wilson caught his only target for 10 yards in Friday's 17-0 preseason win over the Steelers.</t>
         </is>
       </c>
     </row>
@@ -45728,27 +45728,27 @@
       </c>
       <c r="B616" s="5" t="inlineStr">
         <is>
-          <t>Kingsley Jonathan</t>
+          <t>Chase Curtis</t>
         </is>
       </c>
       <c r="C616" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D616" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E616" s="5" t="inlineStr">
         <is>
-          <t>Bruise</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F616" s="5" t="inlineStr">
         <is>
-          <t>Jonathan (thigh) reverted to the Jets' injured reserve Wednesday, Aaron Wilson of KPRC 2 Houston reports.</t>
+          <t>Curtis (knee) is out for the remainder of Friday's preseason contest at Pittsburgh.</t>
         </is>
       </c>
     </row>
@@ -45760,27 +45760,27 @@
       </c>
       <c r="B617" s="4" t="inlineStr">
         <is>
-          <t>Qwan'tez Stiggers</t>
+          <t>Kingsley Jonathan</t>
         </is>
       </c>
       <c r="C617" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D617" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E617" s="4" t="inlineStr">
         <is>
-          <t>Concussion</t>
+          <t>Bruise</t>
         </is>
       </c>
       <c r="F617" s="4" t="inlineStr">
         <is>
-          <t>Stiggers (concussion) was a limited participant in Wednesday's practice, Rich Cimini of ESPN.com reports.</t>
+          <t>Jonathan (thigh) reverted to the Jets' injured reserve Wednesday, Aaron Wilson of KPRC 2 Houston reports.</t>
         </is>
       </c>
     </row>
@@ -45792,27 +45792,27 @@
       </c>
       <c r="B618" s="5" t="inlineStr">
         <is>
-          <t>Junior Bergen</t>
+          <t>Qwan'tez Stiggers</t>
         </is>
       </c>
       <c r="C618" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D618" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E618" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Concussion</t>
         </is>
       </c>
       <c r="F618" s="5" t="inlineStr">
         <is>
-          <t>The Jets signed Bergen to a contract Wednesday, Eric Allen of the team's official site reports.</t>
+          <t>Stiggers (concussion) was a limited participant in Wednesday's practice, Rich Cimini of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -45824,27 +45824,27 @@
       </c>
       <c r="B619" s="4" t="inlineStr">
         <is>
-          <t>Nahshon Wright</t>
+          <t>Junior Bergen</t>
         </is>
       </c>
       <c r="C619" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D619" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E619" s="4" t="inlineStr">
         <is>
-          <t>Strain</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F619" s="4" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>The Jets signed Bergen to a contract Wednesday, Eric Allen of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -45856,12 +45856,12 @@
       </c>
       <c r="B620" s="5" t="inlineStr">
         <is>
-          <t>VJ Payne</t>
+          <t>Nahshon Wright</t>
         </is>
       </c>
       <c r="C620" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D620" s="5" t="inlineStr">
@@ -45871,7 +45871,7 @@
       </c>
       <c r="E620" s="5" t="inlineStr">
         <is>
-          <t>Bruise</t>
+          <t>Strain</t>
         </is>
       </c>
       <c r="F620" s="5" t="inlineStr">
@@ -45888,12 +45888,12 @@
       </c>
       <c r="B621" s="4" t="inlineStr">
         <is>
-          <t>Kenyon Sadiq</t>
+          <t>VJ Payne</t>
         </is>
       </c>
       <c r="C621" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D621" s="4" t="inlineStr">
@@ -45903,7 +45903,7 @@
       </c>
       <c r="E621" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Bruise</t>
         </is>
       </c>
       <c r="F621" s="4" t="inlineStr">
@@ -45920,12 +45920,12 @@
       </c>
       <c r="B622" s="5" t="inlineStr">
         <is>
-          <t>Breece Hall</t>
+          <t>Kenyon Sadiq</t>
         </is>
       </c>
       <c r="C622" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D622" s="5" t="inlineStr">
@@ -45935,7 +45935,7 @@
       </c>
       <c r="E622" s="5" t="inlineStr">
         <is>
-          <t>Strain</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F622" s="5" t="inlineStr">
@@ -45952,12 +45952,12 @@
       </c>
       <c r="B623" s="4" t="inlineStr">
         <is>
-          <t>Mory Bamba</t>
+          <t>Breece Hall</t>
         </is>
       </c>
       <c r="C623" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D623" s="4" t="inlineStr">
@@ -45967,7 +45967,7 @@
       </c>
       <c r="E623" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Strain</t>
         </is>
       </c>
       <c r="F623" s="4" t="inlineStr">
@@ -45984,25 +45984,29 @@
       </c>
       <c r="B624" s="5" t="inlineStr">
         <is>
-          <t>Joseph Ossai</t>
+          <t>Mory Bamba</t>
         </is>
       </c>
       <c r="C624" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D624" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E624" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F624" s="5" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F624" s="5" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="625">
       <c r="A625" s="4" t="inlineStr">
@@ -46012,12 +46016,12 @@
       </c>
       <c r="B625" s="4" t="inlineStr">
         <is>
-          <t>Kiko Mauigoa</t>
+          <t>Joseph Ossai</t>
         </is>
       </c>
       <c r="C625" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D625" s="4" t="inlineStr">
@@ -46040,12 +46044,12 @@
       </c>
       <c r="B626" s="5" t="inlineStr">
         <is>
-          <t>T'Vondre Sweat</t>
+          <t>Kiko Mauigoa</t>
         </is>
       </c>
       <c r="C626" s="5" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D626" s="5" t="inlineStr">
@@ -46068,12 +46072,12 @@
       </c>
       <c r="B627" s="4" t="inlineStr">
         <is>
-          <t>Andre Cisco</t>
+          <t>T'Vondre Sweat</t>
         </is>
       </c>
       <c r="C627" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D627" s="4" t="inlineStr">
@@ -46096,12 +46100,12 @@
       </c>
       <c r="B628" s="5" t="inlineStr">
         <is>
-          <t>Kingsley Enagbare</t>
+          <t>Andre Cisco</t>
         </is>
       </c>
       <c r="C628" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D628" s="5" t="inlineStr">
@@ -46114,11 +46118,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F628" s="5" t="inlineStr">
-        <is>
-          <t>Enagbare (undisclosed) was a full participant in Tuesday's practice, Brian Costello of the New York Post reports.</t>
-        </is>
-      </c>
+      <c r="F628" s="5" t="inlineStr"/>
     </row>
     <row r="629">
       <c r="A629" s="4" t="inlineStr">
@@ -46128,27 +46128,27 @@
       </c>
       <c r="B629" s="4" t="inlineStr">
         <is>
-          <t>D'Angelo Ponds</t>
+          <t>Kingsley Enagbare</t>
         </is>
       </c>
       <c r="C629" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D629" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E629" s="4" t="inlineStr">
         <is>
-          <t>Strain</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F629" s="4" t="inlineStr">
         <is>
-          <t>Ponds (calf) is nearing a return to the field according to head coach Aaron Glenn, Eric Allen of the Jets' official site reports.</t>
+          <t>Enagbare (undisclosed) was a full participant in Tuesday's practice, Brian Costello of the New York Post reports.</t>
         </is>
       </c>
     </row>
@@ -47904,7 +47904,7 @@
       </c>
       <c r="F684" s="5" t="inlineStr">
         <is>
-          <t>Kittle (Achilles) was activated from the Active/PUP list Sunday.</t>
+          <t>Kittle (Achilles) was activated from the active/PUP list Sunday.</t>
         </is>
       </c>
     </row>
@@ -48556,27 +48556,27 @@
       </c>
       <c r="B705" s="4" t="inlineStr">
         <is>
-          <t>Bud Clark</t>
+          <t>Drew Lock</t>
         </is>
       </c>
       <c r="C705" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D705" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E705" s="4" t="inlineStr">
         <is>
-          <t>Leg</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F705" s="4" t="inlineStr">
         <is>
-          <t>Clark was carted off the field with a right leg injury during Sunday's preseason matchup with the Titans, Brady Henderson of ESPN.com reports.</t>
+          <t>Lock completed 12 of 14 passes for 103 yards and a touchdown while rushing twice for eight yards in Sunday's 19-16 preseason loss to the Titans.</t>
         </is>
       </c>
     </row>
@@ -48588,12 +48588,12 @@
       </c>
       <c r="B706" s="5" t="inlineStr">
         <is>
-          <t>Drew Lock</t>
+          <t>Emmanuel Henderson Jr.</t>
         </is>
       </c>
       <c r="C706" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D706" s="5" t="inlineStr">
@@ -48608,7 +48608,7 @@
       </c>
       <c r="F706" s="5" t="inlineStr">
         <is>
-          <t>Lock will start Sunday's preseason game against the Titans, Bob Condotta of The Seattle Times reports.</t>
+          <t>Henderson caught one of two targets for seven yards in Sunday's 19-16 preseason loss to the Titans. He also returned two kickoffs for 47 yards and notched two solo tackles on special teams.</t>
         </is>
       </c>
     </row>
@@ -48620,12 +48620,12 @@
       </c>
       <c r="B707" s="4" t="inlineStr">
         <is>
-          <t>Jadarian Price</t>
+          <t>Elijah Arroyo</t>
         </is>
       </c>
       <c r="C707" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D707" s="4" t="inlineStr">
@@ -48640,7 +48640,7 @@
       </c>
       <c r="F707" s="4" t="inlineStr">
         <is>
-          <t>Price will not play in Sunday's preseason game against the Titans, Gregg Bell of The Tacoma News Tribune reports.</t>
+          <t>Arroyo caught two of four targets for 50 yards and a touchdown in Sunday's 19-16 preseason loss to the Titans.</t>
         </is>
       </c>
     </row>
@@ -48652,27 +48652,27 @@
       </c>
       <c r="B708" s="5" t="inlineStr">
         <is>
-          <t>Julian Hicks</t>
+          <t>Bud Clark</t>
         </is>
       </c>
       <c r="C708" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D708" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E708" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Leg</t>
         </is>
       </c>
       <c r="F708" s="5" t="inlineStr">
         <is>
-          <t>The Seahawks signed Hicks to a contract Saturday, John Boyle of the team's official site reports.</t>
+          <t>Clark was carted off the field with a right leg injury during Sunday's preseason matchup with the Titans, Brady Henderson of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -48684,27 +48684,27 @@
       </c>
       <c r="B709" s="4" t="inlineStr">
         <is>
-          <t>Jake Bobo</t>
+          <t>Jadarian Price</t>
         </is>
       </c>
       <c r="C709" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D709" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E709" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F709" s="4" t="inlineStr">
         <is>
-          <t>The Seahawks placed Bobo (knee) on injured reserve Saturday, John Boyle of the team's official site reports.</t>
+          <t>Price will not play in Sunday's preseason game against the Titans, Gregg Bell of The Tacoma News Tribune reports.</t>
         </is>
       </c>
     </row>
@@ -48716,12 +48716,12 @@
       </c>
       <c r="B710" s="5" t="inlineStr">
         <is>
-          <t>Trevon Diggs</t>
+          <t>Julian Hicks</t>
         </is>
       </c>
       <c r="C710" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D710" s="5" t="inlineStr">
@@ -48736,7 +48736,7 @@
       </c>
       <c r="F710" s="5" t="inlineStr">
         <is>
-          <t>The Seahawks are slated to sign Diggs to a one-year deal, Adam Schefter of ESPN reports.</t>
+          <t>The Seahawks signed Hicks to a contract Saturday, John Boyle of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -48748,12 +48748,12 @@
       </c>
       <c r="B711" s="4" t="inlineStr">
         <is>
-          <t>Joseph Vaughn</t>
+          <t>Jake Bobo</t>
         </is>
       </c>
       <c r="C711" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D711" s="4" t="inlineStr">
@@ -48768,7 +48768,7 @@
       </c>
       <c r="F711" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>The Seahawks placed Bobo (knee) on injured reserve Saturday, John Boyle of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -48780,27 +48780,27 @@
       </c>
       <c r="B712" s="5" t="inlineStr">
         <is>
-          <t>Emanuel Wilson</t>
+          <t>Trevon Diggs</t>
         </is>
       </c>
       <c r="C712" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D712" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E712" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F712" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>The Seahawks are slated to sign Diggs to a one-year deal, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -48812,12 +48812,12 @@
       </c>
       <c r="B713" s="4" t="inlineStr">
         <is>
-          <t>Robbie Ouzts</t>
+          <t>Joseph Vaughn</t>
         </is>
       </c>
       <c r="C713" s="4" t="inlineStr">
         <is>
-          <t>FB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D713" s="4" t="inlineStr">
@@ -48844,12 +48844,12 @@
       </c>
       <c r="B714" s="5" t="inlineStr">
         <is>
-          <t>Tory Horton</t>
+          <t>Emanuel Wilson</t>
         </is>
       </c>
       <c r="C714" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D714" s="5" t="inlineStr">
@@ -48859,7 +48859,7 @@
       </c>
       <c r="E714" s="5" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F714" s="5" t="inlineStr">
@@ -48876,12 +48876,12 @@
       </c>
       <c r="B715" s="4" t="inlineStr">
         <is>
-          <t>Shemar Jean-Charles</t>
+          <t>Robbie Ouzts</t>
         </is>
       </c>
       <c r="C715" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>FB</t>
         </is>
       </c>
       <c r="D715" s="4" t="inlineStr">
@@ -48908,12 +48908,12 @@
       </c>
       <c r="B716" s="5" t="inlineStr">
         <is>
-          <t>Nick Emmanwori</t>
+          <t>Tory Horton</t>
         </is>
       </c>
       <c r="C716" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D716" s="5" t="inlineStr">
@@ -48923,7 +48923,7 @@
       </c>
       <c r="E716" s="5" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Undisclosed</t>
         </is>
       </c>
       <c r="F716" s="5" t="inlineStr">
@@ -48940,27 +48940,27 @@
       </c>
       <c r="B717" s="4" t="inlineStr">
         <is>
-          <t>Anthony Hankerson</t>
+          <t>Shemar Jean-Charles</t>
         </is>
       </c>
       <c r="C717" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D717" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E717" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F717" s="4" t="inlineStr">
         <is>
-          <t>Hankerson and the Seahawks agreed on a contract Monday, John Boyle of the team's official website reports.</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -48972,27 +48972,27 @@
       </c>
       <c r="B718" s="5" t="inlineStr">
         <is>
-          <t>Montorie Foster Jr.</t>
+          <t>Nick Emmanwori</t>
         </is>
       </c>
       <c r="C718" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D718" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E718" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F718" s="5" t="inlineStr">
         <is>
-          <t>Foster caught five of seven targets for 36 yards and a touchdown in Saturday's 17-7 preseason loss to the Cowboys, building on what has been a strong performance in training camp, John Boyle of the Seahawks' official site reports.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -49004,12 +49004,12 @@
       </c>
       <c r="B719" s="4" t="inlineStr">
         <is>
-          <t>Rashid Shaheed</t>
+          <t>Anthony Hankerson</t>
         </is>
       </c>
       <c r="C719" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D719" s="4" t="inlineStr">
@@ -49024,7 +49024,7 @@
       </c>
       <c r="F719" s="4" t="inlineStr">
         <is>
-          <t>Shaheed didn't suit up for Saturday's 17-7 preseason loss to the Cowboys.</t>
+          <t>Hankerson and the Seahawks agreed on a contract Monday, John Boyle of the team's official website reports.</t>
         </is>
       </c>
     </row>
@@ -49036,12 +49036,12 @@
       </c>
       <c r="B720" s="5" t="inlineStr">
         <is>
-          <t>AJ Barner</t>
+          <t>Montorie Foster Jr.</t>
         </is>
       </c>
       <c r="C720" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D720" s="5" t="inlineStr">
@@ -49056,7 +49056,7 @@
       </c>
       <c r="F720" s="5" t="inlineStr">
         <is>
-          <t>Barner was rested for Seattle's 17-7 preseason loss to the Cowboys on Saturday.</t>
+          <t>Foster caught five of seven targets for 36 yards and a touchdown in Saturday's 17-7 preseason loss to the Cowboys, building on what has been a strong performance in training camp, John Boyle of the Seahawks' official site reports.</t>
         </is>
       </c>
     </row>
@@ -49068,27 +49068,27 @@
       </c>
       <c r="B721" s="4" t="inlineStr">
         <is>
-          <t>Zach Charbonnet</t>
+          <t>Rashid Shaheed</t>
         </is>
       </c>
       <c r="C721" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D721" s="4" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E721" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F721" s="4" t="inlineStr">
         <is>
-          <t>Charbonnet (knee) remains on the active/PUP list as the Seahawks' second preseason contest (Sunday, Aug. 23 versus the Titans) approaches.</t>
+          <t>Shaheed didn't suit up for Saturday's 17-7 preseason loss to the Cowboys.</t>
         </is>
       </c>
     </row>
@@ -49100,12 +49100,12 @@
       </c>
       <c r="B722" s="5" t="inlineStr">
         <is>
-          <t>Jason Myers</t>
+          <t>AJ Barner</t>
         </is>
       </c>
       <c r="C722" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D722" s="5" t="inlineStr">
@@ -49120,7 +49120,7 @@
       </c>
       <c r="F722" s="5" t="inlineStr">
         <is>
-          <t>Myers missed his only field-goal attempt from 45 yards out and made his only extra-point try in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
+          <t>Barner was rested for Seattle's 17-7 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -49132,7 +49132,7 @@
       </c>
       <c r="B723" s="4" t="inlineStr">
         <is>
-          <t>George Holani</t>
+          <t>Zach Charbonnet</t>
         </is>
       </c>
       <c r="C723" s="4" t="inlineStr">
@@ -49142,17 +49142,17 @@
       </c>
       <c r="D723" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E723" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F723" s="4" t="inlineStr">
         <is>
-          <t>Holani rushed 12 times for 42 yards in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
+          <t>Charbonnet (knee) remains on the active/PUP list as the Seahawks' second preseason contest (Sunday, Aug. 23 versus the Titans) approaches.</t>
         </is>
       </c>
     </row>
@@ -49164,12 +49164,12 @@
       </c>
       <c r="B724" s="5" t="inlineStr">
         <is>
-          <t>Devon Witherspoon</t>
+          <t>Jason Myers</t>
         </is>
       </c>
       <c r="C724" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D724" s="5" t="inlineStr">
@@ -49184,7 +49184,7 @@
       </c>
       <c r="F724" s="5" t="inlineStr">
         <is>
-          <t>Witherspoon and the Seahawks agreed to a four-year, $132 million contract extension Saturday, Adam Schefter of ESPN reports.</t>
+          <t>Myers missed his only field-goal attempt from 45 yards out and made his only extra-point try in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -49196,12 +49196,12 @@
       </c>
       <c r="B725" s="4" t="inlineStr">
         <is>
-          <t>DeMarcus Lawrence</t>
+          <t>George Holani</t>
         </is>
       </c>
       <c r="C725" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D725" s="4" t="inlineStr">
@@ -49216,7 +49216,7 @@
       </c>
       <c r="F725" s="4" t="inlineStr">
         <is>
-          <t>Lawrence has declared that he will retire after the 2026 season, Jori Epstein of Yahoo Sports reports.</t>
+          <t>Holani rushed 12 times for 42 yards in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -49228,12 +49228,12 @@
       </c>
       <c r="B726" s="5" t="inlineStr">
         <is>
-          <t>Sam Darnold</t>
+          <t>Devon Witherspoon</t>
         </is>
       </c>
       <c r="C726" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D726" s="5" t="inlineStr">
@@ -49248,7 +49248,7 @@
       </c>
       <c r="F726" s="5" t="inlineStr">
         <is>
-          <t>Coach Mike Macdonald said Friday that Darnold won't suit up for Saturday's preseason game versus the Cowboys, Curtis Crabtree of Fox 13 Seattle reports.</t>
+          <t>Witherspoon and the Seahawks agreed to a four-year, $132 million contract extension Saturday, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -49260,12 +49260,12 @@
       </c>
       <c r="B727" s="4" t="inlineStr">
         <is>
-          <t>Jaxon Smith-Njigba</t>
+          <t>DeMarcus Lawrence</t>
         </is>
       </c>
       <c r="C727" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D727" s="4" t="inlineStr">
@@ -49280,7 +49280,7 @@
       </c>
       <c r="F727" s="4" t="inlineStr">
         <is>
-          <t>Smith-Njigba is always willing to be coached up in an attempt to be a better player, Anthony Moeglin of Roundtable Sports reports.</t>
+          <t>Lawrence has declared that he will retire after the 2026 season, Jori Epstein of Yahoo Sports reports.</t>
         </is>
       </c>
     </row>
@@ -49292,12 +49292,12 @@
       </c>
       <c r="B728" s="5" t="inlineStr">
         <is>
-          <t>AJ Finley</t>
+          <t>Sam Darnold</t>
         </is>
       </c>
       <c r="C728" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D728" s="5" t="inlineStr">
@@ -49310,7 +49310,11 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F728" s="5" t="inlineStr"/>
+      <c r="F728" s="5" t="inlineStr">
+        <is>
+          <t>Coach Mike Macdonald said Friday that Darnold won't suit up for Saturday's preseason game versus the Cowboys, Curtis Crabtree of Fox 13 Seattle reports.</t>
+        </is>
+      </c>
     </row>
     <row r="729">
       <c r="A729" s="4" t="inlineStr">
@@ -49320,12 +49324,12 @@
       </c>
       <c r="B729" s="4" t="inlineStr">
         <is>
-          <t>Brock Lampe</t>
+          <t>Jaxon Smith-Njigba</t>
         </is>
       </c>
       <c r="C729" s="4" t="inlineStr">
         <is>
-          <t>FB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D729" s="4" t="inlineStr">
@@ -49340,7 +49344,7 @@
       </c>
       <c r="F729" s="4" t="inlineStr">
         <is>
-          <t>Seattle signed Lampe on Thursday, John Boyle of the Seahawks' official site reports.</t>
+          <t>Smith-Njigba is always willing to be coached up in an attempt to be a better player, Anthony Moeglin of Roundtable Sports reports.</t>
         </is>
       </c>
     </row>
@@ -50144,12 +50148,12 @@
       </c>
       <c r="B755" s="4" t="inlineStr">
         <is>
-          <t>Carnell Tate</t>
+          <t>Joey Slye</t>
         </is>
       </c>
       <c r="C755" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D755" s="4" t="inlineStr">
@@ -50164,7 +50168,7 @@
       </c>
       <c r="F755" s="4" t="inlineStr">
         <is>
-          <t>Tate (undisclosed) is in uniform for Sunday's preseason game against the Seahawks.</t>
+          <t>Slye converted all four of his field-goal attempts and made his only PAT try in Sunday's 19-16 preseason win over the Seahawks.</t>
         </is>
       </c>
     </row>
@@ -50176,27 +50180,27 @@
       </c>
       <c r="B756" s="5" t="inlineStr">
         <is>
-          <t>Nazeeh Johnson</t>
+          <t>Tyjae Spears</t>
         </is>
       </c>
       <c r="C756" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D756" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E756" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F756" s="5" t="inlineStr">
         <is>
-          <t>The Titans placed Johnson (ankle) on injured reserve Friday, Jim Wyatt of the team's official site reports.</t>
+          <t>Spears rushed twice for two yards and caught all three of his targets for 14 yards in Sunday's 19-16 preseason win over the Seahawks.</t>
         </is>
       </c>
     </row>
@@ -50208,7 +50212,7 @@
       </c>
       <c r="B757" s="4" t="inlineStr">
         <is>
-          <t>Mitchell Trubisky</t>
+          <t>Cam Ward</t>
         </is>
       </c>
       <c r="C757" s="4" t="inlineStr">
@@ -50218,17 +50222,17 @@
       </c>
       <c r="D757" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E757" s="4" t="inlineStr">
         <is>
-          <t>Biceps</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F757" s="4" t="inlineStr">
         <is>
-          <t>Trubisky (biceps) did not participate in Wednesday's practice, Terry McCormick of TitanInsider.com reports.</t>
+          <t>Ward completed eight of 12 passes for 69 yards, no touchdowns and no interceptions in Sunday's 19-16 preseason win over the Seahawks.</t>
         </is>
       </c>
     </row>
@@ -50260,7 +50264,7 @@
       </c>
       <c r="F758" s="5" t="inlineStr">
         <is>
-          <t>Pollard (undisclosed) returned to practice Wednesday, Turron Davenport of ESPN.com reports.</t>
+          <t>Pollard rushed twice for 12 yards and caught his only target for 33 yards in Sunday's 19-16 preseason win over the Seahawks.</t>
         </is>
       </c>
     </row>
@@ -50272,12 +50276,12 @@
       </c>
       <c r="B759" s="4" t="inlineStr">
         <is>
-          <t>D'Ernest Johnson</t>
+          <t>Carnell Tate</t>
         </is>
       </c>
       <c r="C759" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D759" s="4" t="inlineStr">
@@ -50292,7 +50296,7 @@
       </c>
       <c r="F759" s="4" t="inlineStr">
         <is>
-          <t>Johnson agreed to a one-year contract with the Titans on Wednesday, NFL reporter Jordan Schultz reports.</t>
+          <t>Tate didn't catch either of his two targets in Sunday's 19-16 preseason win over the Seahawks.</t>
         </is>
       </c>
     </row>
@@ -50304,17 +50308,17 @@
       </c>
       <c r="B760" s="5" t="inlineStr">
         <is>
-          <t>Kalel Mullings</t>
+          <t>Nazeeh Johnson</t>
         </is>
       </c>
       <c r="C760" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D760" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E760" s="5" t="inlineStr">
@@ -50324,7 +50328,7 @@
       </c>
       <c r="F760" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>The Titans placed Johnson (ankle) on injured reserve Friday, Jim Wyatt of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -50336,27 +50340,27 @@
       </c>
       <c r="B761" s="4" t="inlineStr">
         <is>
-          <t>Jaylen Harrell</t>
+          <t>Mitchell Trubisky</t>
         </is>
       </c>
       <c r="C761" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D761" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E761" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Biceps</t>
         </is>
       </c>
       <c r="F761" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>Trubisky (biceps) did not participate in Wednesday's practice, Terry McCormick of TitanInsider.com reports.</t>
         </is>
       </c>
     </row>
@@ -50368,27 +50372,27 @@
       </c>
       <c r="B762" s="5" t="inlineStr">
         <is>
-          <t>Jaren Kanak</t>
+          <t>D'Ernest Johnson</t>
         </is>
       </c>
       <c r="C762" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D762" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E762" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F762" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>Johnson agreed to a one-year contract with the Titans on Wednesday, NFL reporter Jordan Schultz reports.</t>
         </is>
       </c>
     </row>
@@ -50400,27 +50404,27 @@
       </c>
       <c r="B763" s="4" t="inlineStr">
         <is>
-          <t>Calvin Ridley</t>
+          <t>Kalel Mullings</t>
         </is>
       </c>
       <c r="C763" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D763" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E763" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F763" s="4" t="inlineStr">
         <is>
-          <t>Ridley caught his only target for 18 yards in Thursday's preseason win over San Francisco.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -50432,27 +50436,27 @@
       </c>
       <c r="B764" s="5" t="inlineStr">
         <is>
-          <t>Nicholas Singleton</t>
+          <t>Jaylen Harrell</t>
         </is>
       </c>
       <c r="C764" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D764" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E764" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F764" s="5" t="inlineStr">
         <is>
-          <t>Singleton rushed eight times for 31 yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -50464,27 +50468,27 @@
       </c>
       <c r="B765" s="4" t="inlineStr">
         <is>
-          <t>Tyjae Spears</t>
+          <t>Jaren Kanak</t>
         </is>
       </c>
       <c r="C765" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D765" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E765" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F765" s="4" t="inlineStr">
         <is>
-          <t>Spears rushed four times for 35 yards and brought in his only target for four yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -50496,7 +50500,7 @@
       </c>
       <c r="B766" s="5" t="inlineStr">
         <is>
-          <t>Wan'Dale Robinson</t>
+          <t>Calvin Ridley</t>
         </is>
       </c>
       <c r="C766" s="5" t="inlineStr">
@@ -50516,7 +50520,7 @@
       </c>
       <c r="F766" s="5" t="inlineStr">
         <is>
-          <t>Robinson brought in two of four targets for 19 yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
+          <t>Ridley caught his only target for 18 yards in Thursday's preseason win over San Francisco.</t>
         </is>
       </c>
     </row>
@@ -50528,12 +50532,12 @@
       </c>
       <c r="B767" s="4" t="inlineStr">
         <is>
-          <t>Gunnar Helm</t>
+          <t>Nicholas Singleton</t>
         </is>
       </c>
       <c r="C767" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D767" s="4" t="inlineStr">
@@ -50548,7 +50552,7 @@
       </c>
       <c r="F767" s="4" t="inlineStr">
         <is>
-          <t>Helm brought in his only target for 16 yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
+          <t>Singleton rushed eight times for 31 yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
         </is>
       </c>
     </row>
@@ -50560,12 +50564,12 @@
       </c>
       <c r="B768" s="5" t="inlineStr">
         <is>
-          <t>Cam Ward</t>
+          <t>Wan'Dale Robinson</t>
         </is>
       </c>
       <c r="C768" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D768" s="5" t="inlineStr">
@@ -50580,7 +50584,7 @@
       </c>
       <c r="F768" s="5" t="inlineStr">
         <is>
-          <t>Ward completed five of 12 targets for 57 yards with no touchdowns or interceptions and rushed once for two yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
+          <t>Robinson brought in two of four targets for 19 yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
         </is>
       </c>
     </row>
@@ -50592,12 +50596,12 @@
       </c>
       <c r="B769" s="4" t="inlineStr">
         <is>
-          <t>Elic Ayomanor</t>
+          <t>Gunnar Helm</t>
         </is>
       </c>
       <c r="C769" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D769" s="4" t="inlineStr">
@@ -50612,7 +50616,7 @@
       </c>
       <c r="F769" s="4" t="inlineStr">
         <is>
-          <t>Ayomanor (shoulder) is practicing Friday, Turron Davenport of ESPN.com reports.</t>
+          <t>Helm brought in his only target for 16 yards in the Titans' 19-13 preseason win over the 49ers on Thursday.</t>
         </is>
       </c>
     </row>
@@ -50624,12 +50628,12 @@
       </c>
       <c r="B770" s="5" t="inlineStr">
         <is>
-          <t>Mario Goodrich III</t>
+          <t>Elic Ayomanor</t>
         </is>
       </c>
       <c r="C770" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D770" s="5" t="inlineStr">
@@ -50644,7 +50648,7 @@
       </c>
       <c r="F770" s="5" t="inlineStr">
         <is>
-          <t>The Titans signed Goodrich to a contract Saturday, Jim Wyatt of the team's official site reports.</t>
+          <t>Ayomanor (shoulder) is practicing Friday, Turron Davenport of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -50656,27 +50660,27 @@
       </c>
       <c r="B771" s="4" t="inlineStr">
         <is>
-          <t>Sanoussi Kane</t>
+          <t>Mario Goodrich III</t>
         </is>
       </c>
       <c r="C771" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D771" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E771" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F771" s="4" t="inlineStr">
         <is>
-          <t>Kane (undisclosed) reverted to the Titans' injured reserve Friday, per the NFL's transaction log.</t>
+          <t>The Titans signed Goodrich to a contract Saturday, Jim Wyatt of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -50688,27 +50692,27 @@
       </c>
       <c r="B772" s="5" t="inlineStr">
         <is>
-          <t>Marcus Harris</t>
+          <t>Sanoussi Kane</t>
         </is>
       </c>
       <c r="C772" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D772" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E772" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F772" s="5" t="inlineStr">
         <is>
-          <t>Harris (knee) has been participating fully in training camp practices, Jim Wyatt of the Titans' official site reports.</t>
+          <t>Kane (undisclosed) reverted to the Titans' injured reserve Friday, per the NFL's transaction log.</t>
         </is>
       </c>
     </row>
@@ -50720,12 +50724,12 @@
       </c>
       <c r="B773" s="4" t="inlineStr">
         <is>
-          <t>Jeffery Simmons</t>
+          <t>Marcus Harris</t>
         </is>
       </c>
       <c r="C773" s="4" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D773" s="4" t="inlineStr">
@@ -50740,7 +50744,7 @@
       </c>
       <c r="F773" s="4" t="inlineStr">
         <is>
-          <t>Simmons (elbow) is participating at the Titans' training camp, George Walker of the Kingsport Times News reports.</t>
+          <t>Harris (knee) has been participating fully in training camp practices, Jim Wyatt of the Titans' official site reports.</t>
         </is>
       </c>
     </row>
@@ -50752,12 +50756,12 @@
       </c>
       <c r="B774" s="5" t="inlineStr">
         <is>
-          <t>JC Latham</t>
+          <t>Jeffery Simmons</t>
         </is>
       </c>
       <c r="C774" s="5" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D774" s="5" t="inlineStr">
@@ -50772,7 +50776,7 @@
       </c>
       <c r="F774" s="5" t="inlineStr">
         <is>
-          <t>Tennessee took Latham (undisclosed) off its active/PUP list Thursday, Buck Reising of WGFX-FM reports.</t>
+          <t>Simmons (elbow) is participating at the Titans' training camp, George Walker of the Kingsport Times News reports.</t>
         </is>
       </c>
     </row>
@@ -50784,12 +50788,12 @@
       </c>
       <c r="B775" s="4" t="inlineStr">
         <is>
-          <t>Oluwafemi Oladejo</t>
+          <t>JC Latham</t>
         </is>
       </c>
       <c r="C775" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D775" s="4" t="inlineStr">
@@ -50804,7 +50808,7 @@
       </c>
       <c r="F775" s="4" t="inlineStr">
         <is>
-          <t>Oladejo (hamstring) passed his conditioning test and is participating in the Titans' training camp activities, Jim Wyatt of the team's official site reports.</t>
+          <t>Tennessee took Latham (undisclosed) off its active/PUP list Thursday, Buck Reising of WGFX-FM reports.</t>
         </is>
       </c>
     </row>
@@ -50816,12 +50820,12 @@
       </c>
       <c r="B776" s="5" t="inlineStr">
         <is>
-          <t>Will Levis</t>
+          <t>Oluwafemi Oladejo</t>
         </is>
       </c>
       <c r="C776" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D776" s="5" t="inlineStr">
@@ -50836,7 +50840,7 @@
       </c>
       <c r="F776" s="5" t="inlineStr">
         <is>
-          <t>Levis is set to compete with Mitchell Trubisky for the backup quarterback role, Turron Davenport of ESPN.com reports.</t>
+          <t>Oladejo (hamstring) passed his conditioning test and is participating in the Titans' training camp activities, Jim Wyatt of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -50848,12 +50852,12 @@
       </c>
       <c r="B777" s="4" t="inlineStr">
         <is>
-          <t>Amani Hooker</t>
+          <t>Will Levis</t>
         </is>
       </c>
       <c r="C777" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D777" s="4" t="inlineStr">
@@ -50868,7 +50872,7 @@
       </c>
       <c r="F777" s="4" t="inlineStr">
         <is>
-          <t>The Titans activated Hooker (undisclosed) from the active/PUP list Tuesday, Jim Wyatt of the team's official site reports.</t>
+          <t>Levis is set to compete with Mitchell Trubisky for the backup quarterback role, Turron Davenport of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -50880,12 +50884,12 @@
       </c>
       <c r="B778" s="5" t="inlineStr">
         <is>
-          <t>Michael Carter</t>
+          <t>Amani Hooker</t>
         </is>
       </c>
       <c r="C778" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D778" s="5" t="inlineStr">
@@ -50900,7 +50904,7 @@
       </c>
       <c r="F778" s="5" t="inlineStr">
         <is>
-          <t>Carter will enter training camp competing for a depth role in Tennessee's backfield, Mark Mihalko of USA Today reports.</t>
+          <t>The Titans activated Hooker (undisclosed) from the active/PUP list Tuesday, Jim Wyatt of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -50912,12 +50916,12 @@
       </c>
       <c r="B779" s="4" t="inlineStr">
         <is>
-          <t>Chimere Dike</t>
+          <t>Michael Carter</t>
         </is>
       </c>
       <c r="C779" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D779" s="4" t="inlineStr">
@@ -50932,7 +50936,7 @@
       </c>
       <c r="F779" s="4" t="inlineStr">
         <is>
-          <t>As the coming season approaches, Nick Suss of the Nashville Tennessean projects that Dike is in line to compete for a rotational role in the Titans' re-tooled WR corps.</t>
+          <t>Carter will enter training camp competing for a depth role in Tennessee's backfield, Mark Mihalko of USA Today reports.</t>
         </is>
       </c>
     </row>
@@ -51832,26 +51836,30 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>71.8</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>5.8</v>
+        <v>7.1</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>10.1</v>
+        <v>19.7</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>31</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Wind 7 mph (gusts 20)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -51870,20 +51878,20 @@
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>75.09999999999999</v>
+        <v>70.3</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>2.6</v>
+        <v>11.3</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>2.7</v>
+        <v>13.2</v>
       </c>
       <c r="G6" s="17" t="n">
         <v>16</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Drizzle</t>
         </is>
       </c>
       <c r="I6" s="24" t="n">
@@ -51908,13 +51916,13 @@
         </is>
       </c>
       <c r="D7" s="15" t="n">
-        <v>108.3</v>
+        <v>107.6</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>16.9</v>
+        <v>22</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>15.4</v>
+        <v>21.7</v>
       </c>
       <c r="G7" s="15" t="n">
         <v>0</v>
@@ -51950,10 +51958,10 @@
         </is>
       </c>
       <c r="D8" s="17" t="n">
-        <v>79</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>8.6</v>
+        <v>7.5</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>6.7</v>
@@ -51963,7 +51971,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I8" s="24" t="n">
@@ -51988,20 +51996,20 @@
         </is>
       </c>
       <c r="D9" s="15" t="n">
-        <v>82</v>
+        <v>86.3</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>9.800000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="G9" s="15" t="n">
         <v>22</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Thunderstorm</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
@@ -52026,13 +52034,13 @@
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>88.8</v>
+        <v>89.2</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>11.6</v>
+        <v>5.7</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>12.3</v>
+        <v>5.8</v>
       </c>
       <c r="G10" s="17" t="n">
         <v>33</v>
@@ -52064,13 +52072,13 @@
         </is>
       </c>
       <c r="D11" s="15" t="n">
-        <v>83.09999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>5.9</v>
+        <v>4</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>11.9</v>
+        <v>13</v>
       </c>
       <c r="G11" s="15" t="n">
         <v>50</v>
@@ -52102,10 +52110,10 @@
         </is>
       </c>
       <c r="D12" s="17" t="n">
-        <v>83.2</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="F12" s="17" t="n">
         <v>9.4</v>
@@ -52115,7 +52123,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I12" s="24" t="n">
@@ -52140,30 +52148,26 @@
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>88.5</v>
+        <v>87.8</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>12.4</v>
+        <v>10.2</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>17</v>
+        <v>14.3</v>
       </c>
       <c r="G13" s="15" t="n">
         <v>52</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Wind 12 mph (gusts 17)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -52182,20 +52186,20 @@
         </is>
       </c>
       <c r="D14" s="17" t="n">
-        <v>82</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>6.9</v>
+        <v>11</v>
       </c>
       <c r="G14" s="17" t="n">
         <v>30</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I14" s="24" t="n">
@@ -52220,20 +52224,20 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>92.5</v>
+        <v>93.2</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>11.3</v>
+        <v>9.4</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>19</v>
+        <v>18.3</v>
       </c>
       <c r="G15" s="15" t="n">
         <v>4</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I15" s="9" t="n">
@@ -52241,7 +52245,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Wind 11 mph (gusts 19) · 92°F</t>
+          <t>Wind 9 mph (gusts 18) · 93°F</t>
         </is>
       </c>
     </row>
@@ -52262,20 +52266,20 @@
         </is>
       </c>
       <c r="D16" s="17" t="n">
-        <v>105.9</v>
+        <v>102.3</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>6</v>
+        <v>10.2</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="G16" s="17" t="n">
         <v>2</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I16" s="24" t="n">
@@ -52283,7 +52287,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>106°F · retractable roof — effect halved</t>
+          <t>102°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -52304,13 +52308,13 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>64.59999999999999</v>
+        <v>68</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>13</v>
+        <v>12.1</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>20.1</v>
+        <v>18.3</v>
       </c>
       <c r="G17" s="15" t="n">
         <v>2</v>
@@ -52325,7 +52329,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Wind 13 mph (gusts 20)</t>
+          <t>Wind 12 mph (gusts 18)</t>
         </is>
       </c>
     </row>
@@ -52346,26 +52350,30 @@
         </is>
       </c>
       <c r="D18" s="17" t="n">
-        <v>81.3</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>10.9</v>
+        <v>14.3</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>12.8</v>
+        <v>17.7</v>
       </c>
       <c r="G18" s="17" t="n">
         <v>18</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Wind 14 mph (gusts 18)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -52384,13 +52392,13 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>79.59999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>3.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>6.5</v>
+        <v>12.3</v>
       </c>
       <c r="G19" s="15" t="n">
         <v>2</v>
@@ -52422,26 +52430,30 @@
         </is>
       </c>
       <c r="D20" s="17" t="n">
-        <v>91.3</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F20" s="17" t="n">
-        <v>7.2</v>
+        <v>3.6</v>
       </c>
       <c r="G20" s="17" t="n">
         <v>1</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="5" t="inlineStr"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>94°F</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh: 2026-08-24 14:25 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -692,7 +692,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-08-24T08:03:54+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-08-24T14:25:16+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-08-24T08:03:54+00:00</t>
+          <t>2026-08-24T14:25:16+00:00</t>
         </is>
       </c>
     </row>
@@ -2779,16 +2779,16 @@
         <v>154</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4133</v>
+        <v>0.4178</v>
       </c>
       <c r="G10" s="13" t="n">
         <v>0.3937</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>0.0188</v>
+        <v>0.0227</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>0.04928467578930995</v>
+        <v>0.06065052683172301</v>
       </c>
       <c r="J10" s="14" t="n">
         <v>0.5</v>
@@ -2967,33 +2967,33 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Over 40.5</t>
+          <t>NE +3.5</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.5405</v>
+        <v>0.5415</v>
       </c>
       <c r="G15" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>0.0162</v>
+        <v>0.0171</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>0.03192423886530243</v>
+        <v>0.0336946163134072</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>0.5</v>
@@ -3008,33 +3008,33 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>CAR ML</t>
+          <t>Over 40.5</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>124</v>
+        <v>-110</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4611</v>
+        <v>0.5405</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.4464</v>
+        <v>0.5238</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0.0143</v>
+        <v>0.0162</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0.0325138851490685</v>
+        <v>0.03192423886530243</v>
       </c>
       <c r="J16" s="14" t="n">
         <v>0.5</v>
@@ -3049,33 +3049,33 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>CAR ML</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>-105</v>
+        <v>124</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.5266999999999999</v>
+        <v>0.4611</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.4464</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.0141</v>
+        <v>0.0143</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.02824070440763249</v>
+        <v>0.0325138851490685</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>0.5</v>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3100,23 +3100,23 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Over 40.5</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.538</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.0139</v>
+        <v>0.0141</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.02712503029680507</v>
+        <v>0.02824070440763249</v>
       </c>
       <c r="J18" s="14" t="n">
         <v>0.5</v>
@@ -3131,33 +3131,33 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>NE +3.5</t>
+          <t>Over 40.5</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.537</v>
+        <v>0.538</v>
       </c>
       <c r="G19" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.013</v>
+        <v>0.0139</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.0252193678819661</v>
+        <v>0.02712503029680507</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>0.5</v>
@@ -3476,16 +3476,16 @@
         <v>170</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.3741</v>
+        <v>0.3738</v>
       </c>
       <c r="G27" s="8" t="n">
         <v>0.3704</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.0037</v>
+        <v>0.0034</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.01004562953541044</v>
+        <v>0.009105696963362275</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>0.5</v>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>BAL @ IND</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -3551,23 +3551,23 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>WSH +4.5</t>
+          <t>IND +3.5</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>-110</v>
+        <v>-112</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>0.5265</v>
+        <v>0.5309</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5283</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.0027</v>
+        <v>0.0026</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.005078033170534846</v>
+        <v>0.004861104802833471</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>0.5</v>
@@ -3582,7 +3582,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>BAL @ IND</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -3592,23 +3592,23 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>IND +3.5</t>
+          <t>WSH +4.5</t>
         </is>
       </c>
       <c r="E30" s="12" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5309</v>
+        <v>0.5261</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.5283</v>
+        <v>0.5238</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>0.0026</v>
+        <v>0.0023</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>0.004861104802833471</v>
+        <v>0.004391528631370045</v>
       </c>
       <c r="J30" s="14" t="n">
         <v>0.5</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>Under 44.5</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -3649,7 +3649,7 @@
         <v>-0.001</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>-0.001823242235343747</v>
+        <v>-0.001817132797922338</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0.5</v>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -3674,23 +3674,23 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>Under 42.5</t>
         </is>
       </c>
       <c r="E32" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5203</v>
+        <v>0.5229</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>-0.0035</v>
+        <v>-0.001</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>-0.00665550171248247</v>
+        <v>-0.001823242235343747</v>
       </c>
       <c r="J32" s="14" t="n">
         <v>0.5</v>
@@ -4132,16 +4132,16 @@
         <v>124</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>0.4304</v>
+        <v>0.4306</v>
       </c>
       <c r="G43" s="8" t="n">
         <v>0.4464</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>-0.0156</v>
+        <v>-0.0154</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>-0.03563281766189008</v>
+        <v>-0.03523243596438208</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>0.5</v>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -4371,23 +4371,23 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>DAL -2.5</t>
+          <t>HOU +1.5</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
         <v>-115</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>0.5141</v>
+        <v>0.5139</v>
       </c>
       <c r="G49" s="8" t="n">
         <v>0.5349</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>-0.0199</v>
+        <v>-0.02</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>-0.03886992500392589</v>
+        <v>-0.03923258924631812</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>0.5</v>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>HOU +1.5</t>
+          <t>DAL -2.5</t>
         </is>
       </c>
       <c r="E50" s="12" t="n">
@@ -4428,7 +4428,7 @@
         <v>-0.02</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>-0.03923258924631812</v>
+        <v>-0.0392070114276778</v>
       </c>
       <c r="J50" s="14" t="n">
         <v>0.5</v>
@@ -4706,16 +4706,16 @@
         <v>-105</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>0.4859</v>
+        <v>0.4861</v>
       </c>
       <c r="G57" s="8" t="n">
         <v>0.5122</v>
       </c>
       <c r="H57" s="8" t="n">
-        <v>-0.0245</v>
+        <v>-0.0243</v>
       </c>
       <c r="I57" s="8" t="n">
-        <v>-0.0513240982517143</v>
+        <v>-0.05097207998194903</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>0.5</v>
@@ -4788,16 +4788,16 @@
         <v>-148</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>0.5696</v>
+        <v>0.5694</v>
       </c>
       <c r="G59" s="8" t="n">
         <v>0.5968</v>
       </c>
       <c r="H59" s="8" t="n">
-        <v>-0.0251</v>
+        <v>-0.0253</v>
       </c>
       <c r="I59" s="8" t="n">
-        <v>-0.04509709345712926</v>
+        <v>-0.04539652946240208</v>
       </c>
       <c r="J59" s="10" t="n">
         <v>0.5</v>
@@ -5345,33 +5345,33 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>LV ML</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
-        <v>-110</v>
+        <v>-205</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>0.4797</v>
+        <v>0.6269</v>
       </c>
       <c r="G73" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6721</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>-0.0366</v>
+        <v>-0.0372</v>
       </c>
       <c r="I73" s="8" t="n">
-        <v>-0.08425358919660841</v>
+        <v>-0.06667280051647667</v>
       </c>
       <c r="J73" s="10" t="n">
         <v>0.5</v>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -5396,23 +5396,23 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>LV ML</t>
+          <t>PHI ML</t>
         </is>
       </c>
       <c r="E74" s="12" t="n">
         <v>-205</v>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.6269</v>
+        <v>0.6262</v>
       </c>
       <c r="G74" s="13" t="n">
         <v>0.6721</v>
       </c>
       <c r="H74" s="13" t="n">
-        <v>-0.0372</v>
+        <v>-0.0376</v>
       </c>
       <c r="I74" s="13" t="n">
-        <v>-0.06667280051647667</v>
+        <v>-0.06770763182517281</v>
       </c>
       <c r="J74" s="14" t="n">
         <v>0.5</v>
@@ -5427,33 +5427,33 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>PHI ML</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
-        <v>-205</v>
+        <v>-110</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>0.6259</v>
+        <v>0.4771</v>
       </c>
       <c r="G75" s="8" t="n">
-        <v>0.6721</v>
+        <v>0.5238</v>
       </c>
       <c r="H75" s="8" t="n">
-        <v>-0.0377</v>
+        <v>-0.038</v>
       </c>
       <c r="I75" s="8" t="n">
-        <v>-0.06822534515899709</v>
+        <v>-0.08909195811116855</v>
       </c>
       <c r="J75" s="10" t="n">
         <v>0.5</v>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>BAL @ IND</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -5519,23 +5519,23 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>BAL -3.5</t>
+          <t>PHI -4.5</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>0.4691</v>
+        <v>0.4739</v>
       </c>
       <c r="G77" s="8" t="n">
-        <v>0.5192</v>
+        <v>0.5238</v>
       </c>
       <c r="H77" s="8" t="n">
-        <v>-0.0397</v>
+        <v>-0.0396</v>
       </c>
       <c r="I77" s="8" t="n">
-        <v>-0.09649040432769079</v>
+        <v>-0.09530061954046082</v>
       </c>
       <c r="J77" s="10" t="n">
         <v>0.5</v>
@@ -5550,33 +5550,33 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>BAL @ IND</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>LAR ML</t>
+          <t>BAL -3.5</t>
         </is>
       </c>
       <c r="E78" s="12" t="n">
-        <v>-192</v>
+        <v>-108</v>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.6073</v>
+        <v>0.4691</v>
       </c>
       <c r="G78" s="13" t="n">
-        <v>0.6575</v>
+        <v>0.5192</v>
       </c>
       <c r="H78" s="13" t="n">
-        <v>-0.0398</v>
+        <v>-0.0397</v>
       </c>
       <c r="I78" s="13" t="n">
-        <v>-0.07579738296532001</v>
+        <v>-0.09649040432769079</v>
       </c>
       <c r="J78" s="14" t="n">
         <v>0.5</v>
@@ -5591,33 +5591,33 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>PHI -4.5</t>
+          <t>LAR ML</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
-        <v>-110</v>
+        <v>-192</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>0.4735</v>
+        <v>0.6073</v>
       </c>
       <c r="G79" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6575</v>
       </c>
       <c r="H79" s="8" t="n">
         <v>-0.0398</v>
       </c>
       <c r="I79" s="8" t="n">
-        <v>-0.09598712407962567</v>
+        <v>-0.07579738296532001</v>
       </c>
       <c r="J79" s="10" t="n">
         <v>0.5</v>
@@ -5919,33 +5919,33 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>SEA -3.5</t>
+          <t>Under 42.5</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>0.463</v>
+        <v>0.4733</v>
       </c>
       <c r="G87" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H87" s="8" t="n">
-        <v>-0.0441</v>
+        <v>-0.0444</v>
       </c>
       <c r="I87" s="8" t="n">
-        <v>-0.1161284587910569</v>
+        <v>-0.1150597625451667</v>
       </c>
       <c r="J87" s="10" t="n">
         <v>0.5</v>
@@ -5960,38 +5960,42 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>LAC ML</t>
         </is>
       </c>
       <c r="E88" s="12" t="n">
-        <v>-115</v>
+        <v>-575</v>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.4733</v>
+        <v>0.7902</v>
       </c>
       <c r="G88" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.8519</v>
       </c>
       <c r="H88" s="13" t="n">
-        <v>-0.0444</v>
+        <v>-0.0445</v>
       </c>
       <c r="I88" s="13" t="n">
-        <v>-0.1150597625451667</v>
+        <v>-0.07194112640748435</v>
       </c>
       <c r="J88" s="14" t="n">
         <v>0.5</v>
       </c>
-      <c r="K88" s="5" t="inlineStr"/>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>price -575 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -6001,42 +6005,38 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>LAC ML</t>
+          <t>Under 40.5</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
-        <v>-575</v>
+        <v>-110</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>0.7902</v>
+        <v>0.462</v>
       </c>
       <c r="G89" s="8" t="n">
-        <v>0.8519</v>
+        <v>0.5238</v>
       </c>
       <c r="H89" s="8" t="n">
         <v>-0.0445</v>
       </c>
       <c r="I89" s="8" t="n">
-        <v>-0.07194112640748435</v>
+        <v>-0.1180341212058959</v>
       </c>
       <c r="J89" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K89" s="4" t="inlineStr">
-        <is>
-          <t>price -575 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -6063,16 +6063,16 @@
         <v>-110</v>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.462</v>
+        <v>0.4595</v>
       </c>
       <c r="G90" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H90" s="13" t="n">
-        <v>-0.0445</v>
+        <v>-0.0453</v>
       </c>
       <c r="I90" s="13" t="n">
-        <v>-0.1180341212058959</v>
+        <v>-0.1228333297743933</v>
       </c>
       <c r="J90" s="14" t="n">
         <v>0.5</v>
@@ -6092,28 +6092,28 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>SEA ML</t>
+          <t>SEA -3.5</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>-185</v>
+        <v>-110</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>0.5867</v>
+        <v>0.4585</v>
       </c>
       <c r="G91" s="8" t="n">
-        <v>0.6491</v>
+        <v>0.5238</v>
       </c>
       <c r="H91" s="8" t="n">
-        <v>-0.0447</v>
+        <v>-0.0456</v>
       </c>
       <c r="I91" s="8" t="n">
-        <v>-0.09527897345482961</v>
+        <v>-0.1246037072224981</v>
       </c>
       <c r="J91" s="10" t="n">
         <v>0.5</v>
@@ -6128,33 +6128,33 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Under 40.5</t>
+          <t>LAC -10.5</t>
         </is>
       </c>
       <c r="E92" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.4595</v>
+        <v>0.4576</v>
       </c>
       <c r="G92" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H92" s="13" t="n">
-        <v>-0.0453</v>
+        <v>-0.0459</v>
       </c>
       <c r="I92" s="13" t="n">
-        <v>-0.1228333297743933</v>
+        <v>-0.1263306720701867</v>
       </c>
       <c r="J92" s="14" t="n">
         <v>0.5</v>
@@ -6169,33 +6169,33 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>LAC -10.5</t>
+          <t>SEA ML</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
-        <v>-110</v>
+        <v>-185</v>
       </c>
       <c r="F93" s="8" t="n">
-        <v>0.4576</v>
+        <v>0.5822000000000001</v>
       </c>
       <c r="G93" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6491</v>
       </c>
       <c r="H93" s="8" t="n">
-        <v>-0.0459</v>
+        <v>-0.0461</v>
       </c>
       <c r="I93" s="8" t="n">
-        <v>-0.1263306720701867</v>
+        <v>-0.1021708430092774</v>
       </c>
       <c r="J93" s="10" t="n">
         <v>0.5</v>
@@ -7328,7 +7328,7 @@
         </is>
       </c>
       <c r="D9" s="24" t="n">
-        <v>-2.44</v>
+        <v>-2.43</v>
       </c>
       <c r="E9" s="24" t="n">
         <v>2.5</v>
@@ -7464,7 +7464,7 @@
         </is>
       </c>
       <c r="D13" s="24" t="n">
-        <v>4.17</v>
+        <v>4.19</v>
       </c>
       <c r="E13" s="24" t="n">
         <v>-4.5</v>
@@ -7804,13 +7804,13 @@
         </is>
       </c>
       <c r="D23" s="24" t="n">
-        <v>2.41</v>
+        <v>2.16</v>
       </c>
       <c r="E23" s="24" t="n">
         <v>-3.5</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>43.7</v>
+        <v>43.6</v>
       </c>
       <c r="G23" s="25" t="n">
         <v>44.5</v>
@@ -8681,7 +8681,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="18" t="n">
-        <v>-0.8</v>
+        <v>-0.83</v>
       </c>
       <c r="E26" s="18" t="n">
         <v>-0.8100000000000001</v>
@@ -8713,7 +8713,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>-1.39</v>
+        <v>-1.36</v>
       </c>
       <c r="E27" s="16" t="n">
         <v>0.02</v>
@@ -8809,7 +8809,7 @@
         <v>0</v>
       </c>
       <c r="D30" s="18" t="n">
-        <v>-2.31</v>
+        <v>-2.32</v>
       </c>
       <c r="E30" s="18" t="n">
         <v>-0.52</v>
@@ -8905,7 +8905,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>-3.24</v>
+        <v>-3.23</v>
       </c>
       <c r="E33" s="16" t="n">
         <v>-2.1</v>
@@ -14030,10 +14030,10 @@
         <v>45.5</v>
       </c>
       <c r="I104" s="12" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="J104" s="12" t="n">
-        <v>-325</v>
+        <v>-310</v>
       </c>
       <c r="K104" s="17" t="n">
         <v>0</v>
@@ -15190,7 +15190,7 @@
         </is>
       </c>
       <c r="G126" s="24" t="n">
-        <v>-2.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H126" s="25" t="n">
         <v>48.5</v>
@@ -15832,10 +15832,10 @@
         <v>44.5</v>
       </c>
       <c r="I138" s="12" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="J138" s="12" t="n">
-        <v>-142</v>
+        <v>-135</v>
       </c>
       <c r="K138" s="17" t="n">
         <v>0</v>
@@ -18588,10 +18588,10 @@
         <v>47.5</v>
       </c>
       <c r="I190" s="12" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="J190" s="12" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="K190" s="17" t="n">
         <v>0</v>
@@ -24047,10 +24047,10 @@
         <v>49.5</v>
       </c>
       <c r="I293" s="7" t="n">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="J293" s="7" t="n">
-        <v>-218</v>
+        <v>-205</v>
       </c>
       <c r="K293" s="15" t="n">
         <v>0</v>
@@ -25478,10 +25478,10 @@
         <v>41.5</v>
       </c>
       <c r="I320" s="12" t="n">
-        <v>-162</v>
+        <v>-155</v>
       </c>
       <c r="J320" s="12" t="n">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="K320" s="17" t="n">
         <v>0</v>
@@ -31904,7 +31904,7 @@
       </c>
       <c r="B180" s="5" t="inlineStr">
         <is>
-          <t>Taylen Green</t>
+          <t>Shedeur Sanders</t>
         </is>
       </c>
       <c r="C180" s="5" t="inlineStr">
@@ -31924,7 +31924,7 @@
       </c>
       <c r="F180" s="5" t="inlineStr">
         <is>
-          <t>Green is set to play in Thursday night's preseason finale against the Patriots, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
+          <t>Sanders will open the season as the Browns' backup quarterback after the team named Deshaun Watson its starter Monday, multiple sources tell NFL reporter Jordan Schultz.</t>
         </is>
       </c>
     </row>
@@ -31936,7 +31936,7 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Dillon Gabriel</t>
+          <t>Deshaun Watson</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -31956,7 +31956,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>Gabriel will start at quarterback in Thursday's preseason finale against the Patriots, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
+          <t>The Browns named Watson their starting quarterback Monday, multiple sources tell NFL reporter Jordan Schultz.</t>
         </is>
       </c>
     </row>
@@ -31968,12 +31968,12 @@
       </c>
       <c r="B182" s="5" t="inlineStr">
         <is>
-          <t>Shedeur Sanders</t>
+          <t>Denzel Boston</t>
         </is>
       </c>
       <c r="C182" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D182" s="5" t="inlineStr">
@@ -31988,7 +31988,7 @@
       </c>
       <c r="F182" s="5" t="inlineStr">
         <is>
-          <t>Sanders will learn Monday if he or Deshaun Watson will start at quarterback for the Browns, Jeremy Fowler of ESPN reports.</t>
+          <t>Boston went without a target while playing 11 snaps on offense Saturday in the Browns' 31-7 preseason loss to the Bills.</t>
         </is>
       </c>
     </row>
@@ -32000,7 +32000,7 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>Deshaun Watson</t>
+          <t>Taylen Green</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -32020,7 +32020,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>Watson will learn Monday if he or Shedeur Sanders will be named the starting quarterback for the Browns, Jeremy Fowler of ESPN reports.</t>
+          <t>Green is set to play in Thursday night's preseason finale against the Patriots, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
         </is>
       </c>
     </row>
@@ -32032,27 +32032,27 @@
       </c>
       <c r="B184" s="5" t="inlineStr">
         <is>
-          <t>Alex Wright</t>
+          <t>Dillon Gabriel</t>
         </is>
       </c>
       <c r="C184" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D184" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F184" s="5" t="inlineStr">
         <is>
-          <t>The Browns placed Wright on injured reserve Sunday due to a ruptured Achilles, Adam Schefter of ESPN reports.</t>
+          <t>Gabriel will start at quarterback in Thursday's preseason finale against the Patriots, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
         </is>
       </c>
     </row>
@@ -32064,7 +32064,7 @@
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Derek Barnett</t>
+          <t>Alex Wright</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
@@ -32074,17 +32074,17 @@
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>Barnett and the Browns agreed to a one-year contract worth up to $5.5 million Sunday, Jeremy Fowler of ESPN.com reports.</t>
+          <t>The Browns placed Wright on injured reserve Sunday due to a ruptured Achilles, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -32096,12 +32096,12 @@
       </c>
       <c r="B186" s="5" t="inlineStr">
         <is>
-          <t>Isaiah Bond</t>
+          <t>Derek Barnett</t>
         </is>
       </c>
       <c r="C186" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D186" s="5" t="inlineStr">
@@ -32116,7 +32116,7 @@
       </c>
       <c r="F186" s="5" t="inlineStr">
         <is>
-          <t>Bond cleared concussion protocol during Saturday's preseason game against the Bills.</t>
+          <t>Barnett and the Browns agreed to a one-year contract worth up to $5.5 million Sunday, Jeremy Fowler of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -32128,7 +32128,7 @@
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>Jerry Jeudy</t>
+          <t>Isaiah Bond</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
@@ -32148,7 +32148,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>Jeudy will not play in the Browns' preseason game against the Bills on Saturday, Daniel Oyefusi of ESPN.com reports.</t>
+          <t>Bond cleared concussion protocol during Saturday's preseason game against the Bills.</t>
         </is>
       </c>
     </row>
@@ -32160,27 +32160,27 @@
       </c>
       <c r="B188" s="5" t="inlineStr">
         <is>
-          <t>Carson Schwesinger</t>
+          <t>Jerry Jeudy</t>
         </is>
       </c>
       <c r="C188" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D188" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E188" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F188" s="5" t="inlineStr">
         <is>
-          <t>Schwesinger (undisclosed) is not expected to play in Saturday's preseason game against the Bills, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
+          <t>Jeudy will not play in the Browns' preseason game against the Bills on Saturday, Daniel Oyefusi of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -32192,12 +32192,12 @@
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>Cedric Tillman</t>
+          <t>Carson Schwesinger</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
@@ -32212,7 +32212,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>Tillman (undisclosed) is not expected to play in Saturday's preseason game against the Bills, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
+          <t>Schwesinger (undisclosed) is not expected to play in Saturday's preseason game against the Bills, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
         </is>
       </c>
     </row>
@@ -32224,12 +32224,12 @@
       </c>
       <c r="B190" s="5" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Cedric Tillman</t>
         </is>
       </c>
       <c r="C190" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D190" s="5" t="inlineStr">
@@ -32244,7 +32244,7 @@
       </c>
       <c r="F190" s="5" t="inlineStr">
         <is>
-          <t>Judkins (undisclosed) is not expected to play in Saturday's preseason game against the Bills, Kelsey Russo of the Browns' official site reports.</t>
+          <t>Tillman (undisclosed) is not expected to play in Saturday's preseason game against the Bills, Mary Kay Cabot of The Cleveland Plain Dealer reports.</t>
         </is>
       </c>
     </row>
@@ -32256,17 +32256,17 @@
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>Jack Stoll</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr">
@@ -32276,7 +32276,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>The Browns placed Stoll (undisclosed) on injured reserve Thursday.</t>
+          <t>Judkins (undisclosed) is not expected to play in Saturday's preseason game against the Bills, Kelsey Russo of the Browns' official site reports.</t>
         </is>
       </c>
     </row>
@@ -32288,7 +32288,7 @@
       </c>
       <c r="B192" s="5" t="inlineStr">
         <is>
-          <t>Drew Biber</t>
+          <t>Jack Stoll</t>
         </is>
       </c>
       <c r="C192" s="5" t="inlineStr">
@@ -32298,17 +32298,17 @@
       </c>
       <c r="D192" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E192" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F192" s="5" t="inlineStr">
         <is>
-          <t>The Browns signed Biber on Thursday.</t>
+          <t>The Browns placed Stoll (undisclosed) on injured reserve Thursday.</t>
         </is>
       </c>
     </row>
@@ -32320,27 +32320,27 @@
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Jamari Thrash</t>
+          <t>Drew Biber</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>The Browns signed Biber on Thursday.</t>
         </is>
       </c>
     </row>
@@ -32352,17 +32352,17 @@
       </c>
       <c r="B194" s="5" t="inlineStr">
         <is>
-          <t>Joe Royer</t>
+          <t>Jamari Thrash</t>
         </is>
       </c>
       <c r="C194" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D194" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E194" s="5" t="inlineStr">
@@ -32372,7 +32372,7 @@
       </c>
       <c r="F194" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -32384,7 +32384,7 @@
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Carsen Ryan</t>
+          <t>Joe Royer</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -32416,17 +32416,17 @@
       </c>
       <c r="B196" s="5" t="inlineStr">
         <is>
-          <t>Kendrick Green</t>
+          <t>Carsen Ryan</t>
         </is>
       </c>
       <c r="C196" s="5" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -32436,7 +32436,7 @@
       </c>
       <c r="F196" s="5" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -32448,12 +32448,12 @@
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>Tyron Herring</t>
+          <t>Kendrick Green</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
@@ -32480,7 +32480,7 @@
       </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
-          <t>Damarri Mathis</t>
+          <t>Tyron Herring</t>
         </is>
       </c>
       <c r="C198" s="5" t="inlineStr">
@@ -32512,25 +32512,29 @@
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>Nathaniel Watson</t>
+          <t>Damarri Mathis</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F199" s="4" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="inlineStr">
+        <is>
+          <t>ir</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="inlineStr">
@@ -32540,12 +32544,12 @@
       </c>
       <c r="B200" s="5" t="inlineStr">
         <is>
-          <t>Kingsley Eguakun</t>
+          <t>Nathaniel Watson</t>
         </is>
       </c>
       <c r="C200" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D200" s="5" t="inlineStr">
@@ -32568,7 +32572,7 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>Parker Brailsford</t>
+          <t>Kingsley Eguakun</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
@@ -32578,19 +32582,15 @@
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="F201" s="4" t="inlineStr">
-        <is>
-          <t>questionable</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="5" t="inlineStr">
@@ -32600,12 +32600,12 @@
       </c>
       <c r="B202" s="5" t="inlineStr">
         <is>
-          <t>Michael Coats Jr.</t>
+          <t>Parker Brailsford</t>
         </is>
       </c>
       <c r="C202" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D202" s="5" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>Nate Evans</t>
+          <t>Michael Coats Jr.</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -32664,25 +32664,29 @@
       </c>
       <c r="B204" s="5" t="inlineStr">
         <is>
-          <t>KC Concepcion</t>
+          <t>Nate Evans</t>
         </is>
       </c>
       <c r="C204" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D204" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F204" s="5" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F204" s="5" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
@@ -39071,7 +39075,7 @@
       </c>
       <c r="E406" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Sprain</t>
         </is>
       </c>
       <c r="F406" s="5" t="inlineStr">
@@ -42988,27 +42992,27 @@
       </c>
       <c r="B530" s="5" t="inlineStr">
         <is>
-          <t>Behren Morton</t>
+          <t>Bryce Baringer</t>
         </is>
       </c>
       <c r="C530" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D530" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E530" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F530" s="5" t="inlineStr">
         <is>
-          <t>Morton completed 13 of 17 passes for 129 yards with one touchdown and no interceptions while rushing once for minus-1 yard in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -43020,12 +43024,12 @@
       </c>
       <c r="B531" s="4" t="inlineStr">
         <is>
-          <t>Andy Borregales</t>
+          <t>Behren Morton</t>
         </is>
       </c>
       <c r="C531" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D531" s="4" t="inlineStr">
@@ -43040,7 +43044,7 @@
       </c>
       <c r="F531" s="4" t="inlineStr">
         <is>
-          <t>Borregales made his only field-goal attempt, from 41 yards out, and connected on all three extra-point tries in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
+          <t>Morton completed 13 of 17 passes for 129 yards with one touchdown and no interceptions while rushing once for minus-1 yard in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
         </is>
       </c>
     </row>
@@ -43052,12 +43056,12 @@
       </c>
       <c r="B532" s="5" t="inlineStr">
         <is>
-          <t>Kyle Williams</t>
+          <t>Andy Borregales</t>
         </is>
       </c>
       <c r="C532" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D532" s="5" t="inlineStr">
@@ -43072,7 +43076,7 @@
       </c>
       <c r="F532" s="5" t="inlineStr">
         <is>
-          <t>Williams brought in two of six targets for 74 yards and a touchdown in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
+          <t>Borregales made his only field-goal attempt, from 41 yards out, and connected on all three extra-point tries in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
         </is>
       </c>
     </row>
@@ -43084,27 +43088,27 @@
       </c>
       <c r="B533" s="4" t="inlineStr">
         <is>
-          <t>Marcus Bryant</t>
+          <t>Kyle Williams</t>
         </is>
       </c>
       <c r="C533" s="4" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D533" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E533" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F533" s="4" t="inlineStr">
         <is>
-          <t>Bryant has been ruled out for the rest of Saturday's preseason game against the Eagles due to an ankle injury, Evan Lazar of the Patriots' official site reports.</t>
+          <t>Williams brought in two of six targets for 74 yards and a touchdown in the Patriots' 24-21 preseason win over the Eagles on Saturday.</t>
         </is>
       </c>
     </row>
@@ -43116,12 +43120,12 @@
       </c>
       <c r="B534" s="5" t="inlineStr">
         <is>
-          <t>Christian Gonzalez</t>
+          <t>Marcus Bryant</t>
         </is>
       </c>
       <c r="C534" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D534" s="5" t="inlineStr">
@@ -43136,7 +43140,7 @@
       </c>
       <c r="F534" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>Bryant has been ruled out for the rest of Saturday's preseason game against the Eagles due to an ankle injury, Evan Lazar of the Patriots' official site reports.</t>
         </is>
       </c>
     </row>
@@ -43148,17 +43152,17 @@
       </c>
       <c r="B535" s="4" t="inlineStr">
         <is>
-          <t>Myles Montgomery</t>
+          <t>Christian Gonzalez</t>
         </is>
       </c>
       <c r="C535" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D535" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E535" s="4" t="inlineStr">
@@ -43168,7 +43172,7 @@
       </c>
       <c r="F535" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -43180,17 +43184,17 @@
       </c>
       <c r="B536" s="5" t="inlineStr">
         <is>
-          <t>Ben Brown</t>
+          <t>Myles Montgomery</t>
         </is>
       </c>
       <c r="C536" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D536" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E536" s="5" t="inlineStr">
@@ -43200,7 +43204,7 @@
       </c>
       <c r="F536" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -43212,25 +43216,29 @@
       </c>
       <c r="B537" s="4" t="inlineStr">
         <is>
-          <t>Carlton Davis III</t>
+          <t>Ben Brown</t>
         </is>
       </c>
       <c r="C537" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D537" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E537" s="4" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F537" s="4" t="inlineStr"/>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F537" s="4" t="inlineStr">
+        <is>
+          <t>questionable</t>
+        </is>
+      </c>
     </row>
     <row r="538">
       <c r="A538" s="5" t="inlineStr">
@@ -43240,12 +43248,12 @@
       </c>
       <c r="B538" s="5" t="inlineStr">
         <is>
-          <t>Quintayvious Hutchins</t>
+          <t>Carlton Davis III</t>
         </is>
       </c>
       <c r="C538" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D538" s="5" t="inlineStr">
@@ -43268,12 +43276,12 @@
       </c>
       <c r="B539" s="4" t="inlineStr">
         <is>
-          <t>Greg Van Roten</t>
+          <t>Quintayvious Hutchins</t>
         </is>
       </c>
       <c r="C539" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D539" s="4" t="inlineStr">
@@ -43286,11 +43294,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F539" s="4" t="inlineStr">
-        <is>
-          <t>The Patriots signed Van Roten on Tuesday.</t>
-        </is>
-      </c>
+      <c r="F539" s="4" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" s="5" t="inlineStr">
@@ -43300,12 +43304,12 @@
       </c>
       <c r="B540" s="5" t="inlineStr">
         <is>
-          <t>TreVeyon Henderson</t>
+          <t>Greg Van Roten</t>
         </is>
       </c>
       <c r="C540" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D540" s="5" t="inlineStr">
@@ -43320,7 +43324,7 @@
       </c>
       <c r="F540" s="5" t="inlineStr">
         <is>
-          <t>Chad Graff of The Athletic predicts that Rhamondre Stevenson and Henderson seem likely to share New England's backfield work pretty evenly this coming season.</t>
+          <t>The Patriots signed Van Roten on Tuesday.</t>
         </is>
       </c>
     </row>
@@ -43332,7 +43336,7 @@
       </c>
       <c r="B541" s="4" t="inlineStr">
         <is>
-          <t>Rhamondre Stevenson</t>
+          <t>TreVeyon Henderson</t>
         </is>
       </c>
       <c r="C541" s="4" t="inlineStr">
@@ -43352,7 +43356,7 @@
       </c>
       <c r="F541" s="4" t="inlineStr">
         <is>
-          <t>Chad Graff of The Athletic predicts that Stevenson and TreVeyon Henderson are likely to share New England's backfield work pretty evenly this coming season.</t>
+          <t>Chad Graff of The Athletic predicts that Rhamondre Stevenson and Henderson seem likely to share New England's backfield work pretty evenly this coming season.</t>
         </is>
       </c>
     </row>
@@ -43364,12 +43368,12 @@
       </c>
       <c r="B542" s="5" t="inlineStr">
         <is>
-          <t>Drake Maye</t>
+          <t>Rhamondre Stevenson</t>
         </is>
       </c>
       <c r="C542" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D542" s="5" t="inlineStr">
@@ -43384,7 +43388,7 @@
       </c>
       <c r="F542" s="5" t="inlineStr">
         <is>
-          <t>Maye completed every pass during the first two periods of practice Monday, including a deep ball to A.J. Brown, Taylor Kyles of CLNSMedia.com reports.</t>
+          <t>Chad Graff of The Athletic predicts that Stevenson and TreVeyon Henderson are likely to share New England's backfield work pretty evenly this coming season.</t>
         </is>
       </c>
     </row>
@@ -43396,12 +43400,12 @@
       </c>
       <c r="B543" s="4" t="inlineStr">
         <is>
-          <t>Romeo Doubs</t>
+          <t>Drake Maye</t>
         </is>
       </c>
       <c r="C543" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D543" s="4" t="inlineStr">
@@ -43416,7 +43420,7 @@
       </c>
       <c r="F543" s="4" t="inlineStr">
         <is>
-          <t>Doubs was the standout wide receiver during the Patriots' training camp practice Saturday, Taylor Kyles of CLNSMedia.com reports.</t>
+          <t>Maye completed every pass during the first two periods of practice Monday, including a deep ball to A.J. Brown, Taylor Kyles of CLNSMedia.com reports.</t>
         </is>
       </c>
     </row>
@@ -43428,7 +43432,7 @@
       </c>
       <c r="B544" s="5" t="inlineStr">
         <is>
-          <t>Kayshon Boutte</t>
+          <t>Romeo Doubs</t>
         </is>
       </c>
       <c r="C544" s="5" t="inlineStr">
@@ -43448,7 +43452,7 @@
       </c>
       <c r="F544" s="5" t="inlineStr">
         <is>
-          <t>Boutte logged 16 snaps in Thursday's preseason opener against the Colts.</t>
+          <t>Doubs was the standout wide receiver during the Patriots' training camp practice Saturday, Taylor Kyles of CLNSMedia.com reports.</t>
         </is>
       </c>
     </row>
@@ -43460,7 +43464,7 @@
       </c>
       <c r="B545" s="4" t="inlineStr">
         <is>
-          <t>DeMario Douglas</t>
+          <t>Kayshon Boutte</t>
         </is>
       </c>
       <c r="C545" s="4" t="inlineStr">
@@ -43480,7 +43484,7 @@
       </c>
       <c r="F545" s="4" t="inlineStr">
         <is>
-          <t>Douglas was among the Patriots' key skill players who didn't play in Thursday's preseason opener against the Colts,  Mark Daniels of masslive.com reports.</t>
+          <t>Boutte logged 16 snaps in Thursday's preseason opener against the Colts.</t>
         </is>
       </c>
     </row>
@@ -43492,7 +43496,7 @@
       </c>
       <c r="B546" s="5" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeMario Douglas</t>
         </is>
       </c>
       <c r="C546" s="5" t="inlineStr">
@@ -43512,7 +43516,7 @@
       </c>
       <c r="F546" s="5" t="inlineStr">
         <is>
-          <t>Brown was among the Patriots' key skill players who didn't see action in Thursday's preseason opener against the Colts, Evan Lazar of the team's official site reports.</t>
+          <t>Douglas was among the Patriots' key skill players who didn't play in Thursday's preseason opener against the Colts,  Mark Daniels of masslive.com reports.</t>
         </is>
       </c>
     </row>
@@ -43524,12 +43528,12 @@
       </c>
       <c r="B547" s="4" t="inlineStr">
         <is>
-          <t>Jam Miller</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="C547" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D547" s="4" t="inlineStr">
@@ -43544,7 +43548,7 @@
       </c>
       <c r="F547" s="4" t="inlineStr">
         <is>
-          <t>Miller carried the ball 14 times for 55 yards and failed to catch his only target in Thursday's 13-13 preseason tie with the Colts.</t>
+          <t>Brown was among the Patriots' key skill players who didn't see action in Thursday's preseason opener against the Colts, Evan Lazar of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -43556,7 +43560,7 @@
       </c>
       <c r="B548" s="5" t="inlineStr">
         <is>
-          <t>Lan Larison</t>
+          <t>Jam Miller</t>
         </is>
       </c>
       <c r="C548" s="5" t="inlineStr">
@@ -43576,7 +43580,7 @@
       </c>
       <c r="F548" s="5" t="inlineStr">
         <is>
-          <t>Larison gained just one yard on seven carries in Thursday's 13-13 preseason tie with the Colts, but he caught six of eight targets for 38 yards.</t>
+          <t>Miller carried the ball 14 times for 55 yards and failed to catch his only target in Thursday's 13-13 preseason tie with the Colts.</t>
         </is>
       </c>
     </row>
@@ -43588,12 +43592,12 @@
       </c>
       <c r="B549" s="4" t="inlineStr">
         <is>
-          <t>Mack Hollins</t>
+          <t>Lan Larison</t>
         </is>
       </c>
       <c r="C549" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D549" s="4" t="inlineStr">
@@ -43608,7 +43612,7 @@
       </c>
       <c r="F549" s="4" t="inlineStr">
         <is>
-          <t>Hollins caught two of four targets for 24 yards in Thursday's 13-13 preseason tie with the Colts.</t>
+          <t>Larison gained just one yard on seven carries in Thursday's 13-13 preseason tie with the Colts, but he caught six of eight targets for 38 yards.</t>
         </is>
       </c>
     </row>
@@ -43620,12 +43624,12 @@
       </c>
       <c r="B550" s="5" t="inlineStr">
         <is>
-          <t>Jared Wilson</t>
+          <t>Mack Hollins</t>
         </is>
       </c>
       <c r="C550" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D550" s="5" t="inlineStr">
@@ -43640,7 +43644,7 @@
       </c>
       <c r="F550" s="5" t="inlineStr">
         <is>
-          <t>Wilson (knee) was a full participant in Thursday's practice, Brooks Kubena of The Athletic reports.</t>
+          <t>Hollins caught two of four targets for 24 yards in Thursday's 13-13 preseason tie with the Colts.</t>
         </is>
       </c>
     </row>
@@ -43652,12 +43656,12 @@
       </c>
       <c r="B551" s="4" t="inlineStr">
         <is>
-          <t>JaMycal Hasty</t>
+          <t>Jared Wilson</t>
         </is>
       </c>
       <c r="C551" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D551" s="4" t="inlineStr">
@@ -43672,7 +43676,7 @@
       </c>
       <c r="F551" s="4" t="inlineStr">
         <is>
-          <t>Hasty and the Patriots agreed on a one-year contract Wednesday, Aaron Wilson of KPRC 2 Houston reports.</t>
+          <t>Wilson (knee) was a full participant in Thursday's practice, Brooks Kubena of The Athletic reports.</t>
         </is>
       </c>
     </row>
@@ -43684,7 +43688,7 @@
       </c>
       <c r="B552" s="5" t="inlineStr">
         <is>
-          <t>Hassan Haskins</t>
+          <t>JaMycal Hasty</t>
         </is>
       </c>
       <c r="C552" s="5" t="inlineStr">
@@ -43704,7 +43708,7 @@
       </c>
       <c r="F552" s="5" t="inlineStr">
         <is>
-          <t>New England signed Haskins on Wednesday.</t>
+          <t>Hasty and the Patriots agreed on a one-year contract Wednesday, Aaron Wilson of KPRC 2 Houston reports.</t>
         </is>
       </c>
     </row>
@@ -43716,12 +43720,12 @@
       </c>
       <c r="B553" s="4" t="inlineStr">
         <is>
-          <t>Hunter Henry</t>
+          <t>Hassan Haskins</t>
         </is>
       </c>
       <c r="C553" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D553" s="4" t="inlineStr">
@@ -43736,7 +43740,7 @@
       </c>
       <c r="F553" s="4" t="inlineStr">
         <is>
-          <t>Henry agreed to a two-year, $16 million contract extension with the Patriots on Monday, Adam Schefter of ESPN reports.</t>
+          <t>New England signed Haskins on Wednesday.</t>
         </is>
       </c>
     </row>
@@ -43748,7 +43752,7 @@
       </c>
       <c r="B554" s="5" t="inlineStr">
         <is>
-          <t>CJ Dippre</t>
+          <t>Hunter Henry</t>
         </is>
       </c>
       <c r="C554" s="5" t="inlineStr">
@@ -43768,7 +43772,7 @@
       </c>
       <c r="F554" s="5" t="inlineStr">
         <is>
-          <t>The Patriots activated Dippre (undisclosed) off the active/PUP list Wednesday, Mike Reiss of ESPN.com reports.</t>
+          <t>Henry agreed to a two-year, $16 million contract extension with the Patriots on Monday, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -48556,27 +48560,27 @@
       </c>
       <c r="B705" s="4" t="inlineStr">
         <is>
-          <t>Drew Lock</t>
+          <t>Rodney Thomas II</t>
         </is>
       </c>
       <c r="C705" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D705" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E705" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F705" s="4" t="inlineStr">
         <is>
-          <t>Lock completed 12 of 14 passes for 103 yards and a touchdown while rushing twice for eight yards in Sunday's 19-16 preseason loss to the Titans.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -48588,27 +48592,27 @@
       </c>
       <c r="B706" s="5" t="inlineStr">
         <is>
-          <t>Emmanuel Henderson Jr.</t>
+          <t>Mason Richman</t>
         </is>
       </c>
       <c r="C706" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D706" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Doubtful</t>
         </is>
       </c>
       <c r="E706" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F706" s="5" t="inlineStr">
         <is>
-          <t>Henderson caught one of two targets for seven yards in Sunday's 19-16 preseason loss to the Titans. He also returned two kickoffs for 47 yards and notched two solo tackles on special teams.</t>
+          <t>doubtful</t>
         </is>
       </c>
     </row>
@@ -48620,27 +48624,27 @@
       </c>
       <c r="B707" s="4" t="inlineStr">
         <is>
-          <t>Elijah Arroyo</t>
+          <t>Bud Clark</t>
         </is>
       </c>
       <c r="C707" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D707" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E707" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Fracture</t>
         </is>
       </c>
       <c r="F707" s="4" t="inlineStr">
         <is>
-          <t>Arroyo caught two of four targets for 50 yards and a touchdown in Sunday's 19-16 preseason loss to the Titans.</t>
+          <t>Seahawks head coach Mike Macdonald said that Clark will be out for "multiple months" after fracturing his right ankle in Sunday's 19-16 preseason loss to Tennessee, Brady Henderson of ESPN.com reports.</t>
         </is>
       </c>
     </row>
@@ -48652,27 +48656,27 @@
       </c>
       <c r="B708" s="5" t="inlineStr">
         <is>
-          <t>Bud Clark</t>
+          <t>Drew Lock</t>
         </is>
       </c>
       <c r="C708" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D708" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E708" s="5" t="inlineStr">
         <is>
-          <t>Leg</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F708" s="5" t="inlineStr">
         <is>
-          <t>Clark was carted off the field with a right leg injury during Sunday's preseason matchup with the Titans, Brady Henderson of ESPN.com reports.</t>
+          <t>Lock completed 12 of 14 passes for 103 yards and a touchdown while rushing twice for eight yards in Sunday's 19-16 preseason loss to the Titans.</t>
         </is>
       </c>
     </row>
@@ -48684,12 +48688,12 @@
       </c>
       <c r="B709" s="4" t="inlineStr">
         <is>
-          <t>Jadarian Price</t>
+          <t>Emmanuel Henderson Jr.</t>
         </is>
       </c>
       <c r="C709" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D709" s="4" t="inlineStr">
@@ -48704,7 +48708,7 @@
       </c>
       <c r="F709" s="4" t="inlineStr">
         <is>
-          <t>Price will not play in Sunday's preseason game against the Titans, Gregg Bell of The Tacoma News Tribune reports.</t>
+          <t>Henderson caught one of two targets for seven yards in Sunday's 19-16 preseason loss to the Titans. He also returned two kickoffs for 47 yards and notched two solo tackles on special teams.</t>
         </is>
       </c>
     </row>
@@ -48716,12 +48720,12 @@
       </c>
       <c r="B710" s="5" t="inlineStr">
         <is>
-          <t>Julian Hicks</t>
+          <t>Elijah Arroyo</t>
         </is>
       </c>
       <c r="C710" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D710" s="5" t="inlineStr">
@@ -48736,7 +48740,7 @@
       </c>
       <c r="F710" s="5" t="inlineStr">
         <is>
-          <t>The Seahawks signed Hicks to a contract Saturday, John Boyle of the team's official site reports.</t>
+          <t>Arroyo caught two of four targets for 50 yards and a touchdown in Sunday's 19-16 preseason loss to the Titans.</t>
         </is>
       </c>
     </row>
@@ -48748,27 +48752,27 @@
       </c>
       <c r="B711" s="4" t="inlineStr">
         <is>
-          <t>Jake Bobo</t>
+          <t>Jadarian Price</t>
         </is>
       </c>
       <c r="C711" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D711" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E711" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F711" s="4" t="inlineStr">
         <is>
-          <t>The Seahawks placed Bobo (knee) on injured reserve Saturday, John Boyle of the team's official site reports.</t>
+          <t>Price will not play in Sunday's preseason game against the Titans, Gregg Bell of The Tacoma News Tribune reports.</t>
         </is>
       </c>
     </row>
@@ -48780,12 +48784,12 @@
       </c>
       <c r="B712" s="5" t="inlineStr">
         <is>
-          <t>Trevon Diggs</t>
+          <t>Julian Hicks</t>
         </is>
       </c>
       <c r="C712" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D712" s="5" t="inlineStr">
@@ -48800,7 +48804,7 @@
       </c>
       <c r="F712" s="5" t="inlineStr">
         <is>
-          <t>The Seahawks are slated to sign Diggs to a one-year deal, Adam Schefter of ESPN reports.</t>
+          <t>The Seahawks signed Hicks to a contract Saturday, John Boyle of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -48812,12 +48816,12 @@
       </c>
       <c r="B713" s="4" t="inlineStr">
         <is>
-          <t>Joseph Vaughn</t>
+          <t>Jake Bobo</t>
         </is>
       </c>
       <c r="C713" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D713" s="4" t="inlineStr">
@@ -48832,7 +48836,7 @@
       </c>
       <c r="F713" s="4" t="inlineStr">
         <is>
-          <t>ir</t>
+          <t>The Seahawks placed Bobo (knee) on injured reserve Saturday, John Boyle of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -48844,27 +48848,27 @@
       </c>
       <c r="B714" s="5" t="inlineStr">
         <is>
-          <t>Emanuel Wilson</t>
+          <t>Trevon Diggs</t>
         </is>
       </c>
       <c r="C714" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D714" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E714" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F714" s="5" t="inlineStr">
         <is>
-          <t>questionable</t>
+          <t>The Seahawks are slated to sign Diggs to a one-year deal, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -48876,12 +48880,12 @@
       </c>
       <c r="B715" s="4" t="inlineStr">
         <is>
-          <t>Robbie Ouzts</t>
+          <t>Joseph Vaughn</t>
         </is>
       </c>
       <c r="C715" s="4" t="inlineStr">
         <is>
-          <t>FB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D715" s="4" t="inlineStr">
@@ -48908,12 +48912,12 @@
       </c>
       <c r="B716" s="5" t="inlineStr">
         <is>
-          <t>Tory Horton</t>
+          <t>Emanuel Wilson</t>
         </is>
       </c>
       <c r="C716" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D716" s="5" t="inlineStr">
@@ -48923,7 +48927,7 @@
       </c>
       <c r="E716" s="5" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F716" s="5" t="inlineStr">
@@ -48940,12 +48944,12 @@
       </c>
       <c r="B717" s="4" t="inlineStr">
         <is>
-          <t>Shemar Jean-Charles</t>
+          <t>Robbie Ouzts</t>
         </is>
       </c>
       <c r="C717" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>FB</t>
         </is>
       </c>
       <c r="D717" s="4" t="inlineStr">
@@ -48972,12 +48976,12 @@
       </c>
       <c r="B718" s="5" t="inlineStr">
         <is>
-          <t>Nick Emmanwori</t>
+          <t>Tory Horton</t>
         </is>
       </c>
       <c r="C718" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D718" s="5" t="inlineStr">
@@ -48987,7 +48991,7 @@
       </c>
       <c r="E718" s="5" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Undisclosed</t>
         </is>
       </c>
       <c r="F718" s="5" t="inlineStr">
@@ -49004,27 +49008,27 @@
       </c>
       <c r="B719" s="4" t="inlineStr">
         <is>
-          <t>Anthony Hankerson</t>
+          <t>Shemar Jean-Charles</t>
         </is>
       </c>
       <c r="C719" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D719" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E719" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F719" s="4" t="inlineStr">
         <is>
-          <t>Hankerson and the Seahawks agreed on a contract Monday, John Boyle of the team's official website reports.</t>
+          <t>ir</t>
         </is>
       </c>
     </row>
@@ -49036,27 +49040,27 @@
       </c>
       <c r="B720" s="5" t="inlineStr">
         <is>
-          <t>Montorie Foster Jr.</t>
+          <t>Nick Emmanwori</t>
         </is>
       </c>
       <c r="C720" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D720" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E720" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F720" s="5" t="inlineStr">
         <is>
-          <t>Foster caught five of seven targets for 36 yards and a touchdown in Saturday's 17-7 preseason loss to the Cowboys, building on what has been a strong performance in training camp, John Boyle of the Seahawks' official site reports.</t>
+          <t>questionable</t>
         </is>
       </c>
     </row>
@@ -49068,12 +49072,12 @@
       </c>
       <c r="B721" s="4" t="inlineStr">
         <is>
-          <t>Rashid Shaheed</t>
+          <t>Anthony Hankerson</t>
         </is>
       </c>
       <c r="C721" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D721" s="4" t="inlineStr">
@@ -49088,7 +49092,7 @@
       </c>
       <c r="F721" s="4" t="inlineStr">
         <is>
-          <t>Shaheed didn't suit up for Saturday's 17-7 preseason loss to the Cowboys.</t>
+          <t>Hankerson and the Seahawks agreed on a contract Monday, John Boyle of the team's official website reports.</t>
         </is>
       </c>
     </row>
@@ -49100,12 +49104,12 @@
       </c>
       <c r="B722" s="5" t="inlineStr">
         <is>
-          <t>AJ Barner</t>
+          <t>Montorie Foster Jr.</t>
         </is>
       </c>
       <c r="C722" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D722" s="5" t="inlineStr">
@@ -49120,7 +49124,7 @@
       </c>
       <c r="F722" s="5" t="inlineStr">
         <is>
-          <t>Barner was rested for Seattle's 17-7 preseason loss to the Cowboys on Saturday.</t>
+          <t>Foster caught five of seven targets for 36 yards and a touchdown in Saturday's 17-7 preseason loss to the Cowboys, building on what has been a strong performance in training camp, John Boyle of the Seahawks' official site reports.</t>
         </is>
       </c>
     </row>
@@ -49132,27 +49136,27 @@
       </c>
       <c r="B723" s="4" t="inlineStr">
         <is>
-          <t>Zach Charbonnet</t>
+          <t>Rashid Shaheed</t>
         </is>
       </c>
       <c r="C723" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D723" s="4" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E723" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F723" s="4" t="inlineStr">
         <is>
-          <t>Charbonnet (knee) remains on the active/PUP list as the Seahawks' second preseason contest (Sunday, Aug. 23 versus the Titans) approaches.</t>
+          <t>Shaheed didn't suit up for Saturday's 17-7 preseason loss to the Cowboys.</t>
         </is>
       </c>
     </row>
@@ -49164,12 +49168,12 @@
       </c>
       <c r="B724" s="5" t="inlineStr">
         <is>
-          <t>Jason Myers</t>
+          <t>AJ Barner</t>
         </is>
       </c>
       <c r="C724" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D724" s="5" t="inlineStr">
@@ -49184,7 +49188,7 @@
       </c>
       <c r="F724" s="5" t="inlineStr">
         <is>
-          <t>Myers missed his only field-goal attempt from 45 yards out and made his only extra-point try in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
+          <t>Barner was rested for Seattle's 17-7 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -49196,7 +49200,7 @@
       </c>
       <c r="B725" s="4" t="inlineStr">
         <is>
-          <t>George Holani</t>
+          <t>Zach Charbonnet</t>
         </is>
       </c>
       <c r="C725" s="4" t="inlineStr">
@@ -49206,17 +49210,17 @@
       </c>
       <c r="D725" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E725" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F725" s="4" t="inlineStr">
         <is>
-          <t>Holani rushed 12 times for 42 yards in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
+          <t>Charbonnet (knee) remains on the active/PUP list as the Seahawks' second preseason contest (Sunday, Aug. 23 versus the Titans) approaches.</t>
         </is>
       </c>
     </row>
@@ -49228,12 +49232,12 @@
       </c>
       <c r="B726" s="5" t="inlineStr">
         <is>
-          <t>Devon Witherspoon</t>
+          <t>Jason Myers</t>
         </is>
       </c>
       <c r="C726" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D726" s="5" t="inlineStr">
@@ -49248,7 +49252,7 @@
       </c>
       <c r="F726" s="5" t="inlineStr">
         <is>
-          <t>Witherspoon and the Seahawks agreed to a four-year, $132 million contract extension Saturday, Adam Schefter of ESPN reports.</t>
+          <t>Myers missed his only field-goal attempt from 45 yards out and made his only extra-point try in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -49260,12 +49264,12 @@
       </c>
       <c r="B727" s="4" t="inlineStr">
         <is>
-          <t>DeMarcus Lawrence</t>
+          <t>George Holani</t>
         </is>
       </c>
       <c r="C727" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D727" s="4" t="inlineStr">
@@ -49280,7 +49284,7 @@
       </c>
       <c r="F727" s="4" t="inlineStr">
         <is>
-          <t>Lawrence has declared that he will retire after the 2026 season, Jori Epstein of Yahoo Sports reports.</t>
+          <t>Holani rushed 12 times for 42 yards in the Seahawks' 17-7 preseason loss to the Cowboys on Saturday.</t>
         </is>
       </c>
     </row>
@@ -49292,12 +49296,12 @@
       </c>
       <c r="B728" s="5" t="inlineStr">
         <is>
-          <t>Sam Darnold</t>
+          <t>Devon Witherspoon</t>
         </is>
       </c>
       <c r="C728" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D728" s="5" t="inlineStr">
@@ -49312,7 +49316,7 @@
       </c>
       <c r="F728" s="5" t="inlineStr">
         <is>
-          <t>Coach Mike Macdonald said Friday that Darnold won't suit up for Saturday's preseason game versus the Cowboys, Curtis Crabtree of Fox 13 Seattle reports.</t>
+          <t>Witherspoon and the Seahawks agreed to a four-year, $132 million contract extension Saturday, Adam Schefter of ESPN reports.</t>
         </is>
       </c>
     </row>
@@ -49324,12 +49328,12 @@
       </c>
       <c r="B729" s="4" t="inlineStr">
         <is>
-          <t>Jaxon Smith-Njigba</t>
+          <t>DeMarcus Lawrence</t>
         </is>
       </c>
       <c r="C729" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D729" s="4" t="inlineStr">
@@ -49344,7 +49348,7 @@
       </c>
       <c r="F729" s="4" t="inlineStr">
         <is>
-          <t>Smith-Njigba is always willing to be coached up in an attempt to be a better player, Anthony Moeglin of Roundtable Sports reports.</t>
+          <t>Lawrence has declared that he will retire after the 2026 season, Jori Epstein of Yahoo Sports reports.</t>
         </is>
       </c>
     </row>
@@ -51836,16 +51840,16 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>71.40000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>19.7</v>
+        <v>15.7</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -51853,13 +51857,9 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Wind 7 mph (gusts 20)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -51878,20 +51878,20 @@
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>70.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>11.3</v>
+        <v>4.3</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>13.2</v>
+        <v>4.5</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Drizzle</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I6" s="24" t="n">
@@ -51916,20 +51916,20 @@
         </is>
       </c>
       <c r="D7" s="15" t="n">
-        <v>107.6</v>
+        <v>107.4</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>22</v>
+        <v>19.5</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>21.7</v>
+        <v>20.6</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
@@ -51958,20 +51958,20 @@
         </is>
       </c>
       <c r="D8" s="17" t="n">
-        <v>79.59999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>7.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>6.7</v>
+        <v>7.2</v>
       </c>
       <c r="G8" s="17" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I8" s="24" t="n">
@@ -51996,16 +51996,16 @@
         </is>
       </c>
       <c r="D9" s="15" t="n">
-        <v>86.3</v>
+        <v>86.2</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>3.4</v>
+        <v>4.9</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -52034,26 +52034,30 @@
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>89.2</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>5.7</v>
+        <v>13.1</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>5.8</v>
+        <v>13</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="5" t="inlineStr"/>
+        <v>-0.68</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Wind 13 mph (gusts 13) · canopy — wind damped</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -52072,16 +52076,16 @@
         </is>
       </c>
       <c r="D11" s="15" t="n">
-        <v>82.2</v>
+        <v>84.2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>13</v>
+        <v>2.9</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -52110,13 +52114,13 @@
         </is>
       </c>
       <c r="D12" s="17" t="n">
-        <v>82.90000000000001</v>
+        <v>85.8</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>5.9</v>
+        <v>5.3</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>9.4</v>
+        <v>5.8</v>
       </c>
       <c r="G12" s="17" t="n">
         <v>23</v>
@@ -52148,26 +52152,30 @@
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>87.8</v>
+        <v>78.3</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>10.2</v>
+        <v>8.9</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>14.3</v>
+        <v>10.7</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Violent showers</t>
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>55% chance of rain</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -52186,16 +52194,16 @@
         </is>
       </c>
       <c r="D14" s="17" t="n">
-        <v>82.90000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>11</v>
+        <v>12.3</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -52224,30 +52232,26 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>93.2</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>9.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>18.3</v>
+        <v>15.2</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I15" s="9" t="n">
-        <v>-1.3</v>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Wind 9 mph (gusts 18) · 93°F</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -52266,20 +52270,20 @@
         </is>
       </c>
       <c r="D16" s="17" t="n">
-        <v>102.3</v>
+        <v>104.1</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>10.2</v>
+        <v>6</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>7.2</v>
+        <v>10.1</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I16" s="24" t="n">
@@ -52287,7 +52291,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>102°F · retractable roof — effect halved</t>
+          <t>104°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -52308,16 +52312,16 @@
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>68</v>
+        <v>65.7</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>12.1</v>
+        <v>11.4</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>18.3</v>
+        <v>18.6</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -52329,7 +52333,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Wind 12 mph (gusts 18)</t>
+          <t>Wind 11 mph (gusts 19)</t>
         </is>
       </c>
     </row>
@@ -52350,30 +52354,26 @@
         </is>
       </c>
       <c r="D18" s="17" t="n">
-        <v>80.90000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>14.3</v>
+        <v>9.6</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>17.7</v>
+        <v>12.5</v>
       </c>
       <c r="G18" s="17" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I18" s="24" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Wind 14 mph (gusts 18)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -52392,20 +52392,20 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>81.59999999999999</v>
+        <v>81</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>8.300000000000001</v>
+        <v>4.9</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>12.3</v>
+        <v>5.4</v>
       </c>
       <c r="G19" s="15" t="n">
         <v>2</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
@@ -52430,20 +52430,20 @@
         </is>
       </c>
       <c r="D20" s="17" t="n">
-        <v>94.40000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="F20" s="17" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I20" s="24" t="n">
@@ -52451,7 +52451,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>94°F</t>
+          <t>92°F</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh: 2026-09-01 12:04 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -224,8 +224,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBest" displayName="tblBest" ref="A4:N8" headerRowCount="1">
-  <autoFilter ref="A4:N8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBest" displayName="tblBest" ref="A4:N9" headerRowCount="1">
+  <autoFilter ref="A4:N9"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Tier"/>
     <tableColumn id="2" name="Game"/>
@@ -692,7 +692,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-09-01T05:13:27+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-09-01T12:04:47+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-09-01T05:13:27+00:00</t>
+          <t>2026-09-01T12:04:47+00:00</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2466,39 +2466,39 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>Under 49.5</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5849</v>
+        <v>0.5714</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>0.0442</v>
+        <v>0.0436</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>0.0611</v>
+        <v>0.0592</v>
       </c>
       <c r="J6" s="14" t="n">
-        <v>-3.42</v>
+        <v>-3.05</v>
       </c>
       <c r="K6" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="L6" s="16" t="n">
-        <v>18.1</v>
+        <v>19.5</v>
       </c>
       <c r="M6" s="16" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -2510,49 +2510,49 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Under 49.5</t>
+          <t>MIA ML</t>
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>-105</v>
+        <v>470</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.5714</v>
+        <v>0.2336</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.1754</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>0.0436</v>
+        <v>0.0431</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.0592</v>
+        <v>0.0581</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>-3.05</v>
+        <v>-1.79</v>
       </c>
       <c r="K7" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>19.5</v>
+        <v>18.4</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>27</v>
+        <v>27.1</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2564,49 +2564,103 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>MIA ML</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>470</v>
+        <v>-110</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.2336</v>
+        <v>0.5752</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.1754</v>
+        <v>0.5238</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>0.0431</v>
+        <v>0.0403</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>0.0581</v>
+        <v>0.0514</v>
       </c>
       <c r="J8" s="14" t="n">
-        <v>-1.79</v>
+        <v>-3.02</v>
       </c>
       <c r="K8" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="L8" s="16" t="n">
-        <v>18.4</v>
+        <v>21</v>
       </c>
       <c r="M8" s="16" t="n">
-        <v>27.1</v>
+        <v>24.5</v>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>LEAN</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>NYJ @ TEN</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Over 38.5</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>-115</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0.5863</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.5349</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0.0403</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0.0514</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2814,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2770,23 +2824,23 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>Under 49.5</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5849</v>
+        <v>0.5714</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>0.0442</v>
+        <v>0.0436</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>0.1165958889485751</v>
+        <v>0.1156289126830108</v>
       </c>
       <c r="J6" s="15" t="n">
         <v>0.5</v>
@@ -2801,33 +2855,33 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Under 49.5</t>
+          <t>MIA ML</t>
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>-105</v>
+        <v>470</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.5714</v>
+        <v>0.2336</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.1754</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>0.0436</v>
+        <v>0.0431</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.1156289126830108</v>
+        <v>0.3288535048635309</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>0.5</v>
@@ -2842,33 +2896,33 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>MIA ML</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>470</v>
+        <v>-110</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.2336</v>
+        <v>0.5752</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.1754</v>
+        <v>0.5238</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>0.0431</v>
+        <v>0.0403</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>0.3288535048635309</v>
+        <v>0.09813079684167703</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>0.5</v>
@@ -2878,47 +2932,43 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SEA @ ARI</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>ARI ML</t>
+          <t>Over 38.5</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>410</v>
+        <v>-115</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.2556</v>
+        <v>0.5863</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.1961</v>
+        <v>0.5349</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>0.0437</v>
+        <v>0.0403</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.3013869591776513</v>
+        <v>0.09609813123903277</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>correlated with a stronger play on the same game</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2928,33 +2978,33 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>SEA @ ARI</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>MIA +10.5</t>
+          <t>ARI ML</t>
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>-110</v>
+        <v>410</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5784</v>
+        <v>0.2556</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.1961</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>0.0417</v>
+        <v>0.0437</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>0.1041938633967684</v>
+        <v>0.3013869591776513</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>0.5</v>
@@ -2973,38 +3023,42 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>MIA +10.5</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>0.5616</v>
+        <v>0.5784</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>0.0394</v>
+        <v>0.0417</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>0.09650071503637747</v>
+        <v>0.1041938633967684</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>correlated with a stronger play on the same game</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3014,7 +3068,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -3024,23 +3078,23 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Over 38.5</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>-115</v>
+        <v>-105</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5814</v>
+        <v>0.5616</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5122</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>0.0379</v>
+        <v>0.0394</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>0.08704652960204162</v>
+        <v>0.09650071503637747</v>
       </c>
       <c r="J12" s="15" t="n">
         <v>0.5</v>
@@ -3564,16 +3618,16 @@
         <v>300</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>0.2796</v>
+        <v>0.2797</v>
       </c>
       <c r="G25" s="8" t="n">
         <v>0.25</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>0.027</v>
+        <v>0.0271</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.1172753011722295</v>
+        <v>0.1179143496855546</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>0.5</v>
@@ -3711,7 +3765,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -3721,23 +3775,23 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>Under 42.5</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>0.5641</v>
+        <v>0.5505</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.5413</v>
+        <v>0.5238</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.0216</v>
+        <v>0.0248</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.04211539969282557</v>
+        <v>0.05101886947689394</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>0.5</v>
@@ -3752,33 +3806,33 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>LV @ LAC</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>LV ML</t>
+          <t>Under 51.5</t>
         </is>
       </c>
       <c r="E30" s="12" t="n">
-        <v>295</v>
+        <v>-118</v>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.2754</v>
+        <v>0.5641</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.2532</v>
+        <v>0.5413</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>0.0211</v>
+        <v>0.0216</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>0.08718388052155757</v>
+        <v>0.04211539969282557</v>
       </c>
       <c r="J30" s="15" t="n">
         <v>0.5</v>
@@ -3793,33 +3847,33 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>NYG @ LAR</t>
+          <t>LV @ LAC</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>NYG +8.5</t>
+          <t>LV ML</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>-110</v>
+        <v>295</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.5457</v>
+        <v>0.2754</v>
       </c>
       <c r="G31" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.2532</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>0.0208</v>
+        <v>0.0211</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>0.04184409282887513</v>
+        <v>0.08718388052155757</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0.5</v>
@@ -3875,33 +3929,33 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>NYG @ LAR</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>NE ML</t>
+          <t>NYG +8.5</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>150</v>
+        <v>-110</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>0.4203</v>
+        <v>0.5454</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>0.4</v>
+        <v>0.5238</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>0.0194</v>
+        <v>0.0205</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>0.05021125444334651</v>
+        <v>0.04114550651634863</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.5</v>
@@ -3916,7 +3970,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>PHI @ TEN</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -3926,23 +3980,23 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>TEN ML</t>
+          <t>NE ML</t>
         </is>
       </c>
       <c r="E34" s="12" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3762</v>
+        <v>0.4203</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.3571</v>
+        <v>0.4</v>
       </c>
       <c r="H34" s="13" t="n">
-        <v>0.0183</v>
+        <v>0.0194</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>0.05284850326466584</v>
+        <v>0.05021125444334651</v>
       </c>
       <c r="J34" s="15" t="n">
         <v>0.5</v>
@@ -3957,33 +4011,33 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>PHI @ TEN</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>CLE +7.5</t>
+          <t>TEN ML</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>-110</v>
+        <v>180</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.542</v>
+        <v>0.3762</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.3571</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>0.0176</v>
+        <v>0.0183</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>0.0347828407971677</v>
+        <v>0.05284850326466584</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>0.5</v>
@@ -3998,33 +4052,33 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>MIA ML</t>
+          <t>CLE +7.5</t>
         </is>
       </c>
       <c r="E36" s="12" t="n">
-        <v>164</v>
+        <v>-110</v>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.3971</v>
+        <v>0.5422</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.3788</v>
+        <v>0.5238</v>
       </c>
       <c r="H36" s="13" t="n">
-        <v>0.0176</v>
+        <v>0.0177</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>0.04787514855665331</v>
+        <v>0.03512992094286965</v>
       </c>
       <c r="J36" s="15" t="n">
         <v>0.5</v>
@@ -4039,7 +4093,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -4049,23 +4103,23 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>MIN ML</t>
+          <t>MIA ML</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
         <v>164</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>0.3962</v>
+        <v>0.3971</v>
       </c>
       <c r="G37" s="8" t="n">
         <v>0.3788</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0176</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>0.0455345620803117</v>
+        <v>0.04787514855665331</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>0.5</v>
@@ -4080,33 +4134,33 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>IND +6.5</t>
+          <t>MIN ML</t>
         </is>
       </c>
       <c r="E38" s="12" t="n">
-        <v>-110</v>
+        <v>164</v>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5411</v>
+        <v>0.3962</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.3788</v>
       </c>
       <c r="H38" s="13" t="n">
         <v>0.0168</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>0.03303001835355274</v>
+        <v>0.0455345620803117</v>
       </c>
       <c r="J38" s="15" t="n">
         <v>0.5</v>
@@ -4121,33 +4175,33 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>NYG @ LAR</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>NYG ML</t>
+          <t>IND +6.5</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>300</v>
+        <v>-110</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.2672</v>
+        <v>0.5411</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>0.25</v>
+        <v>0.5238</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>0.0166</v>
+        <v>0.0168</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>0.0681184473903711</v>
+        <v>0.03303001835355274</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>0.5</v>
@@ -4162,33 +4216,33 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>NYG @ LAR</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>NYG ML</t>
         </is>
       </c>
       <c r="E40" s="12" t="n">
-        <v>-110</v>
+        <v>300</v>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5405</v>
+        <v>0.2668</v>
       </c>
       <c r="G40" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.25</v>
       </c>
       <c r="H40" s="13" t="n">
-        <v>0.0162</v>
+        <v>0.0163</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>0.0319130781248223</v>
+        <v>0.06687638084325775</v>
       </c>
       <c r="J40" s="15" t="n">
         <v>0.5</v>
@@ -4203,33 +4257,33 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Over 40.5</t>
+          <t>NE +3.5</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>0.538</v>
+        <v>0.5456</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>0.0139</v>
+        <v>0.0106</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>0.02712503029680507</v>
+        <v>0.02004531325434894</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>0.5</v>
@@ -4249,28 +4303,28 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>NE +3.5</t>
+          <t>Under 44.5</t>
         </is>
       </c>
       <c r="E42" s="12" t="n">
         <v>-115</v>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5456</v>
+        <v>0.5443</v>
       </c>
       <c r="G42" s="13" t="n">
         <v>0.5349</v>
       </c>
       <c r="H42" s="13" t="n">
-        <v>0.0106</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>0.02004531325434894</v>
+        <v>0.01763314497491086</v>
       </c>
       <c r="J42" s="15" t="n">
         <v>0.5</v>
@@ -4285,33 +4339,33 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>CAR @ ATL</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>SF ML</t>
+          <t>Under 43.5</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>164</v>
+        <v>-102</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>0.3883</v>
+        <v>0.5142</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>0.3788</v>
+        <v>0.505</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>0.0095</v>
+        <v>0.0092</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>0.02501076933874147</v>
+        <v>0.01840603867218615</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>0.5</v>
@@ -4326,33 +4380,33 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>PHI @ TEN</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>TEN +4.5</t>
         </is>
       </c>
       <c r="E44" s="12" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.5443</v>
+        <v>0.5331</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H44" s="13" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0092</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>0.01763314497491086</v>
+        <v>0.01775328317101132</v>
       </c>
       <c r="J44" s="15" t="n">
         <v>0.5</v>
@@ -4367,33 +4421,33 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>CAR @ ATL</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Under 43.5</t>
+          <t>SF ML</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>-102</v>
+        <v>164</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.5142</v>
+        <v>0.388</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>0.505</v>
+        <v>0.3788</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>0.0092</v>
+        <v>0.0091</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>0.01840603867218615</v>
+        <v>0.02408115735673189</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>0.5</v>
@@ -4408,33 +4462,33 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>PHI @ TEN</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>TEN +4.5</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E46" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.5331</v>
+        <v>0.533</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H46" s="13" t="n">
-        <v>0.0092</v>
+        <v>0.0091</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>0.01775328317101132</v>
+        <v>0.01749282810775288</v>
       </c>
       <c r="J46" s="15" t="n">
         <v>0.5</v>
@@ -4449,7 +4503,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -4459,23 +4513,23 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>0.533</v>
+        <v>0.5191</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>0.0091</v>
+        <v>0.0068</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>0.01749282810775288</v>
+        <v>0.01342415224820337</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>0.5</v>
@@ -4490,7 +4544,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -4500,23 +4554,23 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>Over 40.5</t>
         </is>
       </c>
       <c r="E48" s="12" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5191</v>
+        <v>0.5305</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H48" s="13" t="n">
-        <v>0.0068</v>
+        <v>0.0066</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>0.01342415224820337</v>
+        <v>0.01268771139495323</v>
       </c>
       <c r="J48" s="15" t="n">
         <v>0.5</v>
@@ -4999,16 +5053,16 @@
         <v>-130</v>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.5667</v>
+        <v>0.5666</v>
       </c>
       <c r="G60" s="13" t="n">
         <v>0.5652</v>
       </c>
       <c r="H60" s="13" t="n">
-        <v>0.0015</v>
+        <v>0.0013</v>
       </c>
       <c r="I60" s="13" t="n">
-        <v>0.002661666039075805</v>
+        <v>0.002347016438638383</v>
       </c>
       <c r="J60" s="15" t="n">
         <v>0.5</v>
@@ -5163,16 +5217,16 @@
         <v>-115</v>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.5348000000000001</v>
+        <v>0.5347</v>
       </c>
       <c r="G64" s="13" t="n">
         <v>0.5349</v>
       </c>
       <c r="H64" s="13" t="n">
-        <v>-0</v>
+        <v>-0.0002</v>
       </c>
       <c r="I64" s="13" t="n">
-        <v>-7.207569994466256e-05</v>
+        <v>-0.000408162702336401</v>
       </c>
       <c r="J64" s="15" t="n">
         <v>0.5</v>
@@ -5351,33 +5405,33 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>SF +3.5</t>
+          <t>BUF ML</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
-        <v>-108</v>
+        <v>-118</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>0.5157</v>
+        <v>0.5374</v>
       </c>
       <c r="G69" s="8" t="n">
-        <v>0.5192</v>
+        <v>0.5413</v>
       </c>
       <c r="H69" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0038</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>-0.006886285227016176</v>
+        <v>-0.007024902242636077</v>
       </c>
       <c r="J69" s="10" t="n">
         <v>0.5</v>
@@ -5392,33 +5446,33 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>BUF ML</t>
+          <t>SF +3.5</t>
         </is>
       </c>
       <c r="E70" s="12" t="n">
-        <v>-118</v>
+        <v>-108</v>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.5374</v>
+        <v>0.5153</v>
       </c>
       <c r="G70" s="13" t="n">
-        <v>0.5413</v>
+        <v>0.5192</v>
       </c>
       <c r="H70" s="13" t="n">
-        <v>-0.0038</v>
+        <v>-0.0039</v>
       </c>
       <c r="I70" s="13" t="n">
-        <v>-0.007024902242636077</v>
+        <v>-0.00757828565733093</v>
       </c>
       <c r="J70" s="15" t="n">
         <v>0.5</v>
@@ -5450,16 +5504,16 @@
         <v>124</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>0.4421</v>
+        <v>0.442</v>
       </c>
       <c r="G71" s="8" t="n">
         <v>0.4464</v>
       </c>
       <c r="H71" s="8" t="n">
-        <v>-0.0043</v>
+        <v>-0.0045</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>-0.009524547947419304</v>
+        <v>-0.009927378901474437</v>
       </c>
       <c r="J71" s="10" t="n">
         <v>0.5</v>
@@ -5491,16 +5545,16 @@
         <v>200</v>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.3287</v>
+        <v>0.3286</v>
       </c>
       <c r="G72" s="13" t="n">
         <v>0.3333</v>
       </c>
       <c r="H72" s="13" t="n">
-        <v>-0.0046</v>
+        <v>-0.0047</v>
       </c>
       <c r="I72" s="13" t="n">
-        <v>-0.01364986484133868</v>
+        <v>-0.01414912923927325</v>
       </c>
       <c r="J72" s="15" t="n">
         <v>0.5</v>
@@ -5614,16 +5668,16 @@
         <v>-105</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>0.5058</v>
+        <v>0.5059</v>
       </c>
       <c r="G75" s="8" t="n">
         <v>0.5122</v>
       </c>
       <c r="H75" s="8" t="n">
-        <v>-0.0064</v>
+        <v>-0.0062</v>
       </c>
       <c r="I75" s="8" t="n">
-        <v>-0.01257807639092878</v>
+        <v>-0.01222345728980595</v>
       </c>
       <c r="J75" s="10" t="n">
         <v>0.5</v>
@@ -5761,33 +5815,33 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>BUF ML</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
-        <v>-110</v>
+        <v>-155</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>0.5127</v>
+        <v>0.5962</v>
       </c>
       <c r="G79" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6078</v>
       </c>
       <c r="H79" s="8" t="n">
-        <v>-0.0109</v>
+        <v>-0.0115</v>
       </c>
       <c r="I79" s="8" t="n">
-        <v>-0.02118472397290833</v>
+        <v>-0.01906002789140349</v>
       </c>
       <c r="J79" s="10" t="n">
         <v>0.5</v>
@@ -5802,7 +5856,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>WSH @ DAL</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -5812,23 +5866,23 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>BUF ML</t>
+          <t>DAL ML</t>
         </is>
       </c>
       <c r="E80" s="12" t="n">
-        <v>-155</v>
+        <v>-205</v>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.5962</v>
+        <v>0.6602</v>
       </c>
       <c r="G80" s="13" t="n">
-        <v>0.6078</v>
+        <v>0.6721</v>
       </c>
       <c r="H80" s="13" t="n">
-        <v>-0.0115</v>
+        <v>-0.0117</v>
       </c>
       <c r="I80" s="13" t="n">
-        <v>-0.01906002789140349</v>
+        <v>-0.01757170464578495</v>
       </c>
       <c r="J80" s="15" t="n">
         <v>0.5</v>
@@ -5843,33 +5897,33 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>WSH @ DAL</t>
+          <t>CAR @ ATL</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>DAL ML</t>
+          <t>ATL -1.5</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
-        <v>-205</v>
+        <v>-110</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>0.6601</v>
+        <v>0.5114</v>
       </c>
       <c r="G81" s="8" t="n">
-        <v>0.6721</v>
+        <v>0.5238</v>
       </c>
       <c r="H81" s="8" t="n">
-        <v>-0.0119</v>
+        <v>-0.0122</v>
       </c>
       <c r="I81" s="8" t="n">
-        <v>-0.01781868529128067</v>
+        <v>-0.02369008041236687</v>
       </c>
       <c r="J81" s="10" t="n">
         <v>0.5</v>
@@ -5884,7 +5938,7 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>CAR @ ATL</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -5894,23 +5948,23 @@
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>ATL -1.5</t>
+          <t>BUF -3</t>
         </is>
       </c>
       <c r="E82" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.5114</v>
+        <v>0.5105</v>
       </c>
       <c r="G82" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H82" s="13" t="n">
-        <v>-0.0122</v>
+        <v>-0.0131</v>
       </c>
       <c r="I82" s="13" t="n">
-        <v>-0.02369008041236687</v>
+        <v>-0.02366289073816819</v>
       </c>
       <c r="J82" s="15" t="n">
         <v>0.5</v>
@@ -5925,7 +5979,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -5935,23 +5989,23 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>BUF -3</t>
+          <t>NYG +2.5</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>0.5105</v>
+        <v>0.4974</v>
       </c>
       <c r="G83" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>-0.0131</v>
+        <v>-0.0144</v>
       </c>
       <c r="I83" s="8" t="n">
-        <v>-0.02366289073816819</v>
+        <v>-0.02879040426669344</v>
       </c>
       <c r="J83" s="10" t="n">
         <v>0.5</v>
@@ -5966,33 +6020,33 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>NYG +2.5</t>
+          <t>ATL ML</t>
         </is>
       </c>
       <c r="E84" s="12" t="n">
-        <v>-105</v>
+        <v>145</v>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.4976</v>
+        <v>0.3922</v>
       </c>
       <c r="G84" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.4082</v>
       </c>
       <c r="H84" s="13" t="n">
-        <v>-0.0142</v>
+        <v>-0.0155</v>
       </c>
       <c r="I84" s="13" t="n">
-        <v>-0.02843835042789322</v>
+        <v>-0.03881419460589064</v>
       </c>
       <c r="J84" s="15" t="n">
         <v>0.5</v>
@@ -6007,33 +6061,33 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>ATL ML</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
-        <v>145</v>
+        <v>-110</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>0.3924</v>
+        <v>0.5076000000000001</v>
       </c>
       <c r="G85" s="8" t="n">
-        <v>0.4082</v>
+        <v>0.5238</v>
       </c>
       <c r="H85" s="8" t="n">
-        <v>-0.0154</v>
+        <v>-0.0157</v>
       </c>
       <c r="I85" s="8" t="n">
-        <v>-0.03838502881250883</v>
+        <v>-0.03088766692791661</v>
       </c>
       <c r="J85" s="10" t="n">
         <v>0.5</v>
@@ -6106,16 +6160,16 @@
         <v>-205</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>0.6553</v>
+        <v>0.6556999999999999</v>
       </c>
       <c r="G87" s="8" t="n">
         <v>0.6721</v>
       </c>
       <c r="H87" s="8" t="n">
-        <v>-0.0163</v>
+        <v>-0.016</v>
       </c>
       <c r="I87" s="8" t="n">
-        <v>-0.02476211020273922</v>
+        <v>-0.02426438295817168</v>
       </c>
       <c r="J87" s="10" t="n">
         <v>0.5</v>
@@ -6188,16 +6242,16 @@
         <v>-110</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>0.5062</v>
+        <v>0.5061</v>
       </c>
       <c r="G89" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H89" s="8" t="n">
-        <v>-0.017</v>
+        <v>-0.0172</v>
       </c>
       <c r="I89" s="8" t="n">
-        <v>-0.03353074385385046</v>
+        <v>-0.0338779412367774</v>
       </c>
       <c r="J89" s="10" t="n">
         <v>0.5</v>
@@ -6352,16 +6406,16 @@
         <v>-110</v>
       </c>
       <c r="F93" s="8" t="n">
-        <v>0.5044999999999999</v>
+        <v>0.5048</v>
       </c>
       <c r="G93" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H93" s="8" t="n">
-        <v>-0.0186</v>
+        <v>-0.0183</v>
       </c>
       <c r="I93" s="8" t="n">
-        <v>-0.03694058913192133</v>
+        <v>-0.03624731383348789</v>
       </c>
       <c r="J93" s="10" t="n">
         <v>0.5</v>
@@ -6417,33 +6471,33 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>JAX @ DEN</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>ATL +3</t>
+          <t>JAX ML</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F95" s="8" t="n">
-        <v>0.4794</v>
+        <v>0.4339</v>
       </c>
       <c r="G95" s="8" t="n">
-        <v>0.5</v>
+        <v>0.4545</v>
       </c>
       <c r="H95" s="8" t="n">
         <v>-0.0197</v>
       </c>
       <c r="I95" s="8" t="n">
-        <v>-0.03818131037285988</v>
+        <v>-0.04497708260678568</v>
       </c>
       <c r="J95" s="10" t="n">
         <v>0.5</v>
@@ -6458,33 +6512,33 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>JAX @ DEN</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>JAX ML</t>
+          <t>ATL +3</t>
         </is>
       </c>
       <c r="E96" s="12" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.4339</v>
+        <v>0.4792</v>
       </c>
       <c r="G96" s="13" t="n">
-        <v>0.4545</v>
+        <v>0.5</v>
       </c>
       <c r="H96" s="13" t="n">
-        <v>-0.0197</v>
+        <v>-0.0198</v>
       </c>
       <c r="I96" s="13" t="n">
-        <v>-0.04497708260678568</v>
+        <v>-0.03854042707833383</v>
       </c>
       <c r="J96" s="15" t="n">
         <v>0.5</v>
@@ -6926,16 +6980,16 @@
         <v>-120</v>
       </c>
       <c r="F107" s="8" t="n">
-        <v>0.5206</v>
+        <v>0.5208</v>
       </c>
       <c r="G107" s="8" t="n">
         <v>0.5455</v>
       </c>
       <c r="H107" s="8" t="n">
-        <v>-0.0233</v>
+        <v>-0.0232</v>
       </c>
       <c r="I107" s="8" t="n">
-        <v>-0.04232167579267038</v>
+        <v>-0.04199259833787239</v>
       </c>
       <c r="J107" s="10" t="n">
         <v>0.5</v>
@@ -7032,33 +7086,33 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>JAX @ DEN</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>WSH ML</t>
+          <t>JAX +2.5</t>
         </is>
       </c>
       <c r="E110" s="12" t="n">
-        <v>170</v>
+        <v>-105</v>
       </c>
       <c r="F110" s="13" t="n">
-        <v>0.3447</v>
+        <v>0.4864</v>
       </c>
       <c r="G110" s="13" t="n">
-        <v>0.3704</v>
+        <v>0.5122</v>
       </c>
       <c r="H110" s="13" t="n">
         <v>-0.024</v>
       </c>
       <c r="I110" s="13" t="n">
-        <v>-0.06887082213294937</v>
+        <v>-0.05026802719465456</v>
       </c>
       <c r="J110" s="15" t="n">
         <v>0.5</v>
@@ -7073,33 +7127,33 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>JAX @ DEN</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>JAX +2.5</t>
+          <t>WSH ML</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
-        <v>-105</v>
+        <v>170</v>
       </c>
       <c r="F111" s="8" t="n">
-        <v>0.4864</v>
+        <v>0.3443</v>
       </c>
       <c r="G111" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.3704</v>
       </c>
       <c r="H111" s="8" t="n">
-        <v>-0.024</v>
+        <v>-0.0243</v>
       </c>
       <c r="I111" s="8" t="n">
-        <v>-0.05026802719465456</v>
+        <v>-0.06977463081454904</v>
       </c>
       <c r="J111" s="10" t="n">
         <v>0.5</v>
@@ -7196,33 +7250,33 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>ATL @ PIT</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>WSH +4.5</t>
+          <t>PIT ML</t>
         </is>
       </c>
       <c r="E114" s="12" t="n">
-        <v>-110</v>
+        <v>-175</v>
       </c>
       <c r="F114" s="13" t="n">
-        <v>0.4955</v>
+        <v>0.6078</v>
       </c>
       <c r="G114" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.6364</v>
       </c>
       <c r="H114" s="13" t="n">
-        <v>-0.026</v>
+        <v>-0.0262</v>
       </c>
       <c r="I114" s="13" t="n">
-        <v>-0.0539685017771695</v>
+        <v>-0.04446946701398502</v>
       </c>
       <c r="J114" s="15" t="n">
         <v>0.5</v>
@@ -7237,33 +7291,33 @@
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>ATL @ PIT</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>PIT ML</t>
+          <t>WSH +4.5</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
-        <v>-175</v>
+        <v>-110</v>
       </c>
       <c r="F115" s="8" t="n">
-        <v>0.6076</v>
+        <v>0.4952</v>
       </c>
       <c r="G115" s="8" t="n">
-        <v>0.6364</v>
+        <v>0.5238</v>
       </c>
       <c r="H115" s="8" t="n">
-        <v>-0.0264</v>
+        <v>-0.0263</v>
       </c>
       <c r="I115" s="8" t="n">
-        <v>-0.04474461798234386</v>
+        <v>-0.05466177707560294</v>
       </c>
       <c r="J115" s="10" t="n">
         <v>0.5</v>
@@ -7442,7 +7496,7 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>CLE @ TB</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
@@ -7452,23 +7506,23 @@
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>CIN -3.5</t>
+          <t>TB -5.5</t>
         </is>
       </c>
       <c r="E120" s="12" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.5048</v>
+        <v>0.4939</v>
       </c>
       <c r="G120" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H120" s="13" t="n">
-        <v>-0.0274</v>
+        <v>-0.0272</v>
       </c>
       <c r="I120" s="13" t="n">
-        <v>-0.05622011654448439</v>
+        <v>-0.05703114967231343</v>
       </c>
       <c r="J120" s="15" t="n">
         <v>0.5</v>
@@ -7483,7 +7537,7 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>CLE @ TB</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -7493,23 +7547,23 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>TB -5.5</t>
+          <t>CIN -3.5</t>
         </is>
       </c>
       <c r="E121" s="7" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F121" s="8" t="n">
-        <v>0.4938</v>
+        <v>0.5048</v>
       </c>
       <c r="G121" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H121" s="8" t="n">
         <v>-0.0274</v>
       </c>
       <c r="I121" s="8" t="n">
-        <v>-0.05737834705524036</v>
+        <v>-0.05622011654448439</v>
       </c>
       <c r="J121" s="10" t="n">
         <v>0.5</v>
@@ -7541,16 +7595,16 @@
         <v>170</v>
       </c>
       <c r="F122" s="13" t="n">
-        <v>0.3399</v>
+        <v>0.3398</v>
       </c>
       <c r="G122" s="13" t="n">
         <v>0.3704</v>
       </c>
       <c r="H122" s="13" t="n">
-        <v>-0.0277</v>
+        <v>-0.0278</v>
       </c>
       <c r="I122" s="13" t="n">
-        <v>-0.08147936056166394</v>
+        <v>-0.08192785858412999</v>
       </c>
       <c r="J122" s="15" t="n">
         <v>0.5</v>
@@ -7606,7 +7660,7 @@
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>PIT @ NE</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
@@ -7616,7 +7670,7 @@
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t>Over 43.5</t>
+          <t>Under 44.5</t>
         </is>
       </c>
       <c r="E124" s="12" t="n">
@@ -7632,7 +7686,7 @@
         <v>-0.0284</v>
       </c>
       <c r="I124" s="13" t="n">
-        <v>-0.06001309614417871</v>
+        <v>-0.06002142398117422</v>
       </c>
       <c r="J124" s="15" t="n">
         <v>0.5</v>
@@ -7647,33 +7701,33 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>PIT @ NE</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>DAL -2.5</t>
+          <t>Over 43.5</t>
         </is>
       </c>
       <c r="E125" s="7" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F125" s="8" t="n">
-        <v>0.5024</v>
+        <v>0.4924</v>
       </c>
       <c r="G125" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H125" s="8" t="n">
-        <v>-0.0292</v>
+        <v>-0.0284</v>
       </c>
       <c r="I125" s="8" t="n">
-        <v>-0.06078490939937703</v>
+        <v>-0.06001309614417871</v>
       </c>
       <c r="J125" s="10" t="n">
         <v>0.5</v>
@@ -7688,7 +7742,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
@@ -7698,23 +7752,23 @@
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>DET +3</t>
+          <t>DAL -2.5</t>
         </is>
       </c>
       <c r="E126" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F126" s="13" t="n">
-        <v>0.4895</v>
+        <v>0.5026</v>
       </c>
       <c r="G126" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H126" s="13" t="n">
-        <v>-0.0304</v>
+        <v>-0.0291</v>
       </c>
       <c r="I126" s="13" t="n">
-        <v>-0.06068621837874821</v>
+        <v>-0.06044778891535091</v>
       </c>
       <c r="J126" s="15" t="n">
         <v>0.5</v>
@@ -7729,33 +7783,33 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>CIN ML</t>
+          <t>DET +3</t>
         </is>
       </c>
       <c r="E127" s="7" t="n">
-        <v>-198</v>
+        <v>-110</v>
       </c>
       <c r="F127" s="8" t="n">
-        <v>0.6294</v>
+        <v>0.4895</v>
       </c>
       <c r="G127" s="8" t="n">
-        <v>0.6644</v>
+        <v>0.5238</v>
       </c>
       <c r="H127" s="8" t="n">
-        <v>-0.0309</v>
+        <v>-0.0304</v>
       </c>
       <c r="I127" s="8" t="n">
-        <v>-0.0522151050002545</v>
+        <v>-0.06068621837874821</v>
       </c>
       <c r="J127" s="10" t="n">
         <v>0.5</v>
@@ -7770,33 +7824,33 @@
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>CAR @ ATL</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr">
         <is>
-          <t>CAR +1.5</t>
+          <t>CIN ML</t>
         </is>
       </c>
       <c r="E128" s="12" t="n">
-        <v>-110</v>
+        <v>-198</v>
       </c>
       <c r="F128" s="13" t="n">
-        <v>0.4886</v>
+        <v>0.6294</v>
       </c>
       <c r="G128" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.6644</v>
       </c>
       <c r="H128" s="13" t="n">
-        <v>-0.0311</v>
+        <v>-0.0309</v>
       </c>
       <c r="I128" s="13" t="n">
-        <v>-0.06721901049672396</v>
+        <v>-0.0522151050002545</v>
       </c>
       <c r="J128" s="15" t="n">
         <v>0.5</v>
@@ -7816,28 +7870,28 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>CAR ML</t>
+          <t>CAR +1.5</t>
         </is>
       </c>
       <c r="E129" s="7" t="n">
-        <v>102</v>
+        <v>-110</v>
       </c>
       <c r="F129" s="8" t="n">
-        <v>0.4588</v>
+        <v>0.4886</v>
       </c>
       <c r="G129" s="8" t="n">
-        <v>0.495</v>
+        <v>0.5238</v>
       </c>
       <c r="H129" s="8" t="n">
-        <v>-0.0318</v>
+        <v>-0.0311</v>
       </c>
       <c r="I129" s="8" t="n">
-        <v>-0.07262458964321516</v>
+        <v>-0.06721901049672396</v>
       </c>
       <c r="J129" s="10" t="n">
         <v>0.5</v>
@@ -7852,33 +7906,33 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>CAR @ ATL</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D130" s="5" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>CAR ML</t>
         </is>
       </c>
       <c r="E130" s="12" t="n">
-        <v>-110</v>
+        <v>102</v>
       </c>
       <c r="F130" s="13" t="n">
-        <v>0.4873</v>
+        <v>0.4588</v>
       </c>
       <c r="G130" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.495</v>
       </c>
       <c r="H130" s="13" t="n">
-        <v>-0.032</v>
+        <v>-0.0318</v>
       </c>
       <c r="I130" s="13" t="n">
-        <v>-0.0697243669361825</v>
+        <v>-0.07262458964321516</v>
       </c>
       <c r="J130" s="15" t="n">
         <v>0.5</v>
@@ -7910,16 +7964,16 @@
         <v>-148</v>
       </c>
       <c r="F131" s="8" t="n">
-        <v>0.5579</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="G131" s="8" t="n">
         <v>0.5968</v>
       </c>
       <c r="H131" s="8" t="n">
-        <v>-0.0335</v>
+        <v>-0.0334</v>
       </c>
       <c r="I131" s="8" t="n">
-        <v>-0.06462351467344279</v>
+        <v>-0.06432222647230235</v>
       </c>
       <c r="J131" s="10" t="n">
         <v>0.5</v>
@@ -7951,16 +8005,16 @@
         <v>-245</v>
       </c>
       <c r="F132" s="13" t="n">
-        <v>0.6713</v>
+        <v>0.6714</v>
       </c>
       <c r="G132" s="13" t="n">
         <v>0.7101</v>
       </c>
       <c r="H132" s="13" t="n">
-        <v>-0.0335</v>
+        <v>-0.0334</v>
       </c>
       <c r="I132" s="13" t="n">
-        <v>-0.05431562614774066</v>
+        <v>-0.05408143001598997</v>
       </c>
       <c r="J132" s="15" t="n">
         <v>0.5</v>
@@ -8074,16 +8128,16 @@
         <v>-115</v>
       </c>
       <c r="F135" s="8" t="n">
-        <v>0.4942</v>
+        <v>0.4941</v>
       </c>
       <c r="G135" s="8" t="n">
         <v>0.5349</v>
       </c>
       <c r="H135" s="8" t="n">
-        <v>-0.0346</v>
+        <v>-0.0347</v>
       </c>
       <c r="I135" s="8" t="n">
-        <v>-0.0759724252587396</v>
+        <v>-0.07631200219226442</v>
       </c>
       <c r="J135" s="10" t="n">
         <v>0.5</v>
@@ -8238,16 +8292,16 @@
         <v>110</v>
       </c>
       <c r="F139" s="8" t="n">
-        <v>0.4333</v>
+        <v>0.4334</v>
       </c>
       <c r="G139" s="8" t="n">
         <v>0.4762</v>
       </c>
       <c r="H139" s="8" t="n">
-        <v>-0.0359</v>
+        <v>-0.0358</v>
       </c>
       <c r="I139" s="8" t="n">
-        <v>-0.08935010122584919</v>
+        <v>-0.08897651782496302</v>
       </c>
       <c r="J139" s="10" t="n">
         <v>0.5</v>
@@ -8279,16 +8333,16 @@
         <v>-112</v>
       </c>
       <c r="F140" s="13" t="n">
-        <v>0.4843</v>
+        <v>0.4847</v>
       </c>
       <c r="G140" s="13" t="n">
         <v>0.5283</v>
       </c>
       <c r="H140" s="13" t="n">
-        <v>-0.0365</v>
+        <v>-0.0363</v>
       </c>
       <c r="I140" s="13" t="n">
-        <v>-0.08320448203306302</v>
+        <v>-0.0825243634782688</v>
       </c>
       <c r="J140" s="15" t="n">
         <v>0.5</v>
@@ -8525,16 +8579,16 @@
         <v>-105</v>
       </c>
       <c r="F146" s="13" t="n">
-        <v>0.4652</v>
+        <v>0.4653</v>
       </c>
       <c r="G146" s="13" t="n">
         <v>0.5122</v>
       </c>
       <c r="H146" s="13" t="n">
-        <v>-0.0382</v>
+        <v>-0.0381</v>
       </c>
       <c r="I146" s="13" t="n">
-        <v>-0.0918405676799029</v>
+        <v>-0.09148959310265437</v>
       </c>
       <c r="J146" s="15" t="n">
         <v>0.5</v>
@@ -8976,16 +9030,16 @@
         <v>-198</v>
       </c>
       <c r="F157" s="8" t="n">
-        <v>0.6117</v>
+        <v>0.612</v>
       </c>
       <c r="G157" s="8" t="n">
         <v>0.6644</v>
       </c>
       <c r="H157" s="8" t="n">
-        <v>-0.0409</v>
+        <v>-0.0408</v>
       </c>
       <c r="I157" s="8" t="n">
-        <v>-0.0787361723695737</v>
+        <v>-0.07820640387615446</v>
       </c>
       <c r="J157" s="10" t="n">
         <v>0.5</v>
@@ -9082,7 +9136,7 @@
       </c>
       <c r="B160" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C160" s="5" t="inlineStr">
@@ -9123,7 +9177,7 @@
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>CAR @ ATL</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
@@ -9133,23 +9187,23 @@
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>Over 43.5</t>
+          <t>Under 40.5</t>
         </is>
       </c>
       <c r="E161" s="7" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="F161" s="8" t="n">
-        <v>0.4858</v>
+        <v>0.4695</v>
       </c>
       <c r="G161" s="8" t="n">
-        <v>0.5413</v>
+        <v>0.5238</v>
       </c>
       <c r="H161" s="8" t="n">
-        <v>-0.0421</v>
+        <v>-0.0416</v>
       </c>
       <c r="I161" s="8" t="n">
-        <v>-0.1025875430405576</v>
+        <v>-0.1035968023040441</v>
       </c>
       <c r="J161" s="10" t="n">
         <v>0.5</v>
@@ -9164,7 +9218,7 @@
       </c>
       <c r="B162" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>CAR @ ATL</t>
         </is>
       </c>
       <c r="C162" s="5" t="inlineStr">
@@ -9174,23 +9228,23 @@
       </c>
       <c r="D162" s="5" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>Over 43.5</t>
         </is>
       </c>
       <c r="E162" s="12" t="n">
-        <v>-105</v>
+        <v>-118</v>
       </c>
       <c r="F162" s="13" t="n">
-        <v>0.4557</v>
+        <v>0.4858</v>
       </c>
       <c r="G162" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5413</v>
       </c>
       <c r="H162" s="13" t="n">
-        <v>-0.0425</v>
+        <v>-0.0421</v>
       </c>
       <c r="I162" s="13" t="n">
-        <v>-0.1103300727700344</v>
+        <v>-0.1025875430405576</v>
       </c>
       <c r="J162" s="15" t="n">
         <v>0.5</v>
@@ -9205,7 +9259,7 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -9215,23 +9269,23 @@
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E163" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F163" s="8" t="n">
-        <v>0.467</v>
+        <v>0.4557</v>
       </c>
       <c r="G163" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H163" s="8" t="n">
-        <v>-0.0426</v>
+        <v>-0.0425</v>
       </c>
       <c r="I163" s="8" t="n">
-        <v>-0.1084019190168437</v>
+        <v>-0.1103300727700344</v>
       </c>
       <c r="J163" s="10" t="n">
         <v>0.5</v>
@@ -9246,33 +9300,33 @@
       </c>
       <c r="B164" s="5" t="inlineStr">
         <is>
-          <t>PHI @ TEN</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C164" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D164" s="5" t="inlineStr">
         <is>
-          <t>PHI -4.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E164" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F164" s="13" t="n">
-        <v>0.4669</v>
+        <v>0.467</v>
       </c>
       <c r="G164" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H164" s="13" t="n">
-        <v>-0.0427</v>
+        <v>-0.0426</v>
       </c>
       <c r="I164" s="13" t="n">
-        <v>-0.1086623740801022</v>
+        <v>-0.1084019190168437</v>
       </c>
       <c r="J164" s="15" t="n">
         <v>0.5</v>
@@ -9287,7 +9341,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>PHI @ TEN</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -9297,23 +9351,23 @@
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>SEA -3.5</t>
+          <t>PHI -4.5</t>
         </is>
       </c>
       <c r="E165" s="7" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F165" s="8" t="n">
-        <v>0.4544</v>
+        <v>0.4669</v>
       </c>
       <c r="G165" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H165" s="8" t="n">
-        <v>-0.043</v>
+        <v>-0.0427</v>
       </c>
       <c r="I165" s="8" t="n">
-        <v>-0.1128490923575317</v>
+        <v>-0.1086623740801022</v>
       </c>
       <c r="J165" s="10" t="n">
         <v>0.5</v>
@@ -9328,42 +9382,38 @@
       </c>
       <c r="B166" s="5" t="inlineStr">
         <is>
-          <t>NYG @ LAR</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C166" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D166" s="5" t="inlineStr">
         <is>
-          <t>LAR ML</t>
+          <t>SEA -3.5</t>
         </is>
       </c>
       <c r="E166" s="12" t="n">
-        <v>-380</v>
+        <v>-105</v>
       </c>
       <c r="F166" s="13" t="n">
-        <v>0.7328</v>
+        <v>0.4544</v>
       </c>
       <c r="G166" s="13" t="n">
-        <v>0.7917</v>
+        <v>0.5122</v>
       </c>
       <c r="H166" s="13" t="n">
-        <v>-0.0434</v>
+        <v>-0.043</v>
       </c>
       <c r="I166" s="13" t="n">
-        <v>-0.07374216851612969</v>
+        <v>-0.1128490923575317</v>
       </c>
       <c r="J166" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K166" s="5" t="inlineStr">
-        <is>
-          <t>price -380 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K166" s="5" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -9373,7 +9423,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>NYG @ LAR</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -9383,28 +9433,32 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>CHI ML</t>
+          <t>LAR ML</t>
         </is>
       </c>
       <c r="E167" s="7" t="n">
-        <v>-198</v>
+        <v>-380</v>
       </c>
       <c r="F167" s="8" t="n">
-        <v>0.6038</v>
+        <v>0.7332</v>
       </c>
       <c r="G167" s="8" t="n">
-        <v>0.6644</v>
+        <v>0.7917</v>
       </c>
       <c r="H167" s="8" t="n">
-        <v>-0.0441</v>
+        <v>-0.0433</v>
       </c>
       <c r="I167" s="8" t="n">
-        <v>-0.090432584438073</v>
+        <v>-0.07335026602967182</v>
       </c>
       <c r="J167" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K167" s="4" t="inlineStr"/>
+      <c r="K167" s="4" t="inlineStr">
+        <is>
+          <t>price -380 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="5" t="inlineStr">
@@ -9414,7 +9468,7 @@
       </c>
       <c r="B168" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C168" s="5" t="inlineStr">
@@ -9424,23 +9478,23 @@
       </c>
       <c r="D168" s="5" t="inlineStr">
         <is>
-          <t>LV ML</t>
+          <t>CHI ML</t>
         </is>
       </c>
       <c r="E168" s="12" t="n">
         <v>-198</v>
       </c>
       <c r="F168" s="13" t="n">
-        <v>0.6029</v>
+        <v>0.6038</v>
       </c>
       <c r="G168" s="13" t="n">
         <v>0.6644</v>
       </c>
       <c r="H168" s="13" t="n">
-        <v>-0.0444</v>
+        <v>-0.0441</v>
       </c>
       <c r="I168" s="13" t="n">
-        <v>-0.09176650825332933</v>
+        <v>-0.090432584438073</v>
       </c>
       <c r="J168" s="15" t="n">
         <v>0.5</v>
@@ -9455,33 +9509,33 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>Under 40.5</t>
+          <t>LV ML</t>
         </is>
       </c>
       <c r="E169" s="7" t="n">
-        <v>-110</v>
+        <v>-198</v>
       </c>
       <c r="F169" s="8" t="n">
-        <v>0.462</v>
+        <v>0.6029</v>
       </c>
       <c r="G169" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.6644</v>
       </c>
       <c r="H169" s="8" t="n">
-        <v>-0.0445</v>
+        <v>-0.0444</v>
       </c>
       <c r="I169" s="8" t="n">
-        <v>-0.1180341212058959</v>
+        <v>-0.09176650825332933</v>
       </c>
       <c r="J169" s="10" t="n">
         <v>0.5</v>
@@ -9619,38 +9673,42 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>LV @ LAC</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>Over 48.5</t>
+          <t>LAC ML</t>
         </is>
       </c>
       <c r="E173" s="7" t="n">
-        <v>-110</v>
+        <v>-375</v>
       </c>
       <c r="F173" s="8" t="n">
-        <v>0.4595</v>
+        <v>0.7246</v>
       </c>
       <c r="G173" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.7895</v>
       </c>
       <c r="H173" s="8" t="n">
-        <v>-0.0453</v>
+        <v>-0.0455</v>
       </c>
       <c r="I173" s="8" t="n">
-        <v>-0.1228221690339132</v>
+        <v>-0.08154755880401182</v>
       </c>
       <c r="J173" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K173" s="4" t="inlineStr"/>
+      <c r="K173" s="4" t="inlineStr">
+        <is>
+          <t>price -375 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="5" t="inlineStr">
@@ -9660,42 +9718,38 @@
       </c>
       <c r="B174" s="5" t="inlineStr">
         <is>
-          <t>LV @ LAC</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C174" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D174" s="5" t="inlineStr">
         <is>
-          <t>LAC ML</t>
+          <t>KC -6.5</t>
         </is>
       </c>
       <c r="E174" s="12" t="n">
-        <v>-375</v>
+        <v>-110</v>
       </c>
       <c r="F174" s="13" t="n">
-        <v>0.7246</v>
+        <v>0.4589</v>
       </c>
       <c r="G174" s="13" t="n">
-        <v>0.7895</v>
+        <v>0.5238</v>
       </c>
       <c r="H174" s="13" t="n">
         <v>-0.0455</v>
       </c>
       <c r="I174" s="13" t="n">
-        <v>-0.08154755880401182</v>
+        <v>-0.1239391092626436</v>
       </c>
       <c r="J174" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K174" s="5" t="inlineStr">
-        <is>
-          <t>price -375 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K174" s="5" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -9705,7 +9759,7 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -9715,23 +9769,23 @@
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>KC -6.5</t>
+          <t>JAX -7.5</t>
         </is>
       </c>
       <c r="E175" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F175" s="8" t="n">
-        <v>0.4589</v>
+        <v>0.4578</v>
       </c>
       <c r="G175" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H175" s="8" t="n">
-        <v>-0.0455</v>
+        <v>-0.0459</v>
       </c>
       <c r="I175" s="8" t="n">
-        <v>-0.1239391092626436</v>
+        <v>-0.1260390118519604</v>
       </c>
       <c r="J175" s="10" t="n">
         <v>0.5</v>
@@ -9746,33 +9800,33 @@
       </c>
       <c r="B176" s="5" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C176" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D176" s="5" t="inlineStr">
         <is>
-          <t>JAX -7.5</t>
+          <t>Over 51.5</t>
         </is>
       </c>
       <c r="E176" s="12" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="F176" s="13" t="n">
-        <v>0.458</v>
+        <v>0.4359</v>
       </c>
       <c r="G176" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.505</v>
       </c>
       <c r="H176" s="13" t="n">
-        <v>-0.0458</v>
+        <v>-0.0467</v>
       </c>
       <c r="I176" s="13" t="n">
-        <v>-0.1256919317062585</v>
+        <v>-0.1367090604010699</v>
       </c>
       <c r="J176" s="15" t="n">
         <v>0.5</v>
@@ -9787,33 +9841,33 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>NYG @ LAR</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>Over 51.5</t>
+          <t>LAR -8.5</t>
         </is>
       </c>
       <c r="E177" s="7" t="n">
-        <v>-102</v>
+        <v>-110</v>
       </c>
       <c r="F177" s="8" t="n">
-        <v>0.4359</v>
+        <v>0.4546</v>
       </c>
       <c r="G177" s="8" t="n">
-        <v>0.505</v>
+        <v>0.5238</v>
       </c>
       <c r="H177" s="8" t="n">
-        <v>-0.0467</v>
+        <v>-0.0468</v>
       </c>
       <c r="I177" s="8" t="n">
-        <v>-0.1367090604010699</v>
+        <v>-0.1320545974254394</v>
       </c>
       <c r="J177" s="10" t="n">
         <v>0.5</v>
@@ -9828,38 +9882,42 @@
       </c>
       <c r="B178" s="5" t="inlineStr">
         <is>
-          <t>NYG @ LAR</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C178" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D178" s="5" t="inlineStr">
         <is>
-          <t>LAR -8.5</t>
+          <t>LAC ML</t>
         </is>
       </c>
       <c r="E178" s="12" t="n">
-        <v>-110</v>
+        <v>-575</v>
       </c>
       <c r="F178" s="13" t="n">
-        <v>0.4543</v>
+        <v>0.7819</v>
       </c>
       <c r="G178" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.8519</v>
       </c>
       <c r="H178" s="13" t="n">
-        <v>-0.0469</v>
+        <v>-0.047</v>
       </c>
       <c r="I178" s="13" t="n">
-        <v>-0.132753183737966</v>
+        <v>-0.0815270974192778</v>
       </c>
       <c r="J178" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K178" s="5" t="inlineStr"/>
+      <c r="K178" s="5" t="inlineStr">
+        <is>
+          <t>price -575 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -9869,7 +9927,7 @@
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
@@ -9879,30 +9937,30 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>LAC ML</t>
+          <t>JAX ML</t>
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>-575</v>
+        <v>-380</v>
       </c>
       <c r="F179" s="8" t="n">
-        <v>0.7819</v>
+        <v>0.7203000000000001</v>
       </c>
       <c r="G179" s="8" t="n">
-        <v>0.8519</v>
+        <v>0.7917</v>
       </c>
       <c r="H179" s="8" t="n">
-        <v>-0.047</v>
+        <v>-0.0474</v>
       </c>
       <c r="I179" s="8" t="n">
-        <v>-0.0815270974192778</v>
+        <v>-0.08945465843273717</v>
       </c>
       <c r="J179" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="K179" s="4" t="inlineStr">
         <is>
-          <t>price -575 outside the allowed range</t>
+          <t>price -380 outside the allowed range</t>
         </is>
       </c>
     </row>
@@ -9914,42 +9972,38 @@
       </c>
       <c r="B180" s="5" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C180" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D180" s="5" t="inlineStr">
         <is>
-          <t>JAX ML</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E180" s="12" t="n">
-        <v>-380</v>
+        <v>-110</v>
       </c>
       <c r="F180" s="13" t="n">
-        <v>0.7204</v>
+        <v>0.4495</v>
       </c>
       <c r="G180" s="13" t="n">
-        <v>0.7917</v>
+        <v>0.5238</v>
       </c>
       <c r="H180" s="13" t="n">
-        <v>-0.0473</v>
+        <v>-0.0481</v>
       </c>
       <c r="I180" s="13" t="n">
-        <v>-0.08925300638423508</v>
+        <v>-0.1419279603859848</v>
       </c>
       <c r="J180" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K180" s="5" t="inlineStr">
-        <is>
-          <t>price -380 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K180" s="5" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -10496,7 +10550,7 @@
       </c>
       <c r="B194" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C194" s="5" t="inlineStr">
@@ -10506,23 +10560,23 @@
       </c>
       <c r="D194" s="5" t="inlineStr">
         <is>
-          <t>Under 38.5</t>
+          <t>Over 45.5</t>
         </is>
       </c>
       <c r="E194" s="12" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F194" s="13" t="n">
-        <v>0.4186</v>
+        <v>0.4297</v>
       </c>
       <c r="G194" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H194" s="13" t="n">
         <v>-0.0515</v>
       </c>
       <c r="I194" s="13" t="n">
-        <v>-0.1828182474138708</v>
+        <v>-0.1797102353978136</v>
       </c>
       <c r="J194" s="15" t="n">
         <v>0.5</v>
@@ -10537,7 +10591,7 @@
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -10547,23 +10601,23 @@
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>Over 45.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E195" s="7" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F195" s="8" t="n">
-        <v>0.4297</v>
+        <v>0.4384</v>
       </c>
       <c r="G195" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H195" s="8" t="n">
-        <v>-0.0515</v>
+        <v>-0.0518</v>
       </c>
       <c r="I195" s="8" t="n">
-        <v>-0.1797102353978136</v>
+        <v>-0.1804243326382279</v>
       </c>
       <c r="J195" s="10" t="n">
         <v>0.5</v>
@@ -10578,7 +10632,7 @@
       </c>
       <c r="B196" s="5" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C196" s="5" t="inlineStr">
@@ -10588,23 +10642,23 @@
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>Under 38.5</t>
         </is>
       </c>
       <c r="E196" s="12" t="n">
-        <v>-115</v>
+        <v>-105</v>
       </c>
       <c r="F196" s="13" t="n">
-        <v>0.4384</v>
+        <v>0.4137</v>
       </c>
       <c r="G196" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5122</v>
       </c>
       <c r="H196" s="13" t="n">
-        <v>-0.0518</v>
+        <v>-0.052</v>
       </c>
       <c r="I196" s="13" t="n">
-        <v>-0.1804243326382279</v>
+        <v>-0.1922708059340066</v>
       </c>
       <c r="J196" s="15" t="n">
         <v>0.5</v>
@@ -10619,42 +10673,38 @@
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>SF ML</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>-650</v>
+        <v>-110</v>
       </c>
       <c r="F197" s="8" t="n">
-        <v>0.7664</v>
+        <v>0.4248</v>
       </c>
       <c r="G197" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.5238</v>
       </c>
       <c r="H197" s="8" t="n">
-        <v>-0.0522</v>
+        <v>-0.0521</v>
       </c>
       <c r="I197" s="8" t="n">
-        <v>-0.1147913763618906</v>
+        <v>-0.1890398877507678</v>
       </c>
       <c r="J197" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K197" s="4" t="inlineStr">
-        <is>
-          <t>price -650 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K197" s="4" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="inlineStr">
@@ -10664,7 +10714,7 @@
       </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
-          <t>SEA @ ARI</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C198" s="5" t="inlineStr">
@@ -10674,30 +10724,30 @@
       </c>
       <c r="D198" s="5" t="inlineStr">
         <is>
-          <t>SEA ML</t>
+          <t>SF ML</t>
         </is>
       </c>
       <c r="E198" s="12" t="n">
-        <v>-550</v>
+        <v>-650</v>
       </c>
       <c r="F198" s="13" t="n">
-        <v>0.7444</v>
+        <v>0.7664</v>
       </c>
       <c r="G198" s="13" t="n">
-        <v>0.8462</v>
+        <v>0.8667</v>
       </c>
       <c r="H198" s="13" t="n">
-        <v>-0.0523</v>
+        <v>-0.0522</v>
       </c>
       <c r="I198" s="13" t="n">
-        <v>-0.1193647652869892</v>
+        <v>-0.1147913763618906</v>
       </c>
       <c r="J198" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="K198" s="5" t="inlineStr">
         <is>
-          <t>price -550 outside the allowed range</t>
+          <t>price -650 outside the allowed range</t>
         </is>
       </c>
     </row>
@@ -10709,38 +10759,42 @@
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>SEA @ ARI</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>SF -10.5</t>
+          <t>SEA ML</t>
         </is>
       </c>
       <c r="E199" s="7" t="n">
-        <v>-110</v>
+        <v>-550</v>
       </c>
       <c r="F199" s="8" t="n">
-        <v>0.4216</v>
+        <v>0.7444</v>
       </c>
       <c r="G199" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.8462</v>
       </c>
       <c r="H199" s="8" t="n">
-        <v>-0.0524</v>
+        <v>-0.0523</v>
       </c>
       <c r="I199" s="8" t="n">
-        <v>-0.1951029543058591</v>
+        <v>-0.1193647652869892</v>
       </c>
       <c r="J199" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K199" s="4" t="inlineStr"/>
+      <c r="K199" s="4" t="inlineStr">
+        <is>
+          <t>price -550 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="inlineStr">
@@ -10750,33 +10804,33 @@
       </c>
       <c r="B200" s="5" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C200" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D200" s="5" t="inlineStr">
         <is>
-          <t>Over 49.5</t>
+          <t>SF -10.5</t>
         </is>
       </c>
       <c r="E200" s="12" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F200" s="13" t="n">
-        <v>0.4286</v>
+        <v>0.4216</v>
       </c>
       <c r="G200" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H200" s="13" t="n">
-        <v>-0.0527</v>
+        <v>-0.0524</v>
       </c>
       <c r="I200" s="13" t="n">
-        <v>-0.1987411539265735</v>
+        <v>-0.1951029543058591</v>
       </c>
       <c r="J200" s="15" t="n">
         <v>0.5</v>
@@ -10791,7 +10845,7 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
@@ -10801,23 +10855,23 @@
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>Over 49.5</t>
         </is>
       </c>
       <c r="E201" s="7" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F201" s="8" t="n">
-        <v>0.4151</v>
+        <v>0.4286</v>
       </c>
       <c r="G201" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H201" s="8" t="n">
-        <v>-0.0529</v>
+        <v>-0.0527</v>
       </c>
       <c r="I201" s="8" t="n">
-        <v>-0.2075049798576659</v>
+        <v>-0.1987411539265735</v>
       </c>
       <c r="J201" s="10" t="n">
         <v>0.5</v>
@@ -11776,7 +11830,7 @@
         </is>
       </c>
       <c r="D9" s="14" t="n">
-        <v>8.16</v>
+        <v>8.18</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>-8.5</v>
@@ -11912,7 +11966,7 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>6.16</v>
+        <v>6.17</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>-4.5</v>
@@ -12082,7 +12136,7 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>6.08</v>
+        <v>6.09</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>-5.5</v>
@@ -12326,7 +12380,7 @@
         <v>-3</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>39.1</v>
+        <v>40.5</v>
       </c>
       <c r="G25" s="16" t="n">
         <v>42.5</v>
@@ -12354,7 +12408,7 @@
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>-1.79</v>
+        <v>-1.8</v>
       </c>
       <c r="E26" s="9" t="n">
         <v>2.5</v>
@@ -12490,7 +12544,7 @@
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>5.88</v>
+        <v>5.9</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>-4.5</v>
@@ -12524,7 +12578,7 @@
         </is>
       </c>
       <c r="D31" s="14" t="n">
-        <v>3.84</v>
+        <v>3.85</v>
       </c>
       <c r="E31" s="14" t="n">
         <v>-3</v>
@@ -12598,7 +12652,7 @@
         <v>1.5</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>45</v>
+        <v>44.8</v>
       </c>
       <c r="G33" s="16" t="n">
         <v>44.5</v>
@@ -12660,13 +12714,13 @@
         </is>
       </c>
       <c r="D35" s="14" t="n">
-        <v>7.38</v>
+        <v>7.37</v>
       </c>
       <c r="E35" s="14" t="n">
         <v>-7.5</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>42</v>
+        <v>41.7</v>
       </c>
       <c r="G35" s="16" t="n">
         <v>40.5</v>
@@ -12728,13 +12782,13 @@
         </is>
       </c>
       <c r="D37" s="14" t="n">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
       <c r="E37" s="14" t="n">
         <v>-1.5</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>41.6</v>
+        <v>41.8</v>
       </c>
       <c r="G37" s="16" t="n">
         <v>38.5</v>
@@ -12796,13 +12850,13 @@
         </is>
       </c>
       <c r="D39" s="14" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
       <c r="E39" s="14" t="n">
         <v>-3.5</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>46.9</v>
+        <v>45.5</v>
       </c>
       <c r="G39" s="16" t="n">
         <v>48.5</v>
@@ -13895,7 +13949,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>3.76</v>
+        <v>3.8</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>2.9</v>
@@ -13927,7 +13981,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>3.07</v>
+        <v>3.08</v>
       </c>
       <c r="E6" s="20" t="n">
         <v>2.35</v>
@@ -14084,7 +14138,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>1.93</v>
@@ -14116,7 +14170,7 @@
         </is>
       </c>
       <c r="C12" s="12" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>1.91</v>
@@ -14407,7 +14461,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="18" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="E21" s="18" t="n">
         <v>1.87</v>
@@ -14567,7 +14621,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="20" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.85</v>
       </c>
       <c r="E26" s="20" t="n">
         <v>-0.8100000000000001</v>
@@ -14727,7 +14781,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="18" t="n">
-        <v>-2.66</v>
+        <v>-2.67</v>
       </c>
       <c r="E31" s="18" t="n">
         <v>-1.44</v>
@@ -14887,7 +14941,7 @@
         <v>0</v>
       </c>
       <c r="D36" s="20" t="n">
-        <v>-5.61</v>
+        <v>-5.6</v>
       </c>
       <c r="E36" s="20" t="n">
         <v>-0.88</v>
@@ -19463,10 +19517,10 @@
         <v>46.5</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>-185</v>
+        <v>-192</v>
       </c>
       <c r="J93" s="7" t="n">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="K93" s="17" t="n">
         <v>0</v>
@@ -22270,10 +22324,10 @@
         <v>50.5</v>
       </c>
       <c r="I146" s="12" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="J146" s="12" t="n">
-        <v>-245</v>
+        <v>-250</v>
       </c>
       <c r="K146" s="19" t="n">
         <v>0</v>
@@ -24119,13 +24173,13 @@
         </is>
       </c>
       <c r="G181" s="9" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="H181" s="11" t="n">
         <v>50.5</v>
       </c>
       <c r="I181" s="7" t="n">
-        <v>-218</v>
+        <v>-225</v>
       </c>
       <c r="J181" s="7" t="n">
         <v>180</v>
@@ -24284,10 +24338,10 @@
         <v>43.5</v>
       </c>
       <c r="I184" s="12" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="J184" s="12" t="n">
-        <v>-142</v>
+        <v>-135</v>
       </c>
       <c r="K184" s="19" t="n">
         <v>0</v>
@@ -24602,10 +24656,10 @@
         <v>47.5</v>
       </c>
       <c r="I190" s="12" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="J190" s="12" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="K190" s="19" t="n">
         <v>0</v>
@@ -25980,10 +26034,10 @@
         <v>52.5</v>
       </c>
       <c r="I216" s="12" t="n">
-        <v>-122</v>
+        <v>-125</v>
       </c>
       <c r="J216" s="12" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="K216" s="19" t="n">
         <v>0</v>
@@ -27835,10 +27889,10 @@
         <v>44.5</v>
       </c>
       <c r="I251" s="7" t="n">
-        <v>-122</v>
+        <v>-125</v>
       </c>
       <c r="J251" s="7" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="K251" s="17" t="n">
         <v>0</v>
@@ -28577,10 +28631,10 @@
         <v>46.5</v>
       </c>
       <c r="I265" s="7" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="J265" s="7" t="n">
-        <v>-180</v>
+        <v>-185</v>
       </c>
       <c r="K265" s="17" t="n">
         <v>0</v>
@@ -28842,10 +28896,10 @@
         <v>43.5</v>
       </c>
       <c r="I270" s="12" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="J270" s="12" t="n">
-        <v>-155</v>
+        <v>-162</v>
       </c>
       <c r="K270" s="19" t="n">
         <v>0</v>
@@ -30326,10 +30380,10 @@
         <v>48.5</v>
       </c>
       <c r="I298" s="12" t="n">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="J298" s="12" t="n">
-        <v>-192</v>
+        <v>-185</v>
       </c>
       <c r="K298" s="19" t="n">
         <v>0</v>
@@ -44370,7 +44424,7 @@
       </c>
       <c r="F381" s="4" t="inlineStr">
         <is>
-          <t>Smith (undisclosed) reverted to the Chiefs' injured reserve list Monday, Matt Derrick of ChiefsDigest.com reports.</t>
+          <t>Smith (undisclosed) reverted to the Chiefs' injured-reserve list Monday, Matt Derrick of ChiefsDigest.com reports.</t>
         </is>
       </c>
     </row>
@@ -53106,7 +53160,7 @@
       </c>
       <c r="F655" s="4" t="inlineStr">
         <is>
-          <t>The Steelers placed Driscoll (undisclosed) on injured reserve Monday with a designation to return during the regular season, Teresa Varley of the team's official site reports.</t>
+          <t>The Steelers placed Driscoll (undisclosed) on injured reserve Monday with a designation to return, Teresa Varley of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -57986,20 +58040,20 @@
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>69.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>9.300000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>13.6</v>
+        <v>6.7</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I5" s="9" t="n">
@@ -58024,26 +58078,30 @@
         </is>
       </c>
       <c r="D6" s="19" t="n">
-        <v>66.40000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>4.6</v>
+        <v>10.4</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>12.3</v>
+        <v>29.1</v>
       </c>
       <c r="G6" s="19" t="n">
         <v>7</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="5" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Wind 10 mph (gusts 29)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -58062,20 +58120,20 @@
         </is>
       </c>
       <c r="D7" s="17" t="n">
-        <v>76.5</v>
+        <v>79.3</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>4.5</v>
+        <v>6.4</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Drizzle</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
@@ -58100,16 +58158,16 @@
         </is>
       </c>
       <c r="D8" s="19" t="n">
-        <v>77.59999999999999</v>
+        <v>81</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>8.800000000000001</v>
+        <v>3.3</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>14.1</v>
+        <v>8.5</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -58138,28 +58196,28 @@
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>97.09999999999999</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>10.3</v>
+        <v>12.5</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>12.5</v>
+        <v>8.5</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>-0.25</v>
+        <v>-0.65</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>97°F · retractable roof — effect halved</t>
+          <t>Wind 12 mph (gusts 8) · 96°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -58180,16 +58238,16 @@
         </is>
       </c>
       <c r="D10" s="19" t="n">
-        <v>93</v>
+        <v>95.2</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>5.5</v>
+        <v>4.3</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>8.1</v>
+        <v>6.5</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -58201,7 +58259,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>93°F</t>
+          <t>95°F</t>
         </is>
       </c>
     </row>
@@ -58222,26 +58280,30 @@
         </is>
       </c>
       <c r="D11" s="17" t="n">
-        <v>91.3</v>
+        <v>101.1</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>8.800000000000001</v>
+        <v>3.5</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>6.9</v>
+        <v>12.3</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4" t="inlineStr"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>101°F</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -58260,16 +58322,16 @@
         </is>
       </c>
       <c r="D12" s="19" t="n">
-        <v>81.3</v>
+        <v>74.2</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>4.4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>10.5</v>
+        <v>3.8</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -58302,16 +58364,16 @@
         </is>
       </c>
       <c r="D13" s="17" t="n">
-        <v>93.2</v>
+        <v>90.8</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>9</v>
+        <v>1.1</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>13</v>
+        <v>6.7</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -58319,13 +58381,9 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>93°F</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -58344,20 +58402,20 @@
         </is>
       </c>
       <c r="D14" s="19" t="n">
-        <v>74.59999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>7.2</v>
+        <v>2.5</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>17.7</v>
+        <v>4.7</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I14" s="14" t="n">
@@ -58382,20 +58440,20 @@
         </is>
       </c>
       <c r="D15" s="17" t="n">
-        <v>70.90000000000001</v>
+        <v>73.3</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>7.2</v>
+        <v>10.7</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I15" s="9" t="n">
@@ -58420,20 +58478,20 @@
         </is>
       </c>
       <c r="D16" s="19" t="n">
-        <v>84.90000000000001</v>
+        <v>74</v>
       </c>
       <c r="E16" s="19" t="n">
-        <v>12</v>
+        <v>8.1</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>24.8</v>
+        <v>2.9</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I16" s="14" t="n">
@@ -58462,20 +58520,20 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>89.09999999999999</v>
+        <v>88</v>
       </c>
       <c r="E17" s="17" t="n">
-        <v>15.5</v>
+        <v>1.5</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>19.7</v>
+        <v>14.8</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I17" s="9" t="n">
@@ -58504,16 +58562,16 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>78.7</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>1.8</v>
+        <v>11</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>3.6</v>
+        <v>4.9</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -58542,20 +58600,20 @@
         </is>
       </c>
       <c r="D19" s="17" t="n">
-        <v>74.8</v>
+        <v>77.5</v>
       </c>
       <c r="E19" s="17" t="n">
-        <v>4.8</v>
+        <v>10.7</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>5.4</v>
+        <v>9.6</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
@@ -58580,30 +58638,26 @@
         </is>
       </c>
       <c r="D20" s="19" t="n">
-        <v>98.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>18.2</v>
+        <v>11.1</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>30.9</v>
+        <v>3.4</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I20" s="14" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>Wind 18 mph (gusts 31) · 99°F</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh: 2026-09-02 12:04 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -224,8 +224,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBest" displayName="tblBest" ref="A4:N9" headerRowCount="1">
-  <autoFilter ref="A4:N9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBest" displayName="tblBest" ref="A4:N7" headerRowCount="1">
+  <autoFilter ref="A4:N7"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Tier"/>
     <tableColumn id="2" name="Game"/>
@@ -692,7 +692,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-09-02T05:13:05+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-09-02T12:04:47+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-09-02T05:13:05+00:00</t>
+          <t>2026-09-02T12:04:47+00:00</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2553,114 +2553,6 @@
       <c r="N7" s="4" t="inlineStr">
         <is>
           <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>SF @ LAR</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Under 48.5</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>-115</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>0.5911</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <v>0.5349</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <v>0.0424</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>0.0562</v>
-      </c>
-      <c r="J8" s="14" t="n">
-        <v>-3.53</v>
-      </c>
-      <c r="K8" s="15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L8" s="16" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="M8" s="16" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>NYJ @ TEN</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Over 38.5</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>-115</v>
-      </c>
-      <c r="F9" s="8" t="n">
-        <v>0.5863</v>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>0.5349</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>0.0403</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>0.0514</v>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="K9" s="10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="M9" s="11" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -2891,84 +2783,92 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>LEAN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>SEA @ ARI</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>ARI ML</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>-115</v>
+        <v>400</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5911</v>
+        <v>0.2593</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.2</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>0.0424</v>
+        <v>0.0436</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>0.1050788805197023</v>
+        <v>0.2943176647439902</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>correlated with a stronger play on the same game</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>LEAN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Over 38.5</t>
+          <t>MIA +10.5</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.5863</v>
+        <v>0.5809</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>0.0403</v>
+        <v>0.0427</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.09609813123903277</v>
+        <v>0.108983771024415</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>correlated with a stronger play on the same game</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2978,7 +2878,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>SEA @ ARI</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -2988,32 +2888,28 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>ARI ML</t>
+          <t>IND ML</t>
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>400</v>
+        <v>270</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.2593</v>
+        <v>0.3171</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.2</v>
+        <v>0.2703</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>0.0436</v>
+        <v>0.0381</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>0.2943176647439902</v>
+        <v>0.1718450921457355</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>correlated with a stronger play on the same game</t>
-        </is>
-      </c>
+      <c r="K10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -3023,42 +2919,38 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>MIA +10.5</t>
+          <t>Over 38.5</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>0.5809</v>
+        <v>0.5814</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>0.0427</v>
+        <v>0.0379</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>0.108983771024415</v>
+        <v>0.08704652960204162</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>correlated with a stronger play on the same game</t>
-        </is>
-      </c>
+      <c r="K11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3068,33 +2960,33 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>IND ML</t>
+          <t>Under 45.5</t>
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>270</v>
+        <v>-110</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.3171</v>
+        <v>0.5703</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>0.2703</v>
+        <v>0.5238</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>0.0381</v>
+        <v>0.0379</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>0.1718450921457355</v>
+        <v>0.08880114448872278</v>
       </c>
       <c r="J12" s="15" t="n">
         <v>0.5</v>
@@ -3109,7 +3001,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -3119,7 +3011,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Under 45.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -3135,7 +3027,7 @@
         <v>0.0379</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>0.08880114448872278</v>
+        <v>0.08880644497500201</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>0.5</v>
@@ -3232,33 +3124,33 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>ATL ML</t>
+          <t>Under 50.5</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>295</v>
+        <v>-102</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.2953</v>
+        <v>0.547</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.2532</v>
+        <v>0.505</v>
       </c>
       <c r="H16" s="13" t="n">
         <v>0.0354</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0.1648945902296205</v>
+        <v>0.08318811058747821</v>
       </c>
       <c r="J16" s="15" t="n">
         <v>0.5</v>
@@ -3273,33 +3165,33 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>LV @ LAC</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>ATL ML</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>-110</v>
+        <v>295</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.5654</v>
+        <v>0.2953</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.2532</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.0351</v>
+        <v>0.0354</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.07941221357333128</v>
+        <v>0.1648945902296205</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>0.5</v>
@@ -3314,7 +3206,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>LV @ LAC</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3324,23 +3216,23 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>Under 42.5</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5517</v>
+        <v>0.5654</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.0339</v>
+        <v>0.0351</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.07718415825415337</v>
+        <v>0.07941221357333128</v>
       </c>
       <c r="J18" s="15" t="n">
         <v>0.5</v>
@@ -3355,7 +3247,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -3365,23 +3257,23 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5517</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.0336</v>
+        <v>0.0339</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.07472455202886785</v>
+        <v>0.07718415825415337</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>0.5</v>
@@ -3396,7 +3288,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -3406,23 +3298,23 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Under 50.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="E20" s="12" t="n">
-        <v>-102</v>
+        <v>-110</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.542</v>
+        <v>0.5605</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.505</v>
+        <v>0.5238</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>0.0323</v>
+        <v>0.0321</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>0.0733067893543442</v>
+        <v>0.07000558387848543</v>
       </c>
       <c r="J20" s="15" t="n">
         <v>0.5</v>
@@ -3437,7 +3329,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -3447,7 +3339,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>Under 42.5</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -3460,10 +3352,10 @@
         <v>0.5238</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>0.0321</v>
+        <v>0.032</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>0.07000558387848543</v>
+        <v>0.06999028039567379</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>0.5</v>
@@ -3642,7 +3534,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>WSH @ PHI</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -3652,23 +3544,23 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Under 45.5</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E26" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5555</v>
+        <v>0.5667</v>
       </c>
       <c r="G26" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>0.0286</v>
+        <v>0.0287</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>0.06053638673362371</v>
+        <v>0.05956181484999368</v>
       </c>
       <c r="J26" s="15" t="n">
         <v>0.5</v>
@@ -3683,7 +3575,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>WSH @ PHI</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -3724,7 +3616,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>WSH @ DAL</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -3734,7 +3626,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>Under 45.5</t>
         </is>
       </c>
       <c r="E28" s="12" t="n">
@@ -3750,7 +3642,7 @@
         <v>0.0286</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>0.06054059650663302</v>
+        <v>0.06053638673362371</v>
       </c>
       <c r="J28" s="15" t="n">
         <v>0.5</v>
@@ -3765,33 +3657,33 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>WSH @ DAL</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>MIN ML</t>
+          <t>Under 51.5</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>170</v>
+        <v>-110</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>0.401</v>
+        <v>0.5555</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.3704</v>
+        <v>0.5238</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.0278</v>
+        <v>0.0286</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.08192396663420087</v>
+        <v>0.06054059650663302</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>0.5</v>
@@ -3806,7 +3698,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -3816,23 +3708,23 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>CLE ML</t>
+          <t>MIN ML</t>
         </is>
       </c>
       <c r="E30" s="12" t="n">
-        <v>310</v>
+        <v>170</v>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.2744</v>
+        <v>0.401</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.2439</v>
+        <v>0.3704</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>0.0277</v>
+        <v>0.0278</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>0.1242061252800249</v>
+        <v>0.08192396663420087</v>
       </c>
       <c r="J30" s="15" t="n">
         <v>0.5</v>
@@ -3847,33 +3739,33 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>CLE ML</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>-110</v>
+        <v>310</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.5505</v>
+        <v>0.2744</v>
       </c>
       <c r="G31" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.2439</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>0.0248</v>
+        <v>0.0277</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>0.05101886947689394</v>
+        <v>0.1242061252800249</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0.5</v>
@@ -9886,38 +9778,42 @@
       </c>
       <c r="B178" s="5" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C178" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D178" s="5" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>LAC ML</t>
         </is>
       </c>
       <c r="E178" s="12" t="n">
-        <v>-110</v>
+        <v>-550</v>
       </c>
       <c r="F178" s="13" t="n">
-        <v>0.4495</v>
+        <v>0.7687</v>
       </c>
       <c r="G178" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.8462</v>
       </c>
       <c r="H178" s="13" t="n">
-        <v>-0.0481</v>
+        <v>-0.0488</v>
       </c>
       <c r="I178" s="13" t="n">
-        <v>-0.1419279603859848</v>
+        <v>-0.09083207401703816</v>
       </c>
       <c r="J178" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K178" s="5" t="inlineStr"/>
+      <c r="K178" s="5" t="inlineStr">
+        <is>
+          <t>price -550 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -9927,42 +9823,38 @@
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>LAC ML</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="E179" s="7" t="n">
-        <v>-550</v>
+        <v>-105</v>
       </c>
       <c r="F179" s="8" t="n">
-        <v>0.7687</v>
+        <v>0.4333</v>
       </c>
       <c r="G179" s="8" t="n">
-        <v>0.8462</v>
+        <v>0.5122</v>
       </c>
       <c r="H179" s="8" t="n">
-        <v>-0.0488</v>
+        <v>-0.0491</v>
       </c>
       <c r="I179" s="8" t="n">
-        <v>-0.09083207401703816</v>
+        <v>-0.1541160480659403</v>
       </c>
       <c r="J179" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K179" s="4" t="inlineStr">
-        <is>
-          <t>price -550 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K179" s="4" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="inlineStr">
@@ -10218,7 +10110,7 @@
       </c>
       <c r="B186" s="5" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C186" s="5" t="inlineStr">
@@ -10228,23 +10120,23 @@
       </c>
       <c r="D186" s="5" t="inlineStr">
         <is>
-          <t>Over 50.5</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E186" s="12" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="F186" s="13" t="n">
-        <v>0.458</v>
+        <v>0.4395</v>
       </c>
       <c r="G186" s="13" t="n">
-        <v>0.5413</v>
+        <v>0.5238</v>
       </c>
       <c r="H186" s="13" t="n">
-        <v>-0.0499</v>
+        <v>-0.0501</v>
       </c>
       <c r="I186" s="13" t="n">
-        <v>-0.1538030612553783</v>
+        <v>-0.1608993713047646</v>
       </c>
       <c r="J186" s="15" t="n">
         <v>0.5</v>
@@ -10386,7 +10278,7 @@
       </c>
       <c r="B190" s="5" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C190" s="5" t="inlineStr">
@@ -10396,23 +10288,23 @@
       </c>
       <c r="D190" s="5" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Over 50.5</t>
         </is>
       </c>
       <c r="E190" s="12" t="n">
-        <v>-110</v>
+        <v>-118</v>
       </c>
       <c r="F190" s="13" t="n">
-        <v>0.437</v>
+        <v>0.453</v>
       </c>
       <c r="G190" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5413</v>
       </c>
       <c r="H190" s="13" t="n">
-        <v>-0.0505</v>
+        <v>-0.0507</v>
       </c>
       <c r="I190" s="13" t="n">
-        <v>-0.1656336429379587</v>
+        <v>-0.1630210952770249</v>
       </c>
       <c r="J190" s="15" t="n">
         <v>0.5</v>
@@ -10591,7 +10483,7 @@
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -10601,23 +10493,23 @@
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>Over 45.5</t>
+          <t>Under 38.5</t>
         </is>
       </c>
       <c r="E195" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F195" s="8" t="n">
-        <v>0.4297</v>
+        <v>0.4186</v>
       </c>
       <c r="G195" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H195" s="8" t="n">
         <v>-0.0515</v>
       </c>
       <c r="I195" s="8" t="n">
-        <v>-0.1797102353978136</v>
+        <v>-0.1828182474138708</v>
       </c>
       <c r="J195" s="10" t="n">
         <v>0.5</v>
@@ -10632,7 +10524,7 @@
       </c>
       <c r="B196" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C196" s="5" t="inlineStr">
@@ -10642,23 +10534,23 @@
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>Under 38.5</t>
+          <t>Over 45.5</t>
         </is>
       </c>
       <c r="E196" s="12" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F196" s="13" t="n">
-        <v>0.4137</v>
+        <v>0.4297</v>
       </c>
       <c r="G196" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H196" s="13" t="n">
-        <v>-0.052</v>
+        <v>-0.0515</v>
       </c>
       <c r="I196" s="13" t="n">
-        <v>-0.1922708059340066</v>
+        <v>-0.1797102353978136</v>
       </c>
       <c r="J196" s="15" t="n">
         <v>0.5</v>
@@ -10673,42 +10565,38 @@
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>SEA @ ARI</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>SEA ML</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="E197" s="7" t="n">
-        <v>-535</v>
+        <v>-110</v>
       </c>
       <c r="F197" s="8" t="n">
-        <v>0.7407</v>
+        <v>0.4297</v>
       </c>
       <c r="G197" s="8" t="n">
-        <v>0.8425</v>
+        <v>0.5238</v>
       </c>
       <c r="H197" s="8" t="n">
-        <v>-0.0524</v>
+        <v>-0.0515</v>
       </c>
       <c r="I197" s="8" t="n">
-        <v>-0.1199405621712683</v>
+        <v>-0.1797155358840928</v>
       </c>
       <c r="J197" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K197" s="4" t="inlineStr">
-        <is>
-          <t>price -535 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K197" s="4" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="inlineStr">
@@ -10718,38 +10606,42 @@
       </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>SEA @ ARI</t>
         </is>
       </c>
       <c r="C198" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D198" s="5" t="inlineStr">
         <is>
-          <t>Over 48.5</t>
+          <t>SEA ML</t>
         </is>
       </c>
       <c r="E198" s="12" t="n">
-        <v>-105</v>
+        <v>-535</v>
       </c>
       <c r="F198" s="13" t="n">
-        <v>0.4089</v>
+        <v>0.7407</v>
       </c>
       <c r="G198" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.8425</v>
       </c>
       <c r="H198" s="13" t="n">
-        <v>-0.0525</v>
+        <v>-0.0524</v>
       </c>
       <c r="I198" s="13" t="n">
-        <v>-0.2016493735659793</v>
+        <v>-0.1199405621712683</v>
       </c>
       <c r="J198" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K198" s="5" t="inlineStr"/>
+      <c r="K198" s="5" t="inlineStr">
+        <is>
+          <t>price -535 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -12346,7 +12238,7 @@
         <v>-3</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>50</v>
+        <v>49.7</v>
       </c>
       <c r="G24" s="11" t="n">
         <v>52.5</v>
@@ -12380,7 +12272,7 @@
         <v>-3</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>40.5</v>
+        <v>40.1</v>
       </c>
       <c r="G25" s="16" t="n">
         <v>42.5</v>
@@ -12788,7 +12680,7 @@
         <v>-1.5</v>
       </c>
       <c r="F37" s="16" t="n">
-        <v>41.8</v>
+        <v>41.6</v>
       </c>
       <c r="G37" s="16" t="n">
         <v>38.5</v>
@@ -12822,7 +12714,7 @@
         <v>-3.5</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>48.6</v>
+        <v>48.4</v>
       </c>
       <c r="G38" s="11" t="n">
         <v>50.5</v>
@@ -12856,7 +12748,7 @@
         <v>-3.5</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G39" s="16" t="n">
         <v>48.5</v>
@@ -58044,16 +57936,16 @@
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>71</v>
+        <v>73.3</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>8.5</v>
+        <v>10.1</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>10.3</v>
+        <v>15</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -58082,16 +57974,16 @@
         </is>
       </c>
       <c r="D6" s="19" t="n">
-        <v>66.59999999999999</v>
+        <v>62.5</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>14.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>32.9</v>
+        <v>22.1</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -58099,11 +57991,11 @@
         </is>
       </c>
       <c r="I6" s="14" t="n">
-        <v>-4.5</v>
+        <v>-1.8</v>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Wind 15 mph (gusts 33)</t>
+          <t>Wind 10 mph (gusts 22)</t>
         </is>
       </c>
     </row>
@@ -58124,20 +58016,20 @@
         </is>
       </c>
       <c r="D7" s="17" t="n">
-        <v>63.6</v>
+        <v>84.2</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>6.6</v>
+        <v>2.5</v>
       </c>
       <c r="F7" s="17" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G7" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="G7" s="17" t="n">
-        <v>19</v>
-      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
@@ -58162,20 +58054,20 @@
         </is>
       </c>
       <c r="D8" s="19" t="n">
-        <v>69.59999999999999</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>8.9</v>
+        <v>11.2</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I8" s="14" t="n">
@@ -58200,20 +58092,20 @@
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>96.2</v>
+        <v>96.7</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>1.6</v>
+        <v>7.5</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>3.1</v>
+        <v>8.9</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
@@ -58221,7 +58113,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>96°F · retractable roof — effect halved</t>
+          <t>97°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -58242,20 +58134,20 @@
         </is>
       </c>
       <c r="D10" s="19" t="n">
-        <v>85.8</v>
+        <v>80</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>3.1</v>
+        <v>0.7</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I10" s="14" t="n">
@@ -58280,20 +58172,20 @@
         </is>
       </c>
       <c r="D11" s="17" t="n">
-        <v>95.8</v>
+        <v>97.2</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>8.699999999999999</v>
+        <v>6.3</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>10.7</v>
+        <v>6.3</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
@@ -58301,7 +58193,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>96°F</t>
+          <t>97°F</t>
         </is>
       </c>
     </row>
@@ -58322,20 +58214,20 @@
         </is>
       </c>
       <c r="D12" s="19" t="n">
-        <v>69.40000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I12" s="14" t="n">
@@ -58364,26 +58256,30 @@
         </is>
       </c>
       <c r="D13" s="17" t="n">
-        <v>75.5</v>
+        <v>94.3</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>6.8</v>
+        <v>5.4</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>8.300000000000001</v>
+        <v>4.9</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>94°F</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -58402,26 +58298,30 @@
         </is>
       </c>
       <c r="D14" s="19" t="n">
-        <v>72.59999999999999</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>7</v>
+        <v>3.6</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>10.1</v>
+        <v>4.9</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="5" t="inlineStr"/>
+        <v>-0.5</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>93°F</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -58440,16 +58340,16 @@
         </is>
       </c>
       <c r="D15" s="17" t="n">
-        <v>78.90000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>9.9</v>
+        <v>7.6</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -58478,20 +58378,20 @@
         </is>
       </c>
       <c r="D16" s="19" t="n">
-        <v>77</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="E16" s="19" t="n">
-        <v>9.800000000000001</v>
+        <v>11.9</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>14.5</v>
+        <v>22.8</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I16" s="14" t="n">
@@ -58520,16 +58420,16 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>90.5</v>
+        <v>86.3</v>
       </c>
       <c r="E17" s="17" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -58562,16 +58462,16 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>77</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>9.199999999999999</v>
+        <v>6.4</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>15.2</v>
+        <v>5.1</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -58600,20 +58500,20 @@
         </is>
       </c>
       <c r="D19" s="17" t="n">
-        <v>73.59999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="E19" s="17" t="n">
-        <v>5.9</v>
+        <v>5.2</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>14.3</v>
+        <v>8.5</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
@@ -58638,16 +58538,16 @@
         </is>
       </c>
       <c r="D20" s="19" t="n">
-        <v>85.8</v>
+        <v>91.8</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>6.5</v>
+        <v>10.2</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>6.5</v>
+        <v>20.4</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
@@ -58655,9 +58555,13 @@
         </is>
       </c>
       <c r="I20" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="5" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Wind 10 mph (gusts 20)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -58675,21 +58579,31 @@
           <t>open</t>
         </is>
       </c>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="17" t="n"/>
+      <c r="D21" s="17" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="F21" s="17" t="n">
+        <v>18.3</v>
+      </c>
       <c r="G21" s="17" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I21" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="4" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Wind 8 mph (gusts 18)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Refresh: 2026-09-04 16:03 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -692,7 +692,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-09-04T12:04:49+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-09-04T16:03:52+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04T12:04:49+00:00</t>
+          <t>2026-09-04T16:03:52+00:00</t>
         </is>
       </c>
     </row>
@@ -3290,33 +3290,33 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>ARI ML</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>-110</v>
+        <v>455</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5703</v>
+        <v>0.2249</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.1802</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0.0379</v>
+        <v>0.0369</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0.08880644497500201</v>
+        <v>0.2463009695348195</v>
       </c>
       <c r="J16" s="15" t="n">
         <v>0.5</v>
@@ -3331,33 +3331,33 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>LAC @ BUF</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>ARI ML</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>455</v>
+        <v>-110</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.2249</v>
+        <v>0.5679</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>0.1802</v>
+        <v>0.5238</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.0369</v>
+        <v>0.0366</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.2463009695348195</v>
+        <v>0.08412334085714346</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>0.5</v>
@@ -3372,33 +3372,33 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>LAC @ BUF</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>ATL ML</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>-110</v>
+        <v>295</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5679</v>
+        <v>0.2961</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.2532</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.0366</v>
+        <v>0.0359</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.08412334085714346</v>
+        <v>0.168143930367591</v>
       </c>
       <c r="J18" s="15" t="n">
         <v>0.5</v>
@@ -3413,33 +3413,33 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>ATL ML</t>
+          <t>ARI +10.5</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>295</v>
+        <v>-110</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.2961</v>
+        <v>0.5661</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0.2532</v>
+        <v>0.5238</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.0359</v>
+        <v>0.0355</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.168143930367591</v>
+        <v>0.08067786799365906</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>0.5</v>
@@ -3454,33 +3454,33 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>ARI +10.5</t>
+          <t>Under 45.5</t>
         </is>
       </c>
       <c r="E20" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5661</v>
+        <v>0.5654</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>0.0355</v>
+        <v>0.0351</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>0.08067786799365906</v>
+        <v>0.07942545928218991</v>
       </c>
       <c r="J20" s="15" t="n">
         <v>0.5</v>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -3505,23 +3505,23 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Under 45.5</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>0.5654</v>
+        <v>0.5517</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>0.0351</v>
+        <v>0.0339</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>0.07942545928218991</v>
+        <v>0.07718308579685929</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>0.5</v>
@@ -3536,33 +3536,33 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>CLE @ JAX</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>CLE ML</t>
         </is>
       </c>
       <c r="E22" s="12" t="n">
-        <v>-105</v>
+        <v>310</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5517</v>
+        <v>0.2825</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.2439</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>0.0339</v>
+        <v>0.0333</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>0.07718308579685929</v>
+        <v>0.1570149247846405</v>
       </c>
       <c r="J22" s="15" t="n">
         <v>0.5</v>
@@ -3577,33 +3577,33 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>CLE @ JAX</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>CLE ML</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>310</v>
+        <v>-110</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0.2825</v>
+        <v>0.5605</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>0.2439</v>
+        <v>0.5238</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>0.0333</v>
+        <v>0.0321</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>0.1570149247846405</v>
+        <v>0.07000736159590726</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>0.5</v>
@@ -5063,23 +5063,23 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>Over 41.5</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
-        <v>-105</v>
+        <v>-115</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>0.5241</v>
+        <v>0.5468</v>
       </c>
       <c r="G59" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.5349</v>
       </c>
       <c r="H59" s="8" t="n">
         <v>0.0118</v>
       </c>
       <c r="I59" s="8" t="n">
-        <v>0.02330691394991258</v>
+        <v>0.02233790964424548</v>
       </c>
       <c r="J59" s="10" t="n">
         <v>0.5</v>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>HOU @ IND</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -5473,23 +5473,23 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>IND ML</t>
+          <t>SF ML</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
-        <v>105</v>
+        <v>170</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>0.4943</v>
+        <v>0.3785</v>
       </c>
       <c r="G69" s="8" t="n">
-        <v>0.4878</v>
+        <v>0.3704</v>
       </c>
       <c r="H69" s="8" t="n">
-        <v>0.0065</v>
+        <v>0.0081</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>0.01320091966647718</v>
+        <v>0.02182433071203271</v>
       </c>
       <c r="J69" s="10" t="n">
         <v>0.5</v>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>NO @ BAL</t>
+          <t>HOU @ IND</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -5514,23 +5514,23 @@
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>NO ML</t>
+          <t>IND ML</t>
         </is>
       </c>
       <c r="E70" s="12" t="n">
-        <v>275</v>
+        <v>105</v>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.2726</v>
+        <v>0.4943</v>
       </c>
       <c r="G70" s="13" t="n">
-        <v>0.2667</v>
+        <v>0.4878</v>
       </c>
       <c r="H70" s="13" t="n">
-        <v>0.0059</v>
+        <v>0.0065</v>
       </c>
       <c r="I70" s="13" t="n">
-        <v>0.02200448599510141</v>
+        <v>0.01320091966647718</v>
       </c>
       <c r="J70" s="15" t="n">
         <v>0.5</v>
@@ -5545,7 +5545,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>LAR @ DEN</t>
+          <t>NO @ BAL</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -5555,23 +5555,23 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>DEN ML</t>
+          <t>NO ML</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
-        <v>130</v>
+        <v>275</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>0.4399</v>
+        <v>0.2726</v>
       </c>
       <c r="G71" s="8" t="n">
-        <v>0.4348</v>
+        <v>0.2667</v>
       </c>
       <c r="H71" s="8" t="n">
-        <v>0.0051</v>
+        <v>0.0059</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>0.0117686138551607</v>
+        <v>0.02200448599510141</v>
       </c>
       <c r="J71" s="10" t="n">
         <v>0.5</v>
@@ -5591,28 +5591,28 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>DEN +3</t>
+          <t>DEN ML</t>
         </is>
       </c>
       <c r="E72" s="12" t="n">
-        <v>-110</v>
+        <v>130</v>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.5283</v>
+        <v>0.4399</v>
       </c>
       <c r="G72" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.4348</v>
       </c>
       <c r="H72" s="13" t="n">
-        <v>0.0045</v>
+        <v>0.0051</v>
       </c>
       <c r="I72" s="13" t="n">
-        <v>0.008042139270503401</v>
+        <v>0.0117686138551607</v>
       </c>
       <c r="J72" s="15" t="n">
         <v>0.5</v>
@@ -5627,33 +5627,33 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>LAR @ DEN</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Over 40.5</t>
+          <t>DEN +3</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>0.5279</v>
+        <v>0.5283</v>
       </c>
       <c r="G73" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>0.0041</v>
+        <v>0.0045</v>
       </c>
       <c r="I73" s="8" t="n">
-        <v>0.007863557846305103</v>
+        <v>0.008042139270503401</v>
       </c>
       <c r="J73" s="10" t="n">
         <v>0.5</v>
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>Over 40.5</t>
         </is>
       </c>
       <c r="E74" s="12" t="n">
@@ -5694,7 +5694,7 @@
         <v>0.0041</v>
       </c>
       <c r="I74" s="13" t="n">
-        <v>0.007849378350001934</v>
+        <v>0.007863557846305103</v>
       </c>
       <c r="J74" s="15" t="n">
         <v>0.5</v>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>TEN @ NYG</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -5735,7 +5735,7 @@
         <v>0.0041</v>
       </c>
       <c r="I75" s="8" t="n">
-        <v>0.007853358450957304</v>
+        <v>0.007849378350001934</v>
       </c>
       <c r="J75" s="10" t="n">
         <v>0.5</v>
@@ -5750,33 +5750,33 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>NO @ BAL</t>
+          <t>TEN @ NYG</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>NO +7.5</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E76" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.5276</v>
+        <v>0.5279</v>
       </c>
       <c r="G76" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H76" s="13" t="n">
-        <v>0.0038</v>
+        <v>0.0041</v>
       </c>
       <c r="I76" s="13" t="n">
-        <v>0.007203208278138695</v>
+        <v>0.007853358450957304</v>
       </c>
       <c r="J76" s="15" t="n">
         <v>0.5</v>
@@ -5791,7 +5791,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>NO @ BAL</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -5801,23 +5801,23 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>MIN +3.5</t>
+          <t>NO +7.5</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>0.5385</v>
+        <v>0.5276</v>
       </c>
       <c r="G77" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H77" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0038</v>
       </c>
       <c r="I77" s="8" t="n">
-        <v>0.006757174293596069</v>
+        <v>0.007203208278138695</v>
       </c>
       <c r="J77" s="10" t="n">
         <v>0.5</v>
@@ -5832,7 +5832,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>CIN @ HOU</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -5842,23 +5842,23 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>CIN +2.5</t>
+          <t>MIN +3.5</t>
         </is>
       </c>
       <c r="E78" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.5273</v>
+        <v>0.5385</v>
       </c>
       <c r="G78" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H78" s="13" t="n">
-        <v>0.0035</v>
+        <v>0.0036</v>
       </c>
       <c r="I78" s="13" t="n">
-        <v>0.006708785315947097</v>
+        <v>0.006757174293596069</v>
       </c>
       <c r="J78" s="15" t="n">
         <v>0.5</v>
@@ -5873,33 +5873,33 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>LV @ NO</t>
+          <t>CIN @ HOU</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>LV ML</t>
+          <t>CIN +2.5</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
-        <v>160</v>
+        <v>-110</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>0.3878</v>
+        <v>0.5273</v>
       </c>
       <c r="G79" s="8" t="n">
-        <v>0.3846</v>
+        <v>0.5238</v>
       </c>
       <c r="H79" s="8" t="n">
-        <v>0.0032</v>
+        <v>0.0035</v>
       </c>
       <c r="I79" s="8" t="n">
-        <v>0.008132684100365828</v>
+        <v>0.006708785315947097</v>
       </c>
       <c r="J79" s="10" t="n">
         <v>0.5</v>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>LV @ NO</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -5924,23 +5924,23 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>SF ML</t>
+          <t>LV ML</t>
         </is>
       </c>
       <c r="E80" s="12" t="n">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.3813</v>
+        <v>0.3878</v>
       </c>
       <c r="G80" s="13" t="n">
-        <v>0.3788</v>
+        <v>0.3846</v>
       </c>
       <c r="H80" s="13" t="n">
-        <v>0.0025</v>
+        <v>0.0032</v>
       </c>
       <c r="I80" s="13" t="n">
-        <v>0.006477081760602688</v>
+        <v>0.008132684100365828</v>
       </c>
       <c r="J80" s="15" t="n">
         <v>0.5</v>
@@ -10793,7 +10793,7 @@
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>BAL @ IND</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
@@ -10803,23 +10803,23 @@
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>LAR ML</t>
+          <t>BAL ML</t>
         </is>
       </c>
       <c r="E199" s="7" t="n">
-        <v>-198</v>
+        <v>-175</v>
       </c>
       <c r="F199" s="8" t="n">
-        <v>0.6187</v>
+        <v>0.5907</v>
       </c>
       <c r="G199" s="8" t="n">
-        <v>0.6644</v>
+        <v>0.6364</v>
       </c>
       <c r="H199" s="8" t="n">
         <v>-0.0374</v>
       </c>
       <c r="I199" s="8" t="n">
-        <v>-0.06817438328922104</v>
+        <v>-0.07108657807518826</v>
       </c>
       <c r="J199" s="10" t="n">
         <v>0.5</v>
@@ -10834,33 +10834,33 @@
       </c>
       <c r="B200" s="5" t="inlineStr">
         <is>
-          <t>BAL @ IND</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C200" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D200" s="5" t="inlineStr">
         <is>
-          <t>BAL ML</t>
+          <t>HOU +1.5</t>
         </is>
       </c>
       <c r="E200" s="12" t="n">
-        <v>-175</v>
+        <v>-115</v>
       </c>
       <c r="F200" s="13" t="n">
-        <v>0.5907</v>
+        <v>0.4884</v>
       </c>
       <c r="G200" s="13" t="n">
-        <v>0.6364</v>
+        <v>0.5349</v>
       </c>
       <c r="H200" s="13" t="n">
-        <v>-0.0374</v>
+        <v>-0.0379</v>
       </c>
       <c r="I200" s="13" t="n">
-        <v>-0.07108657807518826</v>
+        <v>-0.08687127655497162</v>
       </c>
       <c r="J200" s="15" t="n">
         <v>0.5</v>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>MIA @ LV</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
@@ -10885,23 +10885,23 @@
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>HOU +1.5</t>
+          <t>LV -3.5</t>
         </is>
       </c>
       <c r="E201" s="7" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F201" s="8" t="n">
-        <v>0.4884</v>
+        <v>0.4771</v>
       </c>
       <c r="G201" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H201" s="8" t="n">
-        <v>-0.0379</v>
+        <v>-0.038</v>
       </c>
       <c r="I201" s="8" t="n">
-        <v>-0.08687127655497162</v>
+        <v>-0.0891968266958536</v>
       </c>
       <c r="J201" s="10" t="n">
         <v>0.5</v>
@@ -10916,17 +10916,17 @@
       </c>
       <c r="B202" s="5" t="inlineStr">
         <is>
-          <t>MIA @ LV</t>
+          <t>ARI @ SF</t>
         </is>
       </c>
       <c r="C202" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D202" s="5" t="inlineStr">
         <is>
-          <t>LV -3.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E202" s="12" t="n">
@@ -10942,7 +10942,7 @@
         <v>-0.038</v>
       </c>
       <c r="I202" s="13" t="n">
-        <v>-0.0891968266958536</v>
+        <v>-0.08909458047419677</v>
       </c>
       <c r="J202" s="15" t="n">
         <v>0.5</v>
@@ -10957,33 +10957,33 @@
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>ARI @ SF</t>
+          <t>BUF @ HOU</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>HOU ML</t>
         </is>
       </c>
       <c r="E203" s="7" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="F203" s="8" t="n">
-        <v>0.4771</v>
+        <v>0.4578</v>
       </c>
       <c r="G203" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.505</v>
       </c>
       <c r="H203" s="8" t="n">
-        <v>-0.038</v>
+        <v>-0.0382</v>
       </c>
       <c r="I203" s="8" t="n">
-        <v>-0.08909458047419677</v>
+        <v>-0.09247330978967083</v>
       </c>
       <c r="J203" s="10" t="n">
         <v>0.5</v>
@@ -10998,7 +10998,7 @@
       </c>
       <c r="B204" s="5" t="inlineStr">
         <is>
-          <t>BUF @ HOU</t>
+          <t>LAR @ DEN</t>
         </is>
       </c>
       <c r="C204" s="5" t="inlineStr">
@@ -11008,23 +11008,23 @@
       </c>
       <c r="D204" s="5" t="inlineStr">
         <is>
-          <t>HOU ML</t>
+          <t>LAR ML</t>
         </is>
       </c>
       <c r="E204" s="12" t="n">
-        <v>-102</v>
+        <v>-155</v>
       </c>
       <c r="F204" s="13" t="n">
-        <v>0.4578</v>
+        <v>0.5601</v>
       </c>
       <c r="G204" s="13" t="n">
-        <v>0.505</v>
+        <v>0.6078</v>
       </c>
       <c r="H204" s="13" t="n">
-        <v>-0.0382</v>
+        <v>-0.0385</v>
       </c>
       <c r="I204" s="13" t="n">
-        <v>-0.09247330978967083</v>
+        <v>-0.07791861190839194</v>
       </c>
       <c r="J204" s="15" t="n">
         <v>0.5</v>
@@ -11039,7 +11039,7 @@
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>LAR @ DEN</t>
+          <t>NO @ BAL</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
@@ -11049,23 +11049,23 @@
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>LAR ML</t>
+          <t>BAL ML</t>
         </is>
       </c>
       <c r="E205" s="7" t="n">
-        <v>-155</v>
+        <v>-345</v>
       </c>
       <c r="F205" s="8" t="n">
-        <v>0.5601</v>
+        <v>0.7274</v>
       </c>
       <c r="G205" s="8" t="n">
-        <v>0.6078</v>
+        <v>0.7753</v>
       </c>
       <c r="H205" s="8" t="n">
-        <v>-0.0385</v>
+        <v>-0.0386</v>
       </c>
       <c r="I205" s="8" t="n">
-        <v>-0.07791861190839194</v>
+        <v>-0.06126342123169412</v>
       </c>
       <c r="J205" s="10" t="n">
         <v>0.5</v>
@@ -11080,33 +11080,33 @@
       </c>
       <c r="B206" s="5" t="inlineStr">
         <is>
-          <t>NO @ BAL</t>
+          <t>NE @ SEA</t>
         </is>
       </c>
       <c r="C206" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D206" s="5" t="inlineStr">
         <is>
-          <t>BAL ML</t>
+          <t>SEA -3.5</t>
         </is>
       </c>
       <c r="E206" s="12" t="n">
-        <v>-345</v>
+        <v>-105</v>
       </c>
       <c r="F206" s="13" t="n">
-        <v>0.7274</v>
+        <v>0.4638</v>
       </c>
       <c r="G206" s="13" t="n">
-        <v>0.7753</v>
+        <v>0.5122</v>
       </c>
       <c r="H206" s="13" t="n">
-        <v>-0.0386</v>
+        <v>-0.0388</v>
       </c>
       <c r="I206" s="13" t="n">
-        <v>-0.06126342123169412</v>
+        <v>-0.09444881622100182</v>
       </c>
       <c r="J206" s="15" t="n">
         <v>0.5</v>
@@ -11126,28 +11126,28 @@
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>SEA -3.5</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E207" s="7" t="n">
         <v>-105</v>
       </c>
       <c r="F207" s="8" t="n">
-        <v>0.4638</v>
+        <v>0.4632</v>
       </c>
       <c r="G207" s="8" t="n">
         <v>0.5122</v>
       </c>
       <c r="H207" s="8" t="n">
-        <v>-0.0388</v>
+        <v>-0.0391</v>
       </c>
       <c r="I207" s="8" t="n">
-        <v>-0.09444881622100182</v>
+        <v>-0.09558459097835359</v>
       </c>
       <c r="J207" s="10" t="n">
         <v>0.5</v>
@@ -11162,33 +11162,33 @@
       </c>
       <c r="B208" s="5" t="inlineStr">
         <is>
-          <t>NE @ SEA</t>
+          <t>PIT @ NE</t>
         </is>
       </c>
       <c r="C208" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D208" s="5" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>NE -4.5</t>
         </is>
       </c>
       <c r="E208" s="12" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F208" s="13" t="n">
-        <v>0.4632</v>
+        <v>0.475</v>
       </c>
       <c r="G208" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5238</v>
       </c>
       <c r="H208" s="13" t="n">
         <v>-0.0391</v>
       </c>
       <c r="I208" s="13" t="n">
-        <v>-0.09558459097835359</v>
+        <v>-0.09324032529484555</v>
       </c>
       <c r="J208" s="15" t="n">
         <v>0.5</v>
@@ -11203,7 +11203,7 @@
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>PIT @ NE</t>
+          <t>BAL @ IND</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -11213,23 +11213,23 @@
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>NE -4.5</t>
+          <t>BAL -3.5</t>
         </is>
       </c>
       <c r="E209" s="7" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="F209" s="8" t="n">
-        <v>0.475</v>
+        <v>0.47</v>
       </c>
       <c r="G209" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5192</v>
       </c>
       <c r="H209" s="8" t="n">
-        <v>-0.0391</v>
+        <v>-0.0393</v>
       </c>
       <c r="I209" s="8" t="n">
-        <v>-0.09324032529484555</v>
+        <v>-0.09476965213035732</v>
       </c>
       <c r="J209" s="10" t="n">
         <v>0.5</v>
@@ -11244,7 +11244,7 @@
       </c>
       <c r="B210" s="5" t="inlineStr">
         <is>
-          <t>BAL @ IND</t>
+          <t>HOU @ IND</t>
         </is>
       </c>
       <c r="C210" s="5" t="inlineStr">
@@ -11254,23 +11254,23 @@
       </c>
       <c r="D210" s="5" t="inlineStr">
         <is>
-          <t>BAL -3.5</t>
+          <t>HOU -1.5</t>
         </is>
       </c>
       <c r="E210" s="12" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="F210" s="13" t="n">
-        <v>0.47</v>
+        <v>0.474</v>
       </c>
       <c r="G210" s="13" t="n">
-        <v>0.5192</v>
+        <v>0.5238</v>
       </c>
       <c r="H210" s="13" t="n">
-        <v>-0.0393</v>
+        <v>-0.0395</v>
       </c>
       <c r="I210" s="13" t="n">
-        <v>-0.09476965213035732</v>
+        <v>-0.09503182085401807</v>
       </c>
       <c r="J210" s="15" t="n">
         <v>0.5</v>
@@ -11285,7 +11285,7 @@
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>HOU @ IND</t>
+          <t>CLE @ TB</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -11295,23 +11295,23 @@
       </c>
       <c r="D211" s="4" t="inlineStr">
         <is>
-          <t>HOU -1.5</t>
+          <t>TB -6.5</t>
         </is>
       </c>
       <c r="E211" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F211" s="8" t="n">
-        <v>0.474</v>
+        <v>0.4739</v>
       </c>
       <c r="G211" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H211" s="8" t="n">
-        <v>-0.0395</v>
+        <v>-0.0396</v>
       </c>
       <c r="I211" s="8" t="n">
-        <v>-0.09503182085401807</v>
+        <v>-0.09535019443157761</v>
       </c>
       <c r="J211" s="10" t="n">
         <v>0.5</v>
@@ -11326,33 +11326,33 @@
       </c>
       <c r="B212" s="5" t="inlineStr">
         <is>
-          <t>CLE @ TB</t>
+          <t>HOU @ IND</t>
         </is>
       </c>
       <c r="C212" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D212" s="5" t="inlineStr">
         <is>
-          <t>TB -6.5</t>
+          <t>HOU ML</t>
         </is>
       </c>
       <c r="E212" s="12" t="n">
-        <v>-110</v>
+        <v>-125</v>
       </c>
       <c r="F212" s="13" t="n">
-        <v>0.4739</v>
+        <v>0.5057</v>
       </c>
       <c r="G212" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5556</v>
       </c>
       <c r="H212" s="13" t="n">
         <v>-0.0396</v>
       </c>
       <c r="I212" s="13" t="n">
-        <v>-0.09535019443157761</v>
+        <v>-0.08893877100947672</v>
       </c>
       <c r="J212" s="15" t="n">
         <v>0.5</v>
@@ -11367,7 +11367,7 @@
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>HOU @ IND</t>
+          <t>CIN @ HOU</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
@@ -11381,19 +11381,19 @@
         </is>
       </c>
       <c r="E213" s="7" t="n">
-        <v>-125</v>
+        <v>-135</v>
       </c>
       <c r="F213" s="8" t="n">
-        <v>0.5057</v>
+        <v>0.5244</v>
       </c>
       <c r="G213" s="8" t="n">
-        <v>0.5556</v>
+        <v>0.5745</v>
       </c>
       <c r="H213" s="8" t="n">
-        <v>-0.0396</v>
+        <v>-0.0397</v>
       </c>
       <c r="I213" s="8" t="n">
-        <v>-0.08893877100947672</v>
+        <v>-0.08636971580093517</v>
       </c>
       <c r="J213" s="10" t="n">
         <v>0.5</v>
@@ -11408,7 +11408,7 @@
       </c>
       <c r="B214" s="5" t="inlineStr">
         <is>
-          <t>CIN @ HOU</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C214" s="5" t="inlineStr">
@@ -11418,23 +11418,23 @@
       </c>
       <c r="D214" s="5" t="inlineStr">
         <is>
-          <t>HOU ML</t>
+          <t>LAR ML</t>
         </is>
       </c>
       <c r="E214" s="12" t="n">
-        <v>-135</v>
+        <v>-205</v>
       </c>
       <c r="F214" s="13" t="n">
-        <v>0.5244</v>
+        <v>0.6215000000000001</v>
       </c>
       <c r="G214" s="13" t="n">
-        <v>0.5745</v>
+        <v>0.6721</v>
       </c>
       <c r="H214" s="13" t="n">
-        <v>-0.0397</v>
+        <v>-0.04</v>
       </c>
       <c r="I214" s="13" t="n">
-        <v>-0.08636971580093517</v>
+        <v>-0.07471312630180416</v>
       </c>
       <c r="J214" s="15" t="n">
         <v>0.5</v>
@@ -12283,23 +12283,23 @@
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>Under 42.5</t>
+          <t>Under 41.5</t>
         </is>
       </c>
       <c r="E235" s="7" t="n">
-        <v>-115</v>
+        <v>-105</v>
       </c>
       <c r="F235" s="8" t="n">
-        <v>0.4759</v>
+        <v>0.4532</v>
       </c>
       <c r="G235" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.5122</v>
       </c>
       <c r="H235" s="8" t="n">
         <v>-0.0435</v>
       </c>
       <c r="I235" s="8" t="n">
-        <v>-0.1103352527007117</v>
+        <v>-0.115243243404788</v>
       </c>
       <c r="J235" s="10" t="n">
         <v>0.5</v>
@@ -13515,7 +13515,7 @@
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>LV @ LAC</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>Over 42.5</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="E265" s="7" t="n">
@@ -13541,7 +13541,7 @@
         <v>-0.0501</v>
       </c>
       <c r="I265" s="8" t="n">
-        <v>-0.1608993713047646</v>
+        <v>-0.1609164525049981</v>
       </c>
       <c r="J265" s="10" t="n">
         <v>0.5</v>
@@ -13556,7 +13556,7 @@
       </c>
       <c r="B266" s="5" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>LV @ LAC</t>
         </is>
       </c>
       <c r="C266" s="5" t="inlineStr">
@@ -13566,7 +13566,7 @@
       </c>
       <c r="D266" s="5" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>Over 42.5</t>
         </is>
       </c>
       <c r="E266" s="12" t="n">
@@ -13582,7 +13582,7 @@
         <v>-0.0501</v>
       </c>
       <c r="I266" s="13" t="n">
-        <v>-0.1609146747875762</v>
+        <v>-0.1608993713047646</v>
       </c>
       <c r="J266" s="15" t="n">
         <v>0.5</v>
@@ -13597,42 +13597,38 @@
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>GB ML</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="E267" s="7" t="n">
-        <v>-375</v>
+        <v>-110</v>
       </c>
       <c r="F267" s="8" t="n">
-        <v>0.7039</v>
+        <v>0.4395</v>
       </c>
       <c r="G267" s="8" t="n">
-        <v>0.7895</v>
+        <v>0.5238</v>
       </c>
       <c r="H267" s="8" t="n">
-        <v>-0.0503</v>
+        <v>-0.0501</v>
       </c>
       <c r="I267" s="8" t="n">
-        <v>-0.1074901842542813</v>
+        <v>-0.1609146747875762</v>
       </c>
       <c r="J267" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K267" s="4" t="inlineStr">
-        <is>
-          <t>price -375 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K267" s="4" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="5" t="inlineStr">
@@ -13642,7 +13638,7 @@
       </c>
       <c r="B268" s="5" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C268" s="5" t="inlineStr">
@@ -13652,30 +13648,30 @@
       </c>
       <c r="D268" s="5" t="inlineStr">
         <is>
-          <t>LAC ML</t>
+          <t>GB ML</t>
         </is>
       </c>
       <c r="E268" s="12" t="n">
-        <v>-625</v>
+        <v>-375</v>
       </c>
       <c r="F268" s="13" t="n">
-        <v>0.7751</v>
+        <v>0.7039</v>
       </c>
       <c r="G268" s="13" t="n">
-        <v>0.8621</v>
+        <v>0.7895</v>
       </c>
       <c r="H268" s="13" t="n">
-        <v>-0.0505</v>
+        <v>-0.0503</v>
       </c>
       <c r="I268" s="13" t="n">
-        <v>-0.1001349534159808</v>
+        <v>-0.1074901842542813</v>
       </c>
       <c r="J268" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="K268" s="5" t="inlineStr">
         <is>
-          <t>price -625 outside the allowed range</t>
+          <t>price -375 outside the allowed range</t>
         </is>
       </c>
     </row>
@@ -13692,33 +13688,37 @@
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>LAC ML</t>
         </is>
       </c>
       <c r="E269" s="7" t="n">
-        <v>-115</v>
+        <v>-625</v>
       </c>
       <c r="F269" s="8" t="n">
-        <v>0.4483</v>
+        <v>0.7751</v>
       </c>
       <c r="G269" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.8621</v>
       </c>
       <c r="H269" s="8" t="n">
         <v>-0.0505</v>
       </c>
       <c r="I269" s="8" t="n">
-        <v>-0.161926115031351</v>
+        <v>-0.1001349534159808</v>
       </c>
       <c r="J269" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K269" s="4" t="inlineStr"/>
+      <c r="K269" s="4" t="inlineStr">
+        <is>
+          <t>price -625 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="5" t="inlineStr">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B270" s="5" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C270" s="5" t="inlineStr">
@@ -13738,23 +13738,23 @@
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>Over 45.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E270" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F270" s="13" t="n">
-        <v>0.4346</v>
+        <v>0.4483</v>
       </c>
       <c r="G270" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H270" s="13" t="n">
-        <v>-0.0509</v>
+        <v>-0.0505</v>
       </c>
       <c r="I270" s="13" t="n">
-        <v>-0.1703345501912807</v>
+        <v>-0.161926115031351</v>
       </c>
       <c r="J270" s="15" t="n">
         <v>0.5</v>
@@ -13769,33 +13769,33 @@
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>LAC -10.5</t>
+          <t>Over 45.5</t>
         </is>
       </c>
       <c r="E271" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F271" s="8" t="n">
-        <v>0.4339</v>
+        <v>0.4346</v>
       </c>
       <c r="G271" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H271" s="8" t="n">
-        <v>-0.051</v>
+        <v>-0.0509</v>
       </c>
       <c r="I271" s="8" t="n">
-        <v>-0.1715869589027499</v>
+        <v>-0.1703345501912807</v>
       </c>
       <c r="J271" s="10" t="n">
         <v>0.5</v>
@@ -13810,33 +13810,33 @@
       </c>
       <c r="B272" s="5" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C272" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>KC ML</t>
+          <t>LAC -10.5</t>
         </is>
       </c>
       <c r="E272" s="12" t="n">
-        <v>-340</v>
+        <v>-110</v>
       </c>
       <c r="F272" s="13" t="n">
-        <v>0.6817</v>
+        <v>0.4339</v>
       </c>
       <c r="G272" s="13" t="n">
-        <v>0.7727000000000001</v>
+        <v>0.5238</v>
       </c>
       <c r="H272" s="13" t="n">
-        <v>-0.0511</v>
+        <v>-0.051</v>
       </c>
       <c r="I272" s="13" t="n">
-        <v>-0.1168151211383064</v>
+        <v>-0.1715869589027499</v>
       </c>
       <c r="J272" s="15" t="n">
         <v>0.5</v>
@@ -13851,33 +13851,33 @@
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>LAC @ BUF</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>Over 48.5</t>
+          <t>KC ML</t>
         </is>
       </c>
       <c r="E273" s="7" t="n">
-        <v>-110</v>
+        <v>-340</v>
       </c>
       <c r="F273" s="8" t="n">
-        <v>0.4321</v>
+        <v>0.6817</v>
       </c>
       <c r="G273" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.7727000000000001</v>
       </c>
       <c r="H273" s="8" t="n">
-        <v>-0.0512</v>
+        <v>-0.0511</v>
       </c>
       <c r="I273" s="8" t="n">
-        <v>-0.1750324317662343</v>
+        <v>-0.1168151211383064</v>
       </c>
       <c r="J273" s="10" t="n">
         <v>0.5</v>
@@ -13892,7 +13892,7 @@
       </c>
       <c r="B274" s="5" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>LAC @ BUF</t>
         </is>
       </c>
       <c r="C274" s="5" t="inlineStr">
@@ -13902,23 +13902,23 @@
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="E274" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F274" s="13" t="n">
-        <v>0.4297</v>
+        <v>0.4321</v>
       </c>
       <c r="G274" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H274" s="13" t="n">
-        <v>-0.0515</v>
+        <v>-0.0512</v>
       </c>
       <c r="I274" s="13" t="n">
-        <v>-0.1797155358840928</v>
+        <v>-0.1750324317662343</v>
       </c>
       <c r="J274" s="15" t="n">
         <v>0.5</v>
@@ -16252,7 +16252,7 @@
         <v>-3</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>49.7</v>
+        <v>50.1</v>
       </c>
       <c r="G38" s="11" t="n">
         <v>52.5</v>
@@ -16490,10 +16490,10 @@
         <v>-3.5</v>
       </c>
       <c r="F45" s="16" t="n">
-        <v>43.6</v>
+        <v>43.2</v>
       </c>
       <c r="G45" s="16" t="n">
-        <v>42.5</v>
+        <v>41.5</v>
       </c>
       <c r="H45" s="12" t="n"/>
       <c r="I45" s="19" t="n"/>
@@ -21409,10 +21409,10 @@
         <v>48.5</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>-198</v>
+        <v>-205</v>
       </c>
       <c r="K55" s="17" t="n">
         <v>0</v>
@@ -21459,7 +21459,7 @@
         <v>-3.5</v>
       </c>
       <c r="H56" s="16" t="n">
-        <v>42.5</v>
+        <v>41.5</v>
       </c>
       <c r="I56" s="12" t="n">
         <v>154</v>
@@ -51474,7 +51474,7 @@
       </c>
       <c r="B480" s="5" t="inlineStr">
         <is>
-          <t>De'Von Achane</t>
+          <t>Jaylen Wright</t>
         </is>
       </c>
       <c r="C480" s="5" t="inlineStr">
@@ -51494,7 +51494,7 @@
       </c>
       <c r="F480" s="5" t="inlineStr">
         <is>
-          <t>Achane is set to lead a Dolphins backfield in 2026 that will also include Jaylen Wright and Ollie Gordon (ribs), based on Miami's initial 53-man roster.</t>
+          <t>Wright is listed as the Dolphins' No. 2 running back on the team's initial depth chart ahead of Week 1 against the Raiders.</t>
         </is>
       </c>
     </row>
@@ -51506,12 +51506,12 @@
       </c>
       <c r="B481" s="4" t="inlineStr">
         <is>
-          <t>Greg Dulcich</t>
+          <t>Caleb Douglas</t>
         </is>
       </c>
       <c r="C481" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D481" s="4" t="inlineStr">
@@ -51526,7 +51526,7 @@
       </c>
       <c r="F481" s="4" t="inlineStr">
         <is>
-          <t>Dulcich did not record a target across his two preseason games.</t>
+          <t>Douglas is listed as a starting wide receiver on Miami's initial depth chart headed into Week 1 against the Raiders.</t>
         </is>
       </c>
     </row>
@@ -51538,7 +51538,7 @@
       </c>
       <c r="B482" s="5" t="inlineStr">
         <is>
-          <t>Ollie Gordon II</t>
+          <t>De'Von Achane</t>
         </is>
       </c>
       <c r="C482" s="5" t="inlineStr">
@@ -51548,17 +51548,17 @@
       </c>
       <c r="D482" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E482" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F482" s="5" t="inlineStr">
         <is>
-          <t>Gordon (ribs) is practicing in a non-contact jersey Wednesday, Alain Poupart of SI.com reports.</t>
+          <t>Achane is set to lead a Dolphins backfield in 2026 that will also include Jaylen Wright and Ollie Gordon (ribs), based on Miami's initial 53-man roster.</t>
         </is>
       </c>
     </row>
@@ -51570,7 +51570,7 @@
       </c>
       <c r="B483" s="4" t="inlineStr">
         <is>
-          <t>Ben Sims</t>
+          <t>Greg Dulcich</t>
         </is>
       </c>
       <c r="C483" s="4" t="inlineStr">
@@ -51580,17 +51580,17 @@
       </c>
       <c r="D483" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E483" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F483" s="4" t="inlineStr">
         <is>
-          <t>Sims (undisclosed) reverted to the Dolphins' injured reserve Tuesday, per the NFL's transaction log.</t>
+          <t>Dulcich did not record a target across his two preseason games.</t>
         </is>
       </c>
     </row>
@@ -51602,27 +51602,27 @@
       </c>
       <c r="B484" s="5" t="inlineStr">
         <is>
-          <t>Chris Bell</t>
+          <t>Ollie Gordon II</t>
         </is>
       </c>
       <c r="C484" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D484" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E484" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F484" s="5" t="inlineStr">
         <is>
-          <t>Coach Jeff Hafley said Tuesday that Bell is still working on getting into football shape, Joe Schad of The Palm Beach Post reports.</t>
+          <t>Gordon (ribs) is practicing in a non-contact jersey Wednesday, Alain Poupart of SI.com reports.</t>
         </is>
       </c>
     </row>
@@ -51634,27 +51634,27 @@
       </c>
       <c r="B485" s="4" t="inlineStr">
         <is>
-          <t>Kyle McCord</t>
+          <t>Ben Sims</t>
         </is>
       </c>
       <c r="C485" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D485" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E485" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F485" s="4" t="inlineStr">
         <is>
-          <t>Dolphins head coach Jeff Hafley confirmed Tuesday that McCord will begin the season as the team's No. 2 quarterback, Joe Schad of The Palm Beach Post reports.</t>
+          <t>Sims (undisclosed) reverted to the Dolphins' injured reserve Tuesday, per the NFL's transaction log.</t>
         </is>
       </c>
     </row>
@@ -51666,12 +51666,12 @@
       </c>
       <c r="B486" s="5" t="inlineStr">
         <is>
-          <t>Chukwuebuka Godrick</t>
+          <t>Chris Bell</t>
         </is>
       </c>
       <c r="C486" s="5" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D486" s="5" t="inlineStr">
@@ -51686,7 +51686,7 @@
       </c>
       <c r="F486" s="5" t="inlineStr">
         <is>
-          <t>The Dolphins claimed Godrick (ankle) off waivers from the Chiefs on Monday.</t>
+          <t>Coach Jeff Hafley said Tuesday that Bell is still working on getting into football shape, Joe Schad of The Palm Beach Post reports.</t>
         </is>
       </c>
     </row>
@@ -51698,12 +51698,12 @@
       </c>
       <c r="B487" s="4" t="inlineStr">
         <is>
-          <t>Reese Taylor</t>
+          <t>Kyle McCord</t>
         </is>
       </c>
       <c r="C487" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D487" s="4" t="inlineStr">
@@ -51718,7 +51718,7 @@
       </c>
       <c r="F487" s="4" t="inlineStr">
         <is>
-          <t>The Dolphins claimed Taylor (concussion) off waivers from the Broncos on Monday.</t>
+          <t>Dolphins head coach Jeff Hafley confirmed Tuesday that McCord will begin the season as the team's No. 2 quarterback, Joe Schad of The Palm Beach Post reports.</t>
         </is>
       </c>
     </row>
@@ -51730,12 +51730,12 @@
       </c>
       <c r="B488" s="5" t="inlineStr">
         <is>
-          <t>Justin Joly</t>
+          <t>Chukwuebuka Godrick</t>
         </is>
       </c>
       <c r="C488" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D488" s="5" t="inlineStr">
@@ -51750,7 +51750,7 @@
       </c>
       <c r="F488" s="5" t="inlineStr">
         <is>
-          <t>The Dolphins claimed Joly off waivers from the Broncos on Monday.</t>
+          <t>The Dolphins claimed Godrick (ankle) off waivers from the Chiefs on Monday.</t>
         </is>
       </c>
     </row>
@@ -51762,12 +51762,12 @@
       </c>
       <c r="B489" s="4" t="inlineStr">
         <is>
-          <t>Brady Cook</t>
+          <t>Reese Taylor</t>
         </is>
       </c>
       <c r="C489" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D489" s="4" t="inlineStr">
@@ -51782,7 +51782,7 @@
       </c>
       <c r="F489" s="4" t="inlineStr">
         <is>
-          <t>The Dolphins claimed Cook off waivers from the Jets on Monday.</t>
+          <t>The Dolphins claimed Taylor (concussion) off waivers from the Broncos on Monday.</t>
         </is>
       </c>
     </row>
@@ -51794,27 +51794,27 @@
       </c>
       <c r="B490" s="5" t="inlineStr">
         <is>
-          <t>Storm Duck</t>
+          <t>Justin Joly</t>
         </is>
       </c>
       <c r="C490" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D490" s="5" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E490" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F490" s="5" t="inlineStr">
         <is>
-          <t>Duck (knee) was moved to the reserve/PUP list by Miami on Sunday.</t>
+          <t>The Dolphins claimed Joly off waivers from the Broncos on Monday.</t>
         </is>
       </c>
     </row>
@@ -51826,27 +51826,27 @@
       </c>
       <c r="B491" s="4" t="inlineStr">
         <is>
-          <t>Trey Moore</t>
+          <t>Brady Cook</t>
         </is>
       </c>
       <c r="C491" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D491" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E491" s="4" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F491" s="4" t="inlineStr">
         <is>
-          <t>Moore (ankle) was placed on injured reserve by the Dolphins on Sunday with a designation to return.</t>
+          <t>The Dolphins claimed Cook off waivers from the Jets on Monday.</t>
         </is>
       </c>
     </row>
@@ -51858,7 +51858,7 @@
       </c>
       <c r="B492" s="5" t="inlineStr">
         <is>
-          <t>Darrell Baker Jr.</t>
+          <t>Storm Duck</t>
         </is>
       </c>
       <c r="C492" s="5" t="inlineStr">
@@ -51878,7 +51878,7 @@
       </c>
       <c r="F492" s="5" t="inlineStr">
         <is>
-          <t>Baker (undisclosed) was moved to the reserve/PUP list by the Dolphins on Sunday.</t>
+          <t>Duck (knee) was moved to the reserve/PUP list by Miami on Sunday.</t>
         </is>
       </c>
     </row>
@@ -51890,12 +51890,12 @@
       </c>
       <c r="B493" s="4" t="inlineStr">
         <is>
-          <t>Kenneth Grant</t>
+          <t>Trey Moore</t>
         </is>
       </c>
       <c r="C493" s="4" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D493" s="4" t="inlineStr">
@@ -51905,12 +51905,12 @@
       </c>
       <c r="E493" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F493" s="4" t="inlineStr">
         <is>
-          <t>Grant (leg) was placed on injured reserve by the Dolphins on Sunday with a designation to return.</t>
+          <t>Moore (ankle) was placed on injured reserve by the Dolphins on Sunday with a designation to return.</t>
         </is>
       </c>
     </row>
@@ -51922,27 +51922,27 @@
       </c>
       <c r="B494" s="5" t="inlineStr">
         <is>
-          <t>Seydou Traore</t>
+          <t>Darrell Baker Jr.</t>
         </is>
       </c>
       <c r="C494" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D494" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E494" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F494" s="5" t="inlineStr">
         <is>
-          <t>Traore failed to catch his sole target in Friday's preseason finale against the Dolphins.</t>
+          <t>Baker (undisclosed) was moved to the reserve/PUP list by the Dolphins on Sunday.</t>
         </is>
       </c>
     </row>
@@ -51954,17 +51954,17 @@
       </c>
       <c r="B495" s="4" t="inlineStr">
         <is>
-          <t>Will Kacmarek</t>
+          <t>Kenneth Grant</t>
         </is>
       </c>
       <c r="C495" s="4" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D495" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E495" s="4" t="inlineStr">
@@ -51974,7 +51974,7 @@
       </c>
       <c r="F495" s="4" t="inlineStr">
         <is>
-          <t>Kacmarek (undisclosed) is considered week-to-week as of Saturday, Barry Jackson of the Miami Herald reports.</t>
+          <t>Grant (leg) was placed on injured reserve by the Dolphins on Sunday with a designation to return.</t>
         </is>
       </c>
     </row>
@@ -51986,12 +51986,12 @@
       </c>
       <c r="B496" s="5" t="inlineStr">
         <is>
-          <t>Jalen Tolbert</t>
+          <t>Seydou Traore</t>
         </is>
       </c>
       <c r="C496" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D496" s="5" t="inlineStr">
@@ -52006,7 +52006,7 @@
       </c>
       <c r="F496" s="5" t="inlineStr">
         <is>
-          <t>Tolbert caught all three of his targets for 27 yards in Friday's 17-12 preseason loss to the Falcons.</t>
+          <t>Traore failed to catch his sole target in Friday's preseason finale against the Dolphins.</t>
         </is>
       </c>
     </row>
@@ -52018,12 +52018,12 @@
       </c>
       <c r="B497" s="4" t="inlineStr">
         <is>
-          <t>Jacob Rodriguez</t>
+          <t>Will Kacmarek</t>
         </is>
       </c>
       <c r="C497" s="4" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D497" s="4" t="inlineStr">
@@ -52038,7 +52038,7 @@
       </c>
       <c r="F497" s="4" t="inlineStr">
         <is>
-          <t>Rodriguez (undisclosed) is considered day-to-day, Joe Schad of The Palm Beach Post reported Friday.</t>
+          <t>Kacmarek (undisclosed) is considered week-to-week as of Saturday, Barry Jackson of the Miami Herald reports.</t>
         </is>
       </c>
     </row>
@@ -52050,27 +52050,27 @@
       </c>
       <c r="B498" s="5" t="inlineStr">
         <is>
-          <t>Cole Turner</t>
+          <t>Jalen Tolbert</t>
         </is>
       </c>
       <c r="C498" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D498" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E498" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F498" s="5" t="inlineStr">
         <is>
-          <t>Turner (undisclosed) reverted to the Dolphins' injured-reserve list Thursday, Aaron Wilson of KPRC 2 Houston reports.</t>
+          <t>Tolbert caught all three of his targets for 27 yards in Friday's 17-12 preseason loss to the Falcons.</t>
         </is>
       </c>
     </row>
@@ -52082,7 +52082,7 @@
       </c>
       <c r="B499" s="4" t="inlineStr">
         <is>
-          <t>Jordyn Brooks</t>
+          <t>Jacob Rodriguez</t>
         </is>
       </c>
       <c r="C499" s="4" t="inlineStr">
@@ -52092,17 +52092,17 @@
       </c>
       <c r="D499" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E499" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F499" s="4" t="inlineStr">
         <is>
-          <t>Brooks (undisclosed) was a full participant in Wednesday's practice, David Furones of the South Florida Sun Sentinel reports.</t>
+          <t>Rodriguez (undisclosed) is considered day-to-day, Joe Schad of The Palm Beach Post reported Friday.</t>
         </is>
       </c>
     </row>
@@ -52114,27 +52114,27 @@
       </c>
       <c r="B500" s="5" t="inlineStr">
         <is>
-          <t>JuJu Brents</t>
+          <t>Cole Turner</t>
         </is>
       </c>
       <c r="C500" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D500" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E500" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F500" s="5" t="inlineStr">
         <is>
-          <t>Brents (undisclosed) was a full participant in Tuesday's practice. C. Isaiah Smalls II of the Miami Herald reports.</t>
+          <t>Turner (undisclosed) reverted to the Dolphins' injured-reserve list Thursday, Aaron Wilson of KPRC 2 Houston reports.</t>
         </is>
       </c>
     </row>
@@ -52146,12 +52146,12 @@
       </c>
       <c r="B501" s="4" t="inlineStr">
         <is>
-          <t>Ryan Miller</t>
+          <t>Jordyn Brooks</t>
         </is>
       </c>
       <c r="C501" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D501" s="4" t="inlineStr">
@@ -52166,7 +52166,7 @@
       </c>
       <c r="F501" s="4" t="inlineStr">
         <is>
-          <t>The Dolphins claimed Miller off waivers from the Giants on Tuesday, David Furones of the South Florida Sun Sentinel reports.</t>
+          <t>Brooks (undisclosed) was a full participant in Wednesday's practice, David Furones of the South Florida Sun Sentinel reports.</t>
         </is>
       </c>
     </row>
@@ -52178,27 +52178,27 @@
       </c>
       <c r="B502" s="5" t="inlineStr">
         <is>
-          <t>Ronnie Harrison Jr.</t>
+          <t>JuJu Brents</t>
         </is>
       </c>
       <c r="C502" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D502" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E502" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F502" s="5" t="inlineStr">
         <is>
-          <t>Harrison is unlikely to play in the Dolphins' preseason finale against the Falcons on Friday due to a hamstring injury, Joe Schad of The Palm Beach Post reports.</t>
+          <t>Brents (undisclosed) was a full participant in Tuesday's practice. C. Isaiah Smalls II of the Miami Herald reports.</t>
         </is>
       </c>
     </row>
@@ -52210,7 +52210,7 @@
       </c>
       <c r="B503" s="4" t="inlineStr">
         <is>
-          <t>Kevin Coleman Jr.</t>
+          <t>Ryan Miller</t>
         </is>
       </c>
       <c r="C503" s="4" t="inlineStr">
@@ -52230,7 +52230,7 @@
       </c>
       <c r="F503" s="4" t="inlineStr">
         <is>
-          <t>Coleman (undisclosed) caught two of five targets for 32 yards in Saturday's 26-3 preseason loss to the Giants.</t>
+          <t>The Dolphins claimed Miller off waivers from the Giants on Tuesday, David Furones of the South Florida Sun Sentinel reports.</t>
         </is>
       </c>
     </row>
@@ -52242,27 +52242,27 @@
       </c>
       <c r="B504" s="5" t="inlineStr">
         <is>
-          <t>Malik Washington</t>
+          <t>Ronnie Harrison Jr.</t>
         </is>
       </c>
       <c r="C504" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D504" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E504" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F504" s="5" t="inlineStr">
         <is>
-          <t>Washington is not playing in Saturday's preseason game against the Giants, C. Isaiah Smalls II of the Miami Herald reports.</t>
+          <t>Harrison is unlikely to play in the Dolphins' preseason finale against the Falcons on Friday due to a hamstring injury, Joe Schad of The Palm Beach Post reports.</t>
         </is>
       </c>
     </row>
@@ -55454,12 +55454,12 @@
       </c>
       <c r="B605" s="4" t="inlineStr">
         <is>
-          <t>Omar Cooper Jr.</t>
+          <t>Mason Taylor</t>
         </is>
       </c>
       <c r="C605" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D605" s="4" t="inlineStr">
@@ -55474,7 +55474,7 @@
       </c>
       <c r="F605" s="4" t="inlineStr">
         <is>
-          <t>Cooper is listed as a backup wide receiver on the Jets' unofficial depth chart.</t>
+          <t>Taylor is listed as a starting tight end on the Jets' initial depth chart ahead of Week 1 against the Titans.</t>
         </is>
       </c>
     </row>
@@ -55486,12 +55486,12 @@
       </c>
       <c r="B606" s="5" t="inlineStr">
         <is>
-          <t>Geno Smith</t>
+          <t>Adonai Mitchell</t>
         </is>
       </c>
       <c r="C606" s="5" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D606" s="5" t="inlineStr">
@@ -55506,7 +55506,7 @@
       </c>
       <c r="F606" s="5" t="inlineStr">
         <is>
-          <t>Smith was voted a Jets captain by his teammates ahead of the 2026 season, Amanda Vogt and Eric Allen of the team's official site reports.</t>
+          <t>Mitchell is listed as a starting wide receiver on the Jets' initial depth chart ahead of Week 1 against the Titans.</t>
         </is>
       </c>
     </row>
@@ -55518,27 +55518,27 @@
       </c>
       <c r="B607" s="4" t="inlineStr">
         <is>
-          <t>Breece Hall</t>
+          <t>Omar Cooper Jr.</t>
         </is>
       </c>
       <c r="C607" s="4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D607" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E607" s="4" t="inlineStr">
         <is>
-          <t>Strain</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F607" s="4" t="inlineStr">
         <is>
-          <t>Hall (groin) is expected to be ready for Week 1 against the Titans on Sunday, Sept. 13, Jack Bell of the Jets' official site reports.</t>
+          <t>Cooper is listed as a backup wide receiver on the Jets' unofficial depth chart.</t>
         </is>
       </c>
     </row>
@@ -55550,12 +55550,12 @@
       </c>
       <c r="B608" s="5" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Geno Smith</t>
         </is>
       </c>
       <c r="C608" s="5" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D608" s="5" t="inlineStr">
@@ -55570,7 +55570,7 @@
       </c>
       <c r="F608" s="5" t="inlineStr">
         <is>
-          <t>Wilson is set to top a Jets wide receiver depth chart that also includes Adonai Mitchell, Omar Cooper, Isaiah Williams, Tim Patrick and Arian Smith, Randy Lange of the Jets' official site reports.</t>
+          <t>Smith was voted a Jets captain by his teammates ahead of the 2026 season, Amanda Vogt and Eric Allen of the team's official site reports.</t>
         </is>
       </c>
     </row>
@@ -55582,7 +55582,7 @@
       </c>
       <c r="B609" s="4" t="inlineStr">
         <is>
-          <t>Isaiah Davis</t>
+          <t>Breece Hall</t>
         </is>
       </c>
       <c r="C609" s="4" t="inlineStr">
@@ -55597,12 +55597,12 @@
       </c>
       <c r="E609" s="4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Strain</t>
         </is>
       </c>
       <c r="F609" s="4" t="inlineStr">
         <is>
-          <t>Davis (knee) did not participate in Wednesday's practice, Zack Rosenblatt of The Athletic reports.</t>
+          <t>Hall (groin) is expected to be ready for Week 1 against the Titans on Sunday, Sept. 13, Jack Bell of the Jets' official site reports.</t>
         </is>
       </c>
     </row>
@@ -55614,27 +55614,27 @@
       </c>
       <c r="B610" s="5" t="inlineStr">
         <is>
-          <t>Tre Brown</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="C610" s="5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D610" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E610" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F610" s="5" t="inlineStr">
         <is>
-          <t>Brown (undisclosed) was placed on the Jets' injured reserve Sunday, Amanda Vogt and Eric Allen of the team's official site report.</t>
+          <t>Wilson is set to top a Jets wide receiver depth chart that also includes Adonai Mitchell, Omar Cooper, Isaiah Williams, Tim Patrick and Arian Smith, Randy Lange of the Jets' official site reports.</t>
         </is>
       </c>
     </row>
@@ -55646,17 +55646,17 @@
       </c>
       <c r="B611" s="4" t="inlineStr">
         <is>
-          <t>Tyler Baron</t>
+          <t>Isaiah Davis</t>
         </is>
       </c>
       <c r="C611" s="4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D611" s="4" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E611" s="4" t="inlineStr">
@@ -55666,7 +55666,7 @@
       </c>
       <c r="F611" s="4" t="inlineStr">
         <is>
-          <t>The Jets moved Baron (knee) to the reserve/PUP list Sunday, Eric Allen and Amanda Vogt of the team's official site report.</t>
+          <t>Davis (knee) did not participate in Wednesday's practice, Zack Rosenblatt of The Athletic reports.</t>
         </is>
       </c>
     </row>
@@ -55678,27 +55678,27 @@
       </c>
       <c r="B612" s="5" t="inlineStr">
         <is>
-          <t>Trevin Wallace</t>
+          <t>Tre Brown</t>
         </is>
       </c>
       <c r="C612" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D612" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E612" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F612" s="5" t="inlineStr">
         <is>
-          <t>The Jets claimed Wallace off waivers from the Panthers on Monday.</t>
+          <t>Brown (undisclosed) was placed on the Jets' injured reserve Sunday, Amanda Vogt and Eric Allen of the team's official site report.</t>
         </is>
       </c>
     </row>
@@ -55710,27 +55710,27 @@
       </c>
       <c r="B613" s="4" t="inlineStr">
         <is>
-          <t>D'Angelo Ponds</t>
+          <t>Tyler Baron</t>
         </is>
       </c>
       <c r="C613" s="4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D613" s="4" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="E613" s="4" t="inlineStr">
         <is>
-          <t>Strain</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F613" s="4" t="inlineStr">
         <is>
-          <t>Head coach Aaron Glenn said Monday that Ponds (calf) is on track to play against the Titans in Week 1, Zack Rosenblatt of The Athletic reports.</t>
+          <t>The Jets moved Baron (knee) to the reserve/PUP list Sunday, Eric Allen and Amanda Vogt of the team's official site report.</t>
         </is>
       </c>
     </row>
@@ -55742,27 +55742,27 @@
       </c>
       <c r="B614" s="5" t="inlineStr">
         <is>
-          <t>Joseph Ossai</t>
+          <t>Trevin Wallace</t>
         </is>
       </c>
       <c r="C614" s="5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D614" s="5" t="inlineStr">
         <is>
-          <t>Questionable</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E614" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F614" s="5" t="inlineStr">
         <is>
-          <t>Head coach Aaron Glenn told reporters Monday that Ossai is week-to-week due to a plantar fascia injury, Brian Costello of the New York Post reports.</t>
+          <t>The Jets claimed Wallace off waivers from the Panthers on Monday.</t>
         </is>
       </c>
     </row>
@@ -55774,27 +55774,27 @@
       </c>
       <c r="B615" s="4" t="inlineStr">
         <is>
-          <t>Blake Grupe</t>
+          <t>D'Angelo Ponds</t>
         </is>
       </c>
       <c r="C615" s="4" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D615" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E615" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Strain</t>
         </is>
       </c>
       <c r="F615" s="4" t="inlineStr">
         <is>
-          <t>Grupe has a clearer path to the Jets' kicking job after the team released Jason Sanders on Monday, Tom Pelissero of NFL Network reports.</t>
+          <t>Head coach Aaron Glenn said Monday that Ponds (calf) is on track to play against the Titans in Week 1, Zack Rosenblatt of The Athletic reports.</t>
         </is>
       </c>
     </row>
@@ -55806,12 +55806,12 @@
       </c>
       <c r="B616" s="5" t="inlineStr">
         <is>
-          <t>Kenyon Sadiq</t>
+          <t>Joseph Ossai</t>
         </is>
       </c>
       <c r="C616" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D616" s="5" t="inlineStr">
@@ -55821,12 +55821,12 @@
       </c>
       <c r="E616" s="5" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F616" s="5" t="inlineStr">
         <is>
-          <t>Coach Aaron Glenn said Monday that Sadiq (hernia) remains on track to play Week 1 against the Titans, Zack Rosenblatt of The Athletic reports.</t>
+          <t>Head coach Aaron Glenn told reporters Monday that Ossai is week-to-week due to a plantar fascia injury, Brian Costello of the New York Post reports.</t>
         </is>
       </c>
     </row>
@@ -55838,12 +55838,12 @@
       </c>
       <c r="B617" s="4" t="inlineStr">
         <is>
-          <t>Cade Klubnik</t>
+          <t>Blake Grupe</t>
         </is>
       </c>
       <c r="C617" s="4" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D617" s="4" t="inlineStr">
@@ -55858,7 +55858,7 @@
       </c>
       <c r="F617" s="4" t="inlineStr">
         <is>
-          <t>Head coach Aaron Glenn confirmed Monday that Klubnik will open the season as the Jets' No. 2 quarterback behind Geno Smith, Zack Rosenblatt of The Athletic reports.</t>
+          <t>Grupe has a clearer path to the Jets' kicking job after the team released Jason Sanders on Monday, Tom Pelissero of NFL Network reports.</t>
         </is>
       </c>
     </row>
@@ -55870,27 +55870,27 @@
       </c>
       <c r="B618" s="5" t="inlineStr">
         <is>
-          <t>Chip Trayanum</t>
+          <t>Kenyon Sadiq</t>
         </is>
       </c>
       <c r="C618" s="5" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D618" s="5" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Questionable</t>
         </is>
       </c>
       <c r="E618" s="5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="F618" s="5" t="inlineStr">
         <is>
-          <t>Trayanum (neck) was placed on injured reserve by the Jets on Sunday, Eric Allen &amp;amp; Amanda Vogt of the team's official website report.</t>
+          <t>Coach Aaron Glenn said Monday that Sadiq (hernia) remains on track to play Week 1 against the Titans, Zack Rosenblatt of The Athletic reports.</t>
         </is>
       </c>
     </row>
@@ -55902,27 +55902,27 @@
       </c>
       <c r="B619" s="4" t="inlineStr">
         <is>
-          <t>VJ Payne</t>
+          <t>Cade Klubnik</t>
         </is>
       </c>
       <c r="C619" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D619" s="4" t="inlineStr">
         <is>
-          <t>Injured Reserve</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E619" s="4" t="inlineStr">
         <is>
-          <t>Bruise</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F619" s="4" t="inlineStr">
         <is>
-          <t>The Jets placed Payne (undisclosed) on injured reserve Sunday with a designation to return, Al Iannazzone of Newsday reports.</t>
+          <t>Head coach Aaron Glenn confirmed Monday that Klubnik will open the season as the Jets' No. 2 quarterback behind Geno Smith, Zack Rosenblatt of The Athletic reports.</t>
         </is>
       </c>
     </row>
@@ -55934,12 +55934,12 @@
       </c>
       <c r="B620" s="5" t="inlineStr">
         <is>
-          <t>Anez Cooper</t>
+          <t>Chip Trayanum</t>
         </is>
       </c>
       <c r="C620" s="5" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D620" s="5" t="inlineStr">
@@ -55954,7 +55954,7 @@
       </c>
       <c r="F620" s="5" t="inlineStr">
         <is>
-          <t>The Jets placed Cooper (shoulder) on injured reserve Sunday with a designation to return, Al Iannazzone of Newsday reports.</t>
+          <t>Trayanum (neck) was placed on injured reserve by the Jets on Sunday, Eric Allen &amp;amp; Amanda Vogt of the team's official website report.</t>
         </is>
       </c>
     </row>
@@ -55966,27 +55966,27 @@
       </c>
       <c r="B621" s="4" t="inlineStr">
         <is>
-          <t>Jordan Meredith</t>
+          <t>VJ Payne</t>
         </is>
       </c>
       <c r="C621" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D621" s="4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E621" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Bruise</t>
         </is>
       </c>
       <c r="F621" s="4" t="inlineStr">
         <is>
-          <t>The Raiders traded Meredith and a 2029 seventh-round pick to the Jets on Sunday in exchange for a 2027 sixth-round pick, Ian Rapoport of ESPN and NFL Network reports.</t>
+          <t>The Jets placed Payne (undisclosed) on injured reserve Sunday with a designation to return, Al Iannazzone of Newsday reports.</t>
         </is>
       </c>
     </row>
@@ -55998,27 +55998,27 @@
       </c>
       <c r="B622" s="5" t="inlineStr">
         <is>
-          <t>Mason Taylor</t>
+          <t>Anez Cooper</t>
         </is>
       </c>
       <c r="C622" s="5" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D622" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Injured Reserve</t>
         </is>
       </c>
       <c r="E622" s="5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F622" s="5" t="inlineStr">
         <is>
-          <t>Taylor caught his only target for 10 yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>The Jets placed Cooper (shoulder) on injured reserve Sunday with a designation to return, Al Iannazzone of Newsday reports.</t>
         </is>
       </c>
     </row>
@@ -56030,12 +56030,12 @@
       </c>
       <c r="B623" s="4" t="inlineStr">
         <is>
-          <t>Adonai Mitchell</t>
+          <t>Jordan Meredith</t>
         </is>
       </c>
       <c r="C623" s="4" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D623" s="4" t="inlineStr">
@@ -56050,7 +56050,7 @@
       </c>
       <c r="F623" s="4" t="inlineStr">
         <is>
-          <t>Mitchell caught both of his targets for 29 yards in Friday's 17-0 preseason win over the Steelers.</t>
+          <t>The Raiders traded Meredith and a 2029 seventh-round pick to the Jets on Sunday in exchange for a 2027 sixth-round pick, Ian Rapoport of ESPN and NFL Network reports.</t>
         </is>
       </c>
     </row>
@@ -61952,7 +61952,7 @@
         <v>7.3</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>12.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G5" s="17" t="n">
         <v>0</v>
@@ -62028,10 +62028,10 @@
         <v>6.5</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>8.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -62066,10 +62066,10 @@
         <v>3.2</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>12.1</v>
+        <v>6</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -62104,10 +62104,10 @@
         <v>4.3</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -62146,10 +62146,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>9.4</v>
+        <v>12.8</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -62187,7 +62187,7 @@
         <v>5.4</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -62226,10 +62226,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>10.5</v>
+        <v>12.8</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -62268,10 +62268,10 @@
         <v>4.7</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>2.2</v>
+        <v>13.6</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -62306,10 +62306,10 @@
         <v>5.4</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>9.6</v>
+        <v>10.3</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -62344,7 +62344,7 @@
         <v>8.5</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>7.6</v>
+        <v>3.8</v>
       </c>
       <c r="G15" s="17" t="n">
         <v>2</v>
@@ -62382,10 +62382,10 @@
         <v>10.1</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>19.2</v>
+        <v>15.9</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
@@ -62424,10 +62424,10 @@
         <v>0.7</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>11.6</v>
+        <v>6.3</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -62466,10 +62466,10 @@
         <v>6</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>6</v>
+        <v>13.9</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -62504,10 +62504,10 @@
         <v>3.3</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
@@ -62542,10 +62542,10 @@
         <v>7</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>3.1</v>
+        <v>12.8</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
@@ -62580,10 +62580,10 @@
         <v>4.4</v>
       </c>
       <c r="F21" s="17" t="n">
-        <v>21</v>
+        <v>3.6</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
@@ -62591,13 +62591,9 @@
         </is>
       </c>
       <c r="I21" s="9" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Wind 4 mph (gusts 21)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Refresh: 2026-09-09 12:04 UTC
</commit_message>
<xml_diff>
--- a/NFL_Edge_Model.xlsx
+++ b/NFL_Edge_Model.xlsx
@@ -715,7 +715,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot of the live model, generated 2026-09-09T05:13:49+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
+          <t>Snapshot of the live model, generated 2026-09-09T12:04:27+00:00. Read-only: the model runs in the pipeline, not in this file.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09T05:13:49+00:00</t>
+          <t>2026-09-09T12:04:27+00:00</t>
         </is>
       </c>
     </row>
@@ -3196,10 +3196,10 @@
         <v>0.5</v>
       </c>
       <c r="L11" s="11" t="n">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>26</v>
+        <v>25.8</v>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
@@ -3304,10 +3304,10 @@
         <v>0.5</v>
       </c>
       <c r="L13" s="11" t="n">
-        <v>19.5</v>
+        <v>20</v>
       </c>
       <c r="M13" s="11" t="n">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -3387,39 +3387,39 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.5792</v>
+        <v>0.5911</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>0.5283</v>
+        <v>0.5349</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>0.05450581629683715</v>
+        <v>0.05463916282647632</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>0.1485227047392428</v>
+        <v>0.1572043852779952</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>-3.12</v>
+        <v>-3.52</v>
       </c>
       <c r="K15" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="L15" s="11" t="n">
-        <v>21.2</v>
+        <v>22.7</v>
       </c>
       <c r="M15" s="11" t="n">
-        <v>22.2</v>
+        <v>26.3</v>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -3431,49 +3431,49 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>NYG @ LAR</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>NYG ML</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>330</v>
+        <v>-112</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.2557</v>
+        <v>0.5792</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.2326</v>
+        <v>0.5283</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0.05445086370722593</v>
+        <v>0.05450581629683715</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0.1456093189964156</v>
+        <v>0.1485227047392428</v>
       </c>
       <c r="J16" s="14" t="n">
-        <v>-0.98</v>
+        <v>-3.12</v>
       </c>
       <c r="K16" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="L16" s="16" t="n">
-        <v>20</v>
+        <v>21.2</v>
       </c>
       <c r="M16" s="16" t="n">
-        <v>28.6</v>
+        <v>22.2</v>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3485,49 +3485,49 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>LAC @ BUF</t>
+          <t>NYG @ LAR</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>NYG ML</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>-110</v>
+        <v>330</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.5703</v>
+        <v>0.2557</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.2326</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.05434180135727222</v>
+        <v>0.05445086370722593</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.1406000000000001</v>
+        <v>0.1456093189964156</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>-2.76</v>
+        <v>-0.98</v>
       </c>
       <c r="K17" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="L17" s="11" t="n">
-        <v>20.8</v>
+        <v>20</v>
       </c>
       <c r="M17" s="11" t="n">
-        <v>24.9</v>
+        <v>28.6</v>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>WSH @ DAL</t>
+          <t>LAC @ BUF</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3549,39 +3549,39 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5703</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.05388541966622874</v>
+        <v>0.05434180135727222</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.1259999999999999</v>
+        <v>0.1406000000000001</v>
       </c>
       <c r="J18" s="14" t="n">
-        <v>-2.54</v>
+        <v>-2.76</v>
       </c>
       <c r="K18" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="L18" s="16" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="M18" s="16" t="n">
-        <v>27</v>
+        <v>24.9</v>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -3593,45 +3593,45 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>GB @ NYJ</t>
+          <t>WSH @ DAL</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>NYJ ML</t>
+          <t>Under 51.5</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>200</v>
+        <v>-110</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.3593</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0.3333</v>
+        <v>0.5238</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.05384131849131323</v>
+        <v>0.05388541966622874</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.1249217282404509</v>
+        <v>0.1259999999999999</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>1.2</v>
+        <v>-2.54</v>
       </c>
       <c r="K19" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="L19" s="11" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="M19" s="11" t="n">
-        <v>19.8</v>
+        <v>27</v>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
@@ -4320,7 +4320,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -4330,23 +4330,23 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.5792</v>
+        <v>0.5911</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>0.5283</v>
+        <v>0.5349</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>0.05450581629683715</v>
+        <v>0.05463916282647632</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>0.09634285714285729</v>
+        <v>0.1050999999999997</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>0.5</v>
@@ -4361,33 +4361,33 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>NYG @ LAR</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>NYG ML</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>330</v>
+        <v>-112</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.2557</v>
+        <v>0.5792</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.2326</v>
+        <v>0.5283</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0.05445086370722593</v>
+        <v>0.05450581629683715</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0.098763675</v>
+        <v>0.09634285714285729</v>
       </c>
       <c r="J16" s="15" t="n">
         <v>0.5</v>
@@ -4402,33 +4402,33 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>LAC @ BUF</t>
+          <t>NYG @ LAR</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>NYG ML</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>-110</v>
+        <v>330</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.5703</v>
+        <v>0.2557</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.2326</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.05434180135727222</v>
+        <v>0.05445086370722593</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.08875454545454553</v>
+        <v>0.098763675</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>0.5</v>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>WSH @ DAL</t>
+          <t>LAC @ BUF</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -4453,23 +4453,23 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5703</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0.05388541966622874</v>
+        <v>0.05434180135727222</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0.07481818181818167</v>
+        <v>0.08875454545454553</v>
       </c>
       <c r="J18" s="15" t="n">
         <v>0.5</v>
@@ -4484,33 +4484,33 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>GB @ NYJ</t>
+          <t>WSH @ DAL</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>NYJ ML</t>
+          <t>Under 51.5</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>200</v>
+        <v>-110</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.3593</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0.3333</v>
+        <v>0.5238</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.05384131849131323</v>
+        <v>0.05388541966622874</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.07723006000000007</v>
+        <v>0.07481818181818167</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>0.5</v>
@@ -4738,33 +4738,33 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>KC @ MIA</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>MIA +7.5</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>0.5703</v>
+        <v>0.5675</v>
       </c>
       <c r="G25" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>0.05434180135727222</v>
+        <v>0.05419423459842903</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.08875454545454553</v>
+        <v>0.08340909090909099</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>0.5</v>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>KC @ MIA</t>
+          <t>MIA @ SF</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -4793,23 +4793,23 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>MIA +7.5</t>
+          <t>MIA +10.5</t>
         </is>
       </c>
       <c r="E26" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5675</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="G26" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>0.05419423459842903</v>
+        <v>0.05403497763408147</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>0.08340909090909099</v>
+        <v>0.07863636363636362</v>
       </c>
       <c r="J26" s="15" t="n">
         <v>0.5</v>
@@ -4828,40 +4828,40 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>MIA @ SF</t>
+          <t>GB @ NYJ</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>MIA +10.5</t>
+          <t>NYJ ML</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>-110</v>
+        <v>200</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.3593</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.3333</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.05403497763408147</v>
+        <v>0.05384131849131323</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.07863636363636362</v>
+        <v>0.07723006000000007</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>correlated with a stronger play on the same game</t>
+          <t>outside the top 6 plays for this week</t>
         </is>
       </c>
     </row>
@@ -5323,40 +5323,40 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>NYJ @ DET</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>NYJ +9.5</t>
         </is>
       </c>
       <c r="E38" s="12" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5643</v>
+        <v>0.5518999999999999</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H38" s="13" t="n">
-        <v>0.05261332294603881</v>
+        <v>0.05253239825206905</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>0.054995652173913</v>
+        <v>0.05362727272727263</v>
       </c>
       <c r="J38" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>outside the top 6 plays for this week</t>
+          <t>correlated with a stronger play on the same game</t>
         </is>
       </c>
     </row>
@@ -5368,40 +5368,40 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>NYJ @ DET</t>
+          <t>PIT @ NE</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>NYJ +9.5</t>
+          <t>PIT ML</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>-110</v>
+        <v>180</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.5518999999999999</v>
+        <v>0.3774</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.3571</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>0.05253239825206905</v>
+        <v>0.05235991280764523</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>0.05362727272727263</v>
+        <v>0.05622653599999988</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>correlated with a stronger play on the same game</t>
+          <t>outside the top 6 plays for this week</t>
         </is>
       </c>
     </row>
@@ -5413,33 +5413,33 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>PIT @ NE</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>PIT ML</t>
+          <t>Under 45.5</t>
         </is>
       </c>
       <c r="E40" s="12" t="n">
-        <v>180</v>
+        <v>-110</v>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.3774</v>
+        <v>0.5505</v>
       </c>
       <c r="G40" s="13" t="n">
-        <v>0.3571</v>
+        <v>0.5238</v>
       </c>
       <c r="H40" s="13" t="n">
-        <v>0.05235991280764523</v>
+        <v>0.05227446863658342</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>0.05622653599999988</v>
+        <v>0.05095454545454547</v>
       </c>
       <c r="J40" s="15" t="n">
         <v>0.5</v>
@@ -5458,40 +5458,40 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Under 45.5</t>
+          <t>ATL +7.5</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>0.5505</v>
+        <v>0.5502</v>
       </c>
       <c r="G41" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>0.05227446863658342</v>
+        <v>0.05221587067561755</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>0.05095454545454547</v>
+        <v>0.05038181818181831</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>outside the top 6 plays for this week</t>
+          <t>correlated with a stronger play on the same game</t>
         </is>
       </c>
     </row>
@@ -5503,33 +5503,33 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>ATL +7.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="E42" s="12" t="n">
-        <v>-110</v>
+        <v>-118</v>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5502</v>
+        <v>0.569</v>
       </c>
       <c r="G42" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5413</v>
       </c>
       <c r="H42" s="13" t="n">
-        <v>0.05221587067561755</v>
+        <v>0.05214892682315637</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>0.05038181818181831</v>
+        <v>0.05120338983050843</v>
       </c>
       <c r="J42" s="15" t="n">
         <v>0.5</v>
@@ -5548,7 +5548,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -5562,19 +5562,19 @@
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>0.569</v>
+        <v>0.548</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>0.5413</v>
+        <v>0.5238</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>0.05214892682315637</v>
+        <v>0.05174707951799837</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>0.05120338983050843</v>
+        <v>0.04618181818181832</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>0.5</v>
@@ -5593,40 +5593,40 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>CIN @ HOU</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>CIN ML</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E44" s="12" t="n">
-        <v>124</v>
+        <v>-110</v>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4682</v>
+        <v>0.548</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.4464</v>
+        <v>0.5238</v>
       </c>
       <c r="H44" s="13" t="n">
-        <v>0.05153163739781726</v>
+        <v>0.05174707951799837</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>0.04832908800000014</v>
+        <v>0.04618181818181832</v>
       </c>
       <c r="J44" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>outside the top 6 plays for this week</t>
+          <t>correlated with a stronger play on the same game</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>SEA @ WSH</t>
+          <t>CIN @ HOU</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -5648,23 +5648,23 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>WSH ML</t>
+          <t>CIN ML</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>160</v>
+        <v>124</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.4033</v>
+        <v>0.4682</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>0.3846</v>
+        <v>0.4464</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>0.0513406961798495</v>
+        <v>0.05153163739781726</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>0.04815249600000007</v>
+        <v>0.04832908800000014</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>0.5</v>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>PHI @ TEN</t>
+          <t>SEA @ WSH</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -5693,23 +5693,23 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>TEN ML</t>
+          <t>WSH ML</t>
         </is>
       </c>
       <c r="E46" s="12" t="n">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.3612</v>
+        <v>0.4033</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.3448</v>
+        <v>0.3846</v>
       </c>
       <c r="H46" s="13" t="n">
-        <v>0.05115367567576327</v>
+        <v>0.0513406961798495</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>0.04707167199999997</v>
+        <v>0.04815249600000007</v>
       </c>
       <c r="J46" s="15" t="n">
         <v>0.5</v>
@@ -5728,33 +5728,33 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>PHI @ TEN</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Under 50.5</t>
+          <t>TEN ML</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>-112</v>
+        <v>190</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>0.5496</v>
+        <v>0.3612</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>0.5283</v>
+        <v>0.3448</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>0.05095858701859107</v>
+        <v>0.05115367567576327</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>0.04031428571428575</v>
+        <v>0.04707167199999997</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>0.5</v>
@@ -5773,7 +5773,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -5783,28 +5783,32 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>Under 50.5</t>
         </is>
       </c>
       <c r="E48" s="12" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5317</v>
+        <v>0.5496</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5283</v>
       </c>
       <c r="H48" s="13" t="n">
-        <v>0.05051943783381651</v>
+        <v>0.05095858701859107</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>0.03808095238095222</v>
+        <v>0.04031428571428575</v>
       </c>
       <c r="J48" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>outside the top 6 plays for this week</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -5814,42 +5818,38 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>NYG ML</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>136</v>
+        <v>-105</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>0.4419</v>
+        <v>0.5317</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>0.4237</v>
+        <v>0.5122</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>0.05051020400110193</v>
+        <v>0.05051943783381651</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>0.04250233240000014</v>
+        <v>0.03808095238095222</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K49" s="4" t="inlineStr">
-        <is>
-          <t>outside the top 6 plays for this week</t>
-        </is>
-      </c>
+      <c r="K49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -5859,38 +5859,42 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>SF +3.5</t>
+          <t>NYG ML</t>
         </is>
       </c>
       <c r="E50" s="12" t="n">
-        <v>-102</v>
+        <v>136</v>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.5224</v>
+        <v>0.4419</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.505</v>
+        <v>0.4237</v>
       </c>
       <c r="H50" s="13" t="n">
-        <v>0.04977772182806617</v>
+        <v>0.05051020400110193</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>0.03455686274509806</v>
+        <v>0.04250233240000014</v>
       </c>
       <c r="J50" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>outside the top 6 plays for this week</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -5900,33 +5904,33 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>NO ML</t>
+          <t>SF +3.5</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>250</v>
+        <v>-102</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>0.2967</v>
+        <v>0.5224</v>
       </c>
       <c r="G51" s="8" t="n">
-        <v>0.2857</v>
+        <v>0.505</v>
       </c>
       <c r="H51" s="8" t="n">
-        <v>0.04970249508856195</v>
+        <v>0.04977772182806617</v>
       </c>
       <c r="I51" s="8" t="n">
-        <v>0.03814624500000009</v>
+        <v>0.03455686274509806</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>0.5</v>
@@ -5941,33 +5945,33 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>MIN @ TB</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>NO ML</t>
         </is>
       </c>
       <c r="E52" s="12" t="n">
-        <v>-110</v>
+        <v>250</v>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.5405</v>
+        <v>0.2967</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.2857</v>
       </c>
       <c r="H52" s="13" t="n">
-        <v>0.04950530390948723</v>
+        <v>0.04970249508856195</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>0.03186363636363643</v>
+        <v>0.03814624500000009</v>
       </c>
       <c r="J52" s="15" t="n">
         <v>0.5</v>
@@ -5982,7 +5986,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>PHI @ CHI</t>
+          <t>MIN @ TB</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -5992,7 +5996,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>Under 44.5</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
@@ -6023,33 +6027,33 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>CIN @ HOU</t>
+          <t>PHI @ CHI</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>CIN +2.5</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="E54" s="12" t="n">
-        <v>-102</v>
+        <v>-110</v>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.5211</v>
+        <v>0.5405</v>
       </c>
       <c r="G54" s="13" t="n">
-        <v>0.505</v>
+        <v>0.5238</v>
       </c>
       <c r="H54" s="13" t="n">
-        <v>0.0492682888966379</v>
+        <v>0.04950530390948723</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>0.03198235294117646</v>
+        <v>0.03186363636363643</v>
       </c>
       <c r="J54" s="15" t="n">
         <v>0.5</v>
@@ -6064,7 +6068,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>GB @ NYJ</t>
+          <t>CIN @ HOU</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -6074,23 +6078,23 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>NYJ +5.5</t>
+          <t>CIN +2.5</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.5384</v>
+        <v>0.5211</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.505</v>
       </c>
       <c r="H55" s="8" t="n">
-        <v>0.04865097072270827</v>
+        <v>0.0492682888966379</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>0.02785454545454558</v>
+        <v>0.03198235294117646</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>0.5</v>
@@ -6105,33 +6109,33 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>GB @ NYJ</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>NYJ +5.5</t>
         </is>
       </c>
       <c r="E56" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.538</v>
+        <v>0.5384</v>
       </c>
       <c r="G56" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H56" s="13" t="n">
-        <v>0.04847467639497067</v>
+        <v>0.04865097072270827</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>0.02709090909090928</v>
+        <v>0.02785454545454558</v>
       </c>
       <c r="J56" s="15" t="n">
         <v>0.5</v>
@@ -6597,33 +6601,33 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>CAR @ ATL</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>NYG +3</t>
+          <t>Under 44.5</t>
         </is>
       </c>
       <c r="E68" s="12" t="n">
-        <v>-112</v>
+        <v>-118</v>
       </c>
       <c r="F68" s="13" t="n">
-        <v>0.5358000000000001</v>
+        <v>0.5491</v>
       </c>
       <c r="G68" s="13" t="n">
-        <v>0.5283</v>
+        <v>0.5413</v>
       </c>
       <c r="H68" s="13" t="n">
-        <v>0.04471262854418794</v>
+        <v>0.0443002028541872</v>
       </c>
       <c r="I68" s="13" t="n">
-        <v>0.01317948714285712</v>
+        <v>0.01443898305084756</v>
       </c>
       <c r="J68" s="15" t="n">
         <v>0.5</v>
@@ -7212,33 +7216,33 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>CAR @ ATL</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>NYG +3</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
-        <v>-118</v>
+        <v>-115</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>0.5441</v>
+        <v>0.5381</v>
       </c>
       <c r="G83" s="8" t="n">
-        <v>0.5413</v>
+        <v>0.5349</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>0.04039314072988053</v>
+        <v>0.04122068107628927</v>
       </c>
       <c r="I83" s="8" t="n">
-        <v>0.00520169491525424</v>
+        <v>0.005583712173912994</v>
       </c>
       <c r="J83" s="10" t="n">
         <v>0.5</v>
@@ -13382,7 +13386,7 @@
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>CAR @ ATL</t>
+          <t>TEN @ NYG</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -13392,23 +13396,23 @@
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>Under 44.5</t>
         </is>
       </c>
       <c r="E233" s="7" t="n">
-        <v>-102</v>
+        <v>-110</v>
       </c>
       <c r="F233" s="8" t="n">
-        <v>0.4559</v>
+        <v>0.4721</v>
       </c>
       <c r="G233" s="8" t="n">
-        <v>0.505</v>
+        <v>0.5238</v>
       </c>
       <c r="H233" s="8" t="n">
-        <v>-0.0420236908336694</v>
+        <v>-0.04221995376217116</v>
       </c>
       <c r="I233" s="8" t="n">
-        <v>-0.09713921568627437</v>
+        <v>-0.09871818181818171</v>
       </c>
       <c r="J233" s="10" t="n">
         <v>0.5</v>
@@ -13423,33 +13427,33 @@
       </c>
       <c r="B234" s="5" t="inlineStr">
         <is>
-          <t>TEN @ NYG</t>
+          <t>DAL @ NYG</t>
         </is>
       </c>
       <c r="C234" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D234" s="5" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>DAL -3</t>
         </is>
       </c>
       <c r="E234" s="12" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F234" s="13" t="n">
-        <v>0.4721</v>
+        <v>0.4619</v>
       </c>
       <c r="G234" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5122</v>
       </c>
       <c r="H234" s="13" t="n">
-        <v>-0.04221995376217116</v>
+        <v>-0.04222217015748686</v>
       </c>
       <c r="I234" s="13" t="n">
-        <v>-0.09871818181818171</v>
+        <v>-0.09118409809523811</v>
       </c>
       <c r="J234" s="15" t="n">
         <v>0.5</v>
@@ -14005,33 +14009,33 @@
       </c>
       <c r="B248" s="5" t="inlineStr">
         <is>
-          <t>DAL @ NYG</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C248" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D248" s="5" t="inlineStr">
         <is>
-          <t>DAL -3</t>
+          <t>KC ML</t>
         </is>
       </c>
       <c r="E248" s="12" t="n">
-        <v>-108</v>
+        <v>-310</v>
       </c>
       <c r="F248" s="13" t="n">
-        <v>0.4642</v>
+        <v>0.6796</v>
       </c>
       <c r="G248" s="13" t="n">
-        <v>0.5192</v>
+        <v>0.7561</v>
       </c>
       <c r="H248" s="13" t="n">
-        <v>-0.04507426620462187</v>
+        <v>-0.04510947619380558</v>
       </c>
       <c r="I248" s="13" t="n">
-        <v>-0.09841784296296296</v>
+        <v>-0.1003344477419356</v>
       </c>
       <c r="J248" s="15" t="n">
         <v>0.5</v>
@@ -14046,7 +14050,7 @@
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
@@ -14056,23 +14060,23 @@
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>KC ML</t>
+          <t>LAR ML</t>
         </is>
       </c>
       <c r="E249" s="7" t="n">
-        <v>-310</v>
+        <v>-205</v>
       </c>
       <c r="F249" s="8" t="n">
-        <v>0.6796</v>
+        <v>0.6031</v>
       </c>
       <c r="G249" s="8" t="n">
-        <v>0.7561</v>
+        <v>0.6721</v>
       </c>
       <c r="H249" s="8" t="n">
-        <v>-0.04510947619380558</v>
+        <v>-0.04539128544485445</v>
       </c>
       <c r="I249" s="8" t="n">
-        <v>-0.1003344477419356</v>
+        <v>-0.1018010751219513</v>
       </c>
       <c r="J249" s="10" t="n">
         <v>0.5</v>
@@ -14087,33 +14091,33 @@
       </c>
       <c r="B250" s="5" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>CAR @ ATL</t>
         </is>
       </c>
       <c r="C250" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>LAR ML</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E250" s="12" t="n">
-        <v>-205</v>
+        <v>-102</v>
       </c>
       <c r="F250" s="13" t="n">
-        <v>0.6031</v>
+        <v>0.4509</v>
       </c>
       <c r="G250" s="13" t="n">
-        <v>0.6721</v>
+        <v>0.505</v>
       </c>
       <c r="H250" s="13" t="n">
-        <v>-0.04539128544485445</v>
+        <v>-0.04575472955737078</v>
       </c>
       <c r="I250" s="13" t="n">
-        <v>-0.1018010751219513</v>
+        <v>-0.1070411764705882</v>
       </c>
       <c r="J250" s="15" t="n">
         <v>0.5</v>
@@ -14587,33 +14591,33 @@
       </c>
       <c r="B262" s="5" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C262" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D262" s="5" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>CHI ML</t>
         </is>
       </c>
       <c r="E262" s="12" t="n">
-        <v>-110</v>
+        <v>-166</v>
       </c>
       <c r="F262" s="13" t="n">
-        <v>0.462</v>
+        <v>0.5538999999999999</v>
       </c>
       <c r="G262" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.6241</v>
       </c>
       <c r="H262" s="13" t="n">
-        <v>-0.04847467639497064</v>
+        <v>-0.04852305056972005</v>
       </c>
       <c r="I262" s="13" t="n">
-        <v>-0.1179999999999999</v>
+        <v>-0.111413473493976</v>
       </c>
       <c r="J262" s="15" t="n">
         <v>0.5</v>
@@ -14628,33 +14632,33 @@
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>GB @ NYJ</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>CHI ML</t>
+          <t>GB -5.5</t>
         </is>
       </c>
       <c r="E263" s="7" t="n">
-        <v>-166</v>
+        <v>-110</v>
       </c>
       <c r="F263" s="8" t="n">
-        <v>0.5538999999999999</v>
+        <v>0.4616</v>
       </c>
       <c r="G263" s="8" t="n">
-        <v>0.6241</v>
+        <v>0.5238</v>
       </c>
       <c r="H263" s="8" t="n">
-        <v>-0.04852305056972005</v>
+        <v>-0.04865097072270827</v>
       </c>
       <c r="I263" s="8" t="n">
-        <v>-0.111413473493976</v>
+        <v>-0.1187636363636363</v>
       </c>
       <c r="J263" s="10" t="n">
         <v>0.5</v>
@@ -14669,7 +14673,7 @@
       </c>
       <c r="B264" s="5" t="inlineStr">
         <is>
-          <t>GB @ NYJ</t>
+          <t>SF @ LAR</t>
         </is>
       </c>
       <c r="C264" s="5" t="inlineStr">
@@ -14679,23 +14683,23 @@
       </c>
       <c r="D264" s="5" t="inlineStr">
         <is>
-          <t>GB -5.5</t>
+          <t>LAR -3.5</t>
         </is>
       </c>
       <c r="E264" s="12" t="n">
-        <v>-110</v>
+        <v>-118</v>
       </c>
       <c r="F264" s="13" t="n">
-        <v>0.4616</v>
+        <v>0.4776</v>
       </c>
       <c r="G264" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5413</v>
       </c>
       <c r="H264" s="13" t="n">
-        <v>-0.04865097072270827</v>
+        <v>-0.04867769293564531</v>
       </c>
       <c r="I264" s="13" t="n">
-        <v>-0.1187636363636363</v>
+        <v>-0.1176542372881356</v>
       </c>
       <c r="J264" s="15" t="n">
         <v>0.5</v>
@@ -14710,38 +14714,42 @@
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>SF @ LAR</t>
+          <t>SEA @ ARI</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>LAR -3.5</t>
+          <t>SEA ML</t>
         </is>
       </c>
       <c r="E265" s="7" t="n">
-        <v>-118</v>
+        <v>-550</v>
       </c>
       <c r="F265" s="8" t="n">
-        <v>0.4776</v>
+        <v>0.7488</v>
       </c>
       <c r="G265" s="8" t="n">
-        <v>0.5413</v>
+        <v>0.8462</v>
       </c>
       <c r="H265" s="8" t="n">
-        <v>-0.04867769293564531</v>
+        <v>-0.04884795285410824</v>
       </c>
       <c r="I265" s="8" t="n">
-        <v>-0.1176542372881356</v>
+        <v>-0.1141686254545454</v>
       </c>
       <c r="J265" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K265" s="4" t="inlineStr"/>
+      <c r="K265" s="4" t="inlineStr">
+        <is>
+          <t>price -550 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="5" t="inlineStr">
@@ -14751,42 +14759,38 @@
       </c>
       <c r="B266" s="5" t="inlineStr">
         <is>
-          <t>SEA @ ARI</t>
+          <t>MIN @ TB</t>
         </is>
       </c>
       <c r="C266" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D266" s="5" t="inlineStr">
         <is>
-          <t>SEA ML</t>
+          <t>Over 44.5</t>
         </is>
       </c>
       <c r="E266" s="12" t="n">
-        <v>-550</v>
+        <v>-110</v>
       </c>
       <c r="F266" s="13" t="n">
-        <v>0.7488</v>
+        <v>0.4595</v>
       </c>
       <c r="G266" s="13" t="n">
-        <v>0.8462</v>
+        <v>0.5238</v>
       </c>
       <c r="H266" s="13" t="n">
-        <v>-0.04884795285410824</v>
+        <v>-0.04950530390948723</v>
       </c>
       <c r="I266" s="13" t="n">
-        <v>-0.1141686254545454</v>
+        <v>-0.1227727272727271</v>
       </c>
       <c r="J266" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K266" s="5" t="inlineStr">
-        <is>
-          <t>price -550 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K266" s="5" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
@@ -14796,7 +14800,7 @@
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>MIN @ TB</t>
+          <t>PHI @ CHI</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
@@ -14806,7 +14810,7 @@
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E267" s="7" t="n">
@@ -14837,7 +14841,7 @@
       </c>
       <c r="B268" s="5" t="inlineStr">
         <is>
-          <t>PHI @ CHI</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C268" s="5" t="inlineStr">
@@ -14851,19 +14855,19 @@
         </is>
       </c>
       <c r="E268" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F268" s="13" t="n">
-        <v>0.4595</v>
+        <v>0.4683</v>
       </c>
       <c r="G268" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H268" s="13" t="n">
-        <v>-0.04950530390948723</v>
+        <v>-0.04990869908255832</v>
       </c>
       <c r="I268" s="13" t="n">
-        <v>-0.1227727272727271</v>
+        <v>-0.1244826086956522</v>
       </c>
       <c r="J268" s="15" t="n">
         <v>0.5</v>
@@ -14878,33 +14882,33 @@
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>MIN @ TB</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>MIN ML</t>
         </is>
       </c>
       <c r="E269" s="7" t="n">
-        <v>-115</v>
+        <v>105</v>
       </c>
       <c r="F269" s="8" t="n">
-        <v>0.4683</v>
+        <v>0.4274</v>
       </c>
       <c r="G269" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.4878</v>
       </c>
       <c r="H269" s="8" t="n">
-        <v>-0.04990869908255832</v>
+        <v>-0.05034413830606997</v>
       </c>
       <c r="I269" s="8" t="n">
-        <v>-0.1244826086956522</v>
+        <v>-0.1227526790000001</v>
       </c>
       <c r="J269" s="10" t="n">
         <v>0.5</v>
@@ -14919,33 +14923,33 @@
       </c>
       <c r="B270" s="5" t="inlineStr">
         <is>
-          <t>MIN @ TB</t>
+          <t>TB @ CIN</t>
         </is>
       </c>
       <c r="C270" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>MIN ML</t>
+          <t>Over 50.5</t>
         </is>
       </c>
       <c r="E270" s="12" t="n">
-        <v>105</v>
+        <v>-108</v>
       </c>
       <c r="F270" s="13" t="n">
-        <v>0.4274</v>
+        <v>0.4504</v>
       </c>
       <c r="G270" s="13" t="n">
-        <v>0.4878</v>
+        <v>0.5192</v>
       </c>
       <c r="H270" s="13" t="n">
-        <v>-0.05034413830606997</v>
+        <v>-0.05117350119118207</v>
       </c>
       <c r="I270" s="13" t="n">
-        <v>-0.1227526790000001</v>
+        <v>-0.1325629629629629</v>
       </c>
       <c r="J270" s="15" t="n">
         <v>0.5</v>
@@ -14960,7 +14964,7 @@
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>TB @ CIN</t>
+          <t>IND @ KC</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
@@ -14970,23 +14974,23 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Over 50.5</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="E271" s="7" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="F271" s="8" t="n">
-        <v>0.4504</v>
+        <v>0.452</v>
       </c>
       <c r="G271" s="8" t="n">
-        <v>0.5192</v>
+        <v>0.5238</v>
       </c>
       <c r="H271" s="8" t="n">
-        <v>-0.05117350119118207</v>
+        <v>-0.05174707951799836</v>
       </c>
       <c r="I271" s="8" t="n">
-        <v>-0.1325629629629629</v>
+        <v>-0.137090909090909</v>
       </c>
       <c r="J271" s="10" t="n">
         <v>0.5</v>
@@ -15001,42 +15005,38 @@
       </c>
       <c r="B272" s="5" t="inlineStr">
         <is>
-          <t>KC @ MIA</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C272" s="5" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>KC ML</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E272" s="12" t="n">
-        <v>-440</v>
+        <v>-110</v>
       </c>
       <c r="F272" s="13" t="n">
-        <v>0.7047</v>
+        <v>0.452</v>
       </c>
       <c r="G272" s="13" t="n">
-        <v>0.8148</v>
+        <v>0.5238</v>
       </c>
       <c r="H272" s="13" t="n">
-        <v>-0.052046642359507</v>
+        <v>-0.05174707951799836</v>
       </c>
       <c r="I272" s="13" t="n">
-        <v>-0.1340327536363636</v>
+        <v>-0.137090909090909</v>
       </c>
       <c r="J272" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="K272" s="5" t="inlineStr">
-        <is>
-          <t>price -440 outside the allowed range</t>
-        </is>
-      </c>
+      <c r="K272" s="5" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
@@ -15046,38 +15046,42 @@
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>ATL @ GB</t>
+          <t>KC @ MIA</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>GB -7.5</t>
+          <t>KC ML</t>
         </is>
       </c>
       <c r="E273" s="7" t="n">
-        <v>-110</v>
+        <v>-440</v>
       </c>
       <c r="F273" s="8" t="n">
-        <v>0.4498</v>
+        <v>0.7047</v>
       </c>
       <c r="G273" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.8148</v>
       </c>
       <c r="H273" s="8" t="n">
-        <v>-0.05221587067561755</v>
+        <v>-0.052046642359507</v>
       </c>
       <c r="I273" s="8" t="n">
-        <v>-0.1412909090909091</v>
+        <v>-0.1340327536363636</v>
       </c>
       <c r="J273" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K273" s="4" t="inlineStr"/>
+      <c r="K273" s="4" t="inlineStr">
+        <is>
+          <t>price -440 outside the allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="5" t="inlineStr">
@@ -15087,33 +15091,33 @@
       </c>
       <c r="B274" s="5" t="inlineStr">
         <is>
-          <t>MIN @ CHI</t>
+          <t>ATL @ GB</t>
         </is>
       </c>
       <c r="C274" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Over 45.5</t>
+          <t>GB -7.5</t>
         </is>
       </c>
       <c r="E274" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F274" s="13" t="n">
-        <v>0.4495</v>
+        <v>0.4498</v>
       </c>
       <c r="G274" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H274" s="13" t="n">
-        <v>-0.05227446863658342</v>
+        <v>-0.05221587067561755</v>
       </c>
       <c r="I274" s="13" t="n">
-        <v>-0.1418636363636363</v>
+        <v>-0.1412909090909091</v>
       </c>
       <c r="J274" s="15" t="n">
         <v>0.5</v>
@@ -15128,33 +15132,33 @@
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>MIN @ CHI</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>LAC -9.5</t>
+          <t>Over 45.5</t>
         </is>
       </c>
       <c r="E275" s="7" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="F275" s="8" t="n">
-        <v>0.4585</v>
+        <v>0.4495</v>
       </c>
       <c r="G275" s="8" t="n">
-        <v>0.5349</v>
+        <v>0.5238</v>
       </c>
       <c r="H275" s="8" t="n">
-        <v>-0.05240549328665507</v>
+        <v>-0.05227446863658342</v>
       </c>
       <c r="I275" s="8" t="n">
-        <v>-0.142804347826087</v>
+        <v>-0.1418636363636363</v>
       </c>
       <c r="J275" s="10" t="n">
         <v>0.5</v>
@@ -15169,7 +15173,7 @@
       </c>
       <c r="B276" s="5" t="inlineStr">
         <is>
-          <t>NYJ @ DET</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C276" s="5" t="inlineStr">
@@ -15179,23 +15183,23 @@
       </c>
       <c r="D276" s="5" t="inlineStr">
         <is>
-          <t>DET -9.5</t>
+          <t>LAC -9.5</t>
         </is>
       </c>
       <c r="E276" s="12" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F276" s="13" t="n">
-        <v>0.4481</v>
+        <v>0.4585</v>
       </c>
       <c r="G276" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5349</v>
       </c>
       <c r="H276" s="13" t="n">
-        <v>-0.05253239825206905</v>
+        <v>-0.05240549328665507</v>
       </c>
       <c r="I276" s="13" t="n">
-        <v>-0.1445363636363636</v>
+        <v>-0.142804347826087</v>
       </c>
       <c r="J276" s="15" t="n">
         <v>0.5</v>
@@ -15210,7 +15214,7 @@
       </c>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>CHI @ CAR</t>
+          <t>NYJ @ DET</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr">
@@ -15220,23 +15224,23 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>CHI -3</t>
+          <t>DET -9.5</t>
         </is>
       </c>
       <c r="E277" s="7" t="n">
-        <v>-120</v>
+        <v>-110</v>
       </c>
       <c r="F277" s="8" t="n">
-        <v>0.4666</v>
+        <v>0.4481</v>
       </c>
       <c r="G277" s="8" t="n">
-        <v>0.5455</v>
+        <v>0.5238</v>
       </c>
       <c r="H277" s="8" t="n">
-        <v>-0.05268679073332724</v>
+        <v>-0.05253239825206905</v>
       </c>
       <c r="I277" s="8" t="n">
-        <v>-0.1342879766666666</v>
+        <v>-0.1445363636363636</v>
       </c>
       <c r="J277" s="10" t="n">
         <v>0.5</v>
@@ -15251,33 +15255,33 @@
       </c>
       <c r="B278" s="5" t="inlineStr">
         <is>
-          <t>DEN @ KC</t>
+          <t>CHI @ CAR</t>
         </is>
       </c>
       <c r="C278" s="5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D278" s="5" t="inlineStr">
         <is>
-          <t>Over 43.5</t>
+          <t>CHI -3</t>
         </is>
       </c>
       <c r="E278" s="12" t="n">
-        <v>-110</v>
+        <v>-120</v>
       </c>
       <c r="F278" s="13" t="n">
-        <v>0.447</v>
+        <v>0.4666</v>
       </c>
       <c r="G278" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5455</v>
       </c>
       <c r="H278" s="13" t="n">
-        <v>-0.05271818101122103</v>
+        <v>-0.05268679073332724</v>
       </c>
       <c r="I278" s="13" t="n">
-        <v>-0.1466363636363636</v>
+        <v>-0.1342879766666666</v>
       </c>
       <c r="J278" s="15" t="n">
         <v>0.5</v>
@@ -15292,7 +15296,7 @@
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>NO @ BAL</t>
+          <t>DEN @ KC</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
@@ -15302,7 +15306,7 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>Over 43.5</t>
         </is>
       </c>
       <c r="E279" s="7" t="n">
@@ -15333,7 +15337,7 @@
       </c>
       <c r="B280" s="5" t="inlineStr">
         <is>
-          <t>ARI @ LAC</t>
+          <t>NO @ BAL</t>
         </is>
       </c>
       <c r="C280" s="5" t="inlineStr">
@@ -15343,23 +15347,23 @@
       </c>
       <c r="D280" s="5" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E280" s="12" t="n">
-        <v>-102</v>
+        <v>-110</v>
       </c>
       <c r="F280" s="13" t="n">
-        <v>0.431</v>
+        <v>0.447</v>
       </c>
       <c r="G280" s="13" t="n">
-        <v>0.505</v>
+        <v>0.5238</v>
       </c>
       <c r="H280" s="13" t="n">
-        <v>-0.0527918148393489</v>
+        <v>-0.05271818101122103</v>
       </c>
       <c r="I280" s="13" t="n">
-        <v>-0.1464509803921569</v>
+        <v>-0.1466363636363636</v>
       </c>
       <c r="J280" s="15" t="n">
         <v>0.5</v>
@@ -15374,7 +15378,7 @@
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>DET @ BUF</t>
+          <t>ARI @ LAC</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
@@ -15384,23 +15388,23 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="E281" s="7" t="n">
-        <v>-105</v>
+        <v>-102</v>
       </c>
       <c r="F281" s="8" t="n">
-        <v>0.4357</v>
+        <v>0.431</v>
       </c>
       <c r="G281" s="8" t="n">
-        <v>0.5122</v>
+        <v>0.505</v>
       </c>
       <c r="H281" s="8" t="n">
-        <v>-0.0529759501677225</v>
+        <v>-0.0527918148393489</v>
       </c>
       <c r="I281" s="8" t="n">
-        <v>-0.1493476190476191</v>
+        <v>-0.1464509803921569</v>
       </c>
       <c r="J281" s="10" t="n">
         <v>0.5</v>
@@ -15743,7 +15747,7 @@
       </c>
       <c r="B290" s="5" t="inlineStr">
         <is>
-          <t>IND @ KC</t>
+          <t>LAC @ BUF</t>
         </is>
       </c>
       <c r="C290" s="5" t="inlineStr">
@@ -15753,7 +15757,7 @@
       </c>
       <c r="D290" s="5" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="E290" s="12" t="n">
@@ -15784,33 +15788,33 @@
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>LAC @ BUF</t>
+          <t>ARI @ SF</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Over 48.5</t>
+          <t>SF -11.5</t>
         </is>
       </c>
       <c r="E291" s="7" t="n">
         <v>-110</v>
       </c>
       <c r="F291" s="8" t="n">
-        <v>0.4297</v>
+        <v>0.4294</v>
       </c>
       <c r="G291" s="8" t="n">
         <v>0.5238</v>
       </c>
       <c r="H291" s="8" t="n">
-        <v>-0.05434180135727222</v>
+        <v>-0.05435592335124494</v>
       </c>
       <c r="I291" s="8" t="n">
-        <v>-0.1796636363636362</v>
+        <v>-0.1802363636363636</v>
       </c>
       <c r="J291" s="10" t="n">
         <v>0.5</v>
@@ -15825,33 +15829,33 @@
       </c>
       <c r="B292" s="5" t="inlineStr">
         <is>
-          <t>ARI @ SF</t>
+          <t>GB @ MIN</t>
         </is>
       </c>
       <c r="C292" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D292" s="5" t="inlineStr">
         <is>
-          <t>SF -11.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E292" s="12" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="F292" s="13" t="n">
-        <v>0.4294</v>
+        <v>0.4208</v>
       </c>
       <c r="G292" s="13" t="n">
-        <v>0.5238</v>
+        <v>0.5192</v>
       </c>
       <c r="H292" s="13" t="n">
-        <v>-0.05435592335124494</v>
+        <v>-0.05454983723766674</v>
       </c>
       <c r="I292" s="13" t="n">
-        <v>-0.1802363636363636</v>
+        <v>-0.1895703703703703</v>
       </c>
       <c r="J292" s="15" t="n">
         <v>0.5</v>
@@ -15866,33 +15870,33 @@
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>GB @ MIN</t>
+          <t>SEA @ ARI</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>SEA -10</t>
         </is>
       </c>
       <c r="E293" s="7" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="F293" s="8" t="n">
-        <v>0.4208</v>
+        <v>0.4202</v>
       </c>
       <c r="G293" s="8" t="n">
-        <v>0.5192</v>
+        <v>0.5238</v>
       </c>
       <c r="H293" s="8" t="n">
-        <v>-0.05454983723766674</v>
+        <v>-0.05466917575370605</v>
       </c>
       <c r="I293" s="8" t="n">
-        <v>-0.1895703703703703</v>
+        <v>-0.18905724</v>
       </c>
       <c r="J293" s="10" t="n">
         <v>0.5</v>
@@ -15907,33 +15911,33 @@
       </c>
       <c r="B294" s="5" t="inlineStr">
         <is>
-          <t>SEA @ ARI</t>
+          <t>NYJ @ TEN</t>
         </is>
       </c>
       <c r="C294" s="5" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D294" s="5" t="inlineStr">
         <is>
-          <t>SEA -10</t>
+          <t>Under 39.5</t>
         </is>
       </c>
       <c r="E294" s="12" t="n">
         <v>-110</v>
       </c>
       <c r="F294" s="13" t="n">
-        <v>0.4202</v>
+        <v>0.4199</v>
       </c>
       <c r="G294" s="13" t="n">
         <v>0.5238</v>
       </c>
       <c r="H294" s="13" t="n">
-        <v>-0.05466917575370605</v>
+        <v>-0.05467629455430777</v>
       </c>
       <c r="I294" s="13" t="n">
-        <v>-0.18905724</v>
+        <v>-0.1983727272727273</v>
       </c>
       <c r="J294" s="15" t="n">
         <v>0.5</v>
@@ -15948,7 +15952,7 @@
       </c>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>NYJ @ TEN</t>
+          <t>NO @ DET</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr">
@@ -15958,23 +15962,23 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Under 39.5</t>
+          <t>Over 49.5</t>
         </is>
       </c>
       <c r="E295" s="7" t="n">
-        <v>-110</v>
+        <v>-118</v>
       </c>
       <c r="F295" s="8" t="n">
-        <v>0.4199</v>
+        <v>0.4333</v>
       </c>
       <c r="G295" s="8" t="n">
-        <v>0.5238</v>
+        <v>0.5413</v>
       </c>
       <c r="H295" s="8" t="n">
-        <v>-0.05467629455430777</v>
+        <v>-0.05470266581608616</v>
       </c>
       <c r="I295" s="8" t="n">
-        <v>-0.1983727272727273</v>
+        <v>-0.1994966101694915</v>
       </c>
       <c r="J295" s="10" t="n">
         <v>0.5</v>
@@ -15989,7 +15993,7 @@
       </c>
       <c r="B296" s="5" t="inlineStr">
         <is>
-          <t>NO @ DET</t>
+          <t>DET @ BUF</t>
         </is>
       </c>
       <c r="C296" s="5" t="inlineStr">
@@ -15999,23 +16003,23 @@
       </c>
       <c r="D296" s="5" t="inlineStr">
         <is>
-          <t>Over 49.5</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="E296" s="12" t="n">
-        <v>-118</v>
+        <v>-105</v>
       </c>
       <c r="F296" s="13" t="n">
-        <v>0.4333</v>
+        <v>0.4089</v>
       </c>
       <c r="G296" s="13" t="n">
-        <v>0.5413</v>
+        <v>0.5122</v>
       </c>
       <c r="H296" s="13" t="n">
-        <v>-0.05470266581608616</v>
+        <v>-0.05471944969032613</v>
       </c>
       <c r="I296" s="13" t="n">
-        <v>-0.1994966101694915</v>
+        <v>-0.2016714285714286</v>
       </c>
       <c r="J296" s="15" t="n">
         <v>0.5</v>
@@ -17447,7 +17451,7 @@
         <v>-7.5</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>45</v>
+        <v>44.6</v>
       </c>
       <c r="G24" s="11" t="n">
         <v>46.5</v>
@@ -17515,7 +17519,7 @@
         <v>-6.5</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>44.7</v>
+        <v>45.6</v>
       </c>
       <c r="G26" s="11" t="n">
         <v>47.5</v>
@@ -17719,7 +17723,7 @@
         <v>-1.5</v>
       </c>
       <c r="F32" s="11" t="n">
-        <v>43</v>
+        <v>42.8</v>
       </c>
       <c r="G32" s="11" t="n">
         <v>44.5</v>
@@ -17991,7 +17995,7 @@
         <v>-3</v>
       </c>
       <c r="F40" s="11" t="n">
-        <v>50.1</v>
+        <v>49</v>
       </c>
       <c r="G40" s="11" t="n">
         <v>52.5</v>
@@ -19779,7 +19783,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
@@ -19789,10 +19793,10 @@
         <v>1.9</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>-0.31</v>
+        <v>0.88</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>0.12</v>
+        <v>2.38</v>
       </c>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="11" t="n"/>
@@ -19811,7 +19815,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
@@ -19821,10 +19825,10 @@
         <v>1.9</v>
       </c>
       <c r="E12" s="20" t="n">
-        <v>0.88</v>
+        <v>-0.31</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>2.38</v>
+        <v>0.12</v>
       </c>
       <c r="G12" s="5" t="n"/>
       <c r="H12" s="16" t="n"/>
@@ -63683,16 +63687,16 @@
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>76.7</v>
+        <v>75.8</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>7</v>
+        <v>7.6</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -63721,20 +63725,20 @@
         </is>
       </c>
       <c r="D6" s="19" t="n">
-        <v>55.3</v>
+        <v>55.5</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="G6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Partly cloudy</t>
         </is>
       </c>
       <c r="I6" s="14" t="n">
@@ -63759,20 +63763,20 @@
         </is>
       </c>
       <c r="D7" s="17" t="n">
-        <v>79.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
@@ -63797,16 +63801,16 @@
         </is>
       </c>
       <c r="D8" s="19" t="n">
-        <v>84.40000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>5.2</v>
+        <v>2.9</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>7.4</v>
+        <v>4.5</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -63835,20 +63839,20 @@
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>93.7</v>
+        <v>93.2</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>9.1</v>
+        <v>8.1</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>12.3</v>
+        <v>12.8</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I9" s="9" t="n">
@@ -63856,7 +63860,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>94°F · retractable roof — effect halved</t>
+          <t>93°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -63877,20 +63881,20 @@
         </is>
       </c>
       <c r="D10" s="19" t="n">
-        <v>87.09999999999999</v>
+        <v>90.5</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>3.5</v>
+        <v>7.3</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>5.8</v>
+        <v>4.5</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I10" s="14" t="n">
@@ -63915,20 +63919,20 @@
         </is>
       </c>
       <c r="D11" s="17" t="n">
-        <v>96.7</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
@@ -63957,20 +63961,20 @@
         </is>
       </c>
       <c r="D12" s="19" t="n">
-        <v>83.90000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>5.5</v>
+        <v>4.9</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>5.4</v>
+        <v>7.4</v>
       </c>
       <c r="G12" s="19" t="n">
         <v>5</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I12" s="14" t="n">
@@ -63999,16 +64003,16 @@
         </is>
       </c>
       <c r="D13" s="17" t="n">
-        <v>90.59999999999999</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>6.9</v>
+        <v>11</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -64037,20 +64041,20 @@
         </is>
       </c>
       <c r="D14" s="19" t="n">
-        <v>87</v>
+        <v>86.7</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I14" s="14" t="n">
@@ -64075,13 +64079,13 @@
         </is>
       </c>
       <c r="D15" s="17" t="n">
-        <v>76.7</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>8.199999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="G15" s="17" t="n">
         <v>0</v>
@@ -64113,20 +64117,20 @@
         </is>
       </c>
       <c r="D16" s="19" t="n">
-        <v>57.1</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="E16" s="19" t="n">
-        <v>7.2</v>
+        <v>10.3</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>16.8</v>
+        <v>10.1</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Light rain</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I16" s="14" t="n">
@@ -64155,13 +64159,13 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>87.2</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="E17" s="17" t="n">
-        <v>5.4</v>
+        <v>6.7</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>6.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G17" s="17" t="n">
         <v>1</v>
@@ -64197,16 +64201,16 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>69.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>15.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -64235,20 +64239,20 @@
         </is>
       </c>
       <c r="D19" s="17" t="n">
-        <v>66.40000000000001</v>
+        <v>74.8</v>
       </c>
       <c r="E19" s="17" t="n">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Drizzle</t>
+          <t>Light drizzle</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
@@ -64273,20 +64277,20 @@
         </is>
       </c>
       <c r="D20" s="19" t="n">
-        <v>78.5</v>
+        <v>87.8</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>4.2</v>
+        <v>6.7</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>2.2</v>
+        <v>17</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Light drizzle</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I20" s="14" t="n">
@@ -64311,26 +64315,30 @@
         </is>
       </c>
       <c r="D21" s="17" t="n">
-        <v>65.90000000000001</v>
+        <v>56.5</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>3.6</v>
+        <v>6.6</v>
       </c>
       <c r="F21" s="17" t="n">
-        <v>3.1</v>
+        <v>28</v>
       </c>
       <c r="G21" s="17" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I21" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="4" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Wind 7 mph (gusts 28)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -64349,26 +64357,30 @@
         </is>
       </c>
       <c r="D22" s="19" t="n">
-        <v>91.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E22" s="19" t="n">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>3.4</v>
+        <v>10.3</v>
       </c>
       <c r="G22" s="19" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="5" t="inlineStr"/>
+        <v>-0.25</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>97°F · retractable roof — effect halved</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -64387,16 +64399,16 @@
         </is>
       </c>
       <c r="D23" s="17" t="n">
-        <v>92.59999999999999</v>
+        <v>94</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>9.4</v>
+        <v>2.9</v>
       </c>
       <c r="F23" s="17" t="n">
-        <v>9.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
@@ -64408,7 +64420,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>93°F · retractable roof — effect halved</t>
+          <t>94°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -64429,20 +64441,20 @@
         </is>
       </c>
       <c r="D24" s="19" t="n">
-        <v>92.3</v>
+        <v>93</v>
       </c>
       <c r="E24" s="19" t="n">
-        <v>11.9</v>
+        <v>2.6</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>14.1</v>
+        <v>12.3</v>
       </c>
       <c r="G24" s="19" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I24" s="14" t="n">
@@ -64450,7 +64462,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>92°F</t>
+          <t>93°F</t>
         </is>
       </c>
     </row>
@@ -64471,20 +64483,20 @@
         </is>
       </c>
       <c r="D25" s="17" t="n">
-        <v>66.8</v>
+        <v>81</v>
       </c>
       <c r="E25" s="17" t="n">
-        <v>10.1</v>
+        <v>6.7</v>
       </c>
       <c r="F25" s="17" t="n">
-        <v>12.8</v>
+        <v>15</v>
       </c>
       <c r="G25" s="17" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I25" s="9" t="n">
@@ -64509,20 +64521,20 @@
         </is>
       </c>
       <c r="D26" s="19" t="n">
-        <v>67.09999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="E26" s="19" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>4.9</v>
+        <v>8.1</v>
       </c>
       <c r="G26" s="19" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Drizzle</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I26" s="14" t="n">
@@ -64547,20 +64559,20 @@
         </is>
       </c>
       <c r="D27" s="17" t="n">
-        <v>71.3</v>
+        <v>80.7</v>
       </c>
       <c r="E27" s="17" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="F27" s="17" t="n">
-        <v>11.2</v>
+        <v>12.8</v>
       </c>
       <c r="G27" s="17" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I27" s="9" t="n">
@@ -64585,20 +64597,20 @@
         </is>
       </c>
       <c r="D28" s="19" t="n">
-        <v>93.09999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="E28" s="19" t="n">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="F28" s="19" t="n">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="G28" s="19" t="n">
         <v>27</v>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Overcast</t>
         </is>
       </c>
       <c r="I28" s="14" t="n">
@@ -64606,7 +64618,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>93°F</t>
+          <t>96°F</t>
         </is>
       </c>
     </row>
@@ -64627,20 +64639,20 @@
         </is>
       </c>
       <c r="D29" s="17" t="n">
-        <v>65</v>
+        <v>83.2</v>
       </c>
       <c r="E29" s="17" t="n">
-        <v>6.8</v>
+        <v>4.4</v>
       </c>
       <c r="F29" s="17" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G29" s="17" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Overcast</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I29" s="9" t="n">
@@ -64665,20 +64677,20 @@
         </is>
       </c>
       <c r="D30" s="19" t="n">
-        <v>65</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E30" s="19" t="n">
-        <v>6.1</v>
+        <v>3.3</v>
       </c>
       <c r="F30" s="19" t="n">
-        <v>5.8</v>
+        <v>4</v>
       </c>
       <c r="G30" s="19" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Rain showers</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I30" s="14" t="n">
@@ -64703,13 +64715,13 @@
         </is>
       </c>
       <c r="D31" s="17" t="n">
-        <v>75.3</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="E31" s="17" t="n">
-        <v>8.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F31" s="17" t="n">
-        <v>5.1</v>
+        <v>8.5</v>
       </c>
       <c r="G31" s="17" t="n">
         <v>0</v>
@@ -64741,13 +64753,13 @@
         </is>
       </c>
       <c r="D32" s="19" t="n">
-        <v>75.40000000000001</v>
+        <v>81</v>
       </c>
       <c r="E32" s="19" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="F32" s="19" t="n">
-        <v>3.6</v>
+        <v>6.5</v>
       </c>
       <c r="G32" s="19" t="n">
         <v>0</v>
@@ -64779,20 +64791,20 @@
         </is>
       </c>
       <c r="D33" s="17" t="n">
-        <v>96.59999999999999</v>
+        <v>101.1</v>
       </c>
       <c r="E33" s="17" t="n">
-        <v>6.9</v>
+        <v>5</v>
       </c>
       <c r="F33" s="17" t="n">
-        <v>10.1</v>
+        <v>5.8</v>
       </c>
       <c r="G33" s="17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Mainly clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I33" s="9" t="n">
@@ -64800,7 +64812,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>97°F · retractable roof — effect halved</t>
+          <t>101°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -64821,16 +64833,16 @@
         </is>
       </c>
       <c r="D34" s="19" t="n">
-        <v>98.3</v>
+        <v>104</v>
       </c>
       <c r="E34" s="19" t="n">
-        <v>7.7</v>
+        <v>8.6</v>
       </c>
       <c r="F34" s="19" t="n">
-        <v>8.5</v>
+        <v>10.1</v>
       </c>
       <c r="G34" s="19" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
@@ -64842,7 +64854,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>98°F · retractable roof — effect halved</t>
+          <t>104°F · retractable roof — effect halved</t>
         </is>
       </c>
     </row>
@@ -64863,30 +64875,26 @@
         </is>
       </c>
       <c r="D35" s="17" t="n">
-        <v>71</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="E35" s="17" t="n">
-        <v>14.4</v>
+        <v>10</v>
       </c>
       <c r="F35" s="17" t="n">
-        <v>23.3</v>
+        <v>14.8</v>
       </c>
       <c r="G35" s="17" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Partly cloudy</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="I35" s="9" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>Wind 14 mph (gusts 23)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -64905,13 +64913,13 @@
         </is>
       </c>
       <c r="D36" s="19" t="n">
-        <v>73.40000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>10.4</v>
+        <v>11.7</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>6.9</v>
+        <v>4.3</v>
       </c>
       <c r="G36" s="19" t="n">
         <v>0</v>
@@ -64942,21 +64950,31 @@
           <t>open</t>
         </is>
       </c>
-      <c r="D37" s="17" t="n"/>
-      <c r="E37" s="17" t="n"/>
-      <c r="F37" s="17" t="n"/>
+      <c r="D37" s="17" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="E37" s="17" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="F37" s="17" t="n">
+        <v>6.7</v>
+      </c>
       <c r="G37" s="17" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Mainly clear</t>
         </is>
       </c>
       <c r="I37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="4" t="inlineStr"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Wind 15 mph (gusts 7)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">

</xml_diff>